<commit_message>
Update dashboards - 2026-03-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -62,12 +62,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -313,6 +319,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -340,9 +349,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -351,10 +357,10 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -873,7 +879,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+      <c r="A3" s="33" t="inlineStr">
         <is>
           <t>RGDP</t>
         </is>
@@ -1006,16 +1012,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q4" s="37" t="n">
+      <c r="Q4" s="38" t="n">
         <v>0.002268304395076705</v>
       </c>
-      <c r="R4" s="37" t="n">
+      <c r="R4" s="38" t="n">
         <v>0.001143283054144875</v>
       </c>
-      <c r="S4" s="37" t="n">
+      <c r="S4" s="38" t="n">
         <v>0.002340601850973247</v>
       </c>
-      <c r="T4" s="37" t="n">
+      <c r="T4" s="38" t="n">
         <v>0.002931400170945582</v>
       </c>
       <c r="U4" s="23" t="n">
@@ -1023,7 +1029,7 @@
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>NGDP</t>
         </is>
@@ -1033,7 +1039,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
+      <c r="C5" s="48" t="n">
         <v>45931</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1102,13 +1108,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="44" t="n"/>
+      <c r="A6" s="33" t="n"/>
       <c r="B6" s="15" t="inlineStr">
         <is>
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
+      <c r="C6" s="48" t="n">
         <v>45931</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1177,7 +1183,7 @@
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>GDP Nowcast</t>
         </is>
@@ -1200,19 +1206,19 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="F7" s="40" t="n">
+      <c r="F7" s="41" t="n">
         <v>4.2373</v>
       </c>
-      <c r="G7" s="40" t="n">
+      <c r="G7" s="41" t="n">
         <v>3.4728</v>
       </c>
-      <c r="H7" s="40" t="n">
+      <c r="H7" s="41" t="n">
         <v>2.902</v>
       </c>
-      <c r="I7" s="40" t="n">
+      <c r="I7" s="41" t="n">
         <v>-2.7318</v>
       </c>
-      <c r="J7" s="40" t="n">
+      <c r="J7" s="41" t="n">
         <v>2.2711</v>
       </c>
       <c r="K7" s="5" t="n"/>
@@ -1256,7 +1262,7 @@
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
-      <c r="A8" s="44" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Smoothed Recession Prob</t>
         </is>
@@ -1335,7 +1341,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="44" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t>RPCE</t>
         </is>
@@ -1414,7 +1420,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="44" t="n"/>
+      <c r="A10" s="33" t="n"/>
       <c r="B10" s="15" t="inlineStr">
         <is>
           <t>PCECC96</t>
@@ -1489,7 +1495,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="44" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>RPCE Dur</t>
         </is>
@@ -1568,7 +1574,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="44" t="n"/>
+      <c r="A12" s="33" t="n"/>
       <c r="B12" s="15" t="inlineStr">
         <is>
           <t>PCEDGC96</t>
@@ -1643,7 +1649,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="44" t="inlineStr">
+      <c r="A13" s="35" t="inlineStr">
         <is>
           <t>RPCE Ndur</t>
         </is>
@@ -1722,7 +1728,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="44" t="n"/>
+      <c r="A14" s="34" t="n"/>
       <c r="B14" s="15" t="inlineStr">
         <is>
           <t>PCENDC96</t>
@@ -1797,7 +1803,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="44" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>RPCE Serv.</t>
         </is>
@@ -1876,7 +1882,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="44" t="n"/>
+      <c r="A16" s="33" t="n"/>
       <c r="B16" s="15" t="inlineStr">
         <is>
           <t>PCESC96</t>
@@ -1923,7 +1929,7 @@
       <c r="U16" s="21" t="n"/>
     </row>
     <row r="17" ht="16.15" customHeight="1" thickBot="1">
-      <c r="A17" s="44" t="inlineStr">
+      <c r="A17" s="33" t="inlineStr">
         <is>
           <t>Retail Sales</t>
         </is>
@@ -2014,7 +2020,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="44" t="n"/>
+      <c r="A18" s="33" t="n"/>
       <c r="B18" s="15" t="inlineStr">
         <is>
           <t>RSAFS</t>
@@ -2072,16 +2078,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q18" s="37" t="n">
+      <c r="Q18" s="38" t="n">
         <v>0.00170842649932057</v>
       </c>
-      <c r="R18" s="37" t="n">
+      <c r="R18" s="38" t="n">
         <v>0.00297788428704604</v>
       </c>
-      <c r="S18" s="37" t="n">
+      <c r="S18" s="38" t="n">
         <v/>
       </c>
-      <c r="T18" s="37" t="n">
+      <c r="T18" s="38" t="n">
         <v/>
       </c>
       <c r="U18" s="23" t="n">
@@ -2089,7 +2095,7 @@
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
-      <c r="A19" s="44" t="inlineStr">
+      <c r="A19" s="33" t="inlineStr">
         <is>
           <t>Real Disposable Personal Income</t>
         </is>
@@ -2147,16 +2153,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q19" s="37" t="n">
+      <c r="Q19" s="38" t="n">
         <v>0.02391201432150015</v>
       </c>
-      <c r="R19" s="37" t="n">
+      <c r="R19" s="38" t="n">
         <v>0.02653304114557758</v>
       </c>
-      <c r="S19" s="37" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.02696443916493949</v>
       </c>
-      <c r="T19" s="37" t="n">
+      <c r="T19" s="38" t="n">
         <v/>
       </c>
       <c r="U19" s="23" t="n">
@@ -2164,7 +2170,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="44" t="n"/>
+      <c r="A20" s="33" t="n"/>
       <c r="B20" s="15" t="inlineStr">
         <is>
           <t>DSPIC96</t>
@@ -2222,16 +2228,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q20" s="37" t="n">
+      <c r="Q20" s="38" t="n">
         <v>0.002950448142634121</v>
       </c>
-      <c r="R20" s="37" t="n">
+      <c r="R20" s="38" t="n">
         <v>0.002329002576704653</v>
       </c>
-      <c r="S20" s="37" t="n">
+      <c r="S20" s="38" t="n">
         <v/>
       </c>
-      <c r="T20" s="37" t="n">
+      <c r="T20" s="38" t="n">
         <v/>
       </c>
       <c r="U20" s="23" t="n">
@@ -2239,7 +2245,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="44" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t>Personal Saving Rate</t>
         </is>
@@ -2297,16 +2303,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q21" s="37" t="n">
+      <c r="Q21" s="38" t="n">
         <v>0.02512028782828883</v>
       </c>
-      <c r="R21" s="37" t="n">
+      <c r="R21" s="38" t="n">
         <v>0.02646484707309002</v>
       </c>
-      <c r="S21" s="37" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.02599044806094405</v>
       </c>
-      <c r="T21" s="37" t="n">
+      <c r="T21" s="38" t="n">
         <v/>
       </c>
       <c r="U21" s="23" t="n">
@@ -2314,7 +2320,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Vehicle Sales</t>
         </is>
@@ -2376,16 +2382,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q22" s="37" t="n">
+      <c r="Q22" s="38" t="n">
         <v>0.00480699391202144</v>
       </c>
-      <c r="R22" s="37" t="n">
+      <c r="R22" s="38" t="n">
         <v>0.004303799147197918</v>
       </c>
-      <c r="S22" s="37" t="n">
+      <c r="S22" s="38" t="n">
         <v>0.00248632190555953</v>
       </c>
-      <c r="T22" s="37" t="n">
+      <c r="T22" s="38" t="n">
         <v>0.001184731605045064</v>
       </c>
       <c r="U22" s="23" t="n">
@@ -2393,7 +2399,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="44" t="n"/>
+      <c r="A23" s="33" t="n"/>
       <c r="B23" s="15" t="inlineStr">
         <is>
           <t>TOTALSA</t>
@@ -2446,16 +2452,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q23" s="37" t="n">
+      <c r="Q23" s="38" t="n">
         <v>0.02837641493495531</v>
       </c>
-      <c r="R23" s="37" t="n">
+      <c r="R23" s="38" t="n">
         <v>0.02988058645921175</v>
       </c>
-      <c r="S23" s="37" t="n">
+      <c r="S23" s="38" t="n">
         <v>0.02970357876911097</v>
       </c>
-      <c r="T23" s="37" t="n">
+      <c r="T23" s="38" t="n">
         <v>0.02822398731321852</v>
       </c>
       <c r="U23" s="23" t="n">
@@ -2463,7 +2469,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="44" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>Cons Credit - Revolving</t>
         </is>
@@ -2486,19 +2492,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F24" s="37" t="n">
+      <c r="F24" s="38" t="n">
         <v>0.0105318556006937</v>
       </c>
-      <c r="G24" s="37" t="n">
+      <c r="G24" s="38" t="n">
         <v>-0.001281418924231392</v>
       </c>
-      <c r="H24" s="37" t="n">
+      <c r="H24" s="38" t="n">
         <v>0.004454853076971466</v>
       </c>
-      <c r="I24" s="37" t="n">
+      <c r="I24" s="38" t="n">
         <v>0.00339828596255809</v>
       </c>
-      <c r="J24" s="37" t="n">
+      <c r="J24" s="38" t="n">
         <v>-0.003651114145611811</v>
       </c>
       <c r="K24" s="5" t="n"/>
@@ -2525,16 +2531,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q24" s="37" t="n">
+      <c r="Q24" s="38" t="n">
         <v>0.003558357849066329</v>
       </c>
-      <c r="R24" s="37" t="n">
+      <c r="R24" s="38" t="n">
         <v>0.002111370905308885</v>
       </c>
-      <c r="S24" s="37" t="n">
+      <c r="S24" s="38" t="n">
         <v>0.001990205680705293</v>
       </c>
-      <c r="T24" s="37" t="n">
+      <c r="T24" s="38" t="n">
         <v>0.002608155986582039</v>
       </c>
       <c r="U24" s="23" t="n">
@@ -2542,7 +2548,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="44" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t>Cons Credit - NonRevolving</t>
         </is>
@@ -2565,19 +2571,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F25" s="37" t="n">
+      <c r="F25" s="38" t="n">
         <v>0.002704782960157415</v>
       </c>
-      <c r="G25" s="37" t="n">
+      <c r="G25" s="38" t="n">
         <v>0.001696137399219255</v>
       </c>
-      <c r="H25" s="37" t="n">
+      <c r="H25" s="38" t="n">
         <v>0.0009232413445350307</v>
       </c>
-      <c r="I25" s="37" t="n">
+      <c r="I25" s="38" t="n">
         <v>0.001873721239173287</v>
       </c>
-      <c r="J25" s="37" t="n">
+      <c r="J25" s="38" t="n">
         <v>0.001994229089696598</v>
       </c>
       <c r="K25" s="5" t="n"/>
@@ -2600,16 +2606,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q25" s="37" t="n">
+      <c r="Q25" s="38" t="n">
         <v>0.02901287416285929</v>
       </c>
-      <c r="R25" s="37" t="n">
+      <c r="R25" s="38" t="n">
         <v>0.02817782841371343</v>
       </c>
-      <c r="S25" s="37" t="n">
+      <c r="S25" s="38" t="n">
         <v>0.02719006538467721</v>
       </c>
-      <c r="T25" s="37" t="n">
+      <c r="T25" s="38" t="n">
         <v>0.02787442414870654</v>
       </c>
       <c r="U25" s="23" t="n">
@@ -2617,7 +2623,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="44" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t>Gross Priv Fixed Inv Non Res</t>
         </is>
@@ -2640,19 +2646,19 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="F26" s="37" t="n">
+      <c r="F26" s="38" t="n">
         <v>0.009152775755367104</v>
       </c>
-      <c r="G26" s="37" t="n">
+      <c r="G26" s="38" t="n">
         <v>0.007794617579222285</v>
       </c>
-      <c r="H26" s="37" t="n">
+      <c r="H26" s="38" t="n">
         <v>0.01778138610314484</v>
       </c>
-      <c r="I26" s="37" t="n">
+      <c r="I26" s="38" t="n">
         <v>0.02303791460563676</v>
       </c>
-      <c r="J26" s="37" t="n">
+      <c r="J26" s="38" t="n">
         <v>-0.009359213919614473</v>
       </c>
       <c r="K26" s="5" t="n"/>
@@ -2679,16 +2685,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q26" s="37" t="n">
+      <c r="Q26" s="38" t="n">
         <v>0.003553916761463993</v>
       </c>
-      <c r="R26" s="37" t="n">
+      <c r="R26" s="38" t="n">
         <v>0.001673844026027105</v>
       </c>
-      <c r="S26" s="37" t="n">
+      <c r="S26" s="38" t="n">
         <v>0.002347306898561774</v>
       </c>
-      <c r="T26" s="37" t="n">
+      <c r="T26" s="38" t="n">
         <v>0.001894029073346237</v>
       </c>
       <c r="U26" s="23" t="n">
@@ -2696,7 +2702,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="44" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>Gross Priv Fixed Inv Res</t>
         </is>
@@ -2719,19 +2725,19 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="F27" s="37" t="n">
+      <c r="F27" s="38" t="n">
         <v>-0.003824604651284313</v>
       </c>
-      <c r="G27" s="37" t="n">
+      <c r="G27" s="38" t="n">
         <v>-0.01832684674964358</v>
       </c>
-      <c r="H27" s="37" t="n">
+      <c r="H27" s="38" t="n">
         <v>-0.01299350008050415</v>
       </c>
-      <c r="I27" s="37" t="n">
+      <c r="I27" s="38" t="n">
         <v>-0.002410568051752549</v>
       </c>
-      <c r="J27" s="37" t="n">
+      <c r="J27" s="38" t="n">
         <v>0.01049622222903812</v>
       </c>
       <c r="K27" s="5" t="n"/>
@@ -2754,16 +2760,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q27" s="37" t="n">
+      <c r="Q27" s="38" t="n">
         <v>0.02996875905826282</v>
       </c>
-      <c r="R27" s="37" t="n">
+      <c r="R27" s="38" t="n">
         <v>0.02825865991190849</v>
       </c>
-      <c r="S27" s="37" t="n">
+      <c r="S27" s="38" t="n">
         <v>0.02761806318237614</v>
       </c>
-      <c r="T27" s="37" t="n">
+      <c r="T27" s="38" t="n">
         <v>0.02825069249833962</v>
       </c>
       <c r="U27" s="23" t="n">
@@ -2771,7 +2777,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="44" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>Dur. Order</t>
         </is>
@@ -2850,7 +2856,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="44" t="n"/>
+      <c r="A29" s="33" t="n"/>
       <c r="B29" s="15" t="inlineStr">
         <is>
           <t>DGORDER</t>
@@ -2925,7 +2931,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="44" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>Dur Orders Non Def x Aicraft</t>
         </is>
@@ -3004,7 +3010,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="44" t="n"/>
+      <c r="A31" s="33" t="n"/>
       <c r="B31" s="15" t="inlineStr">
         <is>
           <t>ADXDNO</t>
@@ -3062,16 +3068,16 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="Q31" s="37" t="n">
+      <c r="Q31" s="38" t="n">
         <v>0.007310493043885868</v>
       </c>
-      <c r="R31" s="37" t="n">
+      <c r="R31" s="38" t="n">
         <v>0.007996957929548465</v>
       </c>
-      <c r="S31" s="37" t="n">
+      <c r="S31" s="38" t="n">
         <v>0.01027939464493599</v>
       </c>
-      <c r="T31" s="37" t="n">
+      <c r="T31" s="38" t="n">
         <v>0.007624633431085215</v>
       </c>
       <c r="U31" s="23" t="n">
@@ -3079,7 +3085,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="44" t="inlineStr">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
@@ -3137,16 +3143,16 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="Q32" s="37" t="n">
+      <c r="Q32" s="38" t="n">
         <v>0.03362463343108507</v>
       </c>
-      <c r="R32" s="37" t="n">
+      <c r="R32" s="38" t="n">
         <v>0.03584369449378332</v>
       </c>
-      <c r="S32" s="37" t="n">
+      <c r="S32" s="38" t="n">
         <v>0.03559665871121723</v>
       </c>
-      <c r="T32" s="37" t="n">
+      <c r="T32" s="38" t="n">
         <v>0.03369434416365838</v>
       </c>
       <c r="U32" s="23" t="n">
@@ -3154,7 +3160,7 @@
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
-      <c r="A33" s="44" t="n"/>
+      <c r="A33" s="33" t="n"/>
       <c r="B33" s="15" t="inlineStr">
         <is>
           <t>INDPRO</t>
@@ -3212,16 +3218,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q33" s="37" t="n">
+      <c r="Q33" s="38" t="n">
         <v>0.004051863857374327</v>
       </c>
-      <c r="R33" s="37" t="n">
+      <c r="R33" s="38" t="n">
         <v>0.000540540540540535</v>
       </c>
-      <c r="S33" s="37" t="n">
+      <c r="S33" s="38" t="n">
         <v>0.00407055630936215</v>
       </c>
-      <c r="T33" s="37" t="n">
+      <c r="T33" s="38" t="n">
         <v>0.004087193460490468</v>
       </c>
       <c r="U33" s="23" t="n">
@@ -3229,7 +3235,7 @@
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
-      <c r="A34" s="44" t="inlineStr">
+      <c r="A34" s="33" t="inlineStr">
         <is>
           <t>Cap Util</t>
         </is>
@@ -3287,16 +3293,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q34" s="37" t="n">
+      <c r="Q34" s="38" t="n">
         <v>0.008019789135629696</v>
       </c>
-      <c r="R34" s="37" t="n">
+      <c r="R34" s="38" t="n">
         <v>0.01084249628307491</v>
       </c>
-      <c r="S34" s="37" t="n">
+      <c r="S34" s="38" t="n">
         <v>0.01169114908209064</v>
       </c>
-      <c r="T34" s="37" t="n">
+      <c r="T34" s="38" t="n">
         <v>0.01032118383222275</v>
       </c>
       <c r="U34" s="23" t="n">
@@ -3304,7 +3310,7 @@
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
-      <c r="A35" s="44" t="inlineStr">
+      <c r="A35" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Productivity </t>
         </is>
@@ -3327,19 +3333,19 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="F35" s="40" t="n">
+      <c r="F35" s="41" t="n">
         <v>4.9</v>
       </c>
-      <c r="G35" s="40" t="n">
+      <c r="G35" s="41" t="n">
         <v>4.1</v>
       </c>
-      <c r="H35" s="40" t="n">
+      <c r="H35" s="41" t="n">
         <v>-2.1</v>
       </c>
-      <c r="I35" s="40" t="n">
+      <c r="I35" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="J35" s="40" t="n">
+      <c r="J35" s="41" t="n">
         <v>3.1</v>
       </c>
       <c r="K35" s="5" t="n"/>
@@ -3366,16 +3372,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q35" s="37" t="n">
+      <c r="Q35" s="38" t="n">
         <v>-0.00300711691046418</v>
       </c>
-      <c r="R35" s="37" t="n">
+      <c r="R35" s="38" t="n">
         <v>0.001955057552418982</v>
       </c>
-      <c r="S35" s="37" t="n">
+      <c r="S35" s="38" t="n">
         <v>0.002092822632293601</v>
       </c>
-      <c r="T35" s="37" t="n">
+      <c r="T35" s="38" t="n">
         <v>-0.0004224555765300897</v>
       </c>
       <c r="U35" s="23" t="n">
@@ -3383,7 +3389,7 @@
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
-      <c r="A36" s="44" t="inlineStr">
+      <c r="A36" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Hou. Starts </t>
         </is>
@@ -3441,16 +3447,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q36" s="37" t="n">
+      <c r="Q36" s="38" t="n">
         <v>0.008019789135629696</v>
       </c>
-      <c r="R36" s="37" t="n">
+      <c r="R36" s="38" t="n">
         <v>0.01084249628307491</v>
       </c>
-      <c r="S36" s="37" t="n">
+      <c r="S36" s="38" t="n">
         <v>0.01169114908209064</v>
       </c>
-      <c r="T36" s="37" t="n">
+      <c r="T36" s="38" t="n">
         <v>0.01032118383222275</v>
       </c>
       <c r="U36" s="23" t="n">
@@ -3458,7 +3464,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="44" t="n"/>
+      <c r="A37" s="33" t="n"/>
       <c r="B37" s="15" t="inlineStr">
         <is>
           <t>HOUST</t>
@@ -3516,16 +3522,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q37" s="37" t="n">
+      <c r="Q37" s="38" t="n">
         <v>-0.00273486156666769</v>
       </c>
-      <c r="R37" s="37" t="n">
+      <c r="R37" s="38" t="n">
         <v>-0.0006239385435752309</v>
       </c>
-      <c r="S37" s="37" t="n">
+      <c r="S37" s="38" t="n">
         <v>-0.001255429809922437</v>
       </c>
-      <c r="T37" s="37" t="n">
+      <c r="T37" s="38" t="n">
         <v>-0.002710199627120158</v>
       </c>
       <c r="U37" s="23" t="n">
@@ -3533,7 +3539,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="44" t="inlineStr">
+      <c r="A38" s="33" t="inlineStr">
         <is>
           <t>Housing Permits</t>
         </is>
@@ -3591,16 +3597,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q38" s="37" t="n">
+      <c r="Q38" s="38" t="n">
         <v>0.01272340965111129</v>
       </c>
-      <c r="R38" s="37" t="n">
+      <c r="R38" s="38" t="n">
         <v>0.01427415269420379</v>
       </c>
-      <c r="S38" s="37" t="n">
+      <c r="S38" s="38" t="n">
         <v>0.01402408537902678</v>
       </c>
-      <c r="T38" s="37" t="n">
+      <c r="T38" s="38" t="n">
         <v>0.01316616157883059</v>
       </c>
       <c r="U38" s="23" t="n">
@@ -3608,7 +3614,7 @@
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
-      <c r="A39" s="44" t="n"/>
+      <c r="A39" s="33" t="n"/>
       <c r="B39" s="15" t="inlineStr">
         <is>
           <t>PERMIT</t>
@@ -3627,19 +3633,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F39" s="37" t="n">
+      <c r="F39" s="38" t="n">
         <v>-0.02162162162162162</v>
       </c>
-      <c r="G39" s="37" t="n">
+      <c r="G39" s="38" t="n">
         <v>-0.07957559681697612</v>
       </c>
-      <c r="H39" s="37" t="n">
+      <c r="H39" s="38" t="n">
         <v>-0.0119047619047619</v>
       </c>
-      <c r="I39" s="37" t="n">
+      <c r="I39" s="38" t="n">
         <v>-0.01324965132496513</v>
       </c>
-      <c r="J39" s="37" t="n">
+      <c r="J39" s="38" t="n">
         <v>-0.0989159891598916</v>
       </c>
       <c r="K39" s="5" t="n"/>
@@ -3683,7 +3689,7 @@
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
-      <c r="A40" s="44" t="inlineStr">
+      <c r="A40" s="33" t="inlineStr">
         <is>
           <t>New Home Sales</t>
         </is>
@@ -3741,16 +3747,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q40" s="37" t="n">
+      <c r="Q40" s="38" t="n">
         <v>-0.07456792269916472</v>
       </c>
-      <c r="R40" s="37" t="n">
+      <c r="R40" s="38" t="n">
         <v>-0.05790675033979801</v>
       </c>
-      <c r="S40" s="37" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.03874237696864814</v>
       </c>
-      <c r="T40" s="37" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.02292562904900106</v>
       </c>
       <c r="U40" s="23" t="n">
@@ -3758,7 +3764,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="44" t="n"/>
+      <c r="A41" s="33" t="n"/>
       <c r="B41" s="15" t="inlineStr">
         <is>
           <t>HSN1F</t>
@@ -3777,19 +3783,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F41" s="37" t="n">
+      <c r="F41" s="38" t="n">
         <v>0.03760445682451254</v>
       </c>
-      <c r="G41" s="37" t="n">
+      <c r="G41" s="38" t="n">
         <v>0.122962962962963</v>
       </c>
-      <c r="H41" s="37" t="n">
+      <c r="H41" s="38" t="n">
         <v>0.05636070853462158</v>
       </c>
-      <c r="I41" s="37" t="n">
+      <c r="I41" s="38" t="n">
         <v>0.002789400278940028</v>
       </c>
-      <c r="J41" s="37" t="n">
+      <c r="J41" s="38" t="n">
         <v>0.01875901875901876</v>
       </c>
       <c r="K41" s="5" t="n"/>
@@ -3816,16 +3822,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q41" s="37" t="n">
+      <c r="Q41" s="38" t="n">
         <v>0.003255208333333259</v>
       </c>
-      <c r="R41" s="37" t="n">
+      <c r="R41" s="38" t="n">
         <v/>
       </c>
-      <c r="S41" s="37" t="n">
+      <c r="S41" s="38" t="n">
         <v/>
       </c>
-      <c r="T41" s="37" t="n">
+      <c r="T41" s="38" t="n">
         <v>0</v>
       </c>
       <c r="U41" s="23" t="n">
@@ -3833,7 +3839,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="44" t="inlineStr">
+      <c r="A42" s="33" t="inlineStr">
         <is>
           <t>Existing Home Sales</t>
         </is>
@@ -3856,19 +3862,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F42" s="38" t="n">
+      <c r="F42" s="39" t="n">
         <v>3910000</v>
       </c>
-      <c r="G42" s="38" t="n">
+      <c r="G42" s="39" t="n">
         <v>4270000</v>
       </c>
-      <c r="H42" s="38" t="n">
+      <c r="H42" s="39" t="n">
         <v>4090000</v>
       </c>
-      <c r="I42" s="38" t="n">
+      <c r="I42" s="39" t="n">
         <v>4110000</v>
       </c>
-      <c r="J42" s="38" t="n">
+      <c r="J42" s="39" t="n">
         <v>4080000</v>
       </c>
       <c r="K42" s="7" t="n"/>
@@ -3891,16 +3897,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q42" s="37" t="n">
+      <c r="Q42" s="38" t="n">
         <v>0.03076923076923073</v>
       </c>
-      <c r="R42" s="37" t="n">
+      <c r="R42" s="38" t="n">
         <v>0.03225806451612891</v>
       </c>
-      <c r="S42" s="37" t="n">
+      <c r="S42" s="38" t="n">
         <v/>
       </c>
-      <c r="T42" s="37" t="n">
+      <c r="T42" s="38" t="n">
         <v>0.03869653767820766</v>
       </c>
       <c r="U42" s="23" t="n">
@@ -3908,7 +3914,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="44" t="n"/>
+      <c r="A43" s="33" t="n"/>
       <c r="B43" s="15" t="inlineStr">
         <is>
           <t>EXHOSLUSM495S</t>
@@ -3927,19 +3933,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F43" s="37" t="n">
+      <c r="F43" s="38" t="n">
         <v>-0.04400977995110025</v>
       </c>
-      <c r="G43" s="37" t="n">
+      <c r="G43" s="38" t="n">
         <v/>
       </c>
-      <c r="H43" s="37" t="n">
+      <c r="H43" s="38" t="n">
         <v/>
       </c>
-      <c r="I43" s="37" t="n">
+      <c r="I43" s="38" t="n">
         <v/>
       </c>
-      <c r="J43" s="37" t="n">
+      <c r="J43" s="38" t="n">
         <v/>
       </c>
       <c r="K43" s="5" t="n"/>
@@ -3966,16 +3972,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q43" s="37" t="n">
+      <c r="Q43" s="38" t="n">
         <v>0.00141643059490093</v>
       </c>
-      <c r="R43" s="37" t="n">
+      <c r="R43" s="38" t="n">
         <v/>
       </c>
-      <c r="S43" s="37" t="n">
+      <c r="S43" s="38" t="n">
         <v/>
       </c>
-      <c r="T43" s="37" t="n">
+      <c r="T43" s="38" t="n">
         <v>-0.001418439716311948</v>
       </c>
       <c r="U43" s="23" t="n">
@@ -3983,7 +3989,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="44" t="inlineStr">
+      <c r="A44" s="33" t="inlineStr">
         <is>
           <t>Gov. Cons</t>
         </is>
@@ -4041,16 +4047,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="Q44" s="37" t="n">
+      <c r="Q44" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="R44" s="37" t="n">
+      <c r="R44" s="38" t="n">
         <v>-0.0007077140835104227</v>
       </c>
-      <c r="S44" s="37" t="n">
+      <c r="S44" s="38" t="n">
         <v/>
       </c>
-      <c r="T44" s="37" t="n">
+      <c r="T44" s="38" t="n">
         <v>-0.0007097232079488595</v>
       </c>
       <c r="U44" s="23" t="n">
@@ -4058,7 +4064,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="44" t="n"/>
+      <c r="A45" s="33" t="n"/>
       <c r="B45" s="15" t="inlineStr">
         <is>
           <t>GCE</t>
@@ -4077,19 +4083,19 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="F45" s="37" t="n">
+      <c r="F45" s="38" t="n">
         <v>0.004135487891410161</v>
       </c>
-      <c r="G45" s="37" t="n">
+      <c r="G45" s="38" t="n">
         <v>0.01669515005814426</v>
       </c>
-      <c r="H45" s="37" t="n">
+      <c r="H45" s="38" t="n">
         <v>0.007978609251013902</v>
       </c>
-      <c r="I45" s="37" t="n">
+      <c r="I45" s="38" t="n">
         <v>0.008696251498575336</v>
       </c>
-      <c r="J45" s="37" t="n">
+      <c r="J45" s="38" t="n">
         <v>0.01254255520332359</v>
       </c>
       <c r="K45" s="5" t="n"/>
@@ -4105,7 +4111,7 @@
       <c r="U45" s="21" t="n"/>
     </row>
     <row r="46" ht="16.15" customHeight="1" thickBot="1">
-      <c r="A46" s="44" t="inlineStr">
+      <c r="A46" s="33" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4196,7 +4202,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="44" t="n"/>
+      <c r="A47" s="33" t="n"/>
       <c r="B47" s="15" t="inlineStr">
         <is>
           <t>BOPTEXP</t>
@@ -4215,19 +4221,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F47" s="37" t="n">
+      <c r="F47" s="38" t="n">
         <v>-0.01711656231824554</v>
       </c>
-      <c r="G47" s="37" t="n">
+      <c r="G47" s="38" t="n">
         <v>-0.03405222839844813</v>
       </c>
-      <c r="H47" s="37" t="n">
+      <c r="H47" s="38" t="n">
         <v>0.02957798714533122</v>
       </c>
-      <c r="I47" s="37" t="n">
+      <c r="I47" s="38" t="n">
         <v>0.03582555615078808</v>
       </c>
-      <c r="J47" s="37" t="n">
+      <c r="J47" s="38" t="n">
         <v>0.0004866042778863822</v>
       </c>
       <c r="K47" s="5" t="n"/>
@@ -4271,7 +4277,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="44" t="inlineStr">
+      <c r="A48" s="33" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4350,7 +4356,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="44" t="n"/>
+      <c r="A49" s="33" t="n"/>
       <c r="B49" s="15" t="inlineStr">
         <is>
           <t>BOPTIMP</t>
@@ -4369,19 +4375,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F49" s="37" t="n">
+      <c r="F49" s="38" t="n">
         <v>0.0355134449547394</v>
       </c>
-      <c r="G49" s="37" t="n">
+      <c r="G49" s="38" t="n">
         <v>0.04222512622871166</v>
       </c>
-      <c r="H49" s="37" t="n">
+      <c r="H49" s="38" t="n">
         <v>-0.02997523288697879</v>
       </c>
-      <c r="I49" s="37" t="n">
+      <c r="I49" s="38" t="n">
         <v>0.007887072931081818</v>
       </c>
-      <c r="J49" s="37" t="n">
+      <c r="J49" s="38" t="n">
         <v>-0.05210885495329198</v>
       </c>
       <c r="K49" s="5" t="n"/>
@@ -4425,7 +4431,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="44" t="inlineStr">
+      <c r="A50" s="33" t="inlineStr">
         <is>
           <t>Trade Balance</t>
         </is>
@@ -4504,7 +4510,7 @@
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
-      <c r="A51" s="44" t="n"/>
+      <c r="A51" s="33" t="n"/>
       <c r="B51" s="15" t="inlineStr">
         <is>
           <t>BOPSTB</t>
@@ -4523,19 +4529,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F51" s="37" t="n">
+      <c r="F51" s="38" t="n">
         <v>-0.05160636663725204</v>
       </c>
-      <c r="G51" s="37" t="n">
+      <c r="G51" s="38" t="n">
         <v>0.02753803270980959</v>
       </c>
-      <c r="H51" s="37" t="n">
+      <c r="H51" s="38" t="n">
         <v>-0.01299347011833341</v>
       </c>
-      <c r="I51" s="37" t="n">
+      <c r="I51" s="38" t="n">
         <v>-0.008120725933719042</v>
       </c>
-      <c r="J51" s="37" t="n">
+      <c r="J51" s="38" t="n">
         <v>0.06327343913864225</v>
       </c>
       <c r="K51" s="5" t="n"/>
@@ -4579,7 +4585,7 @@
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
-      <c r="A52" s="35" t="n"/>
+      <c r="A52" s="36" t="n"/>
       <c r="B52" s="17" t="n"/>
       <c r="C52" s="20" t="n"/>
       <c r="D52" s="9" t="n"/>
@@ -4630,12 +4636,12 @@
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">
-      <c r="A53" s="36" t="inlineStr">
+      <c r="A53" s="37" t="inlineStr">
         <is>
           <t>Footnote: All data is Seasonally Adjusted unless otherwise indicated by NSA</t>
         </is>
       </c>
-      <c r="B53" s="39" t="inlineStr">
+      <c r="B53" s="40" t="inlineStr">
         <is>
           <t>*FRED doesn't include real avg. hourly earning data. Calculated through chained PCE deflator (FRED ticker: PCEPI). Ticker "RCES0500000003" is only for reference in the raw data table</t>
         </is>
@@ -4661,7 +4667,7 @@
       <c r="U53" s="6" t="n"/>
     </row>
     <row r="54" ht="21" customHeight="1">
-      <c r="A54" s="36" t="inlineStr">
+      <c r="A54" s="37" t="inlineStr">
         <is>
           <t>Source: All data collected via FRED from the St. Louis Fed</t>
         </is>
@@ -4687,11 +4693,10 @@
       <c r="T54" s="6" t="n"/>
       <c r="U54" s="6" t="n"/>
     </row>
-    <row r="55" ht="31.5" customHeight="1">
-      <c r="A55" s="36" t="inlineStr">
-        <is>
-          <t>Mike Aguilar | mike.aguilar@duke.edu |
-Jacky Yang    | jacky.yang@duke.edu     | www.market-observatory.com</t>
+    <row r="55" ht="21" customHeight="1">
+      <c r="A55" s="37" t="inlineStr">
+        <is>
+          <t>Mike Aguilar | mike.aguilar@duke.edu | www.market-observatory.com</t>
         </is>
       </c>
       <c r="B55" s="15" t="n"/>

</xml_diff>

<commit_message>
Update dashboards - 2026-03-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,16 +2915,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.14</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.12</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.12</v>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,16 +2994,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.25</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.28</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.28</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.26</v>
@@ -3509,7 +3509,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="49" t="n">
+      <c r="N37" s="48" t="n">
         <v>45992</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3584,7 +3584,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="49" t="n">
+      <c r="N38" s="48" t="n">
         <v>45992</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.42</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.45</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.43</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.43</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.48</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.57</v>
-      </c>
-      <c r="R49" s="6" t="n">
-        <v>3.61</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>3.61</v>
       </c>
       <c r="T49" s="6" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>3.59</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.65</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.02</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.04</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.03</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.08</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46078</v>
+        <v>46080</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,13 +4620,13 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>5.78</v>
+        <v>5.77</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>5.77</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>5.76</v>
+        <v>5.78</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>5.77</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-03-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1078,8 +1078,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
-        <v>46023</v>
+      <c r="N5" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1092,19 +1092,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>22000</v>
+        <v>63000</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>37000</v>
+        <v>11000</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>74000</v>
+        <v>41000</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>20000</v>
+        <v>-29000</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>88000</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="6">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2918,16 +2918,16 @@
         <v>2.12</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.14</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,16 +2997,16 @@
         <v>2.29</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.25</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.28</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.28</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="31">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,16 +4340,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.38</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.42</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.45</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>3.43</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>3.43</v>
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.51</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.57</v>
-      </c>
-      <c r="S49" s="6" t="n">
-        <v>3.61</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>3.61</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>3.59</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.02</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.04</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.03</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>5.77</v>
+        <v>5.83</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>5.77</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>5.78</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.77</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.76</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-05
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1098,13 +1098,13 @@
         <v>11000</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>41000</v>
+        <v>37000</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>-29000</v>
+        <v>74000</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>47000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="6">
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N13" s="49" t="n">
-        <v>46069</v>
+        <v>46076</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1712,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>212000</v>
+        <v>213000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>213000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>208000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>229000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>232000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>209000</v>
       </c>
     </row>
     <row r="14">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46062</v>
+        <v>46069</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1833000</v>
+        <v>1868000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1822000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1864000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1852000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1841000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1819000</v>
       </c>
     </row>
     <row r="15">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2921,13 +2921,13 @@
         <v>2.12</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.13</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.14</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3000,10 +3000,10 @@
         <v>2.29</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.25</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.28</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.28</v>
@@ -3320,8 +3320,8 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="48" t="n">
-        <v>45839</v>
+      <c r="C35" s="49" t="n">
+        <v>45931</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -3334,19 +3334,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>4.9</v>
+        <v>2.8</v>
       </c>
       <c r="G35" s="41" t="n">
-        <v>4.1</v>
+        <v>5.2</v>
       </c>
       <c r="H35" s="41" t="n">
-        <v>-2.1</v>
+        <v>4.2</v>
       </c>
       <c r="I35" s="41" t="n">
-        <v>0.9</v>
+        <v>-0.9</v>
       </c>
       <c r="J35" s="41" t="n">
-        <v>3.1</v>
+        <v>1.4</v>
       </c>
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -3809,8 +3809,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
-        <v>45992</v>
+      <c r="N41" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3823,19 +3823,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.003255208333333259</v>
+        <v>0.006468305304010435</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v/>
+        <v>0.005855562784645496</v>
       </c>
       <c r="S41" s="38" t="n">
         <v/>
       </c>
       <c r="T41" s="38" t="n">
+        <v/>
+      </c>
+      <c r="U41" s="23" t="n">
         <v>0</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0.00130890052356003</v>
       </c>
     </row>
     <row r="42">
@@ -3884,8 +3884,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
-        <v>45992</v>
+      <c r="N42" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3898,19 +3898,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.03076923076923073</v>
+        <v>0.02638522427440633</v>
       </c>
       <c r="R42" s="38" t="n">
-        <v>0.03225806451612891</v>
+        <v>0.0341137123745819</v>
       </c>
       <c r="S42" s="38" t="n">
+        <v>0.03293010752688157</v>
+      </c>
+      <c r="T42" s="38" t="n">
         <v/>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v>0.03869653767820766</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.03238866396761141</v>
       </c>
     </row>
     <row r="43">
@@ -3959,8 +3959,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
-        <v>45992</v>
+      <c r="N43" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3973,19 +3973,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.00141643059490093</v>
+        <v>0.002121640735502028</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v/>
+        <v>0.002126151665485576</v>
       </c>
       <c r="S43" s="38" t="n">
         <v/>
       </c>
       <c r="T43" s="38" t="n">
+        <v/>
+      </c>
+      <c r="U43" s="23" t="n">
         <v>-0.001418439716311948</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>-0.001416430594900819</v>
       </c>
     </row>
     <row r="44">
@@ -4034,8 +4034,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
-        <v>45992</v>
+      <c r="N44" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4048,19 +4048,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
+        <v>-0.0007052186177716695</v>
+      </c>
+      <c r="R44" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="R44" s="38" t="n">
-        <v>-0.0007077140835104227</v>
-      </c>
       <c r="S44" s="38" t="n">
+        <v>-0.001415428167020644</v>
+      </c>
+      <c r="T44" s="38" t="n">
         <v/>
       </c>
-      <c r="T44" s="38" t="n">
+      <c r="U44" s="23" t="n">
         <v>-0.0007097232079488595</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>-0.002828854314002869</v>
       </c>
     </row>
     <row r="45">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.47</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.38</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.42</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.45</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.43</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,16 +4415,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.62</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.51</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.57</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>3.61</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>3.61</v>
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.02</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.05</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.04</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,7 +4555,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46076</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.83</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>5.77</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>5.77</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>5.78</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.77</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-06
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -928,8 +928,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
-        <v>46023</v>
+      <c r="N3" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
@@ -942,19 +942,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>130</v>
+        <v>-92</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>-17</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>41</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>-140</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>76</v>
       </c>
     </row>
     <row r="4">
@@ -999,8 +999,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
-        <v>46023</v>
+      <c r="N4" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
@@ -1013,19 +1013,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.002268304395076705</v>
+        <v>0.0009854083759711957</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.001143283054144875</v>
+        <v>0.001832335026663634</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.0007327117916066601</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.002340601850973247</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.002931400170945582</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.004027559653477886</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1153,8 +1153,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
-        <v>46023</v>
+      <c r="N6" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1167,19 +1167,19 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="R6" s="6" t="n">
         <v>4.3</v>
       </c>
-      <c r="R6" s="6" t="n">
+      <c r="S6" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="S6" s="6" t="n">
+      <c r="T6" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="U6" s="21" t="n">
         <v/>
-      </c>
-      <c r="U6" s="21" t="n">
-        <v>4.4</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1232,8 +1232,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46023</v>
+      <c r="N7" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1246,19 +1246,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="R7" s="6" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>8.4</v>
       </c>
-      <c r="S7" s="6" t="n">
+      <c r="T7" s="6" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="T7" s="6" t="n">
+      <c r="U7" s="21" t="n">
         <v/>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>8.1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1311,8 +1311,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
-        <v>46023</v>
+      <c r="N8" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1325,19 +1325,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="T8" s="6" t="n">
         <v>62.5</v>
       </c>
-      <c r="R8" s="6" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="S8" s="6" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="T8" s="6" t="n">
+      <c r="U8" s="21" t="n">
         <v/>
-      </c>
-      <c r="U8" s="21" t="n">
-        <v>62.5</v>
       </c>
     </row>
     <row r="9">
@@ -1390,8 +1390,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46023</v>
+      <c r="N9" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1404,19 +1404,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.8</v>
+        <v>59.3</v>
       </c>
       <c r="R9" s="6" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="S9" s="6" t="n">
         <v>59.7</v>
       </c>
-      <c r="S9" s="6" t="n">
+      <c r="T9" s="6" t="n">
         <v>59.6</v>
       </c>
-      <c r="T9" s="6" t="n">
+      <c r="U9" s="21" t="n">
         <v/>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>59.7</v>
       </c>
     </row>
     <row r="10">
@@ -1852,8 +1852,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
-        <v>46023</v>
+      <c r="N15" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1869,13 +1869,13 @@
         <v>34.3</v>
       </c>
       <c r="R15" s="24" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="S15" s="24" t="n">
         <v>34.2</v>
       </c>
-      <c r="S15" s="24" t="n">
+      <c r="T15" s="24" t="n">
         <v>34.3</v>
-      </c>
-      <c r="T15" s="24" t="n">
-        <v>34.2</v>
       </c>
       <c r="U15" s="26" t="n">
         <v>34.2</v>
@@ -1939,8 +1939,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
-        <v>45992</v>
+      <c r="C17" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1953,19 +1953,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>-0.000160525653495891</v>
+        <v>-0.0015625744366633</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.005518082869731433</v>
+        <v>-4.49151919511559e-05</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>0.005016065910586232</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>-0.001558334425942887</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>0.0006724067240673204</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>0.00545946488174831</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2026,8 +2026,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
-        <v>45992</v>
+      <c r="C18" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2040,19 +2040,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.02427715536403887</v>
+        <v>0.03155977752620958</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.03263595152369941</v>
+        <v>0.02428670017357602</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.03212039564348258</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.03213514238518121</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.04144341481107452</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.04972605550048132</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2369,7 +2369,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2439,7 +2439,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,7 +2915,7 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.12</v>
@@ -2924,10 +2924,10 @@
         <v>2.12</v>
       </c>
       <c r="T29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.1</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.13</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,7 +2994,7 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.29</v>
+        <v>2.31</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.29</v>
@@ -3003,10 +3003,10 @@
         <v>2.29</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.25</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="31">
@@ -3205,8 +3205,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
-        <v>46023</v>
+      <c r="N33" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
@@ -3219,19 +3219,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
+        <v>0.004035512510088823</v>
+      </c>
+      <c r="R33" s="38" t="n">
         <v>0.004051863857374327</v>
       </c>
-      <c r="R33" s="38" t="n">
+      <c r="S33" s="38" t="n">
         <v>0.000540540540540535</v>
       </c>
-      <c r="S33" s="38" t="n">
+      <c r="T33" s="38" t="n">
         <v>0.00407055630936215</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.004087193460490468</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.002184598580011077</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.51</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.47</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.38</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.42</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.45</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.63</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.62</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.51</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.57</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.61</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.06</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.02</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.05</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,8 +4555,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46076</v>
+      <c r="N51" s="49" t="n">
+        <v>46083</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4569,19 +4569,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>5.98</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.01</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.09</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.11</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.1</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.84</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.83</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>5.77</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>5.77</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>5.78</v>
+        <v>5.77</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2330,8 +2330,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
-        <v>46023</v>
+      <c r="C22" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2344,19 +2344,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>15.199</v>
+        <v>16.118</v>
       </c>
       <c r="G22" s="24" t="n">
+        <v>15.209</v>
+      </c>
+      <c r="H22" s="24" t="n">
         <v>16.401</v>
       </c>
-      <c r="H22" s="24" t="n">
+      <c r="I22" s="24" t="n">
         <v>16.006</v>
       </c>
-      <c r="I22" s="24" t="n">
+      <c r="J22" s="24" t="n">
         <v>15.843</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>16.985</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2405,8 +2405,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
-        <v>46023</v>
+      <c r="C23" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2419,19 +2419,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.04708463949843257</v>
+        <v>-0.01833241975759802</v>
       </c>
       <c r="G23" s="25" t="n">
+        <v>-0.04645768025078368</v>
+      </c>
+      <c r="H23" s="25" t="n">
         <v>-0.0520201144442517</v>
       </c>
-      <c r="H23" s="25" t="n">
+      <c r="I23" s="25" t="n">
         <v>-0.05334752779749237</v>
       </c>
-      <c r="I23" s="25" t="n">
+      <c r="J23" s="25" t="n">
         <v>-0.03941065906748309</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>0.03941007282296054</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2479,8 +2479,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
-        <v>45992</v>
+      <c r="C24" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2493,19 +2493,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.0105318556006937</v>
+        <v>0.003556211510844731</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>-0.001281418924231392</v>
+        <v>0.009446225118119989</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.004454853076971466</v>
+        <v>-0.002377705261307317</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.00339828596255809</v>
+        <v>0.003395368410566313</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>-0.003651114145611811</v>
+        <v>0.003399783954204594</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2558,8 +2558,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="48" t="n">
-        <v>45992</v>
+      <c r="C25" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2572,19 +2572,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.002704782960157415</v>
+        <v>0.0008831408658551698</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.001696137399219255</v>
+        <v>0.003398716336493468</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.0009232413445350307</v>
+        <v>0.001527249410752551</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.001873721239173287</v>
+        <v>0.0007591671161557567</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.001994229089696598</v>
+        <v>0.002887647186711639</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,10 +2915,10 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.11</v>
-      </c>
-      <c r="R29" s="6" t="n">
-        <v>2.12</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.12</v>
@@ -2927,7 +2927,7 @@
         <v>2.12</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.1</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,10 +2994,10 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.31</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.29</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.29</v>
@@ -3006,7 +3006,7 @@
         <v>2.29</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.25</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="31">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.54</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.51</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.47</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.38</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.42</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.67</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.63</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.62</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.51</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.57</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.06</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>3.97</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.02</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,16 +4620,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.83</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.84</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.83</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>5.77</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>5.77</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-03-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,13 +2915,13 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.11</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <v>2.12</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.12</v>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,13 +2994,13 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.35</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.31</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.29</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.29</v>
@@ -3850,7 +3850,7 @@
         </is>
       </c>
       <c r="C42" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3863,19 +3863,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>3910000</v>
+        <v>4090000</v>
       </c>
       <c r="G42" s="39" t="n">
+        <v>4020000</v>
+      </c>
+      <c r="H42" s="39" t="n">
         <v>4270000</v>
       </c>
-      <c r="H42" s="39" t="n">
+      <c r="I42" s="39" t="n">
         <v>4090000</v>
       </c>
-      <c r="I42" s="39" t="n">
+      <c r="J42" s="39" t="n">
         <v>4110000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4080000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="C43" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3934,7 +3934,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.04400977995110025</v>
+        <v>-0.01445783132530121</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.54</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.51</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.47</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.38</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4418,16 +4418,16 @@
         <v>3.72</v>
       </c>
       <c r="R49" s="6" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="S49" s="6" t="n">
         <v>3.67</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.63</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.62</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.51</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.06</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.05</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>3.97</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.89</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.83</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.84</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.83</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.77</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1078,7 +1078,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1272,8 +1272,10 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
-        <v>45992</v>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RECPROUSM156N' not found in values file."</t>
+        </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1286,19 +1288,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>0.62</v>
+        <v>1</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>0.82</v>
+        <v>1</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1505,8 +1507,10 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
-        <v>45992</v>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1519,19 +1523,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>-0.008854919140606765</v>
+        <v>1</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.005152948892116038</v>
+        <v>1</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>-9.368120286679105e-05</v>
+        <v>1</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>-0.00461581499440511</v>
+        <v>1</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>0.001494209936496294</v>
+        <v>1</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1580,8 +1584,10 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
-        <v>45992</v>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1594,19 +1600,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>-0.02783872737246302</v>
+        <v>1</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.006567528263826993</v>
+        <v>1</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.01846374045801518</v>
+        <v>1</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>0.02290259211345895</v>
+        <v>1</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>0.03914728682170551</v>
+        <v>1</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1659,8 +1665,10 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
-        <v>45992</v>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1673,19 +1681,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.002845310871341211</v>
+        <v>1</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.001580090855224148</v>
+        <v>1</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>0.001469383141654124</v>
+        <v>1</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>-0.00357585313661446</v>
+        <v>1</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>0.005207743688441013</v>
+        <v>1</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1734,8 +1742,10 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
-        <v>45992</v>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1748,19 +1758,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.01357310577859232</v>
+        <v>1</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.02625112029836067</v>
+        <v>1</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.02445440092498914</v>
+        <v>1</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>0.02153393181883783</v>
+        <v>1</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>0.03793325150505573</v>
+        <v>1</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1939,8 +1949,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
-        <v>46023</v>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1953,19 +1965,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>-0.0015625744366633</v>
+        <v>1</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>-4.49151919511559e-05</v>
+        <v>1</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>0.005016065910586232</v>
+        <v>1</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>-0.001558334425942887</v>
+        <v>1</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>0.0006724067240673204</v>
+        <v>1</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2026,8 +2038,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
-        <v>46023</v>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2040,19 +2054,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.03155977752620958</v>
+        <v>1</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.02428670017357602</v>
+        <v>1</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>0.03212039564348258</v>
+        <v>1</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>0.03213514238518121</v>
+        <v>1</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>0.04144341481107452</v>
+        <v>1</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2065,8 +2079,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
-        <v>46023</v>
+      <c r="N18" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2079,19 +2093,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>0.00267003074209704</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>0.00170842649932057</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>0.00297788428704604</v>
-      </c>
-      <c r="S18" s="38" t="n">
-        <v/>
       </c>
       <c r="T18" s="38" t="n">
         <v/>
       </c>
       <c r="U18" s="23" t="n">
-        <v>0.002950901819104068</v>
+        <v/>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2105,8 +2119,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
-        <v>45992</v>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2119,19 +2135,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.0002827474178507261</v>
+        <v>1</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.001248973066589665</v>
+        <v>1</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>-0.001280636881233477</v>
+        <v>1</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>0.0005713461581133839</v>
+        <v>1</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>0.001005025125628167</v>
+        <v>1</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2140,8 +2156,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
-        <v>46023</v>
+      <c r="N19" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2154,19 +2170,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.0243400411037322</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.02391201432150015</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.02653304114557758</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.02696443916493949</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v/>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.03022571584713336</v>
       </c>
     </row>
     <row r="20">
@@ -2176,8 +2192,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
-        <v>45992</v>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2190,19 +2208,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.009195260774909153</v>
+        <v>1</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01041374906169812</v>
+        <v>1</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.01147076162937589</v>
+        <v>1</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.01508168307081075</v>
+        <v>1</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01547352826862074</v>
+        <v>1</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2215,8 +2233,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46023</v>
+      <c r="N20" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2229,19 +2247,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>0.002160502174024082</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.002950448142634121</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>0.002329002576704653</v>
-      </c>
-      <c r="S20" s="38" t="n">
-        <v/>
       </c>
       <c r="T20" s="38" t="n">
         <v/>
       </c>
       <c r="U20" s="23" t="n">
-        <v>0.002177737336973129</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2255,8 +2273,10 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
-        <v>45992</v>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
+        </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2269,19 +2289,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>3.6</v>
+        <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>3.7</v>
+        <v>1</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>3.7</v>
+        <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2290,8 +2310,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46023</v>
+      <c r="N21" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2304,19 +2324,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.02472462476764023</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.02512028782828883</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.02646484707309002</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.02599044806094405</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v/>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v>0.03019966825885779</v>
       </c>
     </row>
     <row r="22">
@@ -2330,8 +2350,10 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
-        <v>46054</v>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
+        </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2344,19 +2366,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.118</v>
+        <v>1</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>15.209</v>
+        <v>1</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.401</v>
+        <v>1</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.006</v>
+        <v>1</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>15.843</v>
+        <v>1</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2405,8 +2427,10 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
-        <v>46054</v>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
+        </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2419,19 +2443,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.01833241975759802</v>
+        <v>1</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.04645768025078368</v>
+        <v>1</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.0520201144442517</v>
+        <v>1</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>-0.05334752779749237</v>
+        <v>1</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.03941065906748309</v>
+        <v>1</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2558,8 +2582,10 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
-        <v>46023</v>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2572,19 +2598,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.0008831408658551698</v>
+        <v>1</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.003398716336493468</v>
+        <v>1</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.001527249410752551</v>
+        <v>1</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.0007591671161557567</v>
+        <v>1</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.002887647186711639</v>
+        <v>1</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2902,7 +2928,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,16 +2941,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.11</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.12</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.12</v>
@@ -2981,7 +3007,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,16 +3020,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.35</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.31</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.29</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.29</v>
@@ -3245,8 +3271,10 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46023</v>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TCU' not found in values file."</t>
+        </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3259,19 +3287,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.2119</v>
+        <v>1</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>75.7433</v>
+        <v>1</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.64619999999999</v>
+        <v>1</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.6474</v>
+        <v>1</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>76.0745</v>
+        <v>1</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3660,7 +3688,7 @@
         </is>
       </c>
       <c r="N39" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3673,19 +3701,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
+        <v>117.906</v>
+      </c>
+      <c r="R39" s="6" t="n">
         <v>119.2298</v>
       </c>
-      <c r="R39" s="6" t="n">
+      <c r="S39" s="6" t="n">
         <v>120.1883</v>
       </c>
-      <c r="S39" s="6" t="n">
+      <c r="T39" s="6" t="n">
         <v>121.4177</v>
       </c>
-      <c r="T39" s="6" t="n">
+      <c r="U39" s="21" t="n">
         <v>120.7618</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>120.0291</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3735,7 +3763,7 @@
         </is>
       </c>
       <c r="N40" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3748,19 +3776,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.07796471263522881</v>
+      </c>
+      <c r="R40" s="38" t="n">
         <v>-0.07456792269916472</v>
       </c>
-      <c r="R40" s="38" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.05790675033979801</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.03874237696864814</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.02292562904900106</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.0152258401163721</v>
       </c>
     </row>
     <row r="41">
@@ -4248,7 +4276,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4355,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4343,16 +4371,16 @@
         <v>3.56</v>
       </c>
       <c r="R48" s="6" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="S48" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.54</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.51</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.47</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4430,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4443,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>3.72</v>
+        <v>3.71</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>3.72</v>
       </c>
       <c r="S49" s="6" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="T49" s="6" t="n">
         <v>3.67</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.63</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.62</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4509,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4522,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.06</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.05</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4635,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4623,16 +4651,16 @@
         <v>5.9</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>5.89</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.83</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.84</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.83</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-12
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1272,10 +1272,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RECPROUSM156N' not found in values file."</t>
-        </is>
+      <c r="C8" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1288,19 +1286,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>1</v>
+        <v>0.62</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>1</v>
+        <v>0.86</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>1</v>
+        <v>0.88</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1507,10 +1505,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
-        </is>
+      <c r="C11" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1523,19 +1519,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>1</v>
+        <v>-0.008854919140606765</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>1</v>
+        <v>0.005152948892116038</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>1</v>
+        <v>-9.368120286679105e-05</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>1</v>
+        <v>-0.00461581499440511</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>1</v>
+        <v>0.001494209936496294</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1584,10 +1580,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
-        </is>
+      <c r="C12" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1600,19 +1594,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>1</v>
+        <v>-0.02783872737246302</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>1</v>
+        <v>0.006567528263826993</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>1</v>
+        <v>0.01846374045801518</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>1</v>
+        <v>0.02290259211345895</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>1</v>
+        <v>0.03914728682170551</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1665,10 +1659,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
-        </is>
+      <c r="C13" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1681,19 +1673,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>1</v>
+        <v>-0.002845310871341211</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>1</v>
+        <v>0.001580090855224148</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>1</v>
+        <v>0.001469383141654124</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>1</v>
+        <v>-0.00357585313661446</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>1</v>
+        <v>0.005207743688441013</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1707,7 +1699,7 @@
         </is>
       </c>
       <c r="N13" s="49" t="n">
-        <v>46076</v>
+        <v>46083</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1723,16 +1715,16 @@
         <v>213000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>214000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>213000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>208000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>229000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>232000</v>
       </c>
     </row>
     <row r="14">
@@ -1742,10 +1734,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
-        </is>
+      <c r="C14" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1758,19 +1748,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>1</v>
+        <v>0.01357310577859232</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>1</v>
+        <v>0.02625112029836067</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>1</v>
+        <v>0.02445440092498914</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>1</v>
+        <v>0.02153393181883783</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>1</v>
+        <v>0.03793325150505573</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1784,7 +1774,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46069</v>
+        <v>46076</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1797,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1868000</v>
+        <v>1850000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1871000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1822000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1864000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1852000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1841000</v>
       </c>
     </row>
     <row r="15">
@@ -1949,10 +1939,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C17" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1965,19 +1953,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>1</v>
+        <v>-0.0015625744366633</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>1</v>
+        <v>-4.49151919511559e-05</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>1</v>
+        <v>0.005016065910586232</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>1</v>
+        <v>-0.001558334425942887</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>1</v>
+        <v>0.0006724067240673204</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2038,10 +2026,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C18" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2054,19 +2040,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>1</v>
+        <v>0.03155977752620958</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>1</v>
+        <v>0.02428670017357602</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>1</v>
+        <v>0.03212039564348258</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>1</v>
+        <v>0.03213514238518121</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>1</v>
+        <v>0.04144341481107452</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2119,10 +2105,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C19" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2135,19 +2119,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>1</v>
+        <v>-0.0002827474178507261</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>1</v>
+        <v>0.001248973066589665</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>1</v>
+        <v>-0.001280636881233477</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>1</v>
+        <v>0.0005713461581133839</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>1</v>
+        <v>0.001005025125628167</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2192,10 +2176,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C20" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2208,19 +2190,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>1</v>
+        <v>0.009195260774909153</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>1</v>
+        <v>0.01041374906169812</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>1</v>
+        <v>0.01147076162937589</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>1</v>
+        <v>0.01508168307081075</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>1</v>
+        <v>0.01547352826862074</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2273,10 +2255,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
-        </is>
+      <c r="C21" s="48" t="n">
+        <v>45992</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2289,19 +2269,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1</v>
+        <v>3.6</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1</v>
+        <v>3.7</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1</v>
+        <v>3.7</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>4.1</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2350,10 +2330,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
-        </is>
+      <c r="C22" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2366,19 +2344,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>1</v>
+        <v>16.118</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>1</v>
+        <v>15.209</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>1</v>
+        <v>16.401</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>1</v>
+        <v>16.006</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>1</v>
+        <v>15.843</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2427,10 +2405,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
-        </is>
+      <c r="C23" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2443,19 +2419,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>1</v>
+        <v>-0.01833241975759802</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>1</v>
+        <v>-0.04645768025078368</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>1</v>
+        <v>-0.0520201144442517</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>1</v>
+        <v>-0.05334752779749237</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>1</v>
+        <v>-0.03941065906748309</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2582,10 +2558,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
-        </is>
+      <c r="C25" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2598,19 +2572,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>1</v>
+        <v>0.0008831408658551698</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>1</v>
+        <v>0.003398716336493468</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>1</v>
+        <v>0.001527249410752551</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>1</v>
+        <v>0.0007591671161557567</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>1</v>
+        <v>0.002887647186711639</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2928,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2941,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.11</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -3007,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3020,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.35</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="31">
@@ -3271,10 +3245,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TCU' not found in values file."</t>
-        </is>
+      <c r="C34" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3287,19 +3259,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>1</v>
+        <v>76.2119</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>1</v>
+        <v>75.7433</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>1</v>
+        <v>75.64619999999999</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>1</v>
+        <v>75.6474</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>1</v>
+        <v>76.0745</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3348,7 +3320,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="49" t="n">
+      <c r="C35" s="48" t="n">
         <v>45931</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -3427,8 +3399,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
-        <v>45992</v>
+      <c r="C36" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3441,19 +3413,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1404</v>
+        <v>1487</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1322</v>
+        <v>1387</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1324</v>
+      </c>
+      <c r="I36" s="24" t="n">
         <v>1272</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="J36" s="24" t="n">
         <v>1328</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1291</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3498,8 +3470,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
-        <v>45992</v>
+      <c r="C37" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3512,19 +3484,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>-0.0726552179656539</v>
+        <v>0.09499263622974963</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>0.02084942084942085</v>
+        <v>-0.08388375165125496</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>0.02239382239382239</v>
+      </c>
+      <c r="I37" s="25" t="n">
         <v>-0.05917159763313609</v>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="J37" s="25" t="n">
         <v>-0.02137067059690494</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>-0.07189072609633357</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3577,8 +3549,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>45992</v>
+      <c r="C38" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3591,19 +3563,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1448</v>
+        <v>1376</v>
       </c>
       <c r="G38" s="24" t="n">
+        <v>1455</v>
+      </c>
+      <c r="H38" s="24" t="n">
         <v>1388</v>
       </c>
-      <c r="H38" s="24" t="n">
+      <c r="I38" s="24" t="n">
         <v>1411</v>
       </c>
-      <c r="I38" s="24" t="n">
+      <c r="J38" s="24" t="n">
         <v>1415</v>
-      </c>
-      <c r="J38" s="24" t="n">
-        <v>1330</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3648,8 +3620,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>45992</v>
+      <c r="C39" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3662,19 +3634,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.02162162162162162</v>
+        <v>-0.05753424657534247</v>
       </c>
       <c r="G39" s="38" t="n">
+        <v>-0.01689189189189189</v>
+      </c>
+      <c r="H39" s="38" t="n">
         <v>-0.07957559681697612</v>
       </c>
-      <c r="H39" s="38" t="n">
+      <c r="I39" s="38" t="n">
         <v>-0.0119047619047619</v>
       </c>
-      <c r="I39" s="38" t="n">
+      <c r="J39" s="38" t="n">
         <v>-0.01324965132496513</v>
-      </c>
-      <c r="J39" s="38" t="n">
-        <v>-0.0989159891598916</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3837,7 +3809,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3912,7 +3884,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="49" t="n">
+      <c r="N42" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3987,7 +3959,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4062,7 +4034,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4276,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4355,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4368,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.56</v>
+        <v>3.57</v>
       </c>
       <c r="R48" s="6" t="n">
         <v>3.56</v>
       </c>
       <c r="S48" s="6" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="T48" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.54</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.51</v>
       </c>
     </row>
     <row r="49">
@@ -4430,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4443,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.71</v>
-      </c>
-      <c r="R49" s="6" t="n">
-        <v>3.72</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>3.72</v>
       </c>
       <c r="T49" s="6" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>3.67</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.63</v>
       </c>
     </row>
     <row r="50">
@@ -4509,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4522,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.12</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.09</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.06</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4583,7 +4555,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46083</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4635,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4648,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>5.9</v>
+        <v>5.92</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>5.9</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>5.89</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.83</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.84</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24111.83</v>
+        <v>24065.956</v>
       </c>
       <c r="G3" s="24" t="n">
         <v>24026.834</v>
@@ -928,7 +928,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N3" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.003537544730196407</v>
+        <v>0.001628262799834523</v>
       </c>
       <c r="G4" s="25" t="n">
         <v>0.0107634621312982</v>
@@ -999,7 +999,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="49" t="n">
+      <c r="N4" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1153,7 +1153,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="49" t="n">
+      <c r="N6" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1232,7 +1232,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1311,7 +1311,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="49" t="n">
+      <c r="N8" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16682.486</v>
+        <v>16667.027</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>16585.878</v>
@@ -1390,7 +1390,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="49" t="n">
+      <c r="N9" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1440,7 +1440,7 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.00582471425389719</v>
+        <v>0.004892656270593321</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>0.008524606910566446</v>
@@ -1465,8 +1465,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
-        <v>45992</v>
+      <c r="N10" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1479,16 +1479,16 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="U10" s="21" t="n">
         <v>4.3</v>
@@ -1505,8 +1505,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
-        <v>45992</v>
+      <c r="C11" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1519,19 +1519,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>-0.008854919140606765</v>
+        <v>-0.01147326027910467</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.005152948892116038</v>
+        <v>-0.007021622878400358</v>
       </c>
       <c r="H11" s="25" t="n">
+        <v>0.007401508408675816</v>
+      </c>
+      <c r="I11" s="25" t="n">
         <v>-9.368120286679105e-05</v>
       </c>
-      <c r="I11" s="25" t="n">
+      <c r="J11" s="25" t="n">
         <v>-0.00461581499440511</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>0.001494209936496294</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1544,8 +1544,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
-        <v>45992</v>
+      <c r="N11" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1561,16 +1561,16 @@
         <v>3.3</v>
       </c>
       <c r="R11" s="6" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="S11" s="6" t="n">
-        <v>3.4</v>
-      </c>
       <c r="T11" s="6" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="12">
@@ -1580,8 +1580,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
-        <v>45992</v>
+      <c r="C12" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1594,19 +1594,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>-0.02783872737246302</v>
+        <v>0.01019333843797865</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.006567528263826993</v>
+        <v>-0.02386176631925389</v>
       </c>
       <c r="H12" s="25" t="n">
+        <v>0.008819252239996333</v>
+      </c>
+      <c r="I12" s="25" t="n">
         <v>0.01846374045801518</v>
       </c>
-      <c r="I12" s="25" t="n">
+      <c r="J12" s="25" t="n">
         <v>0.02290259211345895</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>0.03914728682170551</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1619,8 +1619,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
-        <v>45992</v>
+      <c r="N12" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
@@ -1633,19 +1633,19 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R12" s="6" t="n">
         <v>3.3</v>
-      </c>
-      <c r="R12" s="6" t="n">
-        <v>3.2</v>
       </c>
       <c r="S12" s="6" t="n">
         <v>3.2</v>
       </c>
       <c r="T12" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="U12" s="21" t="n">
         <v>3.3</v>
-      </c>
-      <c r="U12" s="21" t="n">
-        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -1659,8 +1659,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
-        <v>45992</v>
+      <c r="C13" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1673,19 +1673,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.002845310871341211</v>
+        <v>-0.0002820635771302316</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.001580090855224148</v>
+        <v>-0.001042547196393295</v>
       </c>
       <c r="H13" s="25" t="n">
+        <v>0.001382579498321101</v>
+      </c>
+      <c r="I13" s="25" t="n">
         <v>0.001469383141654124</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="J13" s="25" t="n">
         <v>-0.00357585313661446</v>
-      </c>
-      <c r="J13" s="25" t="n">
-        <v>0.005207743688441013</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1734,8 +1734,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
-        <v>45992</v>
+      <c r="C14" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1748,19 +1748,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.01357310577859232</v>
+        <v>0.02017730700592953</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.02625112029836067</v>
+        <v>0.01520531470133451</v>
       </c>
       <c r="H14" s="25" t="n">
+        <v>0.02604874382028966</v>
+      </c>
+      <c r="I14" s="25" t="n">
         <v>0.02445440092498914</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="J14" s="25" t="n">
         <v>0.02153393181883783</v>
-      </c>
-      <c r="J14" s="25" t="n">
-        <v>0.03793325150505573</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1813,8 +1813,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
-        <v>45992</v>
+      <c r="C15" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1827,19 +1827,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.003201726937135607</v>
+        <v>0.003326444782829396</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.001180498170227917</v>
+        <v>0.002599007651623797</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.003554081269991682</v>
+        <v>0.0002363292611984313</v>
       </c>
       <c r="I15" s="25" t="n">
+        <v>0.00257898717796845</v>
+      </c>
+      <c r="J15" s="25" t="n">
         <v>0.003374053619106698</v>
-      </c>
-      <c r="J15" s="25" t="n">
-        <v>0.002493308400249195</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1852,7 +1852,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="49" t="n">
+      <c r="N15" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1888,8 +1888,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
-        <v>45992</v>
+      <c r="C16" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1902,19 +1902,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02574422702401932</v>
+        <v>0.02651248191698502</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02586696193462544</v>
+        <v>0.02316609477881844</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02668257801064683</v>
+        <v>0.02390367813311264</v>
       </c>
       <c r="I16" s="25" t="n">
+        <v>0.02568501132750953</v>
+      </c>
+      <c r="J16" s="25" t="n">
         <v>0.0245940671714955</v>
-      </c>
-      <c r="J16" s="25" t="n">
-        <v>0.02312614601653996</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -1939,7 +1939,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
+      <c r="C17" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2026,7 +2026,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
+      <c r="C18" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2105,8 +2105,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
-        <v>45992</v>
+      <c r="C19" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2119,19 +2119,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.0002827474178507261</v>
+        <v>0.00668052913330075</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.001248973066589665</v>
+        <v>-0.0003095975232196846</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>-0.001280636881233477</v>
+        <v>0.001184506215890169</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>0.0005713461581133839</v>
+        <v>-0.001547422988073754</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>0.001005025125628167</v>
+        <v>0.0009791501861489138</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2176,8 +2176,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
-        <v>45992</v>
+      <c r="C20" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2190,19 +2190,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.009195260774909153</v>
+        <v>0.01751836241880857</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01041374906169812</v>
+        <v>0.01200476832755948</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.01147076162937589</v>
+        <v>0.01325386244216132</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.01508168307081075</v>
+        <v>0.01437915836164052</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01547352826862074</v>
+        <v>0.01827247198915003</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2255,8 +2255,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
-        <v>45992</v>
+      <c r="C21" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2269,19 +2269,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2330,7 +2330,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2405,7 +2405,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2479,7 +2479,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
+      <c r="C24" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2518,8 +2518,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
-        <v>45992</v>
+      <c r="N24" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
@@ -2532,19 +2532,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.003558357849066329</v>
+        <v>0.002752400575360525</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.002111370905308885</v>
+        <v>0.003589403456751628</v>
       </c>
       <c r="S24" s="38" t="n">
-        <v>0.001990205680705293</v>
+        <v>0.002205313084075566</v>
       </c>
       <c r="T24" s="38" t="n">
+        <v>0.0019431929480902</v>
+      </c>
+      <c r="U24" s="23" t="n">
         <v>0.002608155986582039</v>
-      </c>
-      <c r="U24" s="23" t="n">
-        <v>0.002622873345935917</v>
       </c>
     </row>
     <row r="25">
@@ -2558,7 +2558,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
+      <c r="C25" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2593,8 +2593,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
-        <v>45992</v>
+      <c r="N25" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
@@ -2607,19 +2607,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.02901287416285929</v>
+        <v>0.02832151941124403</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.02817782841371343</v>
+        <v>0.02909288760511774</v>
       </c>
       <c r="S25" s="38" t="n">
-        <v>0.02719006538467721</v>
+        <v>0.02822596821168675</v>
       </c>
       <c r="T25" s="38" t="n">
+        <v>0.02714187029093776</v>
+      </c>
+      <c r="U25" s="23" t="n">
         <v>0.02787442414870654</v>
-      </c>
-      <c r="U25" s="23" t="n">
-        <v>0.02747620854151709</v>
       </c>
     </row>
     <row r="26">
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.009152775755367104</v>
+        <v>0.005574532321468206</v>
       </c>
       <c r="G26" s="38" t="n">
         <v>0.007794617579222285</v>
@@ -2672,8 +2672,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
-        <v>45992</v>
+      <c r="N26" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2686,19 +2686,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.003553916761463993</v>
+        <v>0.003634828694041303</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.001673844026027105</v>
+        <v>0.003577228118895714</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.002347306898561774</v>
+        <v>0.001791818931981659</v>
       </c>
       <c r="T26" s="38" t="n">
+        <v>0.002292168817051854</v>
+      </c>
+      <c r="U26" s="23" t="n">
         <v>0.001894029073346237</v>
-      </c>
-      <c r="U26" s="23" t="n">
-        <v>0.002246302301668779</v>
       </c>
     </row>
     <row r="27">
@@ -2726,7 +2726,7 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.003824604651284313</v>
+        <v>-0.001337237753545217</v>
       </c>
       <c r="G27" s="38" t="n">
         <v>-0.01832684674964358</v>
@@ -2747,8 +2747,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
-        <v>45992</v>
+      <c r="N27" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2761,19 +2761,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.02996875905826282</v>
+        <v>0.03055696019648922</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.02825865991190849</v>
+        <v>0.03005732873844572</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.02761806318237614</v>
+        <v>0.02832319581807324</v>
       </c>
       <c r="T27" s="38" t="n">
+        <v>0.02756153498288012</v>
+      </c>
+      <c r="U27" s="23" t="n">
         <v>0.02825069249833962</v>
-      </c>
-      <c r="U27" s="23" t="n">
-        <v>0.02912416347215904</v>
       </c>
     </row>
     <row r="28">
@@ -2787,8 +2787,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
-        <v>45992</v>
+      <c r="C28" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2801,19 +2801,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.01358905968147273</v>
+        <v>-0.0004170206674197763</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>-0.009182713803364106</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>0.05441037812530491</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>-0.02093605859677161</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>0.006436255758670795</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>0.03004963172206243</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2862,8 +2862,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
-        <v>45992</v>
+      <c r="C29" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2876,19 +2876,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.1009743287938078</v>
+        <v>0.1030168787238792</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.1058924349271576</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.1247312200873968</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.04877483240471108</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.07412067603746038</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.07661265288383932</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.14</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.11</v>
       </c>
     </row>
     <row r="30">
@@ -2941,8 +2941,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
-        <v>45992</v>
+      <c r="C30" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2955,19 +2955,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.02377629691120575</v>
+        <v>0.004692113383853558</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>-0.0192792268699935</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>0.06592882125886601</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>-0.0128376635658648</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>0.001174064535676367</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>0.01907672443132968</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.36</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -3016,8 +3016,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
-        <v>45992</v>
+      <c r="C31" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3030,19 +3030,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.09596509959750062</v>
+        <v>0.09526923440213324</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.1010137701020375</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.1265306873826442</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.05011084527755218</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.06502168244015354</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.06671073894520346</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3205,7 +3205,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="49" t="n">
+      <c r="N33" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -3281,7 +3281,7 @@
         </is>
       </c>
       <c r="N34" s="48" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
@@ -3294,19 +3294,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>0.008019789135629696</v>
+        <v>0.008545824844536363</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>0.01084249628307491</v>
+        <v>0.007941414156884045</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>0.01169114908209064</v>
+        <v>0.01079517034980899</v>
       </c>
       <c r="T34" s="38" t="n">
+        <v>0.01173861920396547</v>
+      </c>
+      <c r="U34" s="23" t="n">
         <v>0.01032118383222275</v>
-      </c>
-      <c r="U34" s="23" t="n">
-        <v>0.01194571058798364</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="N35" s="48" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
@@ -3373,19 +3373,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.00300711691046418</v>
+        <v>0.001295896455863144</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.001955057552418982</v>
+        <v>-0.003037958457621781</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>0.002092822632293601</v>
+        <v>0.001861138831470432</v>
       </c>
       <c r="T35" s="38" t="n">
+        <v>0.002139842385766366</v>
+      </c>
+      <c r="U35" s="23" t="n">
         <v>-0.0004224555765300897</v>
-      </c>
-      <c r="U35" s="23" t="n">
-        <v>0.001486198108683112</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="N36" s="48" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
@@ -3448,19 +3448,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>0.008019789135629696</v>
+        <v>0.008545824844536363</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>0.01084249628307491</v>
+        <v>0.007941414156884045</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>0.01169114908209064</v>
+        <v>0.01079517034980899</v>
       </c>
       <c r="T36" s="38" t="n">
+        <v>0.01173861920396547</v>
+      </c>
+      <c r="U36" s="23" t="n">
         <v>0.01032118383222275</v>
-      </c>
-      <c r="U36" s="23" t="n">
-        <v>0.01194571058798364</v>
       </c>
     </row>
     <row r="37">
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5346.421</v>
+        <v>5341.129</v>
       </c>
       <c r="G44" s="24" t="n">
         <v>5324.402</v>
@@ -4084,7 +4084,7 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.004135487891410161</v>
+        <v>0.003141573457451141</v>
       </c>
       <c r="G45" s="38" t="n">
         <v>0.01669515005814426</v>
@@ -4121,8 +4121,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
-        <v>45992</v>
+      <c r="C46" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -4135,19 +4135,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>287287</v>
+        <v>302149</v>
       </c>
       <c r="G46" s="24" t="n">
-        <v>292290</v>
+        <v>286301</v>
       </c>
       <c r="H46" s="24" t="n">
-        <v>302594</v>
+        <v>290906</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>293901</v>
+        <v>301177</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>283736</v>
+        <v>293804</v>
       </c>
       <c r="K46" s="5" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4208,8 +4208,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
-        <v>45992</v>
+      <c r="C47" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4222,19 +4222,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>-0.01711656231824554</v>
+        <v>0.05535432988358413</v>
       </c>
       <c r="G47" s="38" t="n">
-        <v>-0.03405222839844813</v>
+        <v>-0.01582985569221673</v>
       </c>
       <c r="H47" s="38" t="n">
-        <v>0.02957798714533122</v>
+        <v>-0.03410286974104926</v>
       </c>
       <c r="I47" s="38" t="n">
-        <v>0.03582555615078808</v>
+        <v>0.02509496126669486</v>
       </c>
       <c r="J47" s="38" t="n">
-        <v>0.0004866042778863822</v>
+        <v>0.03326956081366239</v>
       </c>
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4287,8 +4287,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
-        <v>45992</v>
+      <c r="C48" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4301,19 +4301,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>357598</v>
+        <v>356604</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>345334</v>
+        <v>359201</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>331343</v>
+        <v>346932</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>341582</v>
+        <v>332279</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>338909</v>
+        <v>342972</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.57</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>3.56</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>3.56</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>3.57</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.54</v>
       </c>
     </row>
     <row r="49">
@@ -4362,8 +4362,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
-        <v>45992</v>
+      <c r="C49" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4376,19 +4376,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.0355134449547394</v>
+        <v>-0.007229935328687875</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>0.04222512622871166</v>
+        <v>0.03536427887885818</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>-0.02997523288697879</v>
+        <v>0.04409848350332091</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>0.007887072931081818</v>
+        <v>-0.03117747221347511</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>-0.05210885495329198</v>
+        <v>0.007689030571021327</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.71</v>
-      </c>
-      <c r="S49" s="6" t="n">
-        <v>3.72</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>3.72</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>3.67</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="50">
@@ -4441,8 +4441,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
-        <v>45992</v>
+      <c r="C50" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4455,19 +4455,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>29018</v>
+        <v>27336</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>30597</v>
+        <v>26347</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>29777</v>
+        <v>27608</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>30169</v>
+        <v>27476</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>30416</v>
+        <v>28592</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.12</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.09</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4516,8 +4516,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
-        <v>45992</v>
+      <c r="C51" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4530,19 +4530,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>-0.05160636663725204</v>
+        <v>0.03753748054806993</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>0.02753803270980959</v>
+        <v>-0.04567516661837145</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>-0.01299347011833341</v>
+        <v>0.004804192750036407</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>-0.008120725933719042</v>
+        <v>-0.03903189703413545</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>0.06327343913864225</v>
+        <v>-0.03349896900246763</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4555,8 +4555,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46083</v>
+      <c r="N51" s="49" t="n">
+        <v>46090</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4569,19 +4569,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>5.98</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.01</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.09</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.11</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.92</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>5.9</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>5.9</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>5.89</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.83</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.12</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.14</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.36</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.64</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.57</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.56</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.56</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.57</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,16 +4415,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.71</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>3.72</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>3.72</v>
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.12</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.15</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.92</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>5.9</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>5.9</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>5.89</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -3095,8 +3095,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
-        <v>46023</v>
+      <c r="C32" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3109,19 +3109,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.007001897085101128</v>
+        <v>0.001510796776836631</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.002486745086434317</v>
+        <v>0.007063467944424584</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>0.001190041182338009</v>
+        <v>0.003133370494423415</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>-0.004413706579460941</v>
+        <v>0.001511745671022524</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>0.0007990183488855163</v>
+        <v>-0.004529448794114321</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3166,8 +3166,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
-        <v>46023</v>
+      <c r="C33" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3180,19 +3180,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.02275028056847218</v>
+        <v>0.01435914986552827</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01298051477514099</v>
+        <v>0.02330092430197657</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.02099856484628742</v>
+        <v>0.01346393254876795</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01797033261452011</v>
+        <v>0.02082735352619783</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.01901142589200902</v>
+        <v>0.01747269263442562</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3245,8 +3245,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46023</v>
+      <c r="C34" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3259,19 +3259,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.2119</v>
+        <v>76.2946</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>75.7433</v>
+        <v>76.2529</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.64619999999999</v>
+        <v>75.7794</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.6474</v>
+        <v>75.63339999999999</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>76.0745</v>
+        <v>75.6104</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>

</xml_diff>

<commit_message>
Update dashboards - 2026-03-17
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1078,8 +1078,10 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
-        <v>46054</v>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1092,19 +1094,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>63000</v>
+        <v>1</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>11000</v>
+        <v>1</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>37000</v>
+        <v>1</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>74000</v>
+        <v>1</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>20000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1153,8 +1155,10 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
-        <v>46054</v>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'UNRATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1167,19 +1171,19 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="S6" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="T6" s="6" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="U6" s="21" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1232,8 +1236,10 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46054</v>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1246,19 +1252,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>8.4</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8.699999999999999</v>
+        <v>1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1311,8 +1317,10 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
-        <v>46054</v>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
+        </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1325,19 +1333,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>62.1</v>
+        <v>1</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>62.4</v>
+        <v>1</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>62.5</v>
+        <v>1</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1390,8 +1398,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46054</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1404,19 +1414,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.6</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2105,8 +2115,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="49" t="n">
-        <v>46023</v>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2119,19 +2131,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>0.00668052913330075</v>
+        <v>1</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>-0.0003095975232196846</v>
+        <v>1</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>0.001184506215890169</v>
+        <v>1</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>-0.001547422988073754</v>
+        <v>1</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>0.0009791501861489138</v>
+        <v>1</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2176,8 +2188,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n">
-        <v>46023</v>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2190,19 +2204,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.01751836241880857</v>
+        <v>1</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01200476832755948</v>
+        <v>1</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.01325386244216132</v>
+        <v>1</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.01437915836164052</v>
+        <v>1</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01827247198915003</v>
+        <v>1</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2255,8 +2269,10 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n">
-        <v>46023</v>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
+        </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2269,19 +2285,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2330,8 +2346,10 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
-        <v>46054</v>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
+        </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2344,19 +2362,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.118</v>
+        <v>1</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>15.209</v>
+        <v>1</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.401</v>
+        <v>1</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.006</v>
+        <v>1</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>15.843</v>
+        <v>1</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2369,8 +2387,10 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46023</v>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
+        </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2383,19 +2403,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.00480699391202144</v>
+        <v>1</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.004303799147197918</v>
+        <v>1</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.00248632190555953</v>
+        <v>1</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.001184731605045064</v>
+        <v>1</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.006147582151921682</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2405,8 +2425,10 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
-        <v>46054</v>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
+        </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2419,19 +2441,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.01833241975759802</v>
+        <v>1</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.04645768025078368</v>
+        <v>1</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.0520201144442517</v>
+        <v>1</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>-0.05334752779749237</v>
+        <v>1</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.03941065906748309</v>
+        <v>1</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2439,8 +2461,10 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46023</v>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
+        </is>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2453,19 +2477,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.02837641493495531</v>
+        <v>1</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.02988058645921175</v>
+        <v>1</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.02970357876911097</v>
+        <v>1</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.02822398731321852</v>
+        <v>1</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.03046576545064236</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -2826,8 +2850,10 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
-        <v>46023</v>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'MICH' not found in values file."</t>
+        </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2840,19 +2866,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2902,7 +2928,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2941,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.11</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.13</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +3007,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,16 +3023,16 @@
         <v>2.36</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.36</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -3809,8 +3835,10 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
-        <v>46023</v>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'IQ' not found in values file."</t>
+        </is>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3823,19 +3851,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.006468305304010435</v>
+        <v>1</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v>0.005855562784645496</v>
+        <v>1</v>
       </c>
       <c r="S41" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="T41" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U41" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -3884,8 +3912,10 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
-        <v>46023</v>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'IQ' not found in values file."</t>
+        </is>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3898,19 +3928,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.02638522427440633</v>
+        <v>1</v>
       </c>
       <c r="R42" s="38" t="n">
-        <v>0.0341137123745819</v>
+        <v>1</v>
       </c>
       <c r="S42" s="38" t="n">
-        <v>0.03293010752688157</v>
+        <v>1</v>
       </c>
       <c r="T42" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U42" s="23" t="n">
-        <v>0.03869653767820766</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -3959,8 +3989,10 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
-        <v>46023</v>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'IR' not found in values file."</t>
+        </is>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3973,19 +4005,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.002121640735502028</v>
+        <v>1</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>0.002126151665485576</v>
+        <v>1</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="T43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U43" s="23" t="n">
-        <v>-0.001418439716311948</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -4034,8 +4066,10 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
-        <v>46023</v>
+      <c r="N44" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'IR' not found in values file."</t>
+        </is>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4048,19 +4082,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>-0.0007052186177716695</v>
+        <v>1</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S44" s="38" t="n">
-        <v>-0.001415428167020644</v>
+        <v>1</v>
       </c>
       <c r="T44" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U44" s="23" t="n">
-        <v>-0.0007097232079488595</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -4248,7 +4282,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4287,8 +4321,10 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
-        <v>46023</v>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
+        </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4301,19 +4337,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>356604</v>
+        <v>1</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>359201</v>
+        <v>1</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>346932</v>
+        <v>1</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>332279</v>
+        <v>1</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>342972</v>
+        <v>1</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4327,7 +4363,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,16 +4376,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.76</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.64</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.57</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>3.56</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>3.56</v>
@@ -4362,8 +4398,10 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
-        <v>46023</v>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
+        </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4376,19 +4414,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>-0.007229935328687875</v>
+        <v>1</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>0.03536427887885818</v>
+        <v>1</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>0.04409848350332091</v>
+        <v>1</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>-0.03117747221347511</v>
+        <v>1</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>0.007689030571021327</v>
+        <v>1</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4402,7 +4440,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4453,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.71</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.72</v>
       </c>
     </row>
     <row r="50">
@@ -4441,8 +4479,10 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
-        <v>46023</v>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
+        </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4455,19 +4495,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>27336</v>
+        <v>1</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>26347</v>
+        <v>1</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>27608</v>
+        <v>1</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>27476</v>
+        <v>1</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>28592</v>
+        <v>1</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4481,7 +4521,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4534,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.12</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.15</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4516,8 +4556,10 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
-        <v>46023</v>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
+        </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4530,19 +4572,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.03753748054806993</v>
+        <v>1</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>-0.04567516661837145</v>
+        <v>1</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>0.004804192750036407</v>
+        <v>1</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>-0.03903189703413545</v>
+        <v>1</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>-0.03349896900246763</v>
+        <v>1</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4607,7 +4649,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4623,13 +4665,13 @@
         <v>6.11</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.92</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>5.9</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>5.9</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-03-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1078,10 +1078,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
-        </is>
+      <c r="N5" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1094,19 +1092,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>1</v>
+        <v>63000</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>1</v>
+        <v>11000</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>1</v>
+        <v>37000</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>1</v>
+        <v>74000</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>1</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="6">
@@ -1155,10 +1153,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'UNRATE' not found in values file."</t>
-        </is>
+      <c r="N6" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1171,19 +1167,19 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="S6" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="T6" s="6" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="U6" s="21" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1236,10 +1232,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
-        </is>
+      <c r="N7" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1252,19 +1246,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>8.1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>8.4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1317,10 +1311,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
-        </is>
+      <c r="N8" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1333,19 +1325,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>1</v>
+        <v>62.1</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>1</v>
+        <v>62.4</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>1</v>
+        <v>62.5</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1398,10 +1390,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1414,19 +1404,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.6</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -2075,7 +2065,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
+      <c r="N18" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2115,10 +2105,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C19" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2131,19 +2119,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>1</v>
+        <v>0.00668052913330075</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>1</v>
+        <v>-0.0003095975232196846</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>1</v>
+        <v>0.001184506215890169</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>1</v>
+        <v>-0.001547422988073754</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>1</v>
+        <v>0.0009791501861489138</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2152,7 +2140,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2188,10 +2176,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C20" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2204,19 +2190,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>1</v>
+        <v>0.01751836241880857</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>1</v>
+        <v>0.01200476832755948</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>1</v>
+        <v>0.01325386244216132</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>1</v>
+        <v>0.01437915836164052</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>1</v>
+        <v>0.01827247198915003</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2229,7 +2215,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
+      <c r="N20" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2269,10 +2255,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
-        </is>
+      <c r="C21" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2285,19 +2269,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2306,7 +2290,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
+      <c r="N21" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2346,10 +2330,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
-        </is>
+      <c r="C22" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2362,19 +2344,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>1</v>
+        <v>16.118</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>1</v>
+        <v>15.209</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>1</v>
+        <v>16.401</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>1</v>
+        <v>16.006</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>1</v>
+        <v>15.843</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2387,10 +2369,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
-        </is>
+      <c r="N22" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2403,19 +2383,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>1</v>
+        <v>0.006840134042972679</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>1</v>
+        <v>0.005264444194909901</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>1</v>
+        <v>0.003805886526233593</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>1</v>
+        <v>0.002525940746747724</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>1</v>
+        <v>0.001291224333588303</v>
       </c>
     </row>
     <row r="23">
@@ -2425,10 +2405,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
-        </is>
+      <c r="C23" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2441,19 +2419,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>1</v>
+        <v>-0.01833241975759802</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>1</v>
+        <v>-0.04645768025078368</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>1</v>
+        <v>-0.0520201144442517</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>1</v>
+        <v>-0.05334752779749237</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>1</v>
+        <v>-0.03941065906748309</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2461,10 +2439,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
-        </is>
+      <c r="N23" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2477,19 +2453,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>1</v>
+        <v>0.03371718848029785</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>1</v>
+        <v>0.02848454130765334</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>1</v>
+        <v>0.0295201697358758</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>1</v>
+        <v>0.02985380376518458</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>1</v>
+        <v>0.02833335611850097</v>
       </c>
     </row>
     <row r="24">
@@ -2811,7 +2787,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="49" t="n">
+      <c r="C28" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2825,10 +2801,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.0004170206674197763</v>
+        <v>-8.71345793578282e-05</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.009182713803364106</v>
+        <v>-0.00913646104747079</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>0.05441037812530491</v>
@@ -2850,10 +2826,8 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'MICH' not found in values file."</t>
-        </is>
+      <c r="N28" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2866,19 +2840,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>1</v>
+        <v>4.6</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="29">
@@ -2888,7 +2862,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="49" t="n">
+      <c r="C29" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2902,10 +2876,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.1030168787238792</v>
+        <v>0.103432407836673</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.1058924349271576</v>
+        <v>0.1059440595541697</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.1247312200873968</v>
@@ -2928,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2941,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.11</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.14</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.13</v>
       </c>
     </row>
     <row r="30">
@@ -2967,7 +2941,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="49" t="n">
+      <c r="C30" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2981,10 +2955,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.004692113383853558</v>
+        <v>0.005088320854118145</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>-0.0192792268699935</v>
+        <v>-0.01921059426035288</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>0.06592882125886601</v>
@@ -3007,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3020,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.36</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -3042,7 +3016,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="49" t="n">
+      <c r="C31" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3056,10 +3030,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.09526923440213324</v>
+        <v>0.09577784074808728</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.1010137701020375</v>
+        <v>0.1010908210327026</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>0.1265306873826442</v>
@@ -3835,10 +3809,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'IQ' not found in values file."</t>
-        </is>
+      <c r="N41" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3851,19 +3823,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>1</v>
+        <v>0.006468305304010435</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v>1</v>
+        <v>0.005855562784645496</v>
       </c>
       <c r="S41" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="T41" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="U41" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -3912,10 +3884,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'IQ' not found in values file."</t>
-        </is>
+      <c r="N42" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3928,19 +3898,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>1</v>
+        <v>0.02638522427440633</v>
       </c>
       <c r="R42" s="38" t="n">
-        <v>1</v>
+        <v>0.0341137123745819</v>
       </c>
       <c r="S42" s="38" t="n">
-        <v>1</v>
+        <v>0.03293010752688157</v>
       </c>
       <c r="T42" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="U42" s="23" t="n">
-        <v>1</v>
+        <v>0.03869653767820766</v>
       </c>
     </row>
     <row r="43">
@@ -3989,10 +3959,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'IR' not found in values file."</t>
-        </is>
+      <c r="N43" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -4005,19 +3973,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>1</v>
+        <v>0.002121640735502028</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>1</v>
+        <v>0.002126151665485576</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="T43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="U43" s="23" t="n">
-        <v>1</v>
+        <v>-0.001418439716311948</v>
       </c>
     </row>
     <row r="44">
@@ -4066,10 +4034,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'IR' not found in values file."</t>
-        </is>
+      <c r="N44" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4082,19 +4048,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>1</v>
+        <v>-0.0007052186177716695</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S44" s="38" t="n">
-        <v>1</v>
+        <v>-0.001415428167020644</v>
       </c>
       <c r="T44" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="U44" s="23" t="n">
-        <v>1</v>
+        <v>-0.0007097232079488595</v>
       </c>
     </row>
     <row r="45">
@@ -4282,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4321,10 +4287,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
-        </is>
+      <c r="C48" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4337,19 +4301,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>1</v>
+        <v>356604</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>1</v>
+        <v>359201</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>1</v>
+        <v>346932</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>1</v>
+        <v>332279</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>1</v>
+        <v>342972</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4363,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4376,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.76</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.64</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.57</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.56</v>
       </c>
     </row>
     <row r="49">
@@ -4398,10 +4362,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
-        </is>
+      <c r="C49" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4414,19 +4376,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>1</v>
+        <v>-0.007229935328687875</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>1</v>
+        <v>0.03536427887885818</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>1</v>
+        <v>0.04409848350332091</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>1</v>
+        <v>-0.03117747221347511</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>1</v>
+        <v>0.007689030571021327</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4440,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4453,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.73</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.71</v>
       </c>
     </row>
     <row r="50">
@@ -4479,10 +4441,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
-        </is>
+      <c r="C50" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4495,19 +4455,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>1</v>
+        <v>27336</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>1</v>
+        <v>26347</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>1</v>
+        <v>27608</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>1</v>
+        <v>27476</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>1</v>
+        <v>28592</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4521,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4534,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.28</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.15</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.12</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4556,10 +4516,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
-        </is>
+      <c r="C51" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4572,19 +4530,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>1</v>
+        <v>0.03753748054806993</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>1</v>
+        <v>-0.04567516661837145</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>1</v>
+        <v>0.004804192750036407</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>1</v>
+        <v>-0.03903189703413545</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>1</v>
+        <v>-0.03349896900246763</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4649,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4662,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.11</v>
+        <v>6.08</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.11</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.92</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.9</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-19
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N13" s="49" t="n">
-        <v>46083</v>
+        <v>46090</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1712,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
+        <v>205000</v>
+      </c>
+      <c r="R13" s="24" t="n">
         <v>213000</v>
       </c>
-      <c r="R13" s="24" t="n">
+      <c r="S13" s="24" t="n">
         <v>214000</v>
       </c>
-      <c r="S13" s="24" t="n">
-        <v>213000</v>
-      </c>
       <c r="T13" s="24" t="n">
+        <v>211000</v>
+      </c>
+      <c r="U13" s="26" t="n">
         <v>208000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>229000</v>
       </c>
     </row>
     <row r="14">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46076</v>
+        <v>46083</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1850000</v>
+        <v>1857000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1847000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1871000</v>
       </c>
-      <c r="S14" s="24" t="n">
-        <v>1822000</v>
-      </c>
       <c r="T14" s="24" t="n">
-        <v>1864000</v>
+        <v>1827000</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1852000</v>
+        <v>1865000</v>
       </c>
     </row>
     <row r="15">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.11</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.13</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.14</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.37</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.38</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -3399,7 +3399,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="49" t="n">
+      <c r="C36" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3470,7 +3470,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n">
+      <c r="C37" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3549,7 +3549,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="49" t="n">
+      <c r="C38" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3620,7 +3620,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="49" t="n">
+      <c r="C39" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3699,8 +3699,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
-        <v>45992</v>
+      <c r="C40" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -3713,19 +3713,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>745</v>
+        <v>587</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>758</v>
+        <v>712</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>656</v>
+        <v>764</v>
       </c>
       <c r="I40" s="24" t="n">
+        <v>650</v>
+      </c>
+      <c r="J40" s="24" t="n">
         <v>719</v>
-      </c>
-      <c r="J40" s="24" t="n">
-        <v>706</v>
       </c>
       <c r="K40" s="5" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3770,8 +3770,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
-        <v>45992</v>
+      <c r="C41" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
@@ -3784,19 +3784,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>0.03760445682451254</v>
+        <v>-0.1132930513595166</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>0.122962962962963</v>
+        <v>-0.008356545961002786</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>0.05636070853462158</v>
+        <v>0.1318518518518519</v>
       </c>
       <c r="I41" s="38" t="n">
+        <v>0.04669887278582931</v>
+      </c>
+      <c r="J41" s="38" t="n">
         <v>0.002789400278940028</v>
-      </c>
-      <c r="J41" s="38" t="n">
-        <v>0.01875901875901876</v>
       </c>
       <c r="K41" s="5" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4121,7 +4121,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
+      <c r="C46" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4208,7 +4208,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
+      <c r="C47" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4287,7 +4287,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
+      <c r="C48" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4343,16 +4343,16 @@
         <v>3.68</v>
       </c>
       <c r="R48" s="6" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="S48" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.76</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.64</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.57</v>
       </c>
     </row>
     <row r="49">
@@ -4362,7 +4362,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
+      <c r="C49" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.8</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.79</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.73</v>
       </c>
     </row>
     <row r="50">
@@ -4441,7 +4441,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
+      <c r="C50" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.23</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.28</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.15</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4516,7 +4516,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
+      <c r="C51" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4555,7 +4555,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46090</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.08</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.11</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.11</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.05</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.92</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-20
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1465,7 +1465,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
+      <c r="N10" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1505,7 +1505,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n">
+      <c r="C11" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1544,7 +1544,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1580,7 +1580,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="49" t="n">
+      <c r="C12" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1619,7 +1619,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1659,7 +1659,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="49" t="n">
+      <c r="C13" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1734,7 +1734,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1813,7 +1813,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1888,7 +1888,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2105,7 +2105,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="49" t="n">
+      <c r="C19" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2176,7 +2176,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2255,7 +2255,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n">
+      <c r="C21" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2518,7 +2518,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="49" t="n">
+      <c r="N24" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2593,7 +2593,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="49" t="n">
+      <c r="N25" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2672,7 +2672,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="49" t="n">
+      <c r="N26" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2747,7 +2747,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="49" t="n">
+      <c r="N27" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.11</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.13</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.37</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.68</v>
+        <v>3.76</v>
       </c>
       <c r="R48" s="6" t="n">
         <v>3.68</v>
       </c>
       <c r="S48" s="6" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="T48" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.76</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.64</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.8</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.88</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.79</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.23</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.28</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,8 +4555,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46090</v>
+      <c r="N51" s="49" t="n">
+        <v>46097</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4569,19 +4569,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.11</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>5.98</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.01</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.09</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.08</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.11</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.11</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.05</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-21
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2918,16 +2918,16 @@
         <v>2.13</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.14</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.11</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,16 +2994,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.37</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.37</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.36</v>
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.76</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>3.68</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>3.68</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>3.73</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.76</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.8</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.87</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.88</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.23</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.28</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,16 +4620,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.07</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.08</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.11</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.11</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-03-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7872517.5</v>
+        <v>7860620.8</v>
       </c>
       <c r="G5" s="24" t="n">
         <v>7774506.8</v>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.01260667750653965</v>
+        <v>0.01107645825198844</v>
       </c>
       <c r="G6" s="25" t="n">
         <v>0.02008474181421249</v>
@@ -3095,7 +3095,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="49" t="n">
+      <c r="C32" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3166,7 +3166,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="49" t="n">
+      <c r="C33" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3245,7 +3245,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="49" t="n">
+      <c r="C34" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-24
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2921,13 +2921,13 @@
         <v>2.13</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.12</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.14</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.37</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.37</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -3334,7 +3334,7 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="G35" s="41" t="n">
         <v>5.2</v>
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.76</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.68</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.68</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.73</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.8</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.87</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.25</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.23</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.28</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.07</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.08</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.11</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-25
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2369,7 +2369,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2439,7 +2439,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,7 +2915,7 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.13</v>
@@ -2924,10 +2924,10 @@
         <v>2.13</v>
       </c>
       <c r="T29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.14</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,16 +2997,16 @@
         <v>2.33</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.37</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.4</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -3809,8 +3809,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
-        <v>46023</v>
+      <c r="N41" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3823,19 +3823,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
+        <v>0.01542416452442152</v>
+      </c>
+      <c r="R41" s="38" t="n">
         <v>0.006468305304010435</v>
       </c>
-      <c r="R41" s="38" t="n">
+      <c r="S41" s="38" t="n">
         <v>0.005855562784645496</v>
-      </c>
-      <c r="S41" s="38" t="n">
-        <v/>
       </c>
       <c r="T41" s="38" t="n">
         <v/>
       </c>
       <c r="U41" s="23" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -3884,8 +3884,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
-        <v>46023</v>
+      <c r="N42" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3898,19 +3898,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
+        <v>0.03538663171690699</v>
+      </c>
+      <c r="R42" s="38" t="n">
         <v>0.02638522427440633</v>
       </c>
-      <c r="R42" s="38" t="n">
+      <c r="S42" s="38" t="n">
         <v>0.0341137123745819</v>
       </c>
-      <c r="S42" s="38" t="n">
+      <c r="T42" s="38" t="n">
         <v>0.03293010752688157</v>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v/>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.03869653767820766</v>
       </c>
     </row>
     <row r="43">
@@ -3959,8 +3959,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
-        <v>46023</v>
+      <c r="N43" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3973,19 +3973,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.002121640735502028</v>
+        <v>0.01265822784810133</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>0.002126151665485576</v>
+        <v>0.005657708628005631</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v/>
+        <v>0.00141643059490093</v>
       </c>
       <c r="T43" s="38" t="n">
         <v/>
       </c>
       <c r="U43" s="23" t="n">
-        <v>-0.001418439716311948</v>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -4034,8 +4034,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
-        <v>46023</v>
+      <c r="N44" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4048,19 +4048,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>-0.0007052186177716695</v>
+        <v>0.0133708655876144</v>
       </c>
       <c r="R44" s="38" t="n">
+        <v>0.002820874471085876</v>
+      </c>
+      <c r="S44" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="S44" s="38" t="n">
-        <v>-0.001415428167020644</v>
-      </c>
       <c r="T44" s="38" t="n">
+        <v>-0.0007077140835104227</v>
+      </c>
+      <c r="U44" s="23" t="n">
         <v/>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>-0.0007097232079488595</v>
       </c>
     </row>
     <row r="45">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,16 +4340,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.76</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>3.68</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>3.68</v>
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.01</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.79</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.8</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.25</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.2</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.23</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.18</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.07</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.05</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.08</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-26
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1698,7 +1698,7 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
+      <c r="N13" s="48" t="n">
         <v>46090</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1773,7 +1773,7 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
+      <c r="N14" s="48" t="n">
         <v>46083</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2918,7 +2918,7 @@
         <v>2.11</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.13</v>
@@ -2927,7 +2927,7 @@
         <v>2.13</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.33</v>
+        <v>2.31</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.33</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.37</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.4</v>
       </c>
     </row>
     <row r="31">
@@ -3699,7 +3699,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n">
+      <c r="C40" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3770,7 +3770,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n">
+      <c r="C41" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.83</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.76</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.68</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.01</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.87</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.79</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.34</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.25</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.2</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,7 +4555,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46097</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.13</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.18</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.07</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.05</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1698,8 +1698,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="48" t="n">
-        <v>46090</v>
+      <c r="N13" s="49" t="n">
+        <v>46097</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1712,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
+        <v>210000</v>
+      </c>
+      <c r="R13" s="24" t="n">
         <v>205000</v>
       </c>
-      <c r="R13" s="24" t="n">
+      <c r="S13" s="24" t="n">
         <v>213000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>214000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>211000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>208000</v>
       </c>
     </row>
     <row r="14">
@@ -1773,8 +1773,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="48" t="n">
-        <v>46083</v>
+      <c r="N14" s="49" t="n">
+        <v>46090</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1857000</v>
+        <v>1819000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1851000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1847000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1871000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1827000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1865000</v>
       </c>
     </row>
     <row r="15">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,13 +2915,13 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.11</v>
       </c>
       <c r="S29" s="6" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.13</v>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.31</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.33</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.33</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.38</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.9</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.83</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.76</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.03</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.01</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.88</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.87</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.34</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.25</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,8 +4555,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46097</v>
+      <c r="N51" s="49" t="n">
+        <v>46104</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4569,19 +4569,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.22</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.11</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>5.98</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.01</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.13</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.18</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.06</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.07</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="N28" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2840,19 +2840,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="R28" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="R28" s="6" t="n">
+      <c r="S28" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="S28" s="6" t="n">
+      <c r="T28" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="T28" s="6" t="n">
+      <c r="U28" s="21" t="n">
         <v>4.6</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>4.7</v>
       </c>
     </row>
     <row r="29">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,16 +2915,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.12</v>
-      </c>
-      <c r="R29" s="6" t="n">
-        <v>2.11</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.11</v>
       </c>
       <c r="T29" s="6" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.13</v>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.31</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.33</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.33</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.38</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -3563,7 +3563,7 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1376</v>
+        <v>1386</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1455</v>
@@ -3634,7 +3634,7 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.05753424657534247</v>
+        <v>-0.05068493150684932</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>-0.01689189189189189</v>
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.9</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.83</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.88</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.79</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.96</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.03</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.01</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.88</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.34</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.39</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.25</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.09</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.13</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.18</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.06</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-03-31
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1465,8 +1465,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
-        <v>46023</v>
+      <c r="N10" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1482,13 +1482,13 @@
         <v>4.2</v>
       </c>
       <c r="R10" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S10" s="6" t="n">
+      <c r="T10" s="6" t="n">
         <v>4.1</v>
-      </c>
-      <c r="T10" s="6" t="n">
-        <v>4.3</v>
       </c>
       <c r="U10" s="21" t="n">
         <v>4.3</v>
@@ -1544,8 +1544,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
-        <v>46023</v>
+      <c r="N11" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1558,16 +1558,16 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>3.3</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="S11" s="6" t="n">
+      <c r="T11" s="6" t="n">
         <v>3.2</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>3.3</v>
       </c>
       <c r="U11" s="21" t="n">
         <v>3.3</v>
@@ -1619,8 +1619,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
-        <v>46023</v>
+      <c r="N12" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
@@ -1633,19 +1633,19 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="R12" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="R12" s="6" t="n">
+      <c r="S12" s="6" t="n">
         <v>3.3</v>
-      </c>
-      <c r="S12" s="6" t="n">
-        <v>3.2</v>
       </c>
       <c r="T12" s="6" t="n">
         <v>3.2</v>
       </c>
       <c r="U12" s="21" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -2255,8 +2255,10 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
-        <v>46023</v>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
+        </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2269,19 +2271,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2330,8 +2332,10 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
-        <v>46054</v>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
+        </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2344,19 +2348,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.118</v>
+        <v>1</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>15.209</v>
+        <v>1</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.401</v>
+        <v>1</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.006</v>
+        <v>1</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>15.843</v>
+        <v>1</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2405,8 +2409,10 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
-        <v>46054</v>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
+        </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2419,19 +2425,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.01833241975759802</v>
+        <v>1</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.04645768025078368</v>
+        <v>1</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.0520201144442517</v>
+        <v>1</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>-0.05334752779749237</v>
+        <v>1</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.03941065906748309</v>
+        <v>1</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2902,7 +2908,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2921,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.06</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.12</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <v>2.11</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.11</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2987,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,13 +3003,13 @@
         <v>2.31</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.31</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.33</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.33</v>
@@ -3509,8 +3515,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
-        <v>45992</v>
+      <c r="N37" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3523,19 +3529,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>-0.00273486156666769</v>
+        <v>-0.001091846627661819</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>-0.0006239385435752309</v>
+        <v>-0.002556382261513668</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>-0.001255429809922437</v>
+        <v>-0.001313071612671246</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.002710199627120158</v>
+        <v>-0.001955114463894181</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.003326625695690755</v>
+        <v>-0.002952812599475663</v>
       </c>
     </row>
     <row r="38">
@@ -3584,8 +3590,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
-        <v>45992</v>
+      <c r="N38" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3598,19 +3604,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.01272340965111129</v>
+        <v>0.009101975493255475</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.01427415269420379</v>
+        <v>0.01130167174427415</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.01402408537902678</v>
+        <v>0.01269705928692578</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01316616157883059</v>
+        <v>0.01313965942447244</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01475691239986718</v>
+        <v>0.01298257285949245</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -4248,7 +4254,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4333,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4346,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.96</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.9</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.83</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.88</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4408,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4421,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.08</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.96</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.03</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.95</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.01</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4487,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4500,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.42</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.34</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.39</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4613,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4626,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.15</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.09</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.13</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.18</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1078,8 +1078,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
-        <v>46054</v>
+      <c r="N5" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1092,19 +1092,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>63000</v>
+        <v>62000</v>
       </c>
       <c r="R5" s="24" t="n">
+        <v>66000</v>
+      </c>
+      <c r="S5" s="24" t="n">
         <v>11000</v>
       </c>
-      <c r="S5" s="24" t="n">
+      <c r="T5" s="24" t="n">
         <v>37000</v>
       </c>
-      <c r="T5" s="24" t="n">
+      <c r="U5" s="26" t="n">
         <v>74000</v>
-      </c>
-      <c r="U5" s="26" t="n">
-        <v>20000</v>
       </c>
     </row>
     <row r="6">
@@ -1272,8 +1272,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
-        <v>45992</v>
+      <c r="C8" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1286,19 +1286,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>0.8</v>
+        <v>0.48</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>0.62</v>
+        <v>0.2</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>0.86</v>
+        <v>0.24</v>
       </c>
       <c r="I8" s="24" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J8" s="24" t="n">
         <v>0.82</v>
-      </c>
-      <c r="J8" s="24" t="n">
-        <v>0.88</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1939,8 +1939,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
-        <v>46023</v>
+      <c r="C17" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1953,19 +1953,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>-0.0015625744366633</v>
+        <v>0.00600990523942202</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>-4.49151919511559e-05</v>
+        <v>-0.001037134025754116</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>-1.361066422789214e-06</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>0.005016065910586232</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>-0.001558334425942887</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>0.0006724067240673204</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2026,8 +2026,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
-        <v>46023</v>
+      <c r="C18" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2040,19 +2040,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.03155977752620958</v>
+        <v>0.03714451864108709</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.02428670017357602</v>
+        <v>0.0319081629783764</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.02433131408893505</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.03212039564348258</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.03213514238518121</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.04144341481107452</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2255,10 +2255,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
-        </is>
+      <c r="C21" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2271,19 +2269,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2332,10 +2330,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
-        </is>
+      <c r="C22" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2348,19 +2344,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>1</v>
+        <v>16.118</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>1</v>
+        <v>15.209</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>1</v>
+        <v>16.401</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>1</v>
+        <v>16.006</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>1</v>
+        <v>15.843</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2409,10 +2405,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TOTALSA' not found in values file."</t>
-        </is>
+      <c r="C23" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2425,19 +2419,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>1</v>
+        <v>-0.01833241975759802</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>1</v>
+        <v>-0.04645768025078368</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>1</v>
+        <v>-0.0520201144442517</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>1</v>
+        <v>-0.05334752779749237</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>1</v>
+        <v>-0.03941065906748309</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2908,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2921,16 +2915,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.05</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.06</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.12</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.11</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.11</v>
@@ -2987,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3000,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.31</v>
+        <v>2.3</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.31</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -3815,7 +3809,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3890,7 +3884,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="49" t="n">
+      <c r="N42" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3965,7 +3959,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4040,7 +4034,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4254,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4333,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4346,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.96</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.9</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.83</v>
       </c>
     </row>
     <row r="49">
@@ -4408,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4421,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.06</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.08</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.96</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.03</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.95</v>
       </c>
     </row>
     <row r="50">
@@ -4487,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4500,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.44</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.42</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.39</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.34</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4613,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46108</v>
+        <v>46111</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4626,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.22</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.15</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.09</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.14</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.13</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,9 +358,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1698,8 +1695,10 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
-        <v>46097</v>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1711,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>210000</v>
+        <v>1</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>205000</v>
+        <v>1</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>213000</v>
+        <v>1</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>214000</v>
+        <v>1</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>211000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1773,8 +1772,10 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
-        <v>46090</v>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1788,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1819000</v>
+        <v>1</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1851000</v>
+        <v>1</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1847000</v>
+        <v>1</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1871000</v>
+        <v>1</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1827000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2902,7 +2903,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2916,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.06</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.05</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.06</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.12</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.11</v>
       </c>
     </row>
     <row r="30">
@@ -2980,8 +2981,10 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="49" t="n">
-        <v>46112</v>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'T10YIE' not found in values file."</t>
+        </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2997,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.3</v>
+        <v>1</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>2.31</v>
+        <v>1</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.31</v>
+        <v>1</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.34</v>
+        <v>1</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.31</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -4121,8 +4124,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
-        <v>46023</v>
+      <c r="C46" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -4135,19 +4138,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>302149</v>
+        <v>314787</v>
       </c>
       <c r="G46" s="24" t="n">
+        <v>302224</v>
+      </c>
+      <c r="H46" s="24" t="n">
         <v>286301</v>
       </c>
-      <c r="H46" s="24" t="n">
+      <c r="I46" s="24" t="n">
         <v>290906</v>
       </c>
-      <c r="I46" s="24" t="n">
+      <c r="J46" s="24" t="n">
         <v>301177</v>
-      </c>
-      <c r="J46" s="24" t="n">
-        <v>293804</v>
       </c>
       <c r="K46" s="5" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4208,8 +4211,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
-        <v>46023</v>
+      <c r="C47" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4222,19 +4225,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>0.05535432988358413</v>
+        <v>0.04156850547937951</v>
       </c>
       <c r="G47" s="38" t="n">
+        <v>0.05561629194449202</v>
+      </c>
+      <c r="H47" s="38" t="n">
         <v>-0.01582985569221673</v>
       </c>
-      <c r="H47" s="38" t="n">
+      <c r="I47" s="38" t="n">
         <v>-0.03410286974104926</v>
       </c>
-      <c r="I47" s="38" t="n">
+      <c r="J47" s="38" t="n">
         <v>0.02509496126669486</v>
-      </c>
-      <c r="J47" s="38" t="n">
-        <v>0.03326956081366239</v>
       </c>
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4247,8 +4250,10 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="49" t="n">
-        <v>46111</v>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DFF' not found in values file."</t>
+        </is>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4261,19 +4266,19 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -4287,8 +4292,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
-        <v>46023</v>
+      <c r="C48" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4301,19 +4306,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>356604</v>
+        <v>372135</v>
       </c>
       <c r="G48" s="24" t="n">
+        <v>356901</v>
+      </c>
+      <c r="H48" s="24" t="n">
         <v>359201</v>
       </c>
-      <c r="H48" s="24" t="n">
+      <c r="I48" s="24" t="n">
         <v>346932</v>
       </c>
-      <c r="I48" s="24" t="n">
+      <c r="J48" s="24" t="n">
         <v>332279</v>
-      </c>
-      <c r="J48" s="24" t="n">
-        <v>342972</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4327,7 +4332,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4345,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.82</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.96</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.84</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.9</v>
       </c>
     </row>
     <row r="49">
@@ -4362,8 +4367,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
-        <v>46023</v>
+      <c r="C49" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4376,19 +4381,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>-0.007229935328687875</v>
+        <v>0.04268410567636405</v>
       </c>
       <c r="G49" s="38" t="n">
+        <v>-0.006403100214086299</v>
+      </c>
+      <c r="H49" s="38" t="n">
         <v>0.03536427887885818</v>
       </c>
-      <c r="H49" s="38" t="n">
+      <c r="I49" s="38" t="n">
         <v>0.04409848350332091</v>
       </c>
-      <c r="I49" s="38" t="n">
+      <c r="J49" s="38" t="n">
         <v>-0.03117747221347511</v>
-      </c>
-      <c r="J49" s="38" t="n">
-        <v>0.007689030571021327</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4401,8 +4406,10 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
-        <v>46111</v>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS5' not found in values file."</t>
+        </is>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4422,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>3.97</v>
+        <v>1</v>
       </c>
       <c r="R49" s="6" t="n">
-        <v>4.06</v>
+        <v>1</v>
       </c>
       <c r="S49" s="6" t="n">
-        <v>4.08</v>
+        <v>1</v>
       </c>
       <c r="T49" s="6" t="n">
-        <v>3.96</v>
+        <v>1</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.03</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -4441,8 +4448,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
-        <v>46023</v>
+      <c r="C50" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4455,19 +4462,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>27336</v>
+        <v>27256</v>
       </c>
       <c r="G50" s="24" t="n">
+        <v>27460</v>
+      </c>
+      <c r="H50" s="24" t="n">
         <v>26347</v>
       </c>
-      <c r="H50" s="24" t="n">
+      <c r="I50" s="24" t="n">
         <v>27608</v>
       </c>
-      <c r="I50" s="24" t="n">
+      <c r="J50" s="24" t="n">
         <v>27476</v>
-      </c>
-      <c r="J50" s="24" t="n">
-        <v>28592</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4480,8 +4487,10 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
-        <v>46111</v>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
+        </is>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.35</v>
+        <v>1</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>4.44</v>
+        <v>1</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>4.42</v>
+        <v>1</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>4.33</v>
+        <v>1</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.39</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4516,8 +4525,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
-        <v>46023</v>
+      <c r="C51" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4530,19 +4539,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.03753748054806993</v>
+        <v>-0.007428987618353977</v>
       </c>
       <c r="G51" s="38" t="n">
+        <v>0.04224389873609891</v>
+      </c>
+      <c r="H51" s="38" t="n">
         <v>-0.04567516661837145</v>
       </c>
-      <c r="H51" s="38" t="n">
+      <c r="I51" s="38" t="n">
         <v>0.004804192750036407</v>
       </c>
-      <c r="I51" s="38" t="n">
+      <c r="J51" s="38" t="n">
         <v>-0.03903189703413545</v>
-      </c>
-      <c r="J51" s="38" t="n">
-        <v>-0.03349896900246763</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4555,7 +4564,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46104</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4606,8 +4615,10 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="50" t="n">
-        <v>46111</v>
+      <c r="N52" s="20" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
+        </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4631,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.14</v>
+        <v>1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>6.22</v>
+        <v>1</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>6.15</v>
+        <v>1</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.09</v>
+        <v>1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,6 +358,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -925,8 +928,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
-        <v>46054</v>
+      <c r="N3" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
@@ -939,19 +942,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>-92</v>
+        <v>178</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>126</v>
+        <v>-133</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>160</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>-17</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>41</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>-140</v>
       </c>
     </row>
     <row r="4">
@@ -996,8 +999,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
-        <v>46054</v>
+      <c r="N4" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
@@ -1010,19 +1013,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.0009854083759711957</v>
+        <v>0.001641652512675452</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.001832335026663634</v>
+        <v>0.0009411913334596677</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.002047160512548336</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.0007327117916066601</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.002340601850973247</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.002931400170945582</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1150,8 +1153,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
-        <v>46054</v>
+      <c r="N6" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1164,19 +1167,19 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="R6" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="R6" s="6" t="n">
+      <c r="S6" s="6" t="n">
         <v>4.3</v>
       </c>
-      <c r="S6" s="6" t="n">
+      <c r="T6" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="U6" s="21" t="n">
         <v>4.5</v>
-      </c>
-      <c r="U6" s="21" t="n">
-        <v/>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1229,8 +1232,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46054</v>
+      <c r="N7" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1243,19 +1246,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>7.9</v>
       </c>
-      <c r="R7" s="6" t="n">
+      <c r="S7" s="6" t="n">
         <v>8.1</v>
       </c>
-      <c r="S7" s="6" t="n">
+      <c r="T7" s="6" t="n">
         <v>8.4</v>
       </c>
-      <c r="T7" s="6" t="n">
+      <c r="U7" s="21" t="n">
         <v>8.699999999999999</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v/>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1308,8 +1311,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
-        <v>46054</v>
+      <c r="N8" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1322,19 +1325,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="R8" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="R8" s="6" t="n">
+      <c r="S8" s="6" t="n">
         <v>62.1</v>
       </c>
-      <c r="S8" s="6" t="n">
+      <c r="T8" s="6" t="n">
         <v>62.4</v>
       </c>
-      <c r="T8" s="6" t="n">
+      <c r="U8" s="21" t="n">
         <v>62.5</v>
-      </c>
-      <c r="U8" s="21" t="n">
-        <v/>
       </c>
     </row>
     <row r="9">
@@ -1387,8 +1390,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46054</v>
+      <c r="N9" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1401,19 +1404,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="R9" s="6" t="n">
         <v>59.3</v>
       </c>
-      <c r="R9" s="6" t="n">
+      <c r="S9" s="6" t="n">
         <v>59.4</v>
       </c>
-      <c r="S9" s="6" t="n">
+      <c r="T9" s="6" t="n">
         <v>59.7</v>
       </c>
-      <c r="T9" s="6" t="n">
+      <c r="U9" s="21" t="n">
         <v>59.6</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -1695,10 +1698,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
-        </is>
+      <c r="N13" s="49" t="n">
+        <v>46104</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1711,19 +1712,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>1</v>
+        <v>202000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>1</v>
+        <v>211000</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>1</v>
+        <v>205000</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>1</v>
+        <v>213000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>1</v>
+        <v>214000</v>
       </c>
     </row>
     <row r="14">
@@ -1772,10 +1773,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
-        </is>
+      <c r="N14" s="49" t="n">
+        <v>46097</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1788,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1</v>
+        <v>1841000</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1</v>
+        <v>1816000</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1</v>
+        <v>1851000</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1</v>
+        <v>1847000</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1</v>
+        <v>1871000</v>
       </c>
     </row>
     <row r="15">
@@ -1853,8 +1852,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
-        <v>46054</v>
+      <c r="N15" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1867,19 +1866,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="R15" s="24" t="n">
         <v>34.3</v>
       </c>
       <c r="S15" s="24" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="T15" s="24" t="n">
         <v>34.2</v>
       </c>
-      <c r="T15" s="24" t="n">
+      <c r="U15" s="26" t="n">
         <v>34.3</v>
-      </c>
-      <c r="U15" s="26" t="n">
-        <v>34.2</v>
       </c>
     </row>
     <row r="16">
@@ -2903,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2916,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.07</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.06</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.05</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.06</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2981,10 +2980,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'T10YIE' not found in values file."</t>
-        </is>
+      <c r="N30" s="49" t="n">
+        <v>46114</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>1</v>
+        <v>2.34</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>1</v>
+        <v>2.31</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>1</v>
+        <v>2.3</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>1</v>
+        <v>2.31</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>1</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -3208,8 +3205,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
-        <v>46054</v>
+      <c r="N33" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
@@ -3222,19 +3219,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
-        <v>0.004035512510088823</v>
+        <v>0.002413515687851975</v>
       </c>
       <c r="R33" s="38" t="n">
-        <v>0.004051863857374327</v>
+        <v>0.003768506056527565</v>
       </c>
       <c r="S33" s="38" t="n">
+        <v>0.003511615343057661</v>
+      </c>
+      <c r="T33" s="38" t="n">
         <v>0.000540540540540535</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.00407055630936215</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.004087193460490468</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -3297,7 +3294,7 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>0.008545824844536363</v>
+        <v>0.008003158272115368</v>
       </c>
       <c r="R34" s="38" t="n">
         <v>0.007941414156884045</v>
@@ -3376,7 +3373,7 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>0.001295896455863144</v>
+        <v>0.0007571308403366839</v>
       </c>
       <c r="R35" s="38" t="n">
         <v>-0.003037958457621781</v>
@@ -3451,7 +3448,7 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>0.008545824844536363</v>
+        <v>0.008003158272115368</v>
       </c>
       <c r="R36" s="38" t="n">
         <v>0.007941414156884045</v>
@@ -4250,10 +4247,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DFF' not found in values file."</t>
-        </is>
+      <c r="N47" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4266,19 +4261,19 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="48">
@@ -4332,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4345,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.82</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.88</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.96</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.84</v>
       </c>
     </row>
     <row r="49">
@@ -4406,10 +4401,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS5' not found in values file."</t>
-        </is>
+      <c r="N49" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4422,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>1</v>
+        <v>3.97</v>
       </c>
       <c r="R49" s="6" t="n">
-        <v>1</v>
+        <v>3.92</v>
       </c>
       <c r="S49" s="6" t="n">
-        <v>1</v>
+        <v>3.97</v>
       </c>
       <c r="T49" s="6" t="n">
-        <v>1</v>
+        <v>4.06</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>1</v>
+        <v>4.08</v>
       </c>
     </row>
     <row r="50">
@@ -4487,10 +4480,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
-        </is>
+      <c r="N50" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>1</v>
+        <v>4.33</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>1</v>
+        <v>4.35</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>1</v>
+        <v>4.44</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>1</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4564,8 +4555,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46104</v>
+      <c r="N51" s="49" t="n">
+        <v>46111</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4578,19 +4569,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.38</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.22</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.11</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>5.98</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4615,10 +4606,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="20" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
-        </is>
+      <c r="N52" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4631,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>1</v>
+        <v>6.08</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>1</v>
+        <v>6.09</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>1</v>
+        <v>6.14</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>1</v>
+        <v>6.22</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>1</v>
+        <v>6.15</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1544,8 +1544,10 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
-        <v>46054</v>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
+        </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1558,19 +1560,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -2330,8 +2332,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
-        <v>46054</v>
+      <c r="C22" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2344,19 +2346,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.118</v>
+        <v>16.686</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>15.209</v>
+        <v>16.134</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.401</v>
+        <v>15.215</v>
       </c>
       <c r="I22" s="24" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="J22" s="24" t="n">
         <v>16.006</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>15.843</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2405,8 +2407,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
-        <v>46054</v>
+      <c r="C23" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2419,19 +2421,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.01833241975759802</v>
+        <v>-0.09068119891008182</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.04645768025078368</v>
+        <v>-0.01735793897314088</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.0520201144442517</v>
+        <v>-0.04608150470219433</v>
       </c>
       <c r="I23" s="25" t="n">
+        <v>-0.05207791457141205</v>
+      </c>
+      <c r="J23" s="25" t="n">
         <v>-0.05334752779749237</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>-0.03941065906748309</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2902,7 +2904,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2918,16 +2920,16 @@
         <v>2.11</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.07</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.06</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.05</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.06</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2983,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,16 +2996,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.31</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.3</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.31</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.31</v>
@@ -4248,7 +4250,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4329,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4342,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.81</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.82</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.88</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.96</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4404,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4417,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.06</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.08</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4483,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4496,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.3</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.35</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.44</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.42</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-05
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1544,10 +1544,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
-        </is>
+      <c r="N11" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1560,19 +1558,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-06
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4326,8 +4326,10 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
-        <v>46114</v>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
+        </is>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4342,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.79</v>
+        <v>1</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>3.81</v>
+        <v>1</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>3.79</v>
+        <v>1</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>3.82</v>
+        <v>1</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.88</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1465,7 +1465,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
+      <c r="N10" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1544,7 +1544,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1619,7 +1619,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -2787,8 +2787,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
-        <v>46023</v>
+      <c r="C28" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2801,19 +2801,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-8.71345793578282e-05</v>
+        <v>-0.01370492520749644</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>-0.004534110075869346</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>-0.00913646104747079</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>0.05441037812530491</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>-0.02093605859677161</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>0.006436255758670795</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2862,8 +2862,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
-        <v>46023</v>
+      <c r="C29" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2876,19 +2876,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.103432407836673</v>
+        <v>0.07318740752079188</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.09852504335582685</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.1059440595541697</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.1247312200873968</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.04877483240471108</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.07412067603746038</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46115</v>
+        <v>46118</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.11</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.07</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.06</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.05</v>
       </c>
     </row>
     <row r="30">
@@ -2941,8 +2941,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
-        <v>46023</v>
+      <c r="C30" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2955,19 +2955,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.005088320854118145</v>
+        <v>-0.0121697783836805</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>0.002152622967753981</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>-0.01921059426035288</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>0.06592882125886601</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>-0.0128376635658648</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>0.001174064535676367</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46115</v>
+        <v>46118</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,16 +2997,16 @@
         <v>2.36</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.31</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.3</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -3016,8 +3016,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
-        <v>46023</v>
+      <c r="C31" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3030,19 +3030,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.09577784074808728</v>
+        <v>0.07269103421880246</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.09257725367104795</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.1010908210327026</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.1265306873826442</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.05011084527755218</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.06502168244015354</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3509,7 +3509,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="49" t="n">
+      <c r="N37" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3584,7 +3584,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="49" t="n">
+      <c r="N38" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4326,10 +4326,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
-        </is>
+      <c r="N48" s="49" t="n">
+        <v>46115</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4342,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>1</v>
+        <v>3.84</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>1</v>
+        <v>3.79</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>1</v>
+        <v>3.81</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>1</v>
+        <v>3.79</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>1</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="49">
@@ -4404,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4417,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.97</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.06</v>
       </c>
     </row>
     <row r="50">
@@ -4483,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4496,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.31</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.3</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.35</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.44</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4609,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4622,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.09</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.22</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.15</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1078,7 +1078,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1193,8 +1193,8 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
-        <v>45931</v>
+      <c r="C7" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1207,19 +1207,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
+        <v>1.3205</v>
+      </c>
+      <c r="G7" s="41" t="n">
         <v>4.2373</v>
       </c>
-      <c r="G7" s="41" t="n">
+      <c r="H7" s="41" t="n">
         <v>3.4728</v>
       </c>
-      <c r="H7" s="41" t="n">
+      <c r="I7" s="41" t="n">
         <v>2.902</v>
       </c>
-      <c r="I7" s="41" t="n">
+      <c r="J7" s="41" t="n">
         <v>-2.7318</v>
-      </c>
-      <c r="J7" s="41" t="n">
-        <v>2.2711</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1272,7 +1272,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1939,7 +1939,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
+      <c r="C17" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2026,7 +2026,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
+      <c r="C18" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2479,8 +2479,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
-        <v>46023</v>
+      <c r="C24" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2493,19 +2493,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.003556211510844731</v>
+        <v>0.0005344764598498308</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.009446225118119989</v>
+        <v>0.00193733910205296</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>-0.002377705261307317</v>
+        <v>0.006198592859945062</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.003395368410566313</v>
+        <v>-0.0007477443007701812</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.003399783954204594</v>
+        <v>0.003378223860396545</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2558,8 +2558,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="48" t="n">
-        <v>46023</v>
+      <c r="C25" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2572,19 +2572,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.0008831408658551698</v>
+        <v>0.002321146114863559</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.003398716336493468</v>
+        <v>0.001350696962159503</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.001527249410752551</v>
+        <v>0.002042971180921338</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.0007591671161557567</v>
+        <v>0.001126106640109592</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.002887647186711639</v>
+        <v>0.0009131400161073167</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.12</v>
-      </c>
-      <c r="R29" s="6" t="n">
-        <v>2.11</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.11</v>
       </c>
       <c r="T29" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.07</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.06</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.3</v>
       </c>
     </row>
     <row r="31">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46115</v>
+        <v>46118</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46115</v>
+        <v>46118</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4343,16 +4343,16 @@
         <v>3.84</v>
       </c>
       <c r="R48" s="6" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="S48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.81</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.82</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46115</v>
+        <v>46118</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.92</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.97</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46115</v>
+        <v>46118</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.35</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.31</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.3</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.35</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46114</v>
+        <v>46118</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.09</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.14</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.22</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-09
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24065.956</v>
+        <v>24055.749</v>
       </c>
       <c r="G3" s="24" t="n">
         <v>24026.834</v>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.001628262799834523</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="G4" s="25" t="n">
         <v>0.0107634621312982</v>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16667.027</v>
+        <v>16665.219</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>16585.878</v>
@@ -1440,7 +1440,7 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.004892656270593321</v>
+        <v>0.004783647872002916</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>0.008524606910566446</v>
@@ -1505,8 +1505,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
-        <v>46023</v>
+      <c r="C11" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1519,19 +1519,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>-0.01147326027910467</v>
+        <v>0.008870546938001267</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>-0.007021622878400358</v>
+        <v>-0.01403114915111547</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>0.007401508408675816</v>
+        <v>-0.00581233144238813</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>-9.368120286679105e-05</v>
+        <v>0.007353974425031495</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>-0.00461581499440511</v>
+        <v>0</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1580,8 +1580,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
-        <v>46023</v>
+      <c r="C12" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1594,19 +1594,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.01019333843797865</v>
+        <v>0.01673200114733722</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>-0.02386176631925389</v>
+        <v>0.008853369065849924</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.008819252239996333</v>
+        <v>-0.02262753702687877</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>0.01846374045801518</v>
+        <v>0.008866163156166484</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>0.02290259211345895</v>
+        <v>0.01855916030534355</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1659,8 +1659,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
-        <v>46023</v>
+      <c r="C13" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1673,19 +1673,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.0002820635771302316</v>
+        <v>-0.002351474629571859</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>-0.001042547196393295</v>
+        <v>-0.003219338623591583</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>0.001382579498321101</v>
+        <v>-0.002197864126912585</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>0.001469383141654124</v>
+        <v>0.001326110264657787</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>-0.00357585313661446</v>
+        <v>0.001497640509762865</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1698,8 +1698,10 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
-        <v>46104</v>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1714,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>202000</v>
+        <v>1</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>211000</v>
+        <v>1</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>205000</v>
+        <v>1</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>213000</v>
+        <v>1</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>214000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1734,8 +1736,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
-        <v>46023</v>
+      <c r="C14" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1748,19 +1750,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.02017730700592953</v>
+        <v>0.009141710846826219</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01520531470133451</v>
+        <v>0.01597490069656324</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.02604874382028966</v>
+        <v>0.01400263444247182</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>0.02445440092498914</v>
+        <v>0.02601983289485096</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>0.02153393181883783</v>
+        <v>0.02448330683624796</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1774,7 +1776,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46097</v>
+        <v>46104</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1789,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1841000</v>
+        <v>1794000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1832000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1816000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1851000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1847000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1871000</v>
       </c>
     </row>
     <row r="15">
@@ -1813,8 +1815,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
-        <v>46023</v>
+      <c r="C15" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1827,19 +1829,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.003326444782829396</v>
+        <v>0.0008222569598179685</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.002599007651623797</v>
+        <v>0.003163466942223581</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.0002363292611984313</v>
+        <v>0.002845221754583793</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>0.00257898717796845</v>
+        <v>-9.089339114154438e-05</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>0.003374053619106698</v>
+        <v>0.002606326264660508</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1852,8 +1854,10 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="49" t="n">
-        <v>46082</v>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
+        </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1866,19 +1870,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1888,8 +1892,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
-        <v>46023</v>
+      <c r="C16" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1902,19 +1906,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02651248191698502</v>
+        <v>0.03044004093404044</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02316609477881844</v>
+        <v>0.02628992173300197</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02390367813311264</v>
+        <v>0.02311045163683583</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>0.02568501132750953</v>
+        <v>0.02359662426842094</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>0.0245940671714955</v>
+        <v>0.02571298048684977</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2065,8 +2069,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
-        <v>46054</v>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2079,19 +2085,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>0.00267003074209704</v>
+        <v>1</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>0.00170842649932057</v>
+        <v>1</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>0.00297788428704604</v>
+        <v>1</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2105,8 +2111,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
-        <v>46023</v>
+      <c r="C19" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2119,19 +2125,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>0.00668052913330075</v>
+        <v>-0.004526180904246169</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>-0.0003095975232196846</v>
+        <v>0.006225581884386822</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>0.001184506215890169</v>
+        <v>-0.0004425121414268762</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>-0.001547422988073754</v>
+        <v>0.0008581029834302534</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>0.0009791501861489138</v>
+        <v>-0.001740850861583043</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2140,8 +2146,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
-        <v>46054</v>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2154,19 +2162,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>0.0243400411037322</v>
+        <v>1</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>0.02391201432150015</v>
+        <v>1</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>0.02653304114557758</v>
+        <v>1</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>0.02696443916493949</v>
+        <v>1</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2176,8 +2184,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
-        <v>46023</v>
+      <c r="C20" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2190,19 +2198,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.01751836241880857</v>
+        <v>0.01062505234359729</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01200476832755948</v>
+        <v>0.01639481715838071</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.01325386244216132</v>
+        <v>0.01134436615382877</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.01437915836164052</v>
+        <v>0.01272729309745998</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01827247198915003</v>
+        <v>0.01418264506891994</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2255,8 +2263,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
-        <v>46023</v>
+      <c r="C21" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2269,19 +2277,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="H21" s="6" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2369,8 +2377,10 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46054</v>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
+        </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2383,19 +2393,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.006840134042972679</v>
+        <v>1</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.005264444194909901</v>
+        <v>1</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.003805886526233593</v>
+        <v>1</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.002525940746747724</v>
+        <v>1</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.001291224333588303</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2439,8 +2449,10 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46054</v>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
+        </is>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2453,19 +2465,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.03371718848029785</v>
+        <v>1</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.02848454130765334</v>
+        <v>1</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.0295201697358758</v>
+        <v>1</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.02985380376518458</v>
+        <v>1</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.02833335611850097</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -2518,8 +2530,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
-        <v>46023</v>
+      <c r="N24" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
@@ -2532,19 +2544,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.002752400575360525</v>
+        <v>0.00375295622843419</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.003589403456751628</v>
+        <v>0.003025447984071672</v>
       </c>
       <c r="S24" s="38" t="n">
-        <v>0.002205313084075566</v>
+        <v>0.003308571071852118</v>
       </c>
       <c r="T24" s="38" t="n">
-        <v>0.0019431929480902</v>
+        <v>0.00219752719537647</v>
       </c>
       <c r="U24" s="23" t="n">
-        <v>0.002608155986582039</v>
+        <v>0.001927522037218354</v>
       </c>
     </row>
     <row r="25">
@@ -2593,8 +2605,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
-        <v>46023</v>
+      <c r="N25" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
@@ -2607,19 +2619,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.02832151941124403</v>
+        <v>0.02801756656951585</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.02909288760511774</v>
+        <v>0.02828962580830351</v>
       </c>
       <c r="S25" s="38" t="n">
-        <v>0.02822596821168675</v>
+        <v>0.02878083518031025</v>
       </c>
       <c r="T25" s="38" t="n">
-        <v>0.02714187029093776</v>
+        <v>0.02820189831269997</v>
       </c>
       <c r="U25" s="23" t="n">
-        <v>0.02787442414870654</v>
+        <v>0.02712580525969119</v>
       </c>
     </row>
     <row r="26">
@@ -2647,7 +2659,7 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.005574532321468206</v>
+        <v>0.005923787970366412</v>
       </c>
       <c r="G26" s="38" t="n">
         <v>0.007794617579222285</v>
@@ -2672,8 +2684,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
-        <v>46023</v>
+      <c r="N26" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2686,19 +2698,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.003634828694041303</v>
+        <v>0.003668567155808988</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.003577228118895714</v>
+        <v>0.00392537103357693</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.001791818931981659</v>
+        <v>0.003271383630529812</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>0.002292168817051854</v>
+        <v>0.001776129138734595</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>0.001894029073346237</v>
+        <v>0.002276415079477623</v>
       </c>
     </row>
     <row r="27">
@@ -2726,7 +2738,7 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.001337237753545217</v>
+        <v>-0.004277328978805506</v>
       </c>
       <c r="G27" s="38" t="n">
         <v>-0.01832684674964358</v>
@@ -2747,8 +2759,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
-        <v>46023</v>
+      <c r="N27" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2761,19 +2773,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03055696019648922</v>
+        <v>0.0296775740141437</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03005732873844572</v>
+        <v>0.03050880107876425</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.02832319581807324</v>
+        <v>0.02971110180682146</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>0.02756153498288012</v>
+        <v>0.02829092786499081</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>0.02825069249833962</v>
+        <v>0.0275453840687383</v>
       </c>
     </row>
     <row r="28">
@@ -2902,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.12</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <v>2.11</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.11</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.07</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +3006,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.37</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -3055,8 +3067,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="48" t="n">
-        <v>45931</v>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3069,19 +3083,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>0.007310493043885868</v>
+        <v>1</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>0.007996957929548465</v>
+        <v>1</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>0.01027939464493599</v>
+        <v>1</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>0.007624633431085215</v>
+        <v>1</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>0.009473060982829962</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3130,8 +3144,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="48" t="n">
-        <v>45931</v>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3144,19 +3160,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>0.03362463343108507</v>
+        <v>1</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>0.03584369449378332</v>
+        <v>1</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>0.03559665871121723</v>
+        <v>1</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>0.03369434416365838</v>
+        <v>1</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>0.03710462287104619</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3281,7 +3297,7 @@
         </is>
       </c>
       <c r="N34" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
@@ -3294,19 +3310,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>0.008003158272115368</v>
+        <v>0.009284897536239168</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>0.007941414156884045</v>
+        <v>0.008034422666587262</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>0.01079517034980899</v>
+        <v>0.008247145515396716</v>
       </c>
       <c r="T34" s="38" t="n">
-        <v>0.01173861920396547</v>
+        <v>0.01081883276249912</v>
       </c>
       <c r="U34" s="23" t="n">
-        <v>0.01032118383222275</v>
+        <v>0.01175444356788234</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3320,8 +3336,10 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="48" t="n">
-        <v>45931</v>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PRS85006092' not found in values file."</t>
+        </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -3334,19 +3352,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="G35" s="41" t="n">
-        <v>5.2</v>
+        <v>1</v>
       </c>
       <c r="H35" s="41" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="I35" s="41" t="n">
-        <v>-0.9</v>
+        <v>1</v>
       </c>
       <c r="J35" s="41" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -3360,7 +3378,7 @@
         </is>
       </c>
       <c r="N35" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
@@ -3373,19 +3391,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>0.0007571308403366839</v>
+        <v>1.549168846470828e-05</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>-0.003037958457621781</v>
+        <v>0.0004847009215600551</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>0.001861138831470432</v>
+        <v>-0.002758902506289296</v>
       </c>
       <c r="T35" s="38" t="n">
-        <v>0.002139842385766366</v>
+        <v>0.001868922106829984</v>
       </c>
       <c r="U35" s="23" t="n">
-        <v>-0.0004224555765300897</v>
+        <v>0.00215551661749025</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3435,7 +3453,7 @@
         </is>
       </c>
       <c r="N36" s="48" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
@@ -3448,19 +3466,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>0.008003158272115368</v>
+        <v>0.009284897536239168</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>0.007941414156884045</v>
+        <v>0.008034422666587262</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>0.01079517034980899</v>
+        <v>0.008247145515396716</v>
       </c>
       <c r="T36" s="38" t="n">
-        <v>0.01173861920396547</v>
+        <v>0.01081883276249912</v>
       </c>
       <c r="U36" s="23" t="n">
-        <v>0.01032118383222275</v>
+        <v>0.01175444356788234</v>
       </c>
     </row>
     <row r="37">
@@ -3659,8 +3677,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
-        <v>46054</v>
+      <c r="N39" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3673,19 +3691,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
+        <v>119.9199</v>
+      </c>
+      <c r="R39" s="6" t="n">
         <v>117.906</v>
       </c>
-      <c r="R39" s="6" t="n">
+      <c r="S39" s="6" t="n">
         <v>119.2298</v>
       </c>
-      <c r="S39" s="6" t="n">
+      <c r="T39" s="6" t="n">
         <v>120.1883</v>
       </c>
-      <c r="T39" s="6" t="n">
+      <c r="U39" s="21" t="n">
         <v>121.4177</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>120.7618</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3734,8 +3752,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
-        <v>46054</v>
+      <c r="N40" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3748,19 +3766,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.05008673748247425</v>
+      </c>
+      <c r="R40" s="38" t="n">
         <v>-0.07796471263522881</v>
       </c>
-      <c r="R40" s="38" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.07456792269916472</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.05790675033979801</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.03874237696864814</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.02292562904900106</v>
       </c>
     </row>
     <row r="41">
@@ -4013,7 +4031,7 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5341.129</v>
+        <v>5343.513</v>
       </c>
       <c r="G44" s="24" t="n">
         <v>5324.402</v>
@@ -4084,7 +4102,7 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.003141573457451141</v>
+        <v>0.003589323270481781</v>
       </c>
       <c r="G45" s="38" t="n">
         <v>0.01669515005814426</v>
@@ -4121,7 +4139,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
+      <c r="C46" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4208,7 +4226,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
+      <c r="C47" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4248,7 +4266,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4287,7 +4305,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
+      <c r="C48" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4327,7 +4345,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4358,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.84</v>
+        <v>3.81</v>
       </c>
       <c r="R48" s="6" t="n">
         <v>3.84</v>
       </c>
       <c r="S48" s="6" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="T48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.81</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.79</v>
       </c>
     </row>
     <row r="49">
@@ -4362,7 +4380,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
+      <c r="C49" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4402,7 +4420,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4433,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.97</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.92</v>
       </c>
     </row>
     <row r="50">
@@ -4441,7 +4459,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
+      <c r="C50" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4481,7 +4499,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4512,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.34</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.35</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.31</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.33</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.3</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4516,7 +4534,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
+      <c r="C51" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4555,7 +4573,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46111</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4607,7 +4625,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46118</v>
+        <v>46120</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4638,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.04</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.08</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.09</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.14</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -928,7 +928,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N3" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -999,7 +999,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="49" t="n">
+      <c r="N4" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1153,7 +1153,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="49" t="n">
+      <c r="N6" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1193,7 +1193,7 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="49" t="n">
+      <c r="C7" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.3205</v>
+        <v>1.3078</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>4.2373</v>
@@ -1232,7 +1232,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1311,7 +1311,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="49" t="n">
+      <c r="N8" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -1390,7 +1390,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="49" t="n">
+      <c r="N9" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1698,10 +1698,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
-        </is>
+      <c r="N13" s="49" t="n">
+        <v>46111</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1714,19 +1712,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>1</v>
+        <v>219000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>1</v>
+        <v>203000</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>1</v>
+        <v>211000</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>1</v>
+        <v>205000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>1</v>
+        <v>213000</v>
       </c>
     </row>
     <row r="14">
@@ -1854,10 +1852,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
-        </is>
+      <c r="N15" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1870,19 +1866,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="16">
@@ -2069,10 +2065,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N18" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2085,19 +2079,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>1</v>
+        <v>0.008651438343614481</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>1</v>
+        <v>0.00267003074209704</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>1</v>
+        <v>0.00170842649932057</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>1</v>
+        <v>0.00297788428704604</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2146,10 +2140,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N19" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2162,19 +2154,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>1</v>
+        <v>0.03285957752865201</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>1</v>
+        <v>0.0243400411037322</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>1</v>
+        <v>0.02391201432150015</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>1</v>
+        <v>0.02653304114557758</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>1</v>
+        <v>0.02696443916493949</v>
       </c>
     </row>
     <row r="20">
@@ -2223,8 +2215,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46054</v>
+      <c r="N20" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2237,16 +2229,16 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>0.001957950538511444</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.002160502174024082</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>0.002950448142634121</v>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="T20" s="38" t="n">
         <v>0.002329002576704653</v>
-      </c>
-      <c r="T20" s="38" t="n">
-        <v/>
       </c>
       <c r="U20" s="23" t="n">
         <v/>
@@ -2298,8 +2290,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46054</v>
+      <c r="N21" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2312,19 +2304,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.0260216770548682</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.02472462476764023</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.02512028782828883</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.02646484707309002</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v>0.02599044806094405</v>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="22">
@@ -2338,7 +2330,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2377,10 +2369,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
-        </is>
+      <c r="N22" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2393,19 +2383,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>1</v>
+        <v>0.006840134042972679</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>1</v>
+        <v>0.005264444194909901</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>1</v>
+        <v>0.003805886526233593</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>1</v>
+        <v>0.002525940746747724</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>1</v>
+        <v>0.001291224333588303</v>
       </c>
     </row>
     <row r="23">
@@ -2415,7 +2405,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2449,10 +2439,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
-        </is>
+      <c r="N23" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2465,19 +2453,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>1</v>
+        <v>0.03371718848029785</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>1</v>
+        <v>0.02848454130765334</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>1</v>
+        <v>0.0295201697358758</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>1</v>
+        <v>0.02985380376518458</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>1</v>
+        <v>0.02833335611850097</v>
       </c>
     </row>
     <row r="24">
@@ -2799,7 +2787,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="49" t="n">
+      <c r="C28" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2813,10 +2801,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.01370492520749644</v>
+        <v>-0.01280100007813112</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.004534110075869346</v>
+        <v>-0.004254034642219184</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>-0.00913646104747079</v>
@@ -2874,7 +2862,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="49" t="n">
+      <c r="C29" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2888,10 +2876,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.07318740752079188</v>
+        <v>0.07447318740752079</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.09852504335582685</v>
+        <v>0.09883411459674789</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.1059440595541697</v>
@@ -2914,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,16 +2915,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.12</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.11</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.11</v>
@@ -2953,7 +2941,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="49" t="n">
+      <c r="C30" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2967,10 +2955,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.0121697783836805</v>
+        <v>-0.01149211309276466</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>0.002152622967753981</v>
+        <v>0.002385879326488816</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>-0.01921059426035288</v>
@@ -2993,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.37</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.34</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -3028,7 +3016,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="49" t="n">
+      <c r="C31" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3042,10 +3030,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.07269103421880246</v>
+        <v>0.07367676103887663</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.09257725367104795</v>
+        <v>0.09283155684402497</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>0.1010908210327026</v>
@@ -3067,10 +3055,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N31" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3083,19 +3069,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>1</v>
+        <v>0.007310493043885868</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>1</v>
+        <v>0.007996957929548465</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>1</v>
+        <v>0.01027939464493599</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>1</v>
+        <v>0.007624633431085215</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>1</v>
+        <v>0.009473060982829962</v>
       </c>
     </row>
     <row r="32">
@@ -3144,10 +3130,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N32" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3160,19 +3144,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>1</v>
+        <v>0.03362463343108507</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>1</v>
+        <v>0.03584369449378332</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>1</v>
+        <v>0.03559665871121723</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>1</v>
+        <v>0.03369434416365838</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>1</v>
+        <v>0.03710462287104619</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3221,7 +3205,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="49" t="n">
+      <c r="N33" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -4266,7 +4250,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4345,7 +4329,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4358,19 +4342,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.81</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>3.84</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>3.84</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>3.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.81</v>
       </c>
     </row>
     <row r="49">
@@ -4420,7 +4404,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4433,19 +4417,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.94</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.97</v>
       </c>
     </row>
     <row r="50">
@@ -4499,7 +4483,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4512,19 +4496,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.34</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.35</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.31</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.33</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4573,8 +4557,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46111</v>
+      <c r="N51" s="49" t="n">
+        <v>46118</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4587,19 +4571,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.46</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.38</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.22</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.11</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.12</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.11</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,16 +2994,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.37</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.36</v>
@@ -3320,10 +3320,8 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PRS85006092' not found in values file."</t>
-        </is>
+      <c r="C35" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -3336,19 +3334,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="G35" s="41" t="n">
-        <v>1</v>
+        <v>5.2</v>
       </c>
       <c r="H35" s="41" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="I35" s="41" t="n">
-        <v>1</v>
+        <v>-0.9</v>
       </c>
       <c r="J35" s="41" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -4250,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4329,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4342,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.81</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.84</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.84</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.79</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="49">
@@ -4404,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4417,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.99</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.94</v>
       </c>
     </row>
     <row r="50">
@@ -4483,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4499,16 +4497,16 @@
         <v>4.29</v>
       </c>
       <c r="R50" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.34</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.35</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4609,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4625,16 +4623,16 @@
         <v>6.02</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.04</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.05</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.08</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2558,8 +2558,10 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
-        <v>46054</v>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2572,19 +2574,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.002321146114863559</v>
+        <v>1</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.001350696962159503</v>
+        <v>1</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.002042971180921338</v>
+        <v>1</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.001126106640109592</v>
+        <v>1</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.0009131400161073167</v>
+        <v>1</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2787,8 +2789,10 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
-        <v>46054</v>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
+        </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2801,19 +2805,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.01280100007813112</v>
+        <v>1</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.004254034642219184</v>
+        <v>1</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>-0.00913646104747079</v>
+        <v>1</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>0.05441037812530491</v>
+        <v>1</v>
       </c>
       <c r="J28" s="25" t="n">
-        <v>-0.02093605859677161</v>
+        <v>1</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2862,8 +2866,10 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
-        <v>46054</v>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
+        </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2876,19 +2882,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.07447318740752079</v>
+        <v>1</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.09883411459674789</v>
+        <v>1</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>0.1059440595541697</v>
+        <v>1</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>0.1247312200873968</v>
+        <v>1</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>0.04877483240471108</v>
+        <v>1</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -3659,7 +3665,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="49" t="n">
+      <c r="N39" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3734,7 +3740,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="49" t="n">
+      <c r="N40" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3850,7 +3856,7 @@
         </is>
       </c>
       <c r="C42" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3863,19 +3869,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
+        <v>3980000</v>
+      </c>
+      <c r="G42" s="39" t="n">
+        <v>4130000</v>
+      </c>
+      <c r="H42" s="39" t="n">
+        <v>4020000</v>
+      </c>
+      <c r="I42" s="39" t="n">
+        <v>4270000</v>
+      </c>
+      <c r="J42" s="39" t="n">
         <v>4090000</v>
-      </c>
-      <c r="G42" s="39" t="n">
-        <v>4020000</v>
-      </c>
-      <c r="H42" s="39" t="n">
-        <v>4270000</v>
-      </c>
-      <c r="I42" s="39" t="n">
-        <v>4090000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4110000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3921,7 +3927,7 @@
         </is>
       </c>
       <c r="C43" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3934,7 +3940,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.01445783132530121</v>
+        <v>-0.009950248756218905</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4607,7 +4613,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4626,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.02</v>
+        <v>6.03</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.02</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.04</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.05</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -889,8 +889,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
-        <v>45931</v>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -903,19 +905,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24055.749</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24026.834</v>
+        <v>1</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>23770.976</v>
+        <v>1</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>23548.21</v>
+        <v>1</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23586.542</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -964,8 +966,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
-        <v>45931</v>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -978,19 +982,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>1</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>1</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>1</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>-0.001625164044818495</v>
+        <v>1</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>0.004598746857240599</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1078,8 +1082,10 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
-        <v>46082</v>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1092,19 +1098,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>62000</v>
+        <v>1</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>66000</v>
+        <v>1</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>11000</v>
+        <v>1</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>37000</v>
+        <v>1</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>74000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1232,8 +1238,10 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46082</v>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1246,19 +1254,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8.4</v>
+        <v>1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>8.699999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1390,8 +1398,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46082</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1404,19 +1414,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2065,8 +2075,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
-        <v>46082</v>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2079,19 +2091,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>0.008651438343614481</v>
+        <v>1</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>0.00267003074209704</v>
+        <v>1</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>0.00170842649932057</v>
+        <v>1</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>0.00297788428704604</v>
+        <v>1</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2140,8 +2152,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
-        <v>46082</v>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2154,19 +2168,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>0.03285957752865201</v>
+        <v>1</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>0.0243400411037322</v>
+        <v>1</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>0.02391201432150015</v>
+        <v>1</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>0.02653304114557758</v>
+        <v>1</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>0.02696443916493949</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2369,8 +2383,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46054</v>
+      <c r="N22" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2383,19 +2397,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.006840134042972679</v>
+        <v>0.005123318605152027</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.005264444194909901</v>
+        <v>0.004965106516948259</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.003805886526233593</v>
+        <v>0.005526756624853135</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.002525940746747724</v>
+        <v>0.003786725277053149</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.001291224333588303</v>
+        <v>0.004088035682236812</v>
       </c>
     </row>
     <row r="23">
@@ -2439,8 +2453,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46054</v>
+      <c r="N23" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2453,19 +2467,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.03371718848029785</v>
+        <v>0.04019452230589979</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.02848454130765334</v>
+        <v>0.03364972711879271</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.0295201697358758</v>
+        <v>0.03033620544010816</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.02985380376518458</v>
+        <v>0.03110464325544714</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.02833335611850097</v>
+        <v>0.03145847985960791</v>
       </c>
     </row>
     <row r="24">
@@ -2479,8 +2493,10 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
-        <v>46054</v>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2493,19 +2509,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.0005344764598498308</v>
+        <v>1</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.00193733910205296</v>
+        <v>1</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.006198592859945062</v>
+        <v>1</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>-0.0007477443007701812</v>
+        <v>1</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.003378223860396545</v>
+        <v>1</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2558,10 +2574,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
-        </is>
+      <c r="C25" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2574,19 +2588,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>1</v>
+        <v>0.002321146114863559</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>1</v>
+        <v>0.001350696962159503</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>1</v>
+        <v>0.002042971180921338</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>1</v>
+        <v>0.001126106640109592</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>1</v>
+        <v>0.0009131400161073167</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2635,8 +2649,10 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n">
-        <v>45931</v>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2649,19 +2665,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.005923787970366412</v>
+        <v>1</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>0.007794617579222285</v>
+        <v>1</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>0.01778138610314484</v>
+        <v>1</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>0.02303791460563676</v>
+        <v>1</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>-0.009359213919614473</v>
+        <v>1</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2714,8 +2730,10 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="48" t="n">
-        <v>45931</v>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2728,19 +2746,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.004277328978805506</v>
+        <v>1</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>-0.01832684674964358</v>
+        <v>1</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>-0.01299350008050415</v>
+        <v>1</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>-0.002410568051752549</v>
+        <v>1</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>0.01049622222903812</v>
+        <v>1</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2789,10 +2807,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
-        </is>
+      <c r="C28" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2805,19 +2821,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>1</v>
+        <v>-0.01280100007813112</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>1</v>
+        <v>-0.004254034642219184</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>1</v>
+        <v>-0.00913646104747079</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>1</v>
+        <v>0.05441037812530491</v>
       </c>
       <c r="J28" s="25" t="n">
-        <v>1</v>
+        <v>-0.02093605859677161</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2830,8 +2846,10 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
-        <v>46054</v>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'MICH' not found in values file."</t>
+        </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2844,19 +2862,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2866,10 +2884,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
-        </is>
+      <c r="C29" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2882,19 +2898,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>1</v>
+        <v>0.07447318740752079</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>1</v>
+        <v>0.09883411459674789</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>1</v>
+        <v>0.1059440595541697</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>1</v>
+        <v>0.1247312200873968</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>1</v>
+        <v>0.04877483240471108</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2908,7 +2924,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2921,19 +2937,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.13</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2947,8 +2963,10 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
-        <v>46054</v>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
+        </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2961,19 +2979,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.01149211309276466</v>
+        <v>1</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>0.002385879326488816</v>
+        <v>1</v>
       </c>
       <c r="H30" s="25" t="n">
-        <v>-0.01921059426035288</v>
+        <v>1</v>
       </c>
       <c r="I30" s="25" t="n">
-        <v>0.06592882125886601</v>
+        <v>1</v>
       </c>
       <c r="J30" s="25" t="n">
-        <v>-0.0128376635658648</v>
+        <v>1</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -2987,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3000,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.36</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.37</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -3022,8 +3040,10 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
-        <v>46054</v>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
+        </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3036,19 +3056,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.07367676103887663</v>
+        <v>1</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.09283155684402497</v>
+        <v>1</v>
       </c>
       <c r="H31" s="25" t="n">
-        <v>0.1010908210327026</v>
+        <v>1</v>
       </c>
       <c r="I31" s="25" t="n">
-        <v>0.1265306873826442</v>
+        <v>1</v>
       </c>
       <c r="J31" s="25" t="n">
-        <v>0.05011084527755218</v>
+        <v>1</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3061,8 +3081,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="48" t="n">
-        <v>45931</v>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3075,19 +3097,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>0.007310493043885868</v>
+        <v>1</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>0.007996957929548465</v>
+        <v>1</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>0.01027939464493599</v>
+        <v>1</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>0.007624633431085215</v>
+        <v>1</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>0.009473060982829962</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3101,8 +3123,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
-        <v>46054</v>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3115,19 +3139,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.001510796776836631</v>
+        <v>1</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.007063467944424584</v>
+        <v>1</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>0.003133370494423415</v>
+        <v>1</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.001511745671022524</v>
+        <v>1</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.004529448794114321</v>
+        <v>1</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3136,8 +3160,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="48" t="n">
-        <v>45931</v>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3150,19 +3176,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>0.03362463343108507</v>
+        <v>1</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>0.03584369449378332</v>
+        <v>1</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>0.03559665871121723</v>
+        <v>1</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>0.03369434416365838</v>
+        <v>1</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>0.03710462287104619</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3172,8 +3198,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
-        <v>46054</v>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3186,19 +3214,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.01435914986552827</v>
+        <v>1</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.02330092430197657</v>
+        <v>1</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01346393254876795</v>
+        <v>1</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.02082735352619783</v>
+        <v>1</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.01747269263442562</v>
+        <v>1</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3251,8 +3279,10 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46054</v>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TCU' not found in values file."</t>
+        </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3265,19 +3295,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.2946</v>
+        <v>1</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.2529</v>
+        <v>1</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.7794</v>
+        <v>1</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.63339999999999</v>
+        <v>1</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.6104</v>
+        <v>1</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3405,8 +3435,10 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
-        <v>46023</v>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
+        </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3419,19 +3451,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1487</v>
+        <v>1</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1387</v>
+        <v>1</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1324</v>
+        <v>1</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1272</v>
+        <v>1</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1328</v>
+        <v>1</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3476,8 +3508,10 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
-        <v>46023</v>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
+        </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3490,19 +3524,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.09499263622974963</v>
+        <v>1</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.08388375165125496</v>
+        <v>1</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>0.02239382239382239</v>
+        <v>1</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>-0.05917159763313609</v>
+        <v>1</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>-0.02137067059690494</v>
+        <v>1</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3555,8 +3589,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>46023</v>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3569,19 +3605,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1386</v>
+        <v>1</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1455</v>
+        <v>1</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1388</v>
+        <v>1</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1411</v>
+        <v>1</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1415</v>
+        <v>1</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3626,8 +3662,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>46023</v>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3640,19 +3678,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.05068493150684932</v>
+        <v>1</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>-0.01689189189189189</v>
+        <v>1</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>-0.07957559681697612</v>
+        <v>1</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>-0.0119047619047619</v>
+        <v>1</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>-0.01324965132496513</v>
+        <v>1</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -4005,8 +4043,10 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="48" t="n">
-        <v>45931</v>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GCE' not found in values file."</t>
+        </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4019,19 +4059,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5343.513</v>
+        <v>1</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>5324.402</v>
+        <v>1</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>5236.97</v>
+        <v>1</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>5195.517</v>
+        <v>1</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>5150.725</v>
+        <v>1</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4076,8 +4116,10 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="48" t="n">
-        <v>45931</v>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GCE' not found in values file."</t>
+        </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4090,19 +4132,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.003589323270481781</v>
+        <v>1</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>0.01669515005814426</v>
+        <v>1</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>0.007978609251013902</v>
+        <v>1</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>0.008696251498575336</v>
+        <v>1</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>0.01254255520332359</v>
+        <v>1</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4254,7 +4296,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4333,7 +4375,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4346,16 +4388,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.81</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>3.84</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>3.84</v>
@@ -4408,7 +4450,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4421,19 +4463,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.91</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.98</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.99</v>
       </c>
     </row>
     <row r="50">
@@ -4487,7 +4529,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4500,19 +4542,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.29</v>
+        <v>4.31</v>
       </c>
       <c r="R50" s="6" t="n">
         <v>4.29</v>
       </c>
       <c r="S50" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="T50" s="6" t="n">
         <v>4.33</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.34</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.35</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -889,10 +889,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C3" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -905,19 +903,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>1</v>
+        <v>24055.749</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>1</v>
+        <v>24026.834</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>1</v>
+        <v>23770.976</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>1</v>
+        <v>23548.21</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>1</v>
+        <v>23586.542</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -966,10 +964,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C4" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -982,19 +978,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>1</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>1</v>
+        <v>0.0107634621312982</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>1</v>
+        <v>0.009459997171759493</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>1</v>
+        <v>-0.001625164044818495</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>1</v>
+        <v>0.004598746857240599</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1082,10 +1078,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
-        </is>
+      <c r="N5" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1098,19 +1092,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>1</v>
+        <v>62000</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>1</v>
+        <v>66000</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>1</v>
+        <v>11000</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>1</v>
+        <v>37000</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>1</v>
+        <v>74000</v>
       </c>
     </row>
     <row r="6">
@@ -1238,10 +1232,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
-        </is>
+      <c r="N7" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1254,19 +1246,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>8.1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>8.4</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>1</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1398,10 +1390,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1414,19 +1404,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="10">
@@ -2075,10 +2065,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N18" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2091,19 +2079,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>1</v>
+        <v>0.008651438343614481</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>1</v>
+        <v>0.00267003074209704</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>1</v>
+        <v>0.00170842649932057</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>1</v>
+        <v>0.00297788428704604</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2152,10 +2140,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N19" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2168,19 +2154,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>1</v>
+        <v>0.03285957752865201</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>1</v>
+        <v>0.0243400411037322</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>1</v>
+        <v>0.02391201432150015</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>1</v>
+        <v>0.02653304114557758</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>1</v>
+        <v>0.02696443916493949</v>
       </c>
     </row>
     <row r="20">
@@ -2493,10 +2479,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
-        </is>
+      <c r="C24" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2509,19 +2493,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>1</v>
+        <v>0.0005344764598498308</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>1</v>
+        <v>0.00193733910205296</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>1</v>
+        <v>0.006198592859945062</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>1</v>
+        <v>-0.0007477443007701812</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>1</v>
+        <v>0.003378223860396545</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2649,10 +2633,8 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
-        </is>
+      <c r="C26" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2665,19 +2647,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>1</v>
+        <v>0.005923787970366412</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>1</v>
+        <v>0.007794617579222285</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>1</v>
+        <v>0.01778138610314484</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>1</v>
+        <v>0.02303791460563676</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>1</v>
+        <v>-0.009359213919614473</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2730,10 +2712,8 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
-        </is>
+      <c r="C27" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2746,19 +2726,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>1</v>
+        <v>-0.004277328978805506</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01832684674964358</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01299350008050415</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>1</v>
+        <v>-0.002410568051752549</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>1</v>
+        <v>0.01049622222903812</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2846,10 +2826,8 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'MICH' not found in values file."</t>
-        </is>
+      <c r="N28" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2862,19 +2840,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>1</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="29">
@@ -2924,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2940,16 +2918,16 @@
         <v>2.15</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.12</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.1</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.13</v>
       </c>
     </row>
     <row r="30">
@@ -2963,10 +2941,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
-        </is>
+      <c r="C30" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2979,19 +2955,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>1</v>
+        <v>-0.01149211309276466</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>1</v>
+        <v>0.002385879326488816</v>
       </c>
       <c r="H30" s="25" t="n">
-        <v>1</v>
+        <v>-0.01921059426035288</v>
       </c>
       <c r="I30" s="25" t="n">
-        <v>1</v>
+        <v>0.06592882125886601</v>
       </c>
       <c r="J30" s="25" t="n">
-        <v>1</v>
+        <v>-0.0128376635658648</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3005,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3018,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.36</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.37</v>
       </c>
     </row>
     <row r="31">
@@ -3040,10 +3016,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
-        </is>
+      <c r="C31" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3056,19 +3030,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>1</v>
+        <v>0.07367676103887663</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>1</v>
+        <v>0.09283155684402497</v>
       </c>
       <c r="H31" s="25" t="n">
-        <v>1</v>
+        <v>0.1010908210327026</v>
       </c>
       <c r="I31" s="25" t="n">
-        <v>1</v>
+        <v>0.1265306873826442</v>
       </c>
       <c r="J31" s="25" t="n">
-        <v>1</v>
+        <v>0.05011084527755218</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3081,10 +3055,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N31" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3097,19 +3069,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>1</v>
+        <v>0.007310493043885868</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>1</v>
+        <v>0.007996957929548465</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>1</v>
+        <v>0.01027939464493599</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>1</v>
+        <v>0.007624633431085215</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>1</v>
+        <v>0.009473060982829962</v>
       </c>
     </row>
     <row r="32">
@@ -3123,10 +3095,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C32" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3139,19 +3109,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>1</v>
+        <v>0.001510796776836631</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>1</v>
+        <v>0.007063467944424584</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>1</v>
+        <v>0.003133370494423415</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>1</v>
+        <v>0.001511745671022524</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>1</v>
+        <v>-0.004529448794114321</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3160,10 +3130,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N32" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3176,19 +3144,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>1</v>
+        <v>0.03362463343108507</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>1</v>
+        <v>0.03584369449378332</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>1</v>
+        <v>0.03559665871121723</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>1</v>
+        <v>0.03369434416365838</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>1</v>
+        <v>0.03710462287104619</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3198,10 +3166,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C33" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3214,19 +3180,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>1</v>
+        <v>0.01435914986552827</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>1</v>
+        <v>0.02330092430197657</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>1</v>
+        <v>0.01346393254876795</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>1</v>
+        <v>0.02082735352619783</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>1</v>
+        <v>0.01747269263442562</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3279,10 +3245,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TCU' not found in values file."</t>
-        </is>
+      <c r="C34" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3295,19 +3259,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>1</v>
+        <v>76.2946</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>1</v>
+        <v>76.2529</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>1</v>
+        <v>75.7794</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>1</v>
+        <v>75.63339999999999</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>1</v>
+        <v>75.6104</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3435,10 +3399,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
-        </is>
+      <c r="C36" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3451,19 +3413,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1</v>
+        <v>1487</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1</v>
+        <v>1387</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1</v>
+        <v>1324</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1</v>
+        <v>1272</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1</v>
+        <v>1328</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3508,10 +3470,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
-        </is>
+      <c r="C37" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3524,19 +3484,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>1</v>
+        <v>0.09499263622974963</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>1</v>
+        <v>-0.08388375165125496</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>1</v>
+        <v>0.02239382239382239</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>1</v>
+        <v>-0.05917159763313609</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>1</v>
+        <v>-0.02137067059690494</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3589,10 +3549,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C38" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3605,19 +3563,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>1386</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1</v>
+        <v>1455</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1</v>
+        <v>1388</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1</v>
+        <v>1411</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1</v>
+        <v>1415</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3662,10 +3620,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C39" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3678,19 +3634,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>1</v>
+        <v>-0.05068493150684932</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>1</v>
+        <v>-0.01689189189189189</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07957559681697612</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>1</v>
+        <v>-0.0119047619047619</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>1</v>
+        <v>-0.01324965132496513</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3853,8 +3809,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
-        <v>46054</v>
+      <c r="N41" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3867,16 +3823,16 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.01542416452442152</v>
+        <v>0.01641414141414144</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v>0.006468305304010435</v>
+        <v>0.01930501930501927</v>
       </c>
       <c r="S41" s="38" t="n">
+        <v>0.005174644243208348</v>
+      </c>
+      <c r="T41" s="38" t="n">
         <v>0.005855562784645496</v>
-      </c>
-      <c r="T41" s="38" t="n">
-        <v/>
       </c>
       <c r="U41" s="23" t="n">
         <v/>
@@ -3928,8 +3884,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
-        <v>46054</v>
+      <c r="N42" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3942,19 +3898,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.03538663171690699</v>
+        <v>0.05573770491803279</v>
       </c>
       <c r="R42" s="38" t="n">
-        <v>0.02638522427440633</v>
+        <v>0.03800786369593716</v>
       </c>
       <c r="S42" s="38" t="n">
+        <v>0.02506596306068609</v>
+      </c>
+      <c r="T42" s="38" t="n">
         <v>0.0341137123745819</v>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v>0.03293010752688157</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="43">
@@ -4003,8 +3959,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
-        <v>46054</v>
+      <c r="N43" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -4017,16 +3973,16 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.01265822784810133</v>
+        <v>0.007665505226480906</v>
       </c>
       <c r="R43" s="38" t="n">
+        <v>0.009142053445851062</v>
+      </c>
+      <c r="S43" s="38" t="n">
         <v>0.005657708628005631</v>
       </c>
-      <c r="S43" s="38" t="n">
+      <c r="T43" s="38" t="n">
         <v>0.00141643059490093</v>
-      </c>
-      <c r="T43" s="38" t="n">
-        <v/>
       </c>
       <c r="U43" s="23" t="n">
         <v/>
@@ -4043,10 +3999,8 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GCE' not found in values file."</t>
-        </is>
+      <c r="C44" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4059,19 +4013,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>1</v>
+        <v>5343.513</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>1</v>
+        <v>5324.402</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>1</v>
+        <v>5236.97</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>1</v>
+        <v>5195.517</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>1</v>
+        <v>5150.725</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4080,8 +4034,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
-        <v>46054</v>
+      <c r="N44" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4094,19 +4048,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.0133708655876144</v>
+        <v>0.0211864406779661</v>
       </c>
       <c r="R44" s="38" t="n">
+        <v>0.009852216748768513</v>
+      </c>
+      <c r="S44" s="38" t="n">
         <v>0.002820874471085876</v>
       </c>
-      <c r="S44" s="38" t="n">
+      <c r="T44" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="T44" s="38" t="n">
+      <c r="U44" s="23" t="n">
         <v>-0.0007077140835104227</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="45">
@@ -4116,10 +4070,8 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GCE' not found in values file."</t>
-        </is>
+      <c r="C45" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4132,19 +4084,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>1</v>
+        <v>0.003589323270481781</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>1</v>
+        <v>0.01669515005814426</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>1</v>
+        <v>0.007978609251013902</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>1</v>
+        <v>0.008696251498575336</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>1</v>
+        <v>0.01254255520332359</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4296,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4375,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4388,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.81</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.81</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.84</v>
       </c>
     </row>
     <row r="49">
@@ -4450,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4463,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.91</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.95</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.98</v>
       </c>
     </row>
     <row r="50">
@@ -4529,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4542,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.31</v>
-      </c>
-      <c r="R50" s="6" t="n">
-        <v>4.29</v>
       </c>
       <c r="S50" s="6" t="n">
         <v>4.29</v>
       </c>
       <c r="T50" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.33</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.34</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4655,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4668,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.03</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.02</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.02</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.08</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.04</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,9 +358,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1505,7 +1502,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n">
+      <c r="C11" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1580,7 +1577,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="49" t="n">
+      <c r="C12" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1659,7 +1656,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="49" t="n">
+      <c r="C13" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1699,7 +1696,7 @@
         </is>
       </c>
       <c r="N13" s="49" t="n">
-        <v>46111</v>
+        <v>46118</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1709,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>219000</v>
+        <v>207000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>218000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>203000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>211000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>205000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>213000</v>
       </c>
     </row>
     <row r="14">
@@ -1734,7 +1731,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1774,7 +1771,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46104</v>
+        <v>46111</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1784,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1794000</v>
+        <v>1818000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1787000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1832000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1816000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1851000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1847000</v>
       </c>
     </row>
     <row r="15">
@@ -1813,7 +1810,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1888,7 +1885,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2105,7 +2102,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="49" t="n">
+      <c r="C19" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2176,7 +2173,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2255,7 +2252,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n">
+      <c r="C21" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2518,7 +2515,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="49" t="n">
+      <c r="N24" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2593,7 +2590,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="49" t="n">
+      <c r="N25" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2672,7 +2669,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="49" t="n">
+      <c r="N26" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2747,7 +2744,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="49" t="n">
+      <c r="N27" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2902,7 +2899,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2912,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.15</v>
+        <v>2.17</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.15</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.12</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.1</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2978,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2991,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.37</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.36</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -3095,8 +3092,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
-        <v>46054</v>
+      <c r="C32" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3109,19 +3106,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.001510796776836631</v>
+        <v>-0.005415070741811912</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.007063467944424584</v>
+        <v>0.007368443846867079</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>0.003133370494423415</v>
+        <v>-0.0001564786593617473</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.001511745671022524</v>
+        <v>0.005246287630711999</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.004529448794114321</v>
+        <v>-0.001368313417869027</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3166,8 +3163,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
-        <v>46054</v>
+      <c r="C33" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3180,19 +3177,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.01435914986552827</v>
+        <v>0.007416835246099523</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.02330092430197657</v>
+        <v>0.01231165794421915</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01346393254876795</v>
+        <v>0.01529710277450485</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.02082735352619783</v>
+        <v>0.01279811178014365</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.01747269263442562</v>
+        <v>0.0180124379988418</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3245,8 +3242,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46054</v>
+      <c r="C34" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3259,19 +3256,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.2946</v>
+        <v>75.6596</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.2529</v>
+        <v>76.1407</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.7794</v>
+        <v>75.6564</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.63339999999999</v>
+        <v>75.7296</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.6104</v>
+        <v>75.42489999999999</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -4248,7 +4245,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4326,8 +4323,10 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
-        <v>46125</v>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
+        </is>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4339,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.78</v>
+        <v>1</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>3.81</v>
+        <v>1</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>3.78</v>
+        <v>1</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>3.79</v>
+        <v>1</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.81</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4401,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4414,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.91</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.92</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.95</v>
       </c>
     </row>
     <row r="50">
@@ -4480,8 +4479,10 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
-        <v>46125</v>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
+        </is>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4495,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>4.31</v>
+        <v>1</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>4.29</v>
+        <v>1</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>4.29</v>
+        <v>1</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.33</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,7 +4556,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46118</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4606,8 +4607,10 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="50" t="n">
-        <v>46125</v>
+      <c r="N52" s="20" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
+        </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4623,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.02</v>
+        <v>1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>6.03</v>
+        <v>1</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>6.02</v>
+        <v>1</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.02</v>
+        <v>1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.08</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,6 +358,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2062,7 +2065,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
+      <c r="N18" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2137,7 +2140,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2212,7 +2215,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
+      <c r="N20" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2287,7 +2290,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
+      <c r="N21" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2899,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46127</v>
+        <v>46129</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2912,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.17</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.15</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.15</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.12</v>
       </c>
     </row>
     <row r="30">
@@ -2978,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46127</v>
+        <v>46129</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2991,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.37</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.38</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -4245,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4323,10 +4326,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
-        </is>
+      <c r="N48" s="49" t="n">
+        <v>46128</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4339,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>1</v>
+        <v>3.78</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>1</v>
+        <v>3.76</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>1</v>
+        <v>3.76</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>1</v>
+        <v>3.78</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>1</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="49">
@@ -4401,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4414,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="R49" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="S49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.94</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.92</v>
       </c>
     </row>
     <row r="50">
@@ -4479,10 +4480,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
-        </is>
+      <c r="N50" s="49" t="n">
+        <v>46128</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4495,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>1</v>
+        <v>4.32</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>1</v>
+        <v>4.29</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>1</v>
+        <v>4.26</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>1</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4556,8 +4555,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46118</v>
+      <c r="N51" s="49" t="n">
+        <v>46125</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4570,19 +4569,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.37</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.46</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.38</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.22</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.11</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4607,10 +4606,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="20" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
-        </is>
+      <c r="N52" s="50" t="n">
+        <v>46128</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4623,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>1</v>
+        <v>6.03</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>1</v>
+        <v>5.98</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>1</v>
+        <v>5.96</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>1</v>
+        <v>6.02</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>1</v>
+        <v>6.03</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-20
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7860620.8</v>
+        <v>7855631.5</v>
       </c>
       <c r="G5" s="24" t="n">
         <v>7774506.8</v>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.01107645825198844</v>
+        <v>0.0104347069321491</v>
       </c>
       <c r="G6" s="25" t="n">
         <v>0.02008474181421249</v>
@@ -1232,8 +1232,10 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46082</v>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1246,19 +1248,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8.4</v>
+        <v>1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>8.699999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1311,8 +1313,10 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
-        <v>46082</v>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
+        </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1325,19 +1329,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>61.9</v>
+        <v>1</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>62.1</v>
+        <v>1</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>62.4</v>
+        <v>1</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>62.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1465,8 +1469,10 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
-        <v>46054</v>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
+        </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1479,19 +1485,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1544,8 +1550,10 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
-        <v>46054</v>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
+        </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1558,19 +1566,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1619,8 +1627,10 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
-        <v>46054</v>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSTSR' not found in values file."</t>
+        </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
@@ -1633,19 +1643,19 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="S12" s="6" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
       <c r="T12" s="6" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="U12" s="21" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -2215,8 +2225,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46082</v>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2229,19 +2241,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>0.001957950538511444</v>
+        <v>1</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.002160502174024082</v>
+        <v>1</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>0.002950448142634121</v>
+        <v>1</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>0.002329002576704653</v>
+        <v>1</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2290,8 +2302,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46082</v>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2304,19 +2318,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.0260216770548682</v>
+        <v>1</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.02472462476764023</v>
+        <v>1</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>0.02512028782828883</v>
+        <v>1</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>0.02646484707309002</v>
+        <v>1</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>0.02599044806094405</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2672,8 +2686,10 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
-        <v>46054</v>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
+        </is>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2686,19 +2702,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.003668567155808988</v>
+        <v>1</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.00392537103357693</v>
+        <v>1</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.003271383630529812</v>
+        <v>1</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>0.001776129138734595</v>
+        <v>1</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>0.002276415079477623</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -2747,8 +2763,10 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
-        <v>46054</v>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
+        </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2761,19 +2779,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.0296775740141437</v>
+        <v>1</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03050880107876425</v>
+        <v>1</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.02971110180682146</v>
+        <v>1</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>0.02829092786499081</v>
+        <v>1</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>0.0275453840687383</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -3959,8 +3977,10 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
-        <v>46082</v>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'IR' not found in values file."</t>
+        </is>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3973,19 +3993,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.007665505226480906</v>
+        <v>1</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>0.009142053445851062</v>
+        <v>1</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v>0.005657708628005631</v>
+        <v>1</v>
       </c>
       <c r="T43" s="38" t="n">
-        <v>0.00141643059490093</v>
+        <v>1</v>
       </c>
       <c r="U43" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -4034,8 +4054,10 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
-        <v>46082</v>
+      <c r="N44" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'IR' not found in values file."</t>
+        </is>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4048,19 +4070,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.0211864406779661</v>
+        <v>1</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>0.009852216748768513</v>
+        <v>1</v>
       </c>
       <c r="S44" s="38" t="n">
-        <v>0.002820874471085876</v>
+        <v>1</v>
       </c>
       <c r="T44" s="38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U44" s="23" t="n">
-        <v>-0.0007077140835104227</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -4607,7 +4629,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4642,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.03</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.98</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.96</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.02</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.03</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-21
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1039,8 +1039,10 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="48" t="n">
-        <v>45931</v>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
+        </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1053,19 +1055,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7855631.5</v>
+        <v>1</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>7774506.8</v>
+        <v>1</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>7621432.3</v>
+        <v>1</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>7510528.3</v>
+        <v>1</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>7456295.5</v>
+        <v>1</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1114,8 +1116,10 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="48" t="n">
-        <v>45931</v>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
+        </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1128,19 +1132,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.0104347069321491</v>
+        <v>1</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>0.02008474181421249</v>
+        <v>1</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>0.0147664712214719</v>
+        <v>1</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>0.007273424182290045</v>
+        <v>1</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>0.01062352837847436</v>
+        <v>1</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1193,8 +1197,10 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
-        <v>46023</v>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPNOW' not found in values file."</t>
+        </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1207,19 +1213,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.3078</v>
+        <v>1</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>4.2373</v>
+        <v>1</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>3.4728</v>
+        <v>1</v>
       </c>
       <c r="I7" s="41" t="n">
-        <v>2.902</v>
+        <v>1</v>
       </c>
       <c r="J7" s="41" t="n">
-        <v>-2.7318</v>
+        <v>1</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1232,10 +1238,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
-        </is>
+      <c r="N7" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1248,19 +1252,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>8.1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>8.4</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>1</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1313,10 +1317,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
-        </is>
+      <c r="N8" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1329,19 +1331,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>1</v>
+        <v>61.9</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>1</v>
+        <v>62.1</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>1</v>
+        <v>62.4</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>1</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="9">
@@ -1469,10 +1471,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
-        </is>
+      <c r="N10" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1485,19 +1485,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>1</v>
+        <v>4.1</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="11">
@@ -1550,10 +1550,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
-        </is>
+      <c r="N11" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1566,19 +1564,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="12">
@@ -1627,10 +1625,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSTSR' not found in values file."</t>
-        </is>
+      <c r="N12" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
@@ -1643,19 +1639,19 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="S12" s="6" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="T12" s="6" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="U12" s="21" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -1669,8 +1665,10 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
-        <v>46054</v>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1683,19 +1681,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.002351474629571859</v>
+        <v>1</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>-0.003219338623591583</v>
+        <v>1</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>-0.002197864126912585</v>
+        <v>1</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>0.001326110264657787</v>
+        <v>1</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>0.001497640509762865</v>
+        <v>1</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1744,8 +1742,10 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
-        <v>46054</v>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1758,19 +1758,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.009141710846826219</v>
+        <v>1</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01597490069656324</v>
+        <v>1</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.01400263444247182</v>
+        <v>1</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>0.02601983289485096</v>
+        <v>1</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>0.02448330683624796</v>
+        <v>1</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1823,8 +1823,10 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
-        <v>46054</v>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1837,19 +1839,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.0008222569598179685</v>
+        <v>1</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.003163466942223581</v>
+        <v>1</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.002845221754583793</v>
+        <v>1</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>-9.089339114154438e-05</v>
+        <v>1</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>0.002606326264660508</v>
+        <v>1</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1898,8 +1900,10 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
-        <v>46054</v>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1912,19 +1916,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.03044004093404044</v>
+        <v>1</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02628992173300197</v>
+        <v>1</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02311045163683583</v>
+        <v>1</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>0.02359662426842094</v>
+        <v>1</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>0.02571298048684977</v>
+        <v>1</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -1949,8 +1953,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
-        <v>46054</v>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1963,19 +1969,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.00600990523942202</v>
+        <v>1</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>-0.001037134025754116</v>
+        <v>1</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>-1.361066422789214e-06</v>
+        <v>1</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>0.005016065910586232</v>
+        <v>1</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>-0.001558334425942887</v>
+        <v>1</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2036,8 +2042,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
-        <v>46054</v>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2050,19 +2058,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.03714451864108709</v>
+        <v>1</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.0319081629783764</v>
+        <v>1</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>0.02433131408893505</v>
+        <v>1</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>0.03212039564348258</v>
+        <v>1</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>0.03213514238518121</v>
+        <v>1</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2225,10 +2233,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N20" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2241,19 +2247,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1</v>
+        <v>0.001957950538511444</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>1</v>
+        <v>0.002160502174024082</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>1</v>
+        <v>0.002950448142634121</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>1</v>
+        <v>0.002329002576704653</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2302,10 +2308,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N21" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2318,19 +2322,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1</v>
+        <v>0.0260216770548682</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>1</v>
+        <v>0.02472462476764023</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>1</v>
+        <v>0.02512028782828883</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>1</v>
+        <v>0.02646484707309002</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>1</v>
+        <v>0.02599044806094405</v>
       </c>
     </row>
     <row r="22">
@@ -2383,7 +2387,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2453,7 +2457,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2686,10 +2690,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
-        </is>
+      <c r="N26" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2702,19 +2704,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>1</v>
+        <v>0.003668567155808988</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>1</v>
+        <v>0.00392537103357693</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>1</v>
+        <v>0.003271383630529812</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>1</v>
+        <v>0.001776129138734595</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>1</v>
+        <v>0.002276415079477623</v>
       </c>
     </row>
     <row r="27">
@@ -2763,10 +2765,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
-        </is>
+      <c r="N27" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2779,19 +2779,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>1</v>
+        <v>0.0296775740141437</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>1</v>
+        <v>0.03050880107876425</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>1</v>
+        <v>0.02971110180682146</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>1</v>
+        <v>0.02829092786499081</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>1</v>
+        <v>0.0275453840687383</v>
       </c>
     </row>
     <row r="28">
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2933,16 +2933,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.16</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.18</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.17</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.15</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.15</v>
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.36</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.39</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.39</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.37</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.38</v>
       </c>
     </row>
     <row r="31">
@@ -3977,10 +3977,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'IR' not found in values file."</t>
-        </is>
+      <c r="N43" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3993,19 +3991,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>1</v>
+        <v>0.007665505226480906</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>1</v>
+        <v>0.009142053445851062</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v>1</v>
+        <v>0.005657708628005631</v>
       </c>
       <c r="T43" s="38" t="n">
-        <v>1</v>
+        <v>0.00141643059490093</v>
       </c>
       <c r="U43" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -4054,10 +4052,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'IR' not found in values file."</t>
-        </is>
+      <c r="N44" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4070,19 +4066,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>1</v>
+        <v>0.0211864406779661</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>1</v>
+        <v>0.009852216748768513</v>
       </c>
       <c r="S44" s="38" t="n">
-        <v>1</v>
+        <v>0.002820874471085876</v>
       </c>
       <c r="T44" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U44" s="23" t="n">
-        <v>1</v>
+        <v>-0.0007077140835104227</v>
       </c>
     </row>
     <row r="45">
@@ -4270,7 +4266,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4309,8 +4305,10 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
-        <v>46054</v>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
+        </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4323,19 +4321,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>372135</v>
+        <v>1</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>356901</v>
+        <v>1</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>359201</v>
+        <v>1</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>346932</v>
+        <v>1</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>332279</v>
+        <v>1</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4349,7 +4347,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4362,19 +4360,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.78</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>3.76</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>3.76</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>3.78</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.81</v>
       </c>
     </row>
     <row r="49">
@@ -4384,8 +4382,10 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
-        <v>46054</v>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
+        </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4398,19 +4398,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.04268410567636405</v>
+        <v>1</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>-0.006403100214086299</v>
+        <v>1</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>0.03536427887885818</v>
+        <v>1</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>0.04409848350332091</v>
+        <v>1</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>-0.03117747221347511</v>
+        <v>1</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4424,7 +4424,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4437,19 +4437,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.91</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.9</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.92</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.94</v>
       </c>
     </row>
     <row r="50">
@@ -4463,8 +4463,10 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
-        <v>46054</v>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
+        </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4477,19 +4479,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>27256</v>
+        <v>1</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>27460</v>
+        <v>1</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>26347</v>
+        <v>1</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>27608</v>
+        <v>1</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>27476</v>
+        <v>1</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4503,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4516,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.32</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.29</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.3</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4538,8 +4540,10 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
-        <v>46054</v>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
+        </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4552,19 +4556,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>-0.007428987618353977</v>
+        <v>1</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>0.04224389873609891</v>
+        <v>1</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>-0.04567516661837145</v>
+        <v>1</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>0.004804192750036407</v>
+        <v>1</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>-0.03903189703413545</v>
+        <v>1</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1039,10 +1039,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
-        </is>
+      <c r="C5" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1055,19 +1053,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>1</v>
+        <v>7855631.5</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>1</v>
+        <v>7774506.8</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>1</v>
+        <v>7621432.3</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>1</v>
+        <v>7510528.3</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>1</v>
+        <v>7456295.5</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1116,10 +1114,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
-        </is>
+      <c r="C6" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1132,19 +1128,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>1</v>
+        <v>0.0104347069321491</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>1</v>
+        <v>0.02008474181421249</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>1</v>
+        <v>0.0147664712214719</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>1</v>
+        <v>0.007273424182290045</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>1</v>
+        <v>0.01062352837847436</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1197,10 +1193,8 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPNOW' not found in values file."</t>
-        </is>
+      <c r="C7" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1213,19 +1207,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1</v>
+        <v>1.241</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>1</v>
+        <v>4.2373</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>1</v>
+        <v>3.4728</v>
       </c>
       <c r="I7" s="41" t="n">
-        <v>1</v>
+        <v>2.902</v>
       </c>
       <c r="J7" s="41" t="n">
-        <v>1</v>
+        <v>-2.7318</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1665,10 +1659,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
-        </is>
+      <c r="C13" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1681,19 +1673,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>1</v>
+        <v>-0.002351474629571859</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>1</v>
+        <v>-0.003219338623591583</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>1</v>
+        <v>-0.002197864126912585</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>1</v>
+        <v>0.001326110264657787</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>1</v>
+        <v>0.001497640509762865</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1742,10 +1734,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
-        </is>
+      <c r="C14" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1758,19 +1748,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>1</v>
+        <v>0.009141710846826219</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>1</v>
+        <v>0.01597490069656324</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>1</v>
+        <v>0.01400263444247182</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>1</v>
+        <v>0.02601983289485096</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>1</v>
+        <v>0.02448330683624796</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1823,10 +1813,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
-        </is>
+      <c r="C15" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1839,19 +1827,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>1</v>
+        <v>0.0008222569598179685</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>1</v>
+        <v>0.003163466942223581</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>1</v>
+        <v>0.002845221754583793</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>1</v>
+        <v>-9.089339114154438e-05</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>1</v>
+        <v>0.002606326264660508</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1900,10 +1888,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
-        </is>
+      <c r="C16" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1916,19 +1902,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>1</v>
+        <v>0.03044004093404044</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>1</v>
+        <v>0.02628992173300197</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>1</v>
+        <v>0.02311045163683583</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>1</v>
+        <v>0.02359662426842094</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>1</v>
+        <v>0.02571298048684977</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -1953,10 +1939,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C17" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1969,19 +1953,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>1</v>
+        <v>0.01661457854582227</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>1</v>
+        <v>0.007173558174711436</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>1</v>
+        <v>-0.0002912686109073359</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>1</v>
+        <v>-1.361066422789214e-06</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>1</v>
+        <v>0.005016065910586232</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2042,10 +2026,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C18" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2058,19 +2040,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>1</v>
+        <v>0.03969447708578144</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>1</v>
+        <v>0.03962618135825458</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>1</v>
+        <v>0.03267862666254253</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>1</v>
+        <v>0.02433131408893505</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>1</v>
+        <v>0.03212039564348258</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2920,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2933,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.16</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.18</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.17</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.15</v>
       </c>
     </row>
     <row r="30">
@@ -2999,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3012,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.35</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.36</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.39</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.39</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.37</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="31">
@@ -3827,7 +3809,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3902,7 +3884,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="49" t="n">
+      <c r="N42" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3977,7 +3959,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4052,7 +4034,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4266,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4305,10 +4287,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
-        </is>
+      <c r="C48" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4321,19 +4301,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>1</v>
+        <v>372135</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>1</v>
+        <v>356901</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>1</v>
+        <v>359201</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>1</v>
+        <v>346932</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>1</v>
+        <v>332279</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4347,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4360,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.71</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.78</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.76</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.76</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.78</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="49">
@@ -4382,10 +4362,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
-        </is>
+      <c r="C49" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4398,19 +4376,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>1</v>
+        <v>0.04268410567636405</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>1</v>
+        <v>-0.006403100214086299</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>1</v>
+        <v>0.03536427887885818</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>1</v>
+        <v>0.04409848350332091</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>1</v>
+        <v>-0.03117747221347511</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4424,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4437,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.91</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.9</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.87</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.92</v>
       </c>
     </row>
     <row r="50">
@@ -4463,10 +4441,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
-        </is>
+      <c r="C50" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4479,19 +4455,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>1</v>
+        <v>27256</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>1</v>
+        <v>27460</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>1</v>
+        <v>26347</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>1</v>
+        <v>27608</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>1</v>
+        <v>27476</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4505,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4521,16 +4497,16 @@
         <v>4.26</v>
       </c>
       <c r="R50" s="6" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.32</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.29</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.3</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4540,10 +4516,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
-        </is>
+      <c r="C51" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4556,19 +4530,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>1</v>
+        <v>-0.007428987618353977</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>1</v>
+        <v>0.04224389873609891</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>1</v>
+        <v>-0.04567516661837145</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>1</v>
+        <v>0.004804192750036407</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>1</v>
+        <v>-0.03903189703413545</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4633,7 +4607,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46129</v>
+        <v>46133</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4646,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.98</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.03</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>5.98</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>5.96</v>
+        <v>6.03</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.02</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N13" s="49" t="n">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1712,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>207000</v>
+        <v>214000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>208000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>218000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>203000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>211000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>205000</v>
       </c>
     </row>
     <row r="14">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46111</v>
+        <v>46118</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1818000</v>
+        <v>1821000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1809000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1787000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1832000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1816000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1851000</v>
       </c>
     </row>
     <row r="15">
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.16</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.16</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.18</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.17</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2997,13 +2997,13 @@
         <v>2.38</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.35</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.36</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.39</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.39</v>
@@ -3095,7 +3095,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="49" t="n">
+      <c r="C32" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3166,7 +3166,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="49" t="n">
+      <c r="C33" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3245,7 +3245,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="49" t="n">
+      <c r="C34" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,16 +4340,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.72</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.71</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.78</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>3.76</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>3.76</v>
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.86</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.91</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.9</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.87</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.26</v>
+        <v>4.3</v>
       </c>
       <c r="R50" s="6" t="n">
         <v>4.26</v>
       </c>
       <c r="S50" s="6" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="T50" s="6" t="n">
         <v>4.32</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.29</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,7 +4555,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46125</v>
       </c>
       <c r="O51" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-24
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,9 +358,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -889,8 +886,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
-        <v>45931</v>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -903,19 +902,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24055.749</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24026.834</v>
+        <v>1</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>23770.976</v>
+        <v>1</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>23548.21</v>
+        <v>1</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23586.542</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -964,8 +963,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
-        <v>45931</v>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -978,19 +979,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>1</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>1</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>1</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>-0.001625164044818495</v>
+        <v>1</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>0.004598746857240599</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1773,8 +1774,10 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
-        <v>46118</v>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1790,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1821000</v>
+        <v>1</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1809000</v>
+        <v>1</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1787000</v>
+        <v>1</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1832000</v>
+        <v>1</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1816000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2633,8 +2636,10 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n">
-        <v>45931</v>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2647,19 +2652,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.005923787970366412</v>
+        <v>1</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>0.007794617579222285</v>
+        <v>1</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>0.01778138610314484</v>
+        <v>1</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>0.02303791460563676</v>
+        <v>1</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>-0.009359213919614473</v>
+        <v>1</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2827,7 +2832,7 @@
         </is>
       </c>
       <c r="N28" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2840,19 +2845,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="R28" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="R28" s="6" t="n">
+      <c r="S28" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S28" s="6" t="n">
+      <c r="T28" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="T28" s="6" t="n">
+      <c r="U28" s="21" t="n">
         <v>4.5</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>4.6</v>
       </c>
     </row>
     <row r="29">
@@ -2902,7 +2907,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2915,19 +2920,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.15</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.16</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.13</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.16</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.18</v>
       </c>
     </row>
     <row r="30">
@@ -2981,7 +2986,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2999,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.38</v>
+        <v>2.42</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.38</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.35</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.36</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.39</v>
       </c>
     </row>
     <row r="31">
@@ -3849,8 +3854,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="48" t="n">
-        <v>46082</v>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3863,19 +3870,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>3980000</v>
+        <v>1000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>4130000</v>
+        <v>1000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>4020000</v>
+        <v>1000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>4270000</v>
+        <v>1000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>4090000</v>
+        <v>1000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3920,8 +3927,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="48" t="n">
-        <v>46082</v>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3934,19 +3943,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.009950248756218905</v>
+        <v>1</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="I43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="J43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -4248,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.72</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.71</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.78</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.76</v>
       </c>
     </row>
     <row r="49">
@@ -4401,8 +4410,10 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
-        <v>46133</v>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS5' not found in values file."</t>
+        </is>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,19 +4426,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>3.91</v>
+        <v>1</v>
       </c>
       <c r="R49" s="6" t="n">
-        <v>3.86</v>
+        <v>1</v>
       </c>
       <c r="S49" s="6" t="n">
-        <v>3.84</v>
+        <v>1</v>
       </c>
       <c r="T49" s="6" t="n">
-        <v>3.91</v>
+        <v>1</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>3.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -4480,8 +4491,10 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
-        <v>46133</v>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
+        </is>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4507,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>4.26</v>
+        <v>1</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>4.26</v>
+        <v>1</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>4.32</v>
+        <v>1</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4555,8 +4568,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46125</v>
+      <c r="N51" s="49" t="n">
+        <v>46132</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4569,19 +4582,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.37</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.46</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.38</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.22</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4606,8 +4619,10 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="50" t="n">
-        <v>46133</v>
+      <c r="N52" s="20" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
+        </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4635,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>5.98</v>
+        <v>1</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>5.98</v>
+        <v>1</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.03</v>
+        <v>1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>5.98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-25
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,6 +358,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -886,10 +889,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C3" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -902,19 +903,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>1</v>
+        <v>24055.749</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>1</v>
+        <v>24026.834</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>1</v>
+        <v>23770.976</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>1</v>
+        <v>23548.21</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>1</v>
+        <v>23586.542</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -963,10 +964,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C4" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -979,19 +978,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>1</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>1</v>
+        <v>0.0107634621312982</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>1</v>
+        <v>0.009459997171759493</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>1</v>
+        <v>-0.001625164044818495</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>1</v>
+        <v>0.004598746857240599</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1774,10 +1773,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
-        </is>
+      <c r="N14" s="49" t="n">
+        <v>46118</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1790,19 +1787,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1</v>
+        <v>1821000</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1</v>
+        <v>1809000</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1</v>
+        <v>1787000</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1</v>
+        <v>1832000</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1</v>
+        <v>1816000</v>
       </c>
     </row>
     <row r="15">
@@ -2636,10 +2633,8 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
-        </is>
+      <c r="C26" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2652,19 +2647,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>1</v>
+        <v>0.005923787970366412</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>1</v>
+        <v>0.007794617579222285</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>1</v>
+        <v>0.01778138610314484</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>1</v>
+        <v>0.02303791460563676</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>1</v>
+        <v>-0.009359213919614473</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2907,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2920,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.15</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.16</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.13</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.16</v>
       </c>
     </row>
     <row r="30">
@@ -2986,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3002,16 +2997,16 @@
         <v>2.42</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>2.38</v>
+        <v>2.42</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.38</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -3854,10 +3849,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C42" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3870,19 +3863,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>1000</v>
+        <v>3980000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>1000</v>
+        <v>4130000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>1000</v>
+        <v>4020000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>1000</v>
+        <v>4270000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>1000</v>
+        <v>4090000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3927,10 +3920,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C43" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3943,19 +3934,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>1</v>
+        <v>-0.009950248756218905</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="H43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="I43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="J43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -4257,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.72</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.71</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.78</v>
       </c>
     </row>
     <row r="49">
@@ -4410,10 +4401,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS5' not found in values file."</t>
-        </is>
+      <c r="N49" s="49" t="n">
+        <v>46135</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4426,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>1</v>
+        <v>3.96</v>
       </c>
       <c r="R49" s="6" t="n">
-        <v>1</v>
+        <v>3.91</v>
       </c>
       <c r="S49" s="6" t="n">
-        <v>1</v>
+        <v>3.91</v>
       </c>
       <c r="T49" s="6" t="n">
-        <v>1</v>
+        <v>3.86</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>1</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="50">
@@ -4491,10 +4480,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
-        </is>
+      <c r="N50" s="49" t="n">
+        <v>46135</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4507,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>1</v>
+        <v>4.34</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>1</v>
+        <v>4.26</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>1</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4619,10 +4606,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="20" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
-        </is>
+      <c r="N52" s="50" t="n">
+        <v>46135</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4635,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>1</v>
+        <v>6.02</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>1</v>
+        <v>5.99</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>1</v>
+        <v>5.98</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>1</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1939,8 +1939,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
-        <v>46082</v>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1953,19 +1955,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.01661457854582227</v>
+        <v>1</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.007173558174711436</v>
+        <v>1</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>-0.0002912686109073359</v>
+        <v>1</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>-1.361066422789214e-06</v>
+        <v>1</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>0.005016065910586232</v>
+        <v>1</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2026,8 +2028,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
-        <v>46082</v>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2040,19 +2044,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.03969447708578144</v>
+        <v>1</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.03962618135825458</v>
+        <v>1</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>0.03267862666254253</v>
+        <v>1</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>0.02433131408893505</v>
+        <v>1</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>0.03212039564348258</v>
+        <v>1</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -928,8 +928,10 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
-        <v>46082</v>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
+        </is>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
@@ -942,19 +944,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>178</v>
+        <v>1</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>-133</v>
+        <v>1</v>
       </c>
       <c r="S3" s="24" t="n">
-        <v>160</v>
+        <v>1</v>
       </c>
       <c r="T3" s="24" t="n">
-        <v>-17</v>
+        <v>1</v>
       </c>
       <c r="U3" s="26" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -999,8 +1001,10 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
-        <v>46082</v>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
+        </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
@@ -1013,19 +1017,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.001641652512675452</v>
+        <v>1</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.0009411913334596677</v>
+        <v>1</v>
       </c>
       <c r="S4" s="38" t="n">
-        <v>0.002047160512548336</v>
+        <v>1</v>
       </c>
       <c r="T4" s="38" t="n">
-        <v>0.0007327117916066601</v>
+        <v>1</v>
       </c>
       <c r="U4" s="23" t="n">
-        <v>0.002340601850973247</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1659,8 +1663,10 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
-        <v>46054</v>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1673,19 +1679,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.002351474629571859</v>
+        <v>1</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>-0.003219338623591583</v>
+        <v>1</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>-0.002197864126912585</v>
+        <v>1</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>0.001326110264657787</v>
+        <v>1</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>0.001497640509762865</v>
+        <v>1</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1734,8 +1740,10 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
-        <v>46054</v>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1748,19 +1756,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.009141710846826219</v>
+        <v>1</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01597490069656324</v>
+        <v>1</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.01400263444247182</v>
+        <v>1</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>0.02601983289485096</v>
+        <v>1</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>0.02448330683624796</v>
+        <v>1</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1813,8 +1821,10 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
-        <v>46054</v>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1827,19 +1837,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.0008222569598179685</v>
+        <v>1</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.003163466942223581</v>
+        <v>1</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.002845221754583793</v>
+        <v>1</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>-9.089339114154438e-05</v>
+        <v>1</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>0.002606326264660508</v>
+        <v>1</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1888,8 +1898,10 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
-        <v>46054</v>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1902,19 +1914,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.03044004093404044</v>
+        <v>1</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02628992173300197</v>
+        <v>1</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02311045163683583</v>
+        <v>1</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>0.02359662426842094</v>
+        <v>1</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>0.02571298048684977</v>
+        <v>1</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2259,8 +2271,10 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
-        <v>46054</v>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
+        </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2273,19 +2287,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>3.9</v>
+        <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2906,7 +2920,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2919,19 +2933,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.15</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.16</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.13</v>
       </c>
     </row>
     <row r="30">
@@ -2985,7 +2999,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2998,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.42</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.38</v>
+        <v>2.42</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.38</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.35</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="31">
@@ -3099,8 +3113,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
-        <v>46082</v>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3113,19 +3129,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>-0.005415070741811912</v>
+        <v>1</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.007368443846867079</v>
+        <v>1</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>-0.0001564786593617473</v>
+        <v>1</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.005246287630711999</v>
+        <v>1</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.001368313417869027</v>
+        <v>1</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3170,8 +3186,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
-        <v>46082</v>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3184,19 +3202,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.007416835246099523</v>
+        <v>1</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01231165794421915</v>
+        <v>1</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01529710277450485</v>
+        <v>1</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01279811178014365</v>
+        <v>1</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.0180124379988418</v>
+        <v>1</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3249,8 +3267,10 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46082</v>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TCU' not found in values file."</t>
+        </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3263,19 +3283,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>75.6596</v>
+        <v>1</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.1407</v>
+        <v>1</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.6564</v>
+        <v>1</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.7296</v>
+        <v>1</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.42489999999999</v>
+        <v>1</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3513,8 +3533,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
-        <v>46023</v>
+      <c r="N37" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3527,19 +3547,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>-0.001091846627661819</v>
+        <v>0.002917033083199794</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>-0.002556382261513668</v>
+        <v>-0.001828986686322698</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>-0.001313071612671246</v>
+        <v>-0.002571690054911535</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.001955114463894181</v>
+        <v>-0.001325270004722268</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.002952812599475663</v>
+        <v>-0.001961201654098743</v>
       </c>
     </row>
     <row r="38">
@@ -3553,8 +3573,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>46023</v>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3567,19 +3589,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1386</v>
+        <v>1</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1455</v>
+        <v>1</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1388</v>
+        <v>1</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1411</v>
+        <v>1</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1415</v>
+        <v>1</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3588,8 +3610,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
-        <v>46023</v>
+      <c r="N38" s="49" t="n">
+        <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3602,19 +3624,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.009101975493255475</v>
+        <v>0.00667093146994231</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.01130167174427415</v>
+        <v>0.00830161397958413</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.01269705928692578</v>
+        <v>0.01125517292572641</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01313965942447244</v>
+        <v>0.01266604881062719</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01298257285949245</v>
+        <v>0.01312727250279332</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3624,8 +3646,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>46023</v>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3638,19 +3662,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.05068493150684932</v>
+        <v>1</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>-0.01689189189189189</v>
+        <v>1</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>-0.07957559681697612</v>
+        <v>1</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>-0.0119047619047619</v>
+        <v>1</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>-0.01324965132496513</v>
+        <v>1</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3663,8 +3687,10 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
-        <v>46082</v>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
+        </is>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3677,19 +3703,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>119.9199</v>
+        <v>1</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>117.906</v>
+        <v>1</v>
       </c>
       <c r="S39" s="6" t="n">
-        <v>119.2298</v>
+        <v>1</v>
       </c>
       <c r="T39" s="6" t="n">
-        <v>120.1883</v>
+        <v>1</v>
       </c>
       <c r="U39" s="21" t="n">
-        <v>121.4177</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3738,8 +3764,10 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
-        <v>46082</v>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
+        </is>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3752,19 +3780,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
-        <v>-0.05008673748247425</v>
+        <v>1</v>
       </c>
       <c r="R40" s="38" t="n">
-        <v>-0.07796471263522881</v>
+        <v>1</v>
       </c>
       <c r="S40" s="38" t="n">
-        <v>-0.07456792269916472</v>
+        <v>1</v>
       </c>
       <c r="T40" s="38" t="n">
-        <v>-0.05790675033979801</v>
+        <v>1</v>
       </c>
       <c r="U40" s="23" t="n">
-        <v>-0.03874237696864814</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -3853,8 +3881,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="48" t="n">
-        <v>46082</v>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3867,19 +3897,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>3980000</v>
+        <v>1000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>4130000</v>
+        <v>1000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>4020000</v>
+        <v>1000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>4270000</v>
+        <v>1000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>4090000</v>
+        <v>1000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3924,8 +3954,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="48" t="n">
-        <v>46082</v>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3938,19 +3970,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.009950248756218905</v>
+        <v>1</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="I43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="J43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -4003,8 +4035,10 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="48" t="n">
-        <v>45931</v>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GCE' not found in values file."</t>
+        </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4017,19 +4051,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5343.513</v>
+        <v>1</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>5324.402</v>
+        <v>1</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>5236.97</v>
+        <v>1</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>5195.517</v>
+        <v>1</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>5150.725</v>
+        <v>1</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4074,8 +4108,10 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="48" t="n">
-        <v>45931</v>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GCE' not found in values file."</t>
+        </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4088,19 +4124,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.003589323270481781</v>
+        <v>1</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>0.01669515005814426</v>
+        <v>1</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>0.007978609251013902</v>
+        <v>1</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>0.008696251498575336</v>
+        <v>1</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>0.01254255520332359</v>
+        <v>1</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4252,7 +4288,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4331,7 +4367,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4344,19 +4380,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.83</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.72</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.71</v>
       </c>
     </row>
     <row r="49">
@@ -4406,7 +4442,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4419,19 +4455,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.96</v>
-      </c>
-      <c r="R49" s="6" t="n">
-        <v>3.91</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>3.91</v>
       </c>
       <c r="T49" s="6" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>3.86</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.84</v>
       </c>
     </row>
     <row r="50">
@@ -4485,7 +4521,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4498,16 +4534,16 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.34</v>
-      </c>
-      <c r="R50" s="6" t="n">
-        <v>4.3</v>
       </c>
       <c r="S50" s="6" t="n">
         <v>4.3</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>4.26</v>
+        <v>4.3</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.26</v>
@@ -4611,7 +4647,7 @@
         </is>
       </c>
       <c r="N52" s="50" t="n">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4624,19 +4660,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.02</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.99</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>5.98</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.98</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-29
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -928,10 +928,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
-        </is>
+      <c r="N3" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
@@ -944,19 +942,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>1</v>
+        <v>178</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>1</v>
+        <v>-133</v>
       </c>
       <c r="S3" s="24" t="n">
-        <v>1</v>
+        <v>160</v>
       </c>
       <c r="T3" s="24" t="n">
-        <v>1</v>
+        <v>-17</v>
       </c>
       <c r="U3" s="26" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -1001,10 +999,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
-        </is>
+      <c r="N4" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
@@ -1017,19 +1013,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>1</v>
+        <v>0.001641652512675452</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>1</v>
+        <v>0.0009411913334596677</v>
       </c>
       <c r="S4" s="38" t="n">
-        <v>1</v>
+        <v>0.002047160512548336</v>
       </c>
       <c r="T4" s="38" t="n">
-        <v>1</v>
+        <v>0.0007327117916066601</v>
       </c>
       <c r="U4" s="23" t="n">
-        <v>1</v>
+        <v>0.002340601850973247</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1211,7 +1207,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.241</v>
+        <v>1.2392</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>4.2373</v>
@@ -1663,10 +1659,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
-        </is>
+      <c r="C13" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1679,19 +1673,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>1</v>
+        <v>-0.002351474629571859</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>1</v>
+        <v>-0.003219338623591583</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>1</v>
+        <v>-0.002197864126912585</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>1</v>
+        <v>0.001326110264657787</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>1</v>
+        <v>0.001497640509762865</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1740,10 +1734,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCENDC96' not found in values file."</t>
-        </is>
+      <c r="C14" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1756,19 +1748,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>1</v>
+        <v>0.009141710846826219</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>1</v>
+        <v>0.01597490069656324</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>1</v>
+        <v>0.01400263444247182</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>1</v>
+        <v>0.02601983289485096</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>1</v>
+        <v>0.02448330683624796</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1821,10 +1813,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
-        </is>
+      <c r="C15" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1837,19 +1827,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>1</v>
+        <v>0.0008222569598179685</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>1</v>
+        <v>0.003163466942223581</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>1</v>
+        <v>0.002845221754583793</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>1</v>
+        <v>-9.089339114154438e-05</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>1</v>
+        <v>0.002606326264660508</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1898,10 +1888,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCESC96' not found in values file."</t>
-        </is>
+      <c r="C16" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1914,19 +1902,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>1</v>
+        <v>0.03044004093404044</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>1</v>
+        <v>0.02628992173300197</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>1</v>
+        <v>0.02311045163683583</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>1</v>
+        <v>0.02359662426842094</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>1</v>
+        <v>0.02571298048684977</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -1951,10 +1939,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C17" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1967,19 +1953,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>1</v>
+        <v>0.01661457854582227</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>1</v>
+        <v>0.007173558174711436</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>1</v>
+        <v>-0.0002912686109073359</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>1</v>
+        <v>-1.361066422789214e-06</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>1</v>
+        <v>0.005016065910586232</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2040,10 +2026,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C18" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2056,19 +2040,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>1</v>
+        <v>0.03969447708578144</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>1</v>
+        <v>0.03962618135825458</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>1</v>
+        <v>0.03267862666254253</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>1</v>
+        <v>0.02433131408893505</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>1</v>
+        <v>0.03212039564348258</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2271,10 +2255,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
-        </is>
+      <c r="C21" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2287,19 +2269,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1</v>
+        <v>3.9</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2805,8 +2787,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
-        <v>46054</v>
+      <c r="C28" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2819,19 +2801,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.01280100007813112</v>
+        <v>0.008328906427866656</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>-0.01164778498320185</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>-0.004254034642219184</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>-0.00913646104747079</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>0.05441037812530491</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>-0.02093605859677161</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2880,8 +2862,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
-        <v>46054</v>
+      <c r="C29" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2894,19 +2876,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.07447318740752079</v>
+        <v>0.008434135003083345</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.07572835348742282</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.09883411459674789</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.1059440595541697</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.1247312200873968</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.04877483240471108</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2920,7 +2902,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2933,19 +2915,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.15</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.16</v>
       </c>
     </row>
     <row r="30">
@@ -2959,8 +2941,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
-        <v>46054</v>
+      <c r="C30" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2973,19 +2955,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.01149211309276466</v>
+        <v>-0.002931495230851011</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>-0.01228994564765717</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>0.002385879326488816</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>-0.01921059426035288</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>0.06592882125886601</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>-0.0128376635658648</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -2999,7 +2981,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3015,13 +2997,13 @@
         <v>2.44</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.42</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.38</v>
+        <v>2.42</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.38</v>
@@ -3034,8 +3016,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
-        <v>46054</v>
+      <c r="C31" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3048,19 +3030,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.07367676103887663</v>
+        <v>-0.0184874116629725</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.07281018801024</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.09283155684402497</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.1010908210327026</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.1265306873826442</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.05011084527755218</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3113,10 +3095,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C32" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3129,19 +3109,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>1</v>
+        <v>-0.005415070741811912</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>1</v>
+        <v>0.007368443846867079</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>1</v>
+        <v>-0.0001564786593617473</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>1</v>
+        <v>0.005246287630711999</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>1</v>
+        <v>-0.001368313417869027</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3186,10 +3166,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C33" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3202,19 +3180,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>1</v>
+        <v>0.007416835246099523</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>1</v>
+        <v>0.01231165794421915</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>1</v>
+        <v>0.01529710277450485</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>1</v>
+        <v>0.01279811178014365</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>1</v>
+        <v>0.0180124379988418</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3267,10 +3245,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TCU' not found in values file."</t>
-        </is>
+      <c r="C34" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3283,19 +3259,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>1</v>
+        <v>75.6596</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>1</v>
+        <v>76.1407</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>1</v>
+        <v>75.6564</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>1</v>
+        <v>75.7296</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>1</v>
+        <v>75.42489999999999</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3423,8 +3399,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
-        <v>46023</v>
+      <c r="C36" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3437,19 +3413,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1487</v>
+        <v>1502</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1387</v>
+        <v>1356</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1398</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>1373</v>
+      </c>
+      <c r="J36" s="24" t="n">
         <v>1324</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>1272</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1328</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3494,8 +3470,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
-        <v>46023</v>
+      <c r="C37" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3508,19 +3484,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.09499263622974963</v>
+        <v>0.1084870848708487</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.08388375165125496</v>
+        <v>-0.08993288590604027</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>0.02945508100147275</v>
+      </c>
+      <c r="I37" s="25" t="n">
+        <v>-0.09313077939233817</v>
+      </c>
+      <c r="J37" s="25" t="n">
         <v>0.02239382239382239</v>
-      </c>
-      <c r="I37" s="25" t="n">
-        <v>-0.05917159763313609</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>-0.02137067059690494</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3573,10 +3549,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C38" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3589,19 +3563,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>1372</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1</v>
+        <v>1538</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1</v>
+        <v>1386</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1</v>
+        <v>1455</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1</v>
+        <v>1388</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3646,10 +3620,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C39" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3662,19 +3634,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07359891964888589</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>1</v>
+        <v>0.0577716643741403</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>1</v>
+        <v>-0.05068493150684932</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>1</v>
+        <v>-0.01689189189189189</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07957559681697612</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3687,10 +3659,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
-        </is>
+      <c r="N39" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3703,19 +3673,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>1</v>
+        <v>119.9199</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>1</v>
+        <v>117.906</v>
       </c>
       <c r="S39" s="6" t="n">
-        <v>1</v>
+        <v>119.2298</v>
       </c>
       <c r="T39" s="6" t="n">
-        <v>1</v>
+        <v>120.1883</v>
       </c>
       <c r="U39" s="21" t="n">
-        <v>1</v>
+        <v>121.4177</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3764,10 +3734,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
-        </is>
+      <c r="N40" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3780,19 +3748,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
-        <v>1</v>
+        <v>-0.05008673748247425</v>
       </c>
       <c r="R40" s="38" t="n">
-        <v>1</v>
+        <v>-0.07796471263522881</v>
       </c>
       <c r="S40" s="38" t="n">
-        <v>1</v>
+        <v>-0.07456792269916472</v>
       </c>
       <c r="T40" s="38" t="n">
-        <v>1</v>
+        <v>-0.05790675033979801</v>
       </c>
       <c r="U40" s="23" t="n">
-        <v>1</v>
+        <v>-0.03874237696864814</v>
       </c>
     </row>
     <row r="41">
@@ -3881,10 +3849,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C42" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3897,19 +3863,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>1000</v>
+        <v>3980000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>1000</v>
+        <v>4130000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>1000</v>
+        <v>4020000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>1000</v>
+        <v>4270000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>1000</v>
+        <v>4090000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3954,10 +3920,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C43" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3970,19 +3934,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>1</v>
+        <v>-0.009950248756218905</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="H43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="I43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="J43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -4035,10 +3999,8 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GCE' not found in values file."</t>
-        </is>
+      <c r="C44" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4051,19 +4013,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>1</v>
+        <v>5343.513</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>1</v>
+        <v>5324.402</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>1</v>
+        <v>5236.97</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>1</v>
+        <v>5195.517</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>1</v>
+        <v>5150.725</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4108,10 +4070,8 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GCE' not found in values file."</t>
-        </is>
+      <c r="C45" s="48" t="n">
+        <v>45931</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4124,19 +4084,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>1</v>
+        <v>0.003589323270481781</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>1</v>
+        <v>0.01669515005814426</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>1</v>
+        <v>0.007978609251013902</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>1</v>
+        <v>0.008696251498575336</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>1</v>
+        <v>0.01254255520332359</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4288,7 +4248,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4367,7 +4327,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4383,16 +4343,16 @@
         <v>3.78</v>
       </c>
       <c r="R48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="S48" s="6" t="n">
         <v>3.83</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.79</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.78</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.72</v>
       </c>
     </row>
     <row r="49">
@@ -4442,7 +4402,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4455,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.96</v>
-      </c>
-      <c r="S49" s="6" t="n">
-        <v>3.91</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>3.91</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>3.86</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="50">
@@ -4521,7 +4481,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4534,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.31</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.34</v>
-      </c>
-      <c r="S50" s="6" t="n">
-        <v>4.3</v>
       </c>
       <c r="T50" s="6" t="n">
         <v>4.3</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.26</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-04-30
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -354,13 +354,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -890,7 +887,7 @@
         </is>
       </c>
       <c r="C3" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -903,19 +900,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
+        <v>24174.527</v>
+      </c>
+      <c r="G3" s="24" t="n">
         <v>24055.749</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="H3" s="24" t="n">
         <v>24026.834</v>
       </c>
-      <c r="H3" s="24" t="n">
+      <c r="I3" s="24" t="n">
         <v>23770.976</v>
       </c>
-      <c r="I3" s="24" t="n">
+      <c r="J3" s="24" t="n">
         <v>23548.21</v>
-      </c>
-      <c r="J3" s="24" t="n">
-        <v>23586.542</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -928,7 +925,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
+      <c r="N3" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -965,7 +962,7 @@
         </is>
       </c>
       <c r="C4" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -978,19 +975,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
+        <v>0.004937613873506885</v>
+      </c>
+      <c r="G4" s="25" t="n">
         <v>0.001203446113624551</v>
       </c>
-      <c r="G4" s="25" t="n">
+      <c r="H4" s="25" t="n">
         <v>0.0107634621312982</v>
       </c>
-      <c r="H4" s="25" t="n">
+      <c r="I4" s="25" t="n">
         <v>0.009459997171759493</v>
       </c>
-      <c r="I4" s="25" t="n">
+      <c r="J4" s="25" t="n">
         <v>-0.001625164044818495</v>
-      </c>
-      <c r="J4" s="25" t="n">
-        <v>0.004598746857240599</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -999,7 +996,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
+      <c r="N4" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1039,7 +1036,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="48" t="n">
+      <c r="C5" s="49" t="n">
         <v>45931</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1078,7 +1075,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
+      <c r="N5" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1114,7 +1111,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="48" t="n">
+      <c r="C6" s="49" t="n">
         <v>45931</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1153,7 +1150,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
+      <c r="N6" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1194,7 +1191,7 @@
         </is>
       </c>
       <c r="C7" s="48" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1207,19 +1204,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
+        <v>3.7007</v>
+      </c>
+      <c r="G7" s="41" t="n">
         <v>1.2392</v>
       </c>
-      <c r="G7" s="41" t="n">
+      <c r="H7" s="41" t="n">
         <v>4.2373</v>
       </c>
-      <c r="H7" s="41" t="n">
+      <c r="I7" s="41" t="n">
         <v>3.4728</v>
       </c>
-      <c r="I7" s="41" t="n">
+      <c r="J7" s="41" t="n">
         <v>2.902</v>
-      </c>
-      <c r="J7" s="41" t="n">
-        <v>-2.7318</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1232,7 +1229,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
+      <c r="N7" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1272,7 +1269,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1311,7 +1308,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
+      <c r="N8" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -1351,8 +1348,10 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="48" t="n">
-        <v>45931</v>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -1365,19 +1364,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16665.219</v>
+        <v>1</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>16585.878</v>
+        <v>1</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>16445.685</v>
+        <v>1</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>16345.793</v>
+        <v>1</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>16320.89</v>
+        <v>1</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1390,7 +1389,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
+      <c r="N9" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1426,8 +1425,10 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="48" t="n">
-        <v>45931</v>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -1440,19 +1441,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.004783647872002916</v>
+        <v>1</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>0.008524606910566446</v>
+        <v>1</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>0.006111174905983452</v>
+        <v>1</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>0.001525835907232986</v>
+        <v>1</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>0.009595708660423696</v>
+        <v>1</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1465,7 +1466,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
+      <c r="N10" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1506,7 +1507,7 @@
         </is>
       </c>
       <c r="C11" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1519,19 +1520,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>0.008870546938001267</v>
+        <v>0.009363644833690454</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>-0.01403114915111547</v>
+        <v>0.01734597156398099</v>
       </c>
       <c r="H11" s="25" t="n">
+        <v>-0.01314250970487807</v>
+      </c>
+      <c r="I11" s="25" t="n">
         <v>-0.00581233144238813</v>
       </c>
-      <c r="I11" s="25" t="n">
+      <c r="J11" s="25" t="n">
         <v>0.007353974425031495</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>0</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1544,7 +1545,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1581,7 +1582,7 @@
         </is>
       </c>
       <c r="C12" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1594,19 +1595,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.01673200114733722</v>
+        <v>-0.005690422651553436</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.008853369065849924</v>
+        <v>0.02619753322497357</v>
       </c>
       <c r="H12" s="25" t="n">
+        <v>0.009762633996937256</v>
+      </c>
+      <c r="I12" s="25" t="n">
         <v>-0.02262753702687877</v>
       </c>
-      <c r="I12" s="25" t="n">
+      <c r="J12" s="25" t="n">
         <v>0.008866163156166484</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>0.01855916030534355</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1619,7 +1620,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1660,7 +1661,7 @@
         </is>
       </c>
       <c r="C13" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1673,19 +1674,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>-0.002351474629571859</v>
+        <v>0.003475754493048377</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>-0.003219338623591583</v>
+        <v>0</v>
       </c>
       <c r="H13" s="25" t="n">
+        <v>-0.0006495156872157182</v>
+      </c>
+      <c r="I13" s="25" t="n">
         <v>-0.002197864126912585</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="J13" s="25" t="n">
         <v>0.001326110264657787</v>
-      </c>
-      <c r="J13" s="25" t="n">
-        <v>0.001497640509762865</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1698,8 +1699,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
-        <v>46125</v>
+      <c r="N13" s="48" t="n">
+        <v>46132</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1712,19 +1713,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>214000</v>
+        <v>189000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>215000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>208000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>218000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>203000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>211000</v>
       </c>
     </row>
     <row r="14">
@@ -1735,7 +1736,7 @@
         </is>
       </c>
       <c r="C14" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1748,19 +1749,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.009141710846826219</v>
+        <v>0.0137310876391664</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01597490069656324</v>
+        <v>0.01412809858145871</v>
       </c>
       <c r="H14" s="25" t="n">
+        <v>0.01859420873870254</v>
+      </c>
+      <c r="I14" s="25" t="n">
         <v>0.01400263444247182</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="J14" s="25" t="n">
         <v>0.02601983289485096</v>
-      </c>
-      <c r="J14" s="25" t="n">
-        <v>0.02448330683624796</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1773,8 +1774,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
-        <v>46118</v>
+      <c r="N14" s="48" t="n">
+        <v>46125</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1788,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1821000</v>
+        <v>1785000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1808000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1809000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1787000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1832000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1816000</v>
       </c>
     </row>
     <row r="15">
@@ -1814,7 +1815,7 @@
         </is>
       </c>
       <c r="C15" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1827,19 +1828,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.0008222569598179685</v>
+        <v>0.0009659131941934795</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.003163466942223581</v>
+        <v>0.001283511397942805</v>
       </c>
       <c r="H15" s="25" t="n">
+        <v>0.002828085060096797</v>
+      </c>
+      <c r="I15" s="25" t="n">
         <v>0.002845221754583793</v>
       </c>
-      <c r="I15" s="25" t="n">
+      <c r="J15" s="25" t="n">
         <v>-9.089339114154438e-05</v>
-      </c>
-      <c r="J15" s="25" t="n">
-        <v>0.002606326264660508</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1852,7 +1853,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
+      <c r="N15" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1889,7 +1890,7 @@
         </is>
       </c>
       <c r="C16" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1902,19 +1903,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.03044004093404044</v>
+        <v>0.02780790300603432</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02628992173300197</v>
+        <v>0.03057028560796356</v>
       </c>
       <c r="H16" s="25" t="n">
+        <v>0.02594680811602797</v>
+      </c>
+      <c r="I16" s="25" t="n">
         <v>0.02311045163683583</v>
       </c>
-      <c r="I16" s="25" t="n">
+      <c r="J16" s="25" t="n">
         <v>0.02359662426842094</v>
-      </c>
-      <c r="J16" s="25" t="n">
-        <v>0.02571298048684977</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -1939,7 +1940,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
+      <c r="C17" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2026,7 +2027,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
+      <c r="C18" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2065,7 +2066,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
+      <c r="N18" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2106,7 +2107,7 @@
         </is>
       </c>
       <c r="C19" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2119,19 +2120,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.004526180904246169</v>
+        <v>-0.0005629480818372112</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.006225581884386822</v>
+        <v>-0.003744432836641498</v>
       </c>
       <c r="H19" s="25" t="n">
+        <v>0.006441402056378998</v>
+      </c>
+      <c r="I19" s="25" t="n">
         <v>-0.0004425121414268762</v>
       </c>
-      <c r="I19" s="25" t="n">
+      <c r="J19" s="25" t="n">
         <v>0.0008581029834302534</v>
-      </c>
-      <c r="J19" s="25" t="n">
-        <v>-0.001740850861583043</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2140,7 +2141,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
+      <c r="N19" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2177,7 +2178,7 @@
         </is>
       </c>
       <c r="C20" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2190,19 +2191,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.01062505234359729</v>
+        <v>0.004415084502276996</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01639481715838071</v>
+        <v>0.01163563272940462</v>
       </c>
       <c r="H20" s="25" t="n">
+        <v>0.01661281847756826</v>
+      </c>
+      <c r="I20" s="25" t="n">
         <v>0.01134436615382877</v>
       </c>
-      <c r="I20" s="25" t="n">
+      <c r="J20" s="25" t="n">
         <v>0.01272729309745998</v>
-      </c>
-      <c r="J20" s="25" t="n">
-        <v>0.01418264506891994</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2215,7 +2216,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
+      <c r="N20" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2256,7 +2257,7 @@
         </is>
       </c>
       <c r="C21" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2269,16 +2270,16 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="G21" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H21" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="I21" s="6" t="n">
         <v>3.9</v>
-      </c>
-      <c r="I21" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>4</v>
@@ -2290,7 +2291,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
+      <c r="N21" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2330,7 +2331,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C22" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2344,13 +2345,13 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.686</v>
+        <v>16.696</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.134</v>
+        <v>16.098</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>15.215</v>
+        <v>15.197</v>
       </c>
       <c r="I22" s="24" t="n">
         <v>16.4</v>
@@ -2369,7 +2370,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
+      <c r="N22" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2405,7 +2406,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
+      <c r="C23" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2419,13 +2420,13 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.09068119891008182</v>
+        <v>-0.09013623978201633</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.01735793897314088</v>
+        <v>-0.01955052073816928</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.04608150470219433</v>
+        <v>-0.04721003134796239</v>
       </c>
       <c r="I23" s="25" t="n">
         <v>-0.05207791457141205</v>
@@ -2439,7 +2440,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
+      <c r="N23" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2479,7 +2480,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
+      <c r="C24" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2519,7 +2520,7 @@
         </is>
       </c>
       <c r="N24" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
@@ -2532,19 +2533,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.00375295622843419</v>
+        <v>0.006641747242902563</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.003025447984071672</v>
+        <v>0.003751937984496134</v>
       </c>
       <c r="S24" s="38" t="n">
+        <v>0.003297660527625812</v>
+      </c>
+      <c r="T24" s="38" t="n">
         <v>0.003308571071852118</v>
       </c>
-      <c r="T24" s="38" t="n">
+      <c r="U24" s="23" t="n">
         <v>0.00219752719537647</v>
-      </c>
-      <c r="U24" s="23" t="n">
-        <v>0.001927522037218354</v>
       </c>
     </row>
     <row r="25">
@@ -2558,7 +2559,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="48" t="n">
+      <c r="C25" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2594,7 +2595,7 @@
         </is>
       </c>
       <c r="N25" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
@@ -2607,19 +2608,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.02801756656951585</v>
+        <v>0.0349608149847944</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.02828962580830351</v>
+        <v>0.02829551861881658</v>
       </c>
       <c r="S25" s="38" t="n">
+        <v>0.02856869483403365</v>
+      </c>
+      <c r="T25" s="38" t="n">
         <v>0.02878083518031025</v>
       </c>
-      <c r="T25" s="38" t="n">
+      <c r="U25" s="23" t="n">
         <v>0.02820189831269997</v>
-      </c>
-      <c r="U25" s="23" t="n">
-        <v>0.02712580525969119</v>
       </c>
     </row>
     <row r="26">
@@ -2633,8 +2634,10 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n">
-        <v>45931</v>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2647,19 +2650,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.005923787970366412</v>
+        <v>1</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>0.007794617579222285</v>
+        <v>1</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>0.01778138610314484</v>
+        <v>1</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>0.02303791460563676</v>
+        <v>1</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>-0.009359213919614473</v>
+        <v>1</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2673,7 +2676,7 @@
         </is>
       </c>
       <c r="N26" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2686,19 +2689,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.003668567155808988</v>
+        <v>0.002932483068401215</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.00392537103357693</v>
+        <v>0.003675182396499332</v>
       </c>
       <c r="S26" s="38" t="n">
+        <v>0.004245969066199562</v>
+      </c>
+      <c r="T26" s="38" t="n">
         <v>0.003271383630529812</v>
       </c>
-      <c r="T26" s="38" t="n">
+      <c r="U26" s="23" t="n">
         <v>0.001776129138734595</v>
-      </c>
-      <c r="U26" s="23" t="n">
-        <v>0.002276415079477623</v>
       </c>
     </row>
     <row r="27">
@@ -2713,7 +2716,7 @@
         </is>
       </c>
       <c r="C27" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2726,19 +2729,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
+        <v>-0.02054026778170115</v>
+      </c>
+      <c r="G27" s="38" t="n">
         <v>-0.004277328978805506</v>
       </c>
-      <c r="G27" s="38" t="n">
+      <c r="H27" s="38" t="n">
         <v>-0.01832684674964358</v>
       </c>
-      <c r="H27" s="38" t="n">
+      <c r="I27" s="38" t="n">
         <v>-0.01299350008050415</v>
       </c>
-      <c r="I27" s="38" t="n">
+      <c r="J27" s="38" t="n">
         <v>-0.002410568051752549</v>
-      </c>
-      <c r="J27" s="38" t="n">
-        <v>0.01049622222903812</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2748,7 +2751,7 @@
         </is>
       </c>
       <c r="N27" s="48" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2761,19 +2764,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.0296775740141437</v>
+        <v>0.03202758906974702</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03050880107876425</v>
+        <v>0.03001318470574146</v>
       </c>
       <c r="S27" s="38" t="n">
+        <v>0.03083788838321814</v>
+      </c>
+      <c r="T27" s="38" t="n">
         <v>0.02971110180682146</v>
       </c>
-      <c r="T27" s="38" t="n">
+      <c r="U27" s="23" t="n">
         <v>0.02829092786499081</v>
-      </c>
-      <c r="U27" s="23" t="n">
-        <v>0.0275453840687383</v>
       </c>
     </row>
     <row r="28">
@@ -2787,7 +2790,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="49" t="n">
+      <c r="C28" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2826,7 +2829,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
+      <c r="N28" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -2862,7 +2865,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="49" t="n">
+      <c r="C29" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2901,8 +2904,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="49" t="n">
-        <v>46140</v>
+      <c r="N29" s="48" t="n">
+        <v>46141</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2918,16 +2921,16 @@
         <v>2.25</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.15</v>
       </c>
     </row>
     <row r="30">
@@ -2941,7 +2944,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="49" t="n">
+      <c r="C30" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2980,8 +2983,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="49" t="n">
-        <v>46140</v>
+      <c r="N30" s="48" t="n">
+        <v>46141</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +2997,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.44</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.42</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.38</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="31">
@@ -3016,7 +3019,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="49" t="n">
+      <c r="C31" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3056,7 +3059,7 @@
         </is>
       </c>
       <c r="N31" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3069,19 +3072,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>0.007310493043885868</v>
+        <v>0.007177997310378714</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>0.007996957929548465</v>
+        <v>0.007345039668930076</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>0.01027939464493599</v>
+        <v>0.007979811365325773</v>
       </c>
       <c r="T31" s="38" t="n">
+        <v>0.01026193247962737</v>
+      </c>
+      <c r="U31" s="23" t="n">
         <v>0.007624633431085215</v>
-      </c>
-      <c r="U31" s="23" t="n">
-        <v>0.009473060982829962</v>
       </c>
     </row>
     <row r="32">
@@ -3095,7 +3098,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
+      <c r="C32" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3131,7 +3134,7 @@
         </is>
       </c>
       <c r="N32" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3144,19 +3147,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
+        <v>0.03316647264260756</v>
+      </c>
+      <c r="R32" s="38" t="n">
         <v>0.03362463343108507</v>
       </c>
-      <c r="R32" s="38" t="n">
-        <v>0.03584369449378332</v>
-      </c>
       <c r="S32" s="38" t="n">
-        <v>0.03559665871121723</v>
+        <v>0.0358081705150977</v>
       </c>
       <c r="T32" s="38" t="n">
+        <v>0.03557875894988063</v>
+      </c>
+      <c r="U32" s="23" t="n">
         <v>0.03369434416365838</v>
-      </c>
-      <c r="U32" s="23" t="n">
-        <v>0.03710462287104619</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3166,7 +3169,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
+      <c r="C33" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3205,7 +3208,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
+      <c r="N33" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -3245,7 +3248,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
+      <c r="C34" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -3280,8 +3283,8 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="48" t="n">
-        <v>46054</v>
+      <c r="N34" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
@@ -3294,19 +3297,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>0.009284897536239168</v>
+        <v>0.0002024211398903792</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>0.008034422666587262</v>
+        <v>0.00901208412752658</v>
       </c>
       <c r="S34" s="38" t="n">
+        <v>0.007760924955011093</v>
+      </c>
+      <c r="T34" s="38" t="n">
         <v>0.008247145515396716</v>
       </c>
-      <c r="T34" s="38" t="n">
+      <c r="U34" s="23" t="n">
         <v>0.01081883276249912</v>
-      </c>
-      <c r="U34" s="23" t="n">
-        <v>0.01175444356788234</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3320,7 +3323,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="48" t="n">
+      <c r="C35" s="49" t="n">
         <v>45931</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -3359,8 +3362,8 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="48" t="n">
-        <v>46054</v>
+      <c r="N35" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
@@ -3373,19 +3376,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>1.549168846470828e-05</v>
+        <v>-0.004200333998298111</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.0004847009215600551</v>
+        <v>1.650614201031964e-05</v>
       </c>
       <c r="S35" s="38" t="n">
+        <v>0.0002132515841006821</v>
+      </c>
+      <c r="T35" s="38" t="n">
         <v>-0.002758902506289296</v>
       </c>
-      <c r="T35" s="38" t="n">
+      <c r="U35" s="23" t="n">
         <v>0.001868922106829984</v>
-      </c>
-      <c r="U35" s="23" t="n">
-        <v>0.00215551661749025</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3399,7 +3402,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="49" t="n">
+      <c r="C36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3434,8 +3437,8 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="48" t="n">
-        <v>46054</v>
+      <c r="N36" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
@@ -3448,19 +3451,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>0.009284897536239168</v>
+        <v>0.0002024211398903792</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>0.008034422666587262</v>
+        <v>0.00901208412752658</v>
       </c>
       <c r="S36" s="38" t="n">
+        <v>0.007760924955011093</v>
+      </c>
+      <c r="T36" s="38" t="n">
         <v>0.008247145515396716</v>
       </c>
-      <c r="T36" s="38" t="n">
+      <c r="U36" s="23" t="n">
         <v>0.01081883276249912</v>
-      </c>
-      <c r="U36" s="23" t="n">
-        <v>0.01175444356788234</v>
       </c>
     </row>
     <row r="37">
@@ -3470,7 +3473,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n">
+      <c r="C37" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3509,7 +3512,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="49" t="n">
+      <c r="N37" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3549,7 +3552,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="49" t="n">
+      <c r="C38" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3584,7 +3587,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="49" t="n">
+      <c r="N38" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -3620,7 +3623,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="49" t="n">
+      <c r="C39" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3659,7 +3662,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
+      <c r="N39" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3699,7 +3702,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
+      <c r="C40" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3734,7 +3737,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
+      <c r="N40" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3770,7 +3773,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
+      <c r="C41" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3809,7 +3812,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
+      <c r="N41" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3849,8 +3852,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="48" t="n">
-        <v>46082</v>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3863,19 +3868,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>3980000</v>
+        <v>1000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>4130000</v>
+        <v>1000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>4020000</v>
+        <v>1000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>4270000</v>
+        <v>1000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>4090000</v>
+        <v>1000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3884,7 +3889,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
+      <c r="N42" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3920,8 +3925,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="48" t="n">
-        <v>46082</v>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3934,19 +3941,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.009950248756218905</v>
+        <v>1</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="I43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="J43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -3959,7 +3966,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
+      <c r="N43" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4000,7 +4007,7 @@
         </is>
       </c>
       <c r="C44" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4013,19 +4020,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
+        <v>5418.445</v>
+      </c>
+      <c r="G44" s="24" t="n">
         <v>5343.513</v>
       </c>
-      <c r="G44" s="24" t="n">
+      <c r="H44" s="24" t="n">
         <v>5324.402</v>
       </c>
-      <c r="H44" s="24" t="n">
+      <c r="I44" s="24" t="n">
         <v>5236.97</v>
       </c>
-      <c r="I44" s="24" t="n">
+      <c r="J44" s="24" t="n">
         <v>5195.517</v>
-      </c>
-      <c r="J44" s="24" t="n">
-        <v>5150.725</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4034,7 +4041,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
+      <c r="N44" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4071,7 +4078,7 @@
         </is>
       </c>
       <c r="C45" s="48" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4084,19 +4091,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
+        <v>0.01402298450476303</v>
+      </c>
+      <c r="G45" s="38" t="n">
         <v>0.003589323270481781</v>
       </c>
-      <c r="G45" s="38" t="n">
+      <c r="H45" s="38" t="n">
         <v>0.01669515005814426</v>
       </c>
-      <c r="H45" s="38" t="n">
+      <c r="I45" s="38" t="n">
         <v>0.007978609251013902</v>
       </c>
-      <c r="I45" s="38" t="n">
+      <c r="J45" s="38" t="n">
         <v>0.008696251498575336</v>
-      </c>
-      <c r="J45" s="38" t="n">
-        <v>0.01254255520332359</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4121,7 +4128,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
+      <c r="C46" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4208,7 +4215,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
+      <c r="C47" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4247,8 +4254,10 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="49" t="n">
-        <v>46139</v>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DFF' not found in values file."</t>
+        </is>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4261,19 +4270,19 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -4287,7 +4296,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
+      <c r="C48" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4326,8 +4335,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
-        <v>46139</v>
+      <c r="N48" s="48" t="n">
+        <v>46140</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4340,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.78</v>
+        <v>3.84</v>
       </c>
       <c r="R48" s="6" t="n">
         <v>3.78</v>
       </c>
       <c r="S48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="T48" s="6" t="n">
         <v>3.83</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.79</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.78</v>
       </c>
     </row>
     <row r="49">
@@ -4362,7 +4371,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
+      <c r="C49" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4401,8 +4410,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
-        <v>46139</v>
+      <c r="N49" s="48" t="n">
+        <v>46140</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4415,16 +4424,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.96</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>3.91</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>3.91</v>
@@ -4441,7 +4450,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
+      <c r="C50" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4480,8 +4489,10 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
-        <v>46139</v>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
+        </is>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4494,19 +4505,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.35</v>
+        <v>1</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>4.31</v>
+        <v>1</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>4.34</v>
+        <v>1</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4516,7 +4527,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
+      <c r="C51" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4606,8 +4617,10 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="50" t="n">
-        <v>46139</v>
+      <c r="N52" s="20" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
+        </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4633,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.05</v>
+        <v>1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>6.01</v>
+        <v>1</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>6.02</v>
+        <v>1</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>5.99</v>
+        <v>1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -354,10 +354,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -886,8 +886,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
-        <v>46023</v>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -900,19 +902,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24174.527</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24055.749</v>
+        <v>1</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>24026.834</v>
+        <v>1</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>23770.976</v>
+        <v>1</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23548.21</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -925,7 +927,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N3" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -961,8 +963,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
-        <v>46023</v>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -975,19 +979,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.004937613873506885</v>
+        <v>1</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>1</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>1</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>1</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>-0.001625164044818495</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -996,7 +1000,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="49" t="n">
+      <c r="N4" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1036,8 +1040,10 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
-        <v>45931</v>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
+        </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1050,19 +1056,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7855631.5</v>
+        <v>1</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>7774506.8</v>
+        <v>1</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>7621432.3</v>
+        <v>1</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>7510528.3</v>
+        <v>1</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>7456295.5</v>
+        <v>1</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1075,7 +1081,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1111,8 +1117,10 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
-        <v>45931</v>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
+        </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1125,19 +1133,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.0104347069321491</v>
+        <v>1</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>0.02008474181421249</v>
+        <v>1</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>0.0147664712214719</v>
+        <v>1</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>0.007273424182290045</v>
+        <v>1</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>0.01062352837847436</v>
+        <v>1</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1150,7 +1158,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="49" t="n">
+      <c r="N6" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1190,8 +1198,10 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
-        <v>46113</v>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPNOW' not found in values file."</t>
+        </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1204,19 +1214,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.7007</v>
+        <v>1</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>1.2392</v>
+        <v>1</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>4.2373</v>
+        <v>1</v>
       </c>
       <c r="I7" s="41" t="n">
-        <v>3.4728</v>
+        <v>1</v>
       </c>
       <c r="J7" s="41" t="n">
-        <v>2.902</v>
+        <v>1</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1229,7 +1239,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1270,7 +1280,7 @@
         </is>
       </c>
       <c r="C8" s="49" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1283,19 +1293,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>0.48</v>
+        <v>1.82</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>0.2</v>
+        <v>0.46</v>
       </c>
       <c r="H8" s="24" t="n">
         <v>0.24</v>
       </c>
       <c r="I8" s="24" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="J8" s="24" t="n">
         <v>0.34</v>
-      </c>
-      <c r="J8" s="24" t="n">
-        <v>0.82</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1308,7 +1318,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="49" t="n">
+      <c r="N8" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -1348,10 +1358,8 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
-        </is>
+      <c r="C9" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -1364,19 +1372,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>1</v>
+        <v>16731.167</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1</v>
+        <v>16665.219</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>1</v>
+        <v>16585.878</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>1</v>
+        <v>16445.685</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>1</v>
+        <v>16345.793</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1389,7 +1397,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="49" t="n">
+      <c r="N9" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1425,10 +1433,8 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
-        </is>
+      <c r="C10" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -1441,19 +1447,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>1</v>
+        <v>0.00395722372445273</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>1</v>
+        <v>0.004783647872002916</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>1</v>
+        <v>0.008524606910566446</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>1</v>
+        <v>0.006111174905983452</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>1</v>
+        <v>0.001525835907232986</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1466,7 +1472,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
+      <c r="N10" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1506,7 +1512,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
+      <c r="C11" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1545,7 +1551,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1581,7 +1587,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
+      <c r="C12" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1620,7 +1626,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1660,7 +1666,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
+      <c r="C13" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1699,7 +1705,7 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="48" t="n">
+      <c r="N13" s="49" t="n">
         <v>46132</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1735,7 +1741,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1774,7 +1780,7 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="48" t="n">
+      <c r="N14" s="49" t="n">
         <v>46125</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -1814,7 +1820,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
+      <c r="C15" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1853,7 +1859,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="49" t="n">
+      <c r="N15" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1889,7 +1895,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1940,7 +1946,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
+      <c r="C17" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2027,7 +2033,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
+      <c r="C18" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2066,7 +2072,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
+      <c r="N18" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2106,7 +2112,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2141,7 +2147,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2177,7 +2183,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
+      <c r="C20" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2216,7 +2222,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
+      <c r="N20" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2256,7 +2262,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
+      <c r="C21" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2291,7 +2297,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
+      <c r="N21" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2331,7 +2337,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2370,7 +2376,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2406,7 +2412,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2440,7 +2446,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2480,7 +2486,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
+      <c r="C24" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2519,7 +2525,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
+      <c r="N24" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2559,7 +2565,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
+      <c r="C25" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2594,7 +2600,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
+      <c r="N25" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2675,7 +2681,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
+      <c r="N26" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2715,8 +2721,10 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="48" t="n">
-        <v>46023</v>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2729,19 +2737,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.02054026778170115</v>
+        <v>1</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>-0.004277328978805506</v>
+        <v>1</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>-0.01832684674964358</v>
+        <v>1</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>-0.01299350008050415</v>
+        <v>1</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>-0.002410568051752549</v>
+        <v>1</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2750,7 +2758,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
+      <c r="N27" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2790,7 +2798,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
+      <c r="C28" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2829,7 +2837,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="49" t="n">
+      <c r="N28" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -2865,7 +2873,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
+      <c r="C29" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2904,8 +2912,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="48" t="n">
-        <v>46141</v>
+      <c r="N29" s="49" t="n">
+        <v>46142</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,13 +2932,13 @@
         <v>2.25</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="30">
@@ -2944,7 +2952,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
+      <c r="C30" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2983,8 +2991,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="48" t="n">
-        <v>46141</v>
+      <c r="N30" s="49" t="n">
+        <v>46142</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3000,13 +3008,13 @@
         <v>2.46</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.44</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.42</v>
@@ -3019,7 +3027,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
+      <c r="C31" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3058,8 +3066,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="48" t="n">
-        <v>46023</v>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3072,19 +3082,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>0.007177997310378714</v>
+        <v>1</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>0.007345039668930076</v>
+        <v>1</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>0.007979811365325773</v>
+        <v>1</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>0.01026193247962737</v>
+        <v>1</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>0.007624633431085215</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3098,7 +3108,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="49" t="n">
+      <c r="C32" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3133,8 +3143,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="48" t="n">
-        <v>46023</v>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3147,19 +3159,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>0.03316647264260756</v>
+        <v>1</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>0.03362463343108507</v>
+        <v>1</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>0.0358081705150977</v>
+        <v>1</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>0.03557875894988063</v>
+        <v>1</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>0.03369434416365838</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3169,7 +3181,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="49" t="n">
+      <c r="C33" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3208,7 +3220,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="49" t="n">
+      <c r="N33" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -3248,7 +3260,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="49" t="n">
+      <c r="C34" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -3283,7 +3295,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="49" t="n">
+      <c r="N34" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
@@ -3323,7 +3335,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="49" t="n">
+      <c r="C35" s="48" t="n">
         <v>45931</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -3362,7 +3374,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="49" t="n">
+      <c r="N35" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
@@ -3402,7 +3414,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
+      <c r="C36" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3437,7 +3449,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="49" t="n">
+      <c r="N36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
@@ -3473,7 +3485,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
+      <c r="C37" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3512,8 +3524,10 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
-        <v>46054</v>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3526,19 +3540,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.002917033083199794</v>
+        <v>1</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>-0.001828986686322698</v>
+        <v>1</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>-0.002571690054911535</v>
+        <v>1</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.001325270004722268</v>
+        <v>1</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.001961201654098743</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -3552,7 +3566,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
+      <c r="C38" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3587,8 +3601,10 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
-        <v>46054</v>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3601,19 +3617,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.00667093146994231</v>
+        <v>1</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.00830161397958413</v>
+        <v>1</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.01125517292572641</v>
+        <v>1</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01266604881062719</v>
+        <v>1</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01312727250279332</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3623,7 +3639,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
+      <c r="C39" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3662,8 +3678,10 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="49" t="n">
-        <v>46082</v>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
+        </is>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3676,19 +3694,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>119.9199</v>
+        <v>1</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>117.906</v>
+        <v>1</v>
       </c>
       <c r="S39" s="6" t="n">
-        <v>119.2298</v>
+        <v>1</v>
       </c>
       <c r="T39" s="6" t="n">
-        <v>120.1883</v>
+        <v>1</v>
       </c>
       <c r="U39" s="21" t="n">
-        <v>121.4177</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3702,7 +3720,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n">
+      <c r="C40" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3737,8 +3755,10 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="49" t="n">
-        <v>46082</v>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
+        </is>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3751,19 +3771,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
-        <v>-0.05008673748247425</v>
+        <v>1</v>
       </c>
       <c r="R40" s="38" t="n">
-        <v>-0.07796471263522881</v>
+        <v>1</v>
       </c>
       <c r="S40" s="38" t="n">
-        <v>-0.07456792269916472</v>
+        <v>1</v>
       </c>
       <c r="T40" s="38" t="n">
-        <v>-0.05790675033979801</v>
+        <v>1</v>
       </c>
       <c r="U40" s="23" t="n">
-        <v>-0.03874237696864814</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -3773,7 +3793,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n">
+      <c r="C41" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3812,7 +3832,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3889,7 +3909,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="49" t="n">
+      <c r="N42" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3966,7 +3986,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4006,7 +4026,7 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="48" t="n">
+      <c r="C44" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -4041,7 +4061,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4077,7 +4097,7 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="48" t="n">
+      <c r="C45" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -4128,7 +4148,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
+      <c r="C46" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4215,7 +4235,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
+      <c r="C47" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4254,10 +4274,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DFF' not found in values file."</t>
-        </is>
+      <c r="N47" s="49" t="n">
+        <v>46141</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4270,19 +4288,19 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>1</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="48">
@@ -4296,7 +4314,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
+      <c r="C48" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4335,8 +4353,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="48" t="n">
-        <v>46140</v>
+      <c r="N48" s="49" t="n">
+        <v>46141</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.84</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>3.78</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>3.78</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>3.83</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.79</v>
       </c>
     </row>
     <row r="49">
@@ -4371,7 +4389,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
+      <c r="C49" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4410,8 +4428,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="48" t="n">
-        <v>46140</v>
+      <c r="N49" s="49" t="n">
+        <v>46141</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.96</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.91</v>
       </c>
     </row>
     <row r="50">
@@ -4450,7 +4468,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
+      <c r="C50" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4527,7 +4545,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
+      <c r="C51" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4567,7 +4585,7 @@
         </is>
       </c>
       <c r="N51" s="49" t="n">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4580,19 +4598,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.23</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.37</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.46</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.38</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -354,10 +354,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -886,10 +889,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C3" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -902,19 +903,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>1</v>
+        <v>24174.527</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>1</v>
+        <v>24055.749</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>1</v>
+        <v>24026.834</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>1</v>
+        <v>23770.976</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>1</v>
+        <v>23548.21</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -927,7 +928,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
+      <c r="N3" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -963,10 +964,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C4" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -979,19 +978,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>1</v>
+        <v>0.004937613873506885</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>1</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>1</v>
+        <v>0.0107634621312982</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>1</v>
+        <v>0.009459997171759493</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>1</v>
+        <v>-0.001625164044818495</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1000,7 +999,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
+      <c r="N4" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1040,10 +1039,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
-        </is>
+      <c r="C5" s="49" t="n">
+        <v>45931</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1056,19 +1053,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>1</v>
+        <v>7855631.5</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>1</v>
+        <v>7774506.8</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>1</v>
+        <v>7621432.3</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>1</v>
+        <v>7510528.3</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>1</v>
+        <v>7456295.5</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1081,7 +1078,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
+      <c r="N5" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1117,10 +1114,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
-        </is>
+      <c r="C6" s="49" t="n">
+        <v>45931</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1133,19 +1128,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>1</v>
+        <v>0.0104347069321491</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>1</v>
+        <v>0.02008474181421249</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>1</v>
+        <v>0.0147664712214719</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>1</v>
+        <v>0.007273424182290045</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>1</v>
+        <v>0.01062352837847436</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1158,7 +1153,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
+      <c r="N6" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1198,10 +1193,8 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPNOW' not found in values file."</t>
-        </is>
+      <c r="C7" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1214,19 +1207,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1</v>
+        <v>3.5185</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>1</v>
+        <v>1.2392</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>1</v>
+        <v>4.2373</v>
       </c>
       <c r="I7" s="41" t="n">
-        <v>1</v>
+        <v>3.4728</v>
       </c>
       <c r="J7" s="41" t="n">
-        <v>1</v>
+        <v>2.902</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1239,7 +1232,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
+      <c r="N7" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1279,7 +1272,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1318,7 +1311,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
+      <c r="N8" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -1358,7 +1351,7 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="49" t="n">
+      <c r="C9" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1397,7 +1390,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
+      <c r="N9" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1433,7 +1426,7 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="49" t="n">
+      <c r="C10" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1472,7 +1465,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
+      <c r="N10" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1512,7 +1505,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n">
+      <c r="C11" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1551,7 +1544,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1587,7 +1580,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="49" t="n">
+      <c r="C12" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1626,7 +1619,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1666,7 +1659,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="49" t="n">
+      <c r="C13" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1705,7 +1698,7 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
+      <c r="N13" s="48" t="n">
         <v>46132</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1741,7 +1734,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1780,7 +1773,7 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
+      <c r="N14" s="48" t="n">
         <v>46125</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -1820,7 +1813,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1859,7 +1852,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
+      <c r="N15" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1895,7 +1888,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1946,7 +1939,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
+      <c r="C17" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2033,7 +2026,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
+      <c r="C18" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2072,7 +2065,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
+      <c r="N18" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2112,7 +2105,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="49" t="n">
+      <c r="C19" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2147,7 +2140,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
+      <c r="N19" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2183,7 +2176,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2222,7 +2215,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
+      <c r="N20" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2262,7 +2255,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n">
+      <c r="C21" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2297,7 +2290,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
+      <c r="N21" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2337,7 +2330,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C22" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2376,7 +2369,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
+      <c r="N22" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2412,7 +2405,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
+      <c r="C23" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2446,7 +2439,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
+      <c r="N23" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2486,7 +2479,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
+      <c r="C24" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2525,7 +2518,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="49" t="n">
+      <c r="N24" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2565,7 +2558,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="48" t="n">
+      <c r="C25" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2600,7 +2593,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="49" t="n">
+      <c r="N25" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2640,10 +2633,8 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
-        </is>
+      <c r="C26" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2656,19 +2647,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>1</v>
+        <v>0.02495869599850553</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>1</v>
+        <v>0.005923787970366412</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>1</v>
+        <v>0.007794617579222285</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>1</v>
+        <v>0.01778138610314484</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>1</v>
+        <v>0.02303791460563676</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2681,7 +2672,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="49" t="n">
+      <c r="N26" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2721,10 +2712,8 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
-        </is>
+      <c r="C27" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2737,19 +2726,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>1</v>
+        <v>-0.02054026778170115</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>1</v>
+        <v>-0.004277328978805506</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01832684674964358</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01299350008050415</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>1</v>
+        <v>-0.002410568051752549</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2758,7 +2747,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="49" t="n">
+      <c r="N27" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2798,7 +2787,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="49" t="n">
+      <c r="C28" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2837,7 +2826,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
+      <c r="N28" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -2873,7 +2862,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="49" t="n">
+      <c r="C29" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2912,8 +2901,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="49" t="n">
-        <v>46142</v>
+      <c r="N29" s="48" t="n">
+        <v>46143</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2926,7 +2915,7 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.25</v>
@@ -2935,10 +2924,10 @@
         <v>2.25</v>
       </c>
       <c r="T29" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="30">
@@ -2952,7 +2941,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="49" t="n">
+      <c r="C30" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2991,8 +2980,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="49" t="n">
-        <v>46142</v>
+      <c r="N30" s="48" t="n">
+        <v>46143</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3005,19 +2994,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.46</v>
+        <v>2.48</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.46</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.44</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="31">
@@ -3027,7 +3016,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="49" t="n">
+      <c r="C31" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3066,10 +3055,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N31" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3082,19 +3069,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>1</v>
+        <v>0.007177997310378714</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>1</v>
+        <v>0.007345039668930076</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>1</v>
+        <v>0.007979811365325773</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>1</v>
+        <v>0.01026193247962737</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>1</v>
+        <v>0.007624633431085215</v>
       </c>
     </row>
     <row r="32">
@@ -3108,7 +3095,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
+      <c r="C32" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3143,10 +3130,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N32" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3159,19 +3144,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>1</v>
+        <v>0.03316647264260756</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>1</v>
+        <v>0.03362463343108507</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>1</v>
+        <v>0.0358081705150977</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>1</v>
+        <v>0.03557875894988063</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>1</v>
+        <v>0.03369434416365838</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3181,7 +3166,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
+      <c r="C33" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3220,7 +3205,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
+      <c r="N33" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -3260,7 +3245,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
+      <c r="C34" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -3295,7 +3280,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="48" t="n">
+      <c r="N34" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
@@ -3335,7 +3320,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="48" t="n">
+      <c r="C35" s="49" t="n">
         <v>45931</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -3374,7 +3359,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="48" t="n">
+      <c r="N35" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
@@ -3414,7 +3399,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="49" t="n">
+      <c r="C36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3449,7 +3434,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="48" t="n">
+      <c r="N36" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
@@ -3485,7 +3470,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n">
+      <c r="C37" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3524,10 +3509,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
-        </is>
+      <c r="N37" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3540,19 +3523,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>1</v>
+        <v>0.002917033083199794</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>1</v>
+        <v>-0.001828986686322698</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>1</v>
+        <v>-0.002571690054911535</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>1</v>
+        <v>-0.001325270004722268</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>1</v>
+        <v>-0.001961201654098743</v>
       </c>
     </row>
     <row r="38">
@@ -3566,7 +3549,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="49" t="n">
+      <c r="C38" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3601,10 +3584,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
-        </is>
+      <c r="N38" s="48" t="n">
+        <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3617,19 +3598,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>1</v>
+        <v>0.00667093146994231</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>1</v>
+        <v>0.00830161397958413</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>1</v>
+        <v>0.01125517292572641</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>1</v>
+        <v>0.01266604881062719</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>1</v>
+        <v>0.01312727250279332</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3639,7 +3620,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="49" t="n">
+      <c r="C39" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3678,10 +3659,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
-        </is>
+      <c r="N39" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3694,19 +3673,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>1</v>
+        <v>119.9199</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>1</v>
+        <v>117.906</v>
       </c>
       <c r="S39" s="6" t="n">
-        <v>1</v>
+        <v>119.2298</v>
       </c>
       <c r="T39" s="6" t="n">
-        <v>1</v>
+        <v>120.1883</v>
       </c>
       <c r="U39" s="21" t="n">
-        <v>1</v>
+        <v>121.4177</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3720,7 +3699,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
+      <c r="C40" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3755,10 +3734,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TWEXBGSMTH' not found in values file."</t>
-        </is>
+      <c r="N40" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3771,19 +3748,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
-        <v>1</v>
+        <v>-0.05008673748247425</v>
       </c>
       <c r="R40" s="38" t="n">
-        <v>1</v>
+        <v>-0.07796471263522881</v>
       </c>
       <c r="S40" s="38" t="n">
-        <v>1</v>
+        <v>-0.07456792269916472</v>
       </c>
       <c r="T40" s="38" t="n">
-        <v>1</v>
+        <v>-0.05790675033979801</v>
       </c>
       <c r="U40" s="23" t="n">
-        <v>1</v>
+        <v>-0.03874237696864814</v>
       </c>
     </row>
     <row r="41">
@@ -3793,7 +3770,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
+      <c r="C41" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3832,7 +3809,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
+      <c r="N41" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3872,10 +3849,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C42" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3888,19 +3863,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>1000</v>
+        <v>3980000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>1000</v>
+        <v>4130000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>1000</v>
+        <v>4020000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>1000</v>
+        <v>4270000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>1000</v>
+        <v>4090000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3909,7 +3884,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
+      <c r="N42" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3945,10 +3920,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C43" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3961,19 +3934,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>1</v>
+        <v>-0.009950248756218905</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="H43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="I43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="J43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -3986,7 +3959,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
+      <c r="N43" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4026,7 +3999,7 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="49" t="n">
+      <c r="C44" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -4061,7 +4034,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
+      <c r="N44" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4097,7 +4070,7 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="49" t="n">
+      <c r="C45" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -4148,7 +4121,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
+      <c r="C46" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4235,7 +4208,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
+      <c r="C47" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4274,8 +4247,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="49" t="n">
-        <v>46141</v>
+      <c r="N47" s="48" t="n">
+        <v>46142</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4314,7 +4287,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
+      <c r="C48" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4353,8 +4326,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
-        <v>46141</v>
+      <c r="N48" s="48" t="n">
+        <v>46142</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4367,19 +4340,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.92</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.84</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.78</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.78</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.83</v>
+        <v>3.78</v>
       </c>
     </row>
     <row r="49">
@@ -4389,7 +4362,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
+      <c r="C49" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4428,8 +4401,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
-        <v>46141</v>
+      <c r="N49" s="48" t="n">
+        <v>46142</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4442,19 +4415,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>3.97</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.94</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.92</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.96</v>
       </c>
     </row>
     <row r="50">
@@ -4468,7 +4441,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
+      <c r="C50" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4507,10 +4480,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
-        </is>
+      <c r="N50" s="48" t="n">
+        <v>46142</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4523,19 +4494,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="R50" s="6" t="n">
-        <v>1</v>
+        <v>4.42</v>
       </c>
       <c r="S50" s="6" t="n">
-        <v>1</v>
+        <v>4.36</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>1</v>
+        <v>4.35</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>1</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4545,7 +4516,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
+      <c r="C51" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4584,7 +4555,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="48" t="n">
         <v>46139</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4635,10 +4606,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="20" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
-        </is>
+      <c r="N52" s="50" t="n">
+        <v>46142</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4651,19 +4620,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>1</v>
+        <v>6.1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>1</v>
+        <v>6.11</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>1</v>
+        <v>6.06</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>1</v>
+        <v>6.05</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>1</v>
+        <v>6.01</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,9 +358,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1039,8 +1036,10 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
-        <v>45931</v>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
+        </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1053,19 +1052,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7855631.5</v>
+        <v>1</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>7774506.8</v>
+        <v>1</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>7621432.3</v>
+        <v>1</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>7510528.3</v>
+        <v>1</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>7456295.5</v>
+        <v>1</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1114,8 +1113,10 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
-        <v>45931</v>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
+        </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1128,19 +1129,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.0104347069321491</v>
+        <v>1</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>0.02008474181421249</v>
+        <v>1</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>0.0147664712214719</v>
+        <v>1</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>0.007273424182290045</v>
+        <v>1</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>0.01062352837847436</v>
+        <v>1</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1272,8 +1273,10 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
-        <v>46082</v>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RECPROUSM156N' not found in values file."</t>
+        </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1286,19 +1289,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>1.82</v>
+        <v>1</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>0.46</v>
+        <v>1</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>0.24</v>
+        <v>1</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>0.16</v>
+        <v>1</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>0.34</v>
+        <v>1</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1505,8 +1508,10 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
-        <v>46082</v>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1519,19 +1524,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>0.009363644833690454</v>
+        <v>1</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.01734597156398099</v>
+        <v>1</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>-0.01314250970487807</v>
+        <v>1</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>-0.00581233144238813</v>
+        <v>1</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>0.007353974425031495</v>
+        <v>1</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1580,8 +1585,10 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
-        <v>46082</v>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1594,19 +1601,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>-0.005690422651553436</v>
+        <v>1</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.02619753322497357</v>
+        <v>1</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.009762633996937256</v>
+        <v>1</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>-0.02262753702687877</v>
+        <v>1</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>0.008866163156166484</v>
+        <v>1</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1773,8 +1780,10 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="48" t="n">
-        <v>46125</v>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1787,19 +1796,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1785000</v>
+        <v>1</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1808000</v>
+        <v>1</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1809000</v>
+        <v>1</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1787000</v>
+        <v>1</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1832000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1939,8 +1948,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
-        <v>46082</v>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1953,19 +1964,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.01661457854582227</v>
+        <v>1</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.007173558174711436</v>
+        <v>1</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>-0.0002912686109073359</v>
+        <v>1</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>-1.361066422789214e-06</v>
+        <v>1</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>0.005016065910586232</v>
+        <v>1</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2026,8 +2037,10 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
-        <v>46082</v>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
+        </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2040,19 +2053,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.03969447708578144</v>
+        <v>1</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.03962618135825458</v>
+        <v>1</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>0.03267862666254253</v>
+        <v>1</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>0.02433131408893505</v>
+        <v>1</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>0.03212039564348258</v>
+        <v>1</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2215,8 +2228,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
-        <v>46082</v>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2229,19 +2244,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>0.001957950538511444</v>
+        <v>1</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.002160502174024082</v>
+        <v>1</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>0.002950448142634121</v>
+        <v>1</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>0.002329002576704653</v>
+        <v>1</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2290,8 +2305,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
-        <v>46082</v>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2304,19 +2321,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.0260216770548682</v>
+        <v>1</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.02472462476764023</v>
+        <v>1</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>0.02512028782828883</v>
+        <v>1</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>0.02646484707309002</v>
+        <v>1</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>0.02599044806094405</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2672,8 +2689,10 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
-        <v>46082</v>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
+        </is>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2686,19 +2705,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.002932483068401215</v>
+        <v>1</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.003675182396499332</v>
+        <v>1</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.004245969066199562</v>
+        <v>1</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>0.003271383630529812</v>
+        <v>1</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>0.001776129138734595</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -2747,8 +2766,10 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
-        <v>46082</v>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
+        </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2761,19 +2782,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03202758906974702</v>
+        <v>1</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03001318470574146</v>
+        <v>1</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.03083788838321814</v>
+        <v>1</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>0.02971110180682146</v>
+        <v>1</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>0.02829092786499081</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2787,7 +2808,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
+      <c r="C28" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2801,10 +2822,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.008328906427866656</v>
+        <v>0.008462114959539413</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.01164778498320185</v>
+        <v>-0.01169466364559735</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>-0.004254034642219184</v>
@@ -2862,7 +2883,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
+      <c r="C29" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2876,10 +2897,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.008434135003083345</v>
+        <v>0.008519519946871591</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.07572835348742282</v>
+        <v>0.07567733047604469</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.09883411459674789</v>
@@ -2941,7 +2962,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
+      <c r="C30" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2955,10 +2976,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.002931495230851011</v>
+        <v>-0.002810142088861101</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>-0.01228994564765717</v>
+        <v>-0.01222345960141613</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>0.002385879326488816</v>
@@ -2980,8 +3001,10 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="48" t="n">
-        <v>46143</v>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'T10YIE' not found in values file."</t>
+        </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -2994,19 +3017,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.48</v>
+        <v>1</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>2.46</v>
+        <v>1</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.46</v>
+        <v>1</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.44</v>
+        <v>1</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -3016,7 +3039,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
+      <c r="C31" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3030,10 +3053,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>-0.0184874116629725</v>
+        <v>-0.01830187491510037</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.07281018801024</v>
+        <v>0.07288240242929306</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>0.09283155684402497</v>
@@ -4555,8 +4578,10 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46139</v>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'MORTGAGE30US' not found in values file."</t>
+        </is>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4569,19 +4594,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="R51" s="6" t="n">
-        <v>6.23</v>
+        <v>1</v>
       </c>
       <c r="S51" s="6" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="T51" s="6" t="n">
-        <v>6.37</v>
+        <v>1</v>
       </c>
       <c r="U51" s="21" t="n">
-        <v>6.46</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4606,8 +4631,10 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="50" t="n">
-        <v>46142</v>
+      <c r="N52" s="20" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
+        </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4620,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.1</v>
+        <v>1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>6.11</v>
+        <v>1</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>6.06</v>
+        <v>1</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.05</v>
+        <v>1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-06
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -217,7 +217,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -358,6 +358,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1036,10 +1039,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
-        </is>
+      <c r="C5" s="49" t="n">
+        <v>45931</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1052,19 +1053,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>1</v>
+        <v>7855631.5</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>1</v>
+        <v>7774506.8</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>1</v>
+        <v>7621432.3</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>1</v>
+        <v>7510528.3</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>1</v>
+        <v>7456295.5</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1077,8 +1078,10 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
-        <v>46082</v>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1091,19 +1094,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>62000</v>
+        <v>1</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>66000</v>
+        <v>1</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>11000</v>
+        <v>1</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>37000</v>
+        <v>1</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>74000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1113,10 +1116,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NGDPSAXDCUSQ' not found in values file."</t>
-        </is>
+      <c r="C6" s="49" t="n">
+        <v>45931</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1129,19 +1130,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>1</v>
+        <v>0.0104347069321491</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>1</v>
+        <v>0.02008474181421249</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>1</v>
+        <v>0.0147664712214719</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>1</v>
+        <v>0.007273424182290045</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>1</v>
+        <v>0.01062352837847436</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1154,8 +1155,10 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="49" t="n">
-        <v>46082</v>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'UNRATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1168,19 +1171,19 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="S6" s="6" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="T6" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="U6" s="21" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1208,7 +1211,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.5185</v>
+        <v>3.7425</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1273,10 +1276,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RECPROUSM156N' not found in values file."</t>
-        </is>
+      <c r="C8" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1289,19 +1290,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>1</v>
+        <v>1.82</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>1</v>
+        <v>0.46</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>1</v>
+        <v>0.24</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>1</v>
+        <v>0.16</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>1</v>
+        <v>0.34</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1314,8 +1315,10 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="49" t="n">
-        <v>46082</v>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
+        </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1328,19 +1331,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>61.9</v>
+        <v>1</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>62.1</v>
+        <v>1</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>62.4</v>
+        <v>1</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>62.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1393,8 +1396,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="49" t="n">
-        <v>46082</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1407,19 +1412,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1468,8 +1473,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
-        <v>46054</v>
+      <c r="N10" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1482,19 +1487,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="R10" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="R10" s="6" t="n">
+      <c r="S10" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="S10" s="6" t="n">
+      <c r="T10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T10" s="6" t="n">
+      <c r="U10" s="21" t="n">
         <v>4.1</v>
-      </c>
-      <c r="U10" s="21" t="n">
-        <v>4.3</v>
       </c>
     </row>
     <row r="11">
@@ -1508,10 +1513,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
-        </is>
+      <c r="C11" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1524,19 +1527,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>1</v>
+        <v>0.009363644833690454</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>1</v>
+        <v>0.01734597156398099</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>1</v>
+        <v>-0.01314250970487807</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>1</v>
+        <v>-0.00581233144238813</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>1</v>
+        <v>0.007353974425031495</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1549,8 +1552,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
-        <v>46054</v>
+      <c r="N11" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1563,19 +1566,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>3.1</v>
       </c>
-      <c r="R11" s="6" t="n">
+      <c r="S11" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="S11" s="6" t="n">
+      <c r="T11" s="6" t="n">
         <v>3.3</v>
       </c>
-      <c r="T11" s="6" t="n">
+      <c r="U11" s="21" t="n">
         <v>3.2</v>
-      </c>
-      <c r="U11" s="21" t="n">
-        <v>3.3</v>
       </c>
     </row>
     <row r="12">
@@ -1585,10 +1588,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEDGC96' not found in values file."</t>
-        </is>
+      <c r="C12" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1601,19 +1602,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>1</v>
+        <v>-0.005690422651553436</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>1</v>
+        <v>0.02619753322497357</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>1</v>
+        <v>0.009762633996937256</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>1</v>
+        <v>-0.02262753702687877</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>1</v>
+        <v>0.008866163156166484</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1626,8 +1627,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
-        <v>46054</v>
+      <c r="N12" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
@@ -1640,16 +1641,16 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="R12" s="6" t="n">
         <v>3.2</v>
       </c>
       <c r="S12" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="T12" s="6" t="n">
         <v>3.3</v>
-      </c>
-      <c r="T12" s="6" t="n">
-        <v>3.2</v>
       </c>
       <c r="U12" s="21" t="n">
         <v>3.2</v>
@@ -1861,8 +1862,10 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="49" t="n">
-        <v>46082</v>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
+        </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1875,19 +1878,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2118,8 +2121,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
-        <v>46082</v>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2132,19 +2137,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.0005629480818372112</v>
+        <v>1</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>-0.003744432836641498</v>
+        <v>1</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>0.006441402056378998</v>
+        <v>1</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>-0.0004425121414268762</v>
+        <v>1</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>0.0008581029834302534</v>
+        <v>1</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2189,8 +2194,10 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
-        <v>46082</v>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2203,19 +2210,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.004415084502276996</v>
+        <v>1</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01163563272940462</v>
+        <v>1</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.01661281847756826</v>
+        <v>1</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.01134436615382877</v>
+        <v>1</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01272729309745998</v>
+        <v>1</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2228,10 +2235,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N20" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2244,19 +2249,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1</v>
+        <v>0.001957950538511444</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>1</v>
+        <v>0.002160502174024082</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>1</v>
+        <v>0.002950448142634121</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>1</v>
+        <v>0.002329002576704653</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2305,10 +2310,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N21" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2321,19 +2324,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1</v>
+        <v>0.0260216770548682</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>1</v>
+        <v>0.02472462476764023</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>1</v>
+        <v>0.02512028782828883</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>1</v>
+        <v>0.02646484707309002</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>1</v>
+        <v>0.02599044806094405</v>
       </c>
     </row>
     <row r="22">
@@ -2689,10 +2692,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
-        </is>
+      <c r="N26" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2705,19 +2706,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>1</v>
+        <v>0.002932483068401215</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>1</v>
+        <v>0.003675182396499332</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>1</v>
+        <v>0.004245969066199562</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>1</v>
+        <v>0.003271383630529812</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>1</v>
+        <v>0.001776129138734595</v>
       </c>
     </row>
     <row r="27">
@@ -2766,10 +2767,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCEPILFE' not found in values file."</t>
-        </is>
+      <c r="N27" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2782,19 +2781,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>1</v>
+        <v>0.03202758906974702</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>1</v>
+        <v>0.03001318470574146</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>1</v>
+        <v>0.03083788838321814</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>1</v>
+        <v>0.02971110180682146</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>1</v>
+        <v>0.02829092786499081</v>
       </c>
     </row>
     <row r="28">
@@ -2808,8 +2807,10 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="49" t="n">
-        <v>46082</v>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
+        </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2822,19 +2823,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.008462114959539413</v>
+        <v>1</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.01169466364559735</v>
+        <v>1</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>-0.004254034642219184</v>
+        <v>1</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>-0.00913646104747079</v>
+        <v>1</v>
       </c>
       <c r="J28" s="25" t="n">
-        <v>0.05441037812530491</v>
+        <v>1</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2883,8 +2884,10 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="49" t="n">
-        <v>46082</v>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
+        </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2897,19 +2900,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.008519519946871591</v>
+        <v>1</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.07567733047604469</v>
+        <v>1</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>0.09883411459674789</v>
+        <v>1</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>0.1059440595541697</v>
+        <v>1</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>0.1247312200873968</v>
+        <v>1</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2923,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="48" t="n">
-        <v>46143</v>
+        <v>46147</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2939,16 +2942,16 @@
         <v>2.27</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>2.25</v>
+        <v>2.28</v>
       </c>
       <c r="S29" s="6" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.25</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="30">
@@ -2962,8 +2965,10 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="49" t="n">
-        <v>46082</v>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
+        </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2976,19 +2981,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.002810142088861101</v>
+        <v>1</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>-0.01222345960141613</v>
+        <v>1</v>
       </c>
       <c r="H30" s="25" t="n">
-        <v>0.002385879326488816</v>
+        <v>1</v>
       </c>
       <c r="I30" s="25" t="n">
-        <v>-0.01921059426035288</v>
+        <v>1</v>
       </c>
       <c r="J30" s="25" t="n">
-        <v>0.06592882125886601</v>
+        <v>1</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3001,10 +3006,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'T10YIE' not found in values file."</t>
-        </is>
+      <c r="N30" s="48" t="n">
+        <v>46147</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3017,19 +3020,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>1</v>
+        <v>2.47</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>1</v>
+        <v>2.48</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>1</v>
+        <v>2.46</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>1</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="31">
@@ -3039,8 +3042,10 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="49" t="n">
-        <v>46082</v>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
+        </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3053,19 +3058,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>-0.01830187491510037</v>
+        <v>1</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.07288240242929306</v>
+        <v>1</v>
       </c>
       <c r="H31" s="25" t="n">
-        <v>0.09283155684402497</v>
+        <v>1</v>
       </c>
       <c r="I31" s="25" t="n">
-        <v>0.1010908210327026</v>
+        <v>1</v>
       </c>
       <c r="J31" s="25" t="n">
-        <v>0.1265306873826442</v>
+        <v>1</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3118,8 +3123,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="49" t="n">
-        <v>46082</v>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3132,19 +3139,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>-0.005415070741811912</v>
+        <v>1</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.007368443846867079</v>
+        <v>1</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>-0.0001564786593617473</v>
+        <v>1</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.005246287630711999</v>
+        <v>1</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.001368313417869027</v>
+        <v>1</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3189,8 +3196,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="49" t="n">
-        <v>46082</v>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3203,19 +3212,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.007416835246099523</v>
+        <v>1</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01231165794421915</v>
+        <v>1</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01529710277450485</v>
+        <v>1</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01279811178014365</v>
+        <v>1</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.0180124379988418</v>
+        <v>1</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3268,8 +3277,10 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="49" t="n">
-        <v>46082</v>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TCU' not found in values file."</t>
+        </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3282,19 +3293,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>75.6596</v>
+        <v>1</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.1407</v>
+        <v>1</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.6564</v>
+        <v>1</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.7296</v>
+        <v>1</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.42489999999999</v>
+        <v>1</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3422,7 +3433,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
+      <c r="C36" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3493,7 +3504,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
+      <c r="C37" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3532,7 +3543,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
+      <c r="N37" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3572,8 +3583,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>46082</v>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3586,19 +3599,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1372</v>
+        <v>1</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1538</v>
+        <v>1</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1386</v>
+        <v>1</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1455</v>
+        <v>1</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1388</v>
+        <v>1</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3607,7 +3620,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
+      <c r="N38" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -3643,8 +3656,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>46082</v>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3657,19 +3672,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.07359891964888589</v>
+        <v>1</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>0.0577716643741403</v>
+        <v>1</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>-0.05068493150684932</v>
+        <v>1</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>-0.01689189189189189</v>
+        <v>1</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>-0.07957559681697612</v>
+        <v>1</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3682,8 +3697,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="49" t="n">
-        <v>46082</v>
+      <c r="N39" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3696,19 +3711,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
+        <v>119.0363</v>
+      </c>
+      <c r="R39" s="6" t="n">
         <v>119.9199</v>
       </c>
-      <c r="R39" s="6" t="n">
+      <c r="S39" s="6" t="n">
         <v>117.906</v>
       </c>
-      <c r="S39" s="6" t="n">
+      <c r="T39" s="6" t="n">
         <v>119.2298</v>
       </c>
-      <c r="T39" s="6" t="n">
+      <c r="U39" s="21" t="n">
         <v>120.1883</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>121.4177</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3722,8 +3737,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n">
-        <v>46023</v>
+      <c r="C40" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -3736,19 +3751,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>587</v>
+        <v>682</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>712</v>
+        <v>635</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>764</v>
+        <v>583</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>650</v>
+        <v>728</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>719</v>
+        <v>748</v>
       </c>
       <c r="K40" s="5" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3757,8 +3772,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="49" t="n">
-        <v>46082</v>
+      <c r="N40" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3771,19 +3786,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.04111399852747133</v>
+      </c>
+      <c r="R40" s="38" t="n">
         <v>-0.05008673748247425</v>
       </c>
-      <c r="R40" s="38" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.07796471263522881</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.07456792269916472</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.05790675033979801</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.03874237696864814</v>
       </c>
     </row>
     <row r="41">
@@ -3793,8 +3808,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n">
-        <v>46023</v>
+      <c r="C41" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
@@ -3807,19 +3822,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.1132930513595166</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.008356545961002786</v>
+        <v>-0.01090342679127726</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>0.1318518518518519</v>
+        <v>-0.1193353474320242</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>0.04669887278582931</v>
+        <v>0.01392757660167131</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>0.002789400278940028</v>
+        <v>0.1081481481481481</v>
       </c>
       <c r="K41" s="5" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4144,8 +4159,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
-        <v>46054</v>
+      <c r="C46" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -4158,19 +4173,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>314787</v>
+        <v>320859</v>
       </c>
       <c r="G46" s="24" t="n">
+        <v>314673</v>
+      </c>
+      <c r="H46" s="24" t="n">
         <v>302224</v>
       </c>
-      <c r="H46" s="24" t="n">
+      <c r="I46" s="24" t="n">
         <v>286301</v>
       </c>
-      <c r="I46" s="24" t="n">
+      <c r="J46" s="24" t="n">
         <v>290906</v>
-      </c>
-      <c r="J46" s="24" t="n">
-        <v>301177</v>
       </c>
       <c r="K46" s="5" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4231,8 +4246,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
-        <v>46054</v>
+      <c r="C47" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4245,19 +4260,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>0.04156850547937951</v>
+        <v>0.01965850263606983</v>
       </c>
       <c r="G47" s="38" t="n">
+        <v>0.04119130181587161</v>
+      </c>
+      <c r="H47" s="38" t="n">
         <v>0.05561629194449202</v>
       </c>
-      <c r="H47" s="38" t="n">
+      <c r="I47" s="38" t="n">
         <v>-0.01582985569221673</v>
       </c>
-      <c r="I47" s="38" t="n">
+      <c r="J47" s="38" t="n">
         <v>-0.03410286974104926</v>
-      </c>
-      <c r="J47" s="38" t="n">
-        <v>0.02509496126669486</v>
       </c>
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4271,7 +4286,7 @@
         </is>
       </c>
       <c r="N47" s="48" t="n">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4310,8 +4325,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
-        <v>46054</v>
+      <c r="C48" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4324,19 +4339,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>372135</v>
+        <v>381165</v>
       </c>
       <c r="G48" s="24" t="n">
+        <v>372449</v>
+      </c>
+      <c r="H48" s="24" t="n">
         <v>356901</v>
       </c>
-      <c r="H48" s="24" t="n">
+      <c r="I48" s="24" t="n">
         <v>359201</v>
       </c>
-      <c r="I48" s="24" t="n">
+      <c r="J48" s="24" t="n">
         <v>346932</v>
-      </c>
-      <c r="J48" s="24" t="n">
-        <v>332279</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4349,8 +4364,10 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="48" t="n">
-        <v>46142</v>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
+        </is>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4363,19 +4380,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.88</v>
+        <v>1</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>3.92</v>
+        <v>1</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>3.84</v>
+        <v>1</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>3.78</v>
+        <v>1</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -4385,8 +4402,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
-        <v>46054</v>
+      <c r="C49" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4399,19 +4416,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.04268410567636405</v>
+        <v>0.0234018617314049</v>
       </c>
       <c r="G49" s="38" t="n">
+        <v>0.04356390147407829</v>
+      </c>
+      <c r="H49" s="38" t="n">
         <v>-0.006403100214086299</v>
       </c>
-      <c r="H49" s="38" t="n">
+      <c r="I49" s="38" t="n">
         <v>0.03536427887885818</v>
       </c>
-      <c r="I49" s="38" t="n">
+      <c r="J49" s="38" t="n">
         <v>0.04409848350332091</v>
-      </c>
-      <c r="J49" s="38" t="n">
-        <v>-0.03117747221347511</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4425,7 +4442,7 @@
         </is>
       </c>
       <c r="N49" s="48" t="n">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4438,19 +4455,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.02</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="T49" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.97</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>3.94</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.92</v>
       </c>
     </row>
     <row r="50">
@@ -4464,8 +4481,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
-        <v>46054</v>
+      <c r="C50" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4478,19 +4495,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>27256</v>
+        <v>28406</v>
       </c>
       <c r="G50" s="24" t="n">
+        <v>26846</v>
+      </c>
+      <c r="H50" s="24" t="n">
         <v>27460</v>
       </c>
-      <c r="H50" s="24" t="n">
+      <c r="I50" s="24" t="n">
         <v>26347</v>
       </c>
-      <c r="I50" s="24" t="n">
+      <c r="J50" s="24" t="n">
         <v>27608</v>
-      </c>
-      <c r="J50" s="24" t="n">
-        <v>27476</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4504,7 +4521,7 @@
         </is>
       </c>
       <c r="N50" s="48" t="n">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4517,19 +4534,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="R50" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.42</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.36</v>
-      </c>
-      <c r="T50" s="6" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4539,8 +4556,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
-        <v>46054</v>
+      <c r="C51" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4553,19 +4570,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>-0.007428987618353977</v>
+        <v>0.05810921552559045</v>
       </c>
       <c r="G51" s="38" t="n">
+        <v>-0.02235979606700655</v>
+      </c>
+      <c r="H51" s="38" t="n">
         <v>0.04224389873609891</v>
       </c>
-      <c r="H51" s="38" t="n">
+      <c r="I51" s="38" t="n">
         <v>-0.04567516661837145</v>
       </c>
-      <c r="I51" s="38" t="n">
+      <c r="J51" s="38" t="n">
         <v>0.004804192750036407</v>
-      </c>
-      <c r="J51" s="38" t="n">
-        <v>-0.03903189703413545</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4578,10 +4595,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'MORTGAGE30US' not found in values file."</t>
-        </is>
+      <c r="N51" s="48" t="n">
+        <v>46139</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4594,19 +4609,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>1</v>
+        <v>6.3</v>
       </c>
       <c r="R51" s="6" t="n">
-        <v>1</v>
+        <v>6.23</v>
       </c>
       <c r="S51" s="6" t="n">
-        <v>1</v>
+        <v>6.3</v>
       </c>
       <c r="T51" s="6" t="n">
-        <v>1</v>
+        <v>6.37</v>
       </c>
       <c r="U51" s="21" t="n">
-        <v>1</v>
+        <v>6.46</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4631,10 +4646,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="20" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
-        </is>
+      <c r="N52" s="50" t="n">
+        <v>46147</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,19 +4660,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>1</v>
+        <v>6.08</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>1</v>
+        <v>6.14</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>1</v>
+        <v>6.08</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>1</v>
+        <v>6.1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>1</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -62,7 +62,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +79,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
         <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -354,14 +360,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -928,7 +934,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N3" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -999,7 +1005,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="49" t="n">
+      <c r="N4" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1039,7 +1045,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
+      <c r="C5" s="48" t="n">
         <v>45931</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1078,10 +1084,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
-        </is>
+      <c r="N5" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1094,19 +1098,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>1</v>
+        <v>109000</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="S5" s="24" t="n">
-        <v>1</v>
+        <v>61000</v>
+      </c>
+      <c r="S5" s="50" t="n">
+        <v>66000</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>1</v>
+        <v>11000</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>1</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="6">
@@ -1116,7 +1120,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
+      <c r="C6" s="48" t="n">
         <v>45931</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1155,10 +1159,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'UNRATE' not found in values file."</t>
-        </is>
+      <c r="N6" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1171,19 +1173,19 @@
         </is>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="S6" s="6" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="T6" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="U6" s="21" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1197,7 +1199,7 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="49" t="n">
+      <c r="C7" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1236,8 +1238,10 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="49" t="n">
-        <v>46082</v>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1250,19 +1254,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8.4</v>
+        <v>1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>8.699999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1276,7 +1280,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1396,10 +1400,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1412,19 +1414,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="10">
@@ -1473,7 +1475,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
+      <c r="N10" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1552,7 +1554,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1627,7 +1629,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1706,8 +1708,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="48" t="n">
-        <v>46132</v>
+      <c r="N13" s="49" t="n">
+        <v>46139</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1720,19 +1722,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>189000</v>
+        <v>200000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>190000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>215000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>208000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>218000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>203000</v>
       </c>
     </row>
     <row r="14">
@@ -1862,10 +1864,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
-        </is>
+      <c r="N15" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1878,19 +1878,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="16">
@@ -1951,10 +1951,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C17" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1967,19 +1965,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>1</v>
+        <v>0.01661457854582227</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>1</v>
+        <v>0.007173558174711436</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>1</v>
+        <v>-0.0002912686109073359</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>1</v>
+        <v>-1.361066422789214e-06</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>1</v>
+        <v>0.005016065910586232</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2040,10 +2038,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'RSAFS' not found in values file."</t>
-        </is>
+      <c r="C18" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2056,19 +2052,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>1</v>
+        <v>0.03969447708578144</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>1</v>
+        <v>0.03962618135825458</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>1</v>
+        <v>0.03267862666254253</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>1</v>
+        <v>0.02433131408893505</v>
       </c>
       <c r="J18" s="25" t="n">
-        <v>1</v>
+        <v>0.03212039564348258</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2081,8 +2077,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
-        <v>46082</v>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2095,19 +2093,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>0.008651438343614481</v>
+        <v>1</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>0.00267003074209704</v>
+        <v>1</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>0.00170842649932057</v>
+        <v>1</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>0.00297788428704604</v>
+        <v>1</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2121,10 +2119,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C19" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2137,19 +2133,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>1</v>
+        <v>-0.0005629480818372112</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>1</v>
+        <v>-0.003744432836641498</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>1</v>
+        <v>0.006441402056378998</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>1</v>
+        <v>-0.0004425121414268762</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>1</v>
+        <v>0.0008581029834302534</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2158,8 +2154,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
-        <v>46082</v>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2172,19 +2170,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>0.03285957752865201</v>
+        <v>1</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>0.0243400411037322</v>
+        <v>1</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>0.02391201432150015</v>
+        <v>1</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>0.02653304114557758</v>
+        <v>1</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>0.02696443916493949</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2194,10 +2192,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DSPIC96' not found in values file."</t>
-        </is>
+      <c r="C20" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2210,19 +2206,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>1</v>
+        <v>0.004415084502276996</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>1</v>
+        <v>0.01163563272940462</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>1</v>
+        <v>0.01661281847756826</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>1</v>
+        <v>0.01134436615382877</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>1</v>
+        <v>0.01272729309745998</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2235,8 +2231,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
-        <v>46082</v>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2249,19 +2247,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>0.001957950538511444</v>
+        <v>1</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.002160502174024082</v>
+        <v>1</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>0.002950448142634121</v>
+        <v>1</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>0.002329002576704653</v>
+        <v>1</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2310,8 +2308,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
-        <v>46082</v>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2324,19 +2324,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.0260216770548682</v>
+        <v>1</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.02472462476764023</v>
+        <v>1</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>0.02512028782828883</v>
+        <v>1</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>0.02646484707309002</v>
+        <v>1</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>0.02599044806094405</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2350,7 +2350,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2389,7 +2389,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2425,7 +2425,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2459,7 +2459,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2499,7 +2499,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
+      <c r="C24" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2578,8 +2578,10 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
-        <v>46054</v>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2592,19 +2594,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.002321146114863559</v>
+        <v>1</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.001350696962159503</v>
+        <v>1</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.002042971180921338</v>
+        <v>1</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.001126106640109592</v>
+        <v>1</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.0009131400161073167</v>
+        <v>1</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2732,8 +2734,10 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="48" t="n">
-        <v>46023</v>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2746,19 +2750,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.02054026778170115</v>
+        <v>1</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>-0.004277328978805506</v>
+        <v>1</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>-0.01832684674964358</v>
+        <v>1</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>-0.01299350008050415</v>
+        <v>1</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>-0.002410568051752549</v>
+        <v>1</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2848,7 +2852,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="49" t="n">
+      <c r="N28" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -2925,8 +2929,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="48" t="n">
-        <v>46147</v>
+      <c r="N29" s="49" t="n">
+        <v>46148</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2939,16 +2943,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.27</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.25</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.25</v>
@@ -3006,8 +3010,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="48" t="n">
-        <v>46147</v>
+      <c r="N30" s="49" t="n">
+        <v>46148</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3020,16 +3024,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.47</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.5</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.48</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.46</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.46</v>
@@ -3237,7 +3241,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="49" t="n">
+      <c r="N33" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -3277,10 +3281,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TCU' not found in values file."</t>
-        </is>
+      <c r="C34" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3293,19 +3295,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>1</v>
+        <v>75.6596</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>1</v>
+        <v>76.1407</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>1</v>
+        <v>75.6564</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>1</v>
+        <v>75.7296</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>1</v>
+        <v>75.42489999999999</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3314,7 +3316,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="49" t="n">
+      <c r="N34" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
@@ -3355,7 +3357,7 @@
         </is>
       </c>
       <c r="C35" s="49" t="n">
-        <v>45931</v>
+        <v>46023</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -3368,19 +3370,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="G35" s="41" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H35" s="41" t="n">
         <v>5.2</v>
       </c>
-      <c r="H35" s="41" t="n">
+      <c r="I35" s="41" t="n">
         <v>4.2</v>
       </c>
-      <c r="I35" s="41" t="n">
+      <c r="J35" s="41" t="n">
         <v>-0.9</v>
-      </c>
-      <c r="J35" s="41" t="n">
-        <v>1.4</v>
       </c>
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -3393,7 +3395,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="49" t="n">
+      <c r="N35" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
@@ -3433,7 +3435,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="49" t="n">
+      <c r="C36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3468,7 +3470,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="49" t="n">
+      <c r="N36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
@@ -3504,7 +3506,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n">
+      <c r="C37" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3543,7 +3545,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="49" t="n">
+      <c r="N37" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3583,10 +3585,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C38" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3599,19 +3599,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>1363</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1</v>
+        <v>1538</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1</v>
+        <v>1386</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1</v>
+        <v>1455</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1</v>
+        <v>1388</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3620,7 +3620,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="49" t="n">
+      <c r="N38" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -3656,10 +3656,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C39" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3672,19 +3670,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07967589466576637</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>1</v>
+        <v>0.0577716643741403</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>1</v>
+        <v>-0.05068493150684932</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>1</v>
+        <v>-0.01689189189189189</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07957559681697612</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3697,7 +3695,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
+      <c r="N39" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3737,8 +3735,10 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
-        <v>46082</v>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
+        </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -3751,19 +3751,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>682</v>
+        <v>1</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>635</v>
+        <v>1</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>583</v>
+        <v>1</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>728</v>
+        <v>1</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>748</v>
+        <v>1</v>
       </c>
       <c r="K40" s="5" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3772,7 +3772,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
+      <c r="N40" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3808,8 +3808,10 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
-        <v>46082</v>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
+        </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
@@ -3822,19 +3824,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>0.03333333333333333</v>
+        <v>1</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.01090342679127726</v>
+        <v>1</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>-0.1193353474320242</v>
+        <v>1</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>0.01392757660167131</v>
+        <v>1</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>0.1081481481481481</v>
+        <v>1</v>
       </c>
       <c r="K41" s="5" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -3847,7 +3849,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3887,7 +3889,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="49" t="n">
+      <c r="C42" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -3922,7 +3924,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="49" t="n">
+      <c r="N42" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3958,7 +3960,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="49" t="n">
+      <c r="C43" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -3997,7 +3999,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4072,7 +4074,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4159,7 +4161,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
+      <c r="C46" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4246,7 +4248,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
+      <c r="C47" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4285,8 +4287,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="48" t="n">
-        <v>46146</v>
+      <c r="N47" s="49" t="n">
+        <v>46147</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4325,7 +4327,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
+      <c r="C48" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4364,10 +4366,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
-        </is>
+      <c r="N48" s="49" t="n">
+        <v>46147</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4380,19 +4380,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>1</v>
+        <v>3.93</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>1</v>
+        <v>3.95</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>1</v>
+        <v>3.88</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>1</v>
+        <v>3.88</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>1</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="49">
@@ -4402,7 +4402,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
+      <c r="C49" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4441,8 +4441,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="48" t="n">
-        <v>46146</v>
+      <c r="N49" s="49" t="n">
+        <v>46147</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4458,16 +4458,16 @@
         <v>4.08</v>
       </c>
       <c r="R49" s="6" t="n">
-        <v>4.02</v>
+        <v>4.08</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>4.02</v>
       </c>
       <c r="T49" s="6" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.05</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.97</v>
       </c>
     </row>
     <row r="50">
@@ -4481,7 +4481,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
+      <c r="C50" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4520,8 +4520,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="48" t="n">
-        <v>46146</v>
+      <c r="N50" s="49" t="n">
+        <v>46147</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4534,19 +4534,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.45</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.42</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.36</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4556,7 +4556,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
+      <c r="C51" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4646,8 +4646,10 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="50" t="n">
-        <v>46147</v>
+      <c r="N52" s="20" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
+        </is>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4660,19 +4662,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.08</v>
+        <v>1</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>6.14</v>
+        <v>1</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>6.08</v>
+        <v>1</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.1</v>
+        <v>1</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -368,6 +368,9 @@
     </xf>
     <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -934,8 +937,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
-        <v>46082</v>
+      <c r="N3" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
@@ -948,19 +951,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>178</v>
+        <v>115</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>-133</v>
+        <v>185</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>-156</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>160</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>-17</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -1005,8 +1008,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
-        <v>46082</v>
+      <c r="N4" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
@@ -1019,19 +1022,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.001641652512675452</v>
+        <v>0.001583746095845033</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.0009411913334596677</v>
+        <v>0.001540627742664655</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.0007959067652075042</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.002047160512548336</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.0007327117916066601</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.002340601850973247</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1159,8 +1162,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
-        <v>46082</v>
+      <c r="N6" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1176,16 +1179,16 @@
         <v>4.3</v>
       </c>
       <c r="R6" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="S6" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="S6" s="6" t="n">
+      <c r="T6" s="6" t="n">
         <v>4.3</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="U6" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U6" s="21" t="n">
-        <v>4.5</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1213,7 +1216,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.7425</v>
+        <v>3.6693</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1238,10 +1241,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
-        </is>
+      <c r="N7" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1254,19 +1255,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>8.1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>1</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1280,7 +1281,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1319,10 +1320,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
-        </is>
+      <c r="N8" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1335,19 +1334,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>1</v>
+        <v>61.8</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>1</v>
+        <v>61.9</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>1</v>
+        <v>62.1</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>1</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="9">
@@ -1400,8 +1399,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46082</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1414,19 +1415,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1475,8 +1476,10 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
-        <v>46082</v>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
+        </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1489,19 +1492,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1783,10 +1786,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
-        </is>
+      <c r="N14" s="49" t="n">
+        <v>46132</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1799,19 +1800,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1</v>
+        <v>1766000</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1</v>
+        <v>1776000</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1</v>
+        <v>1808000</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1</v>
+        <v>1809000</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1</v>
+        <v>1787000</v>
       </c>
     </row>
     <row r="15">
@@ -1864,8 +1865,10 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
-        <v>46082</v>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
+        </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1878,19 +1881,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2077,10 +2080,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N18" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2093,19 +2094,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>1</v>
+        <v>0.008651438343614481</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>1</v>
+        <v>0.00267003074209704</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>1</v>
+        <v>0.00170842649932057</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>1</v>
+        <v>0.00297788428704604</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2154,10 +2155,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N19" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2170,19 +2169,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>1</v>
+        <v>0.03285957752865201</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>1</v>
+        <v>0.0243400411037322</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>1</v>
+        <v>0.02391201432150015</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>1</v>
+        <v>0.02653304114557758</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>1</v>
+        <v>0.02696443916493949</v>
       </c>
     </row>
     <row r="20">
@@ -2231,10 +2230,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N20" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2247,19 +2244,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1</v>
+        <v>0.001957950538511444</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>1</v>
+        <v>0.002160502174024082</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>1</v>
+        <v>0.002950448142634121</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>1</v>
+        <v>0.002329002576704653</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2308,10 +2305,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N21" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2324,19 +2319,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1</v>
+        <v>0.0260216770548682</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>1</v>
+        <v>0.02472462476764023</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>1</v>
+        <v>0.02512028782828883</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>1</v>
+        <v>0.02646484707309002</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>1</v>
+        <v>0.02599044806094405</v>
       </c>
     </row>
     <row r="22">
@@ -2499,8 +2494,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
-        <v>46054</v>
+      <c r="C24" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2513,19 +2508,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.0005344764598498308</v>
+        <v>0.007561302505515899</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.00193733910205296</v>
+        <v>0.0002854040755513321</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.006198592859945062</v>
+        <v>0.001701852596202258</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>-0.0007477443007701812</v>
+        <v>0.006198562656960505</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.003378223860396545</v>
+        <v>-0.0007477594964454548</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2578,10 +2573,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
-        </is>
+      <c r="C25" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2594,19 +2587,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>1</v>
+        <v>0.003911989748358602</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>1</v>
+        <v>0.0022395833833464</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>1</v>
+        <v>0.001310703086948806</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>1</v>
+        <v>0.001967095543671693</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>1</v>
+        <v>0.001164097695629751</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2734,10 +2727,8 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
-        </is>
+      <c r="C27" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2750,19 +2741,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>1</v>
+        <v>-0.02054026778170115</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>1</v>
+        <v>-0.004277328978805506</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01832684674964358</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01299350008050415</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>1</v>
+        <v>-0.002410568051752549</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2811,10 +2802,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
-        </is>
+      <c r="C28" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2827,19 +2816,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>1</v>
+        <v>0.008462114959539413</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>1</v>
+        <v>-0.01169466364559735</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>1</v>
+        <v>-0.004254034642219184</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>1</v>
+        <v>-0.00913646104747079</v>
       </c>
       <c r="J28" s="25" t="n">
-        <v>1</v>
+        <v>0.05441037812530491</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2888,10 +2877,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
-        </is>
+      <c r="C29" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2904,19 +2891,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>1</v>
+        <v>0.008519519946871591</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>1</v>
+        <v>0.07567733047604469</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>1</v>
+        <v>0.09883411459674789</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>1</v>
+        <v>0.1059440595541697</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>1</v>
+        <v>0.1247312200873968</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2930,7 +2917,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2943,19 +2930,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="30">
@@ -2969,10 +2956,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
-        </is>
+      <c r="C30" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2985,19 +2970,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>1</v>
+        <v>-0.002810142088861101</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>1</v>
+        <v>-0.01222345960141613</v>
       </c>
       <c r="H30" s="25" t="n">
-        <v>1</v>
+        <v>0.002385879326488816</v>
       </c>
       <c r="I30" s="25" t="n">
-        <v>1</v>
+        <v>-0.01921059426035288</v>
       </c>
       <c r="J30" s="25" t="n">
-        <v>1</v>
+        <v>0.06592882125886601</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3011,7 +2996,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3024,19 +3009,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.42</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.47</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.5</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.48</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.46</v>
       </c>
     </row>
     <row r="31">
@@ -3046,10 +3031,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADXDNO' not found in values file."</t>
-        </is>
+      <c r="C31" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3062,19 +3045,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>1</v>
+        <v>-0.01830187491510037</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>1</v>
+        <v>0.07288240242929306</v>
       </c>
       <c r="H31" s="25" t="n">
-        <v>1</v>
+        <v>0.09283155684402497</v>
       </c>
       <c r="I31" s="25" t="n">
-        <v>1</v>
+        <v>0.1010908210327026</v>
       </c>
       <c r="J31" s="25" t="n">
-        <v>1</v>
+        <v>0.1265306873826442</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3127,10 +3110,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C32" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3143,19 +3124,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>1</v>
+        <v>-0.005415070741811912</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>1</v>
+        <v>0.007368443846867079</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>1</v>
+        <v>-0.0001564786593617473</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>1</v>
+        <v>0.005246287630711999</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>1</v>
+        <v>-0.001368313417869027</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3200,10 +3181,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C33" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3216,19 +3195,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>1</v>
+        <v>0.007416835246099523</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>1</v>
+        <v>0.01231165794421915</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>1</v>
+        <v>0.01529710277450485</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>1</v>
+        <v>0.01279811178014365</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>1</v>
+        <v>0.0180124379988418</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3241,8 +3220,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
-        <v>46082</v>
+      <c r="N33" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
@@ -3255,19 +3234,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
-        <v>0.002413515687851975</v>
+        <v>0.001606425702811221</v>
       </c>
       <c r="R33" s="38" t="n">
-        <v>0.003768506056527565</v>
+        <v>0.002146498524282281</v>
       </c>
       <c r="S33" s="38" t="n">
+        <v>0.003230148048452453</v>
+      </c>
+      <c r="T33" s="38" t="n">
         <v>0.003511615343057661</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.000540540540540535</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.00407055630936215</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -3330,10 +3309,10 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>0.0002024211398903792</v>
+        <v>-0.0006003095351817524</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>0.00901208412752658</v>
+        <v>0.008470913795465586</v>
       </c>
       <c r="S34" s="38" t="n">
         <v>0.007760924955011093</v>
@@ -3409,10 +3388,10 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.004200333998298111</v>
+        <v>-0.004465589402518066</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>1.650614201031964e-05</v>
+        <v>-0.0005198395303640524</v>
       </c>
       <c r="S35" s="38" t="n">
         <v>0.0002132515841006821</v>
@@ -3435,8 +3414,10 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
-        <v>46082</v>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
+        </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3449,19 +3430,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1502</v>
+        <v>1</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1356</v>
+        <v>1</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1398</v>
+        <v>1</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1373</v>
+        <v>1</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1324</v>
+        <v>1</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3484,10 +3465,10 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>0.0002024211398903792</v>
+        <v>-0.0006003095351817524</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>0.00901208412752658</v>
+        <v>0.008470913795465586</v>
       </c>
       <c r="S36" s="38" t="n">
         <v>0.007760924955011093</v>
@@ -3506,8 +3487,10 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
-        <v>46082</v>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
+        </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3520,19 +3503,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.1084870848708487</v>
+        <v>1</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.08993288590604027</v>
+        <v>1</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>0.02945508100147275</v>
+        <v>1</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>-0.09313077939233817</v>
+        <v>1</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>0.02239382239382239</v>
+        <v>1</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3585,8 +3568,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>46082</v>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3599,19 +3584,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1363</v>
+        <v>1</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1538</v>
+        <v>1</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1386</v>
+        <v>1</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1455</v>
+        <v>1</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1388</v>
+        <v>1</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3656,8 +3641,10 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>46082</v>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
+        </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3670,19 +3657,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.07967589466576637</v>
+        <v>1</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>0.0577716643741403</v>
+        <v>1</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>-0.05068493150684932</v>
+        <v>1</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>-0.01689189189189189</v>
+        <v>1</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>-0.07957559681697612</v>
+        <v>1</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -4288,7 +4275,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4367,7 +4354,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4380,19 +4367,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.93</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.95</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>3.88</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>3.88</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.92</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="49">
@@ -4442,7 +4429,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4455,19 +4442,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>4.08</v>
+        <v>3.99</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>4.08</v>
       </c>
       <c r="S49" s="6" t="n">
-        <v>4.02</v>
+        <v>4.08</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>4.02</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.05</v>
+        <v>4.02</v>
       </c>
     </row>
     <row r="50">
@@ -4521,7 +4508,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4534,19 +4521,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.43</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.45</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.39</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.42</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4595,8 +4582,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="48" t="n">
-        <v>46139</v>
+      <c r="N51" s="49" t="n">
+        <v>46146</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4609,19 +4596,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.23</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.37</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.46</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4646,10 +4633,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="20" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DBAA' not found in values file."</t>
-        </is>
+      <c r="N52" s="51" t="n">
+        <v>46149</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4662,19 +4647,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>1</v>
+        <v>6.06</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>1</v>
+        <v>6.02</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>1</v>
+        <v>6.08</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>1</v>
+        <v>6.14</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>1</v>
+        <v>6.08</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-09
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.6693</v>
+        <v>3.7469</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1399,10 +1399,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1415,19 +1413,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="10">
@@ -1476,10 +1474,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
-        </is>
+      <c r="N10" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1492,19 +1488,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>1</v>
+        <v>4.1</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>1</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="11">
@@ -1865,10 +1861,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
-        </is>
+      <c r="N15" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1881,19 +1875,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="16">
@@ -2917,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2930,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -2996,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3012,16 +3006,16 @@
         <v>2.45</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.42</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.47</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.5</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.48</v>
       </c>
     </row>
     <row r="31">
@@ -3414,10 +3408,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
-        </is>
+      <c r="C36" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3430,19 +3422,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1</v>
+        <v>1502</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1</v>
+        <v>1356</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1</v>
+        <v>1398</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1</v>
+        <v>1373</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1</v>
+        <v>1324</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3487,10 +3479,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
-        </is>
+      <c r="C37" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3503,19 +3493,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>1</v>
+        <v>0.1084870848708487</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>1</v>
+        <v>-0.08993288590604027</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>1</v>
+        <v>0.02945508100147275</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>1</v>
+        <v>-0.09313077939233817</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>1</v>
+        <v>0.02239382239382239</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3568,10 +3558,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C38" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3584,19 +3572,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>1363</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>1</v>
+        <v>1538</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>1</v>
+        <v>1386</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1</v>
+        <v>1455</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1</v>
+        <v>1388</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3641,10 +3629,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PERMIT' not found in values file."</t>
-        </is>
+      <c r="C39" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3657,19 +3643,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07967589466576637</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>1</v>
+        <v>0.0577716643741403</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>1</v>
+        <v>-0.05068493150684932</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>1</v>
+        <v>-0.01689189189189189</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>1</v>
+        <v>-0.07957559681697612</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3722,10 +3708,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
-        </is>
+      <c r="C40" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -3738,19 +3722,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>682</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>1</v>
+        <v>635</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>1</v>
+        <v>583</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>1</v>
+        <v>728</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>1</v>
+        <v>748</v>
       </c>
       <c r="K40" s="5" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3795,10 +3779,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
-        </is>
+      <c r="C41" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
@@ -3811,19 +3793,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>1</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>1</v>
+        <v>-0.01090342679127726</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>1</v>
+        <v>-0.1193353474320242</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>1</v>
+        <v>0.01392757660167131</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>1</v>
+        <v>0.1081481481481481</v>
       </c>
       <c r="K41" s="5" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4275,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4288,7 +4270,7 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>3.64</v>
+        <v>3.63</v>
       </c>
       <c r="R47" s="6" t="n">
         <v>3.64</v>
@@ -4354,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4367,16 +4349,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.87</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.93</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.95</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>3.88</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>3.88</v>
@@ -4429,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4442,16 +4424,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>3.99</v>
-      </c>
-      <c r="R49" s="6" t="n">
-        <v>4.08</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>4.08</v>
       </c>
       <c r="T49" s="6" t="n">
-        <v>4.02</v>
+        <v>4.08</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.02</v>
@@ -4508,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4521,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.36</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.43</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.45</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.39</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.4</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1048,8 +1048,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="48" t="n">
-        <v>45931</v>
+      <c r="C5" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -1062,19 +1062,19 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
+        <v>7964064.3</v>
+      </c>
+      <c r="G5" s="24" t="n">
         <v>7855631.5</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="H5" s="24" t="n">
         <v>7774506.8</v>
       </c>
-      <c r="H5" s="24" t="n">
+      <c r="I5" s="24" t="n">
         <v>7621432.3</v>
       </c>
-      <c r="I5" s="24" t="n">
+      <c r="J5" s="24" t="n">
         <v>7510528.3</v>
-      </c>
-      <c r="J5" s="24" t="n">
-        <v>7456295.5</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="28" t="inlineStr">
@@ -1087,7 +1087,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1123,8 +1123,8 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="48" t="n">
-        <v>45931</v>
+      <c r="C6" s="49" t="n">
+        <v>46023</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1137,19 +1137,19 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
+        <v>0.01380319328878898</v>
+      </c>
+      <c r="G6" s="25" t="n">
         <v>0.0104347069321491</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="H6" s="25" t="n">
         <v>0.02008474181421249</v>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="I6" s="25" t="n">
         <v>0.0147664712214719</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="J6" s="25" t="n">
         <v>0.007273424182290045</v>
-      </c>
-      <c r="J6" s="25" t="n">
-        <v>0.01062352837847436</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="28" t="inlineStr">
@@ -1474,7 +1474,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
+      <c r="N10" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1553,7 +1553,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1628,7 +1628,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1707,8 +1707,10 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
-        <v>46139</v>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1721,19 +1723,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>200000</v>
+        <v>1</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>190000</v>
+        <v>1</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>215000</v>
+        <v>1</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>208000</v>
+        <v>1</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>218000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2074,8 +2076,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
-        <v>46082</v>
+      <c r="N18" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2088,19 +2090,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>0.006400377846336402</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>0.008651438343614481</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>0.00267003074209704</v>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="T18" s="38" t="n">
         <v>0.00170842649932057</v>
       </c>
-      <c r="T18" s="38" t="n">
+      <c r="U18" s="23" t="n">
         <v>0.00297788428704604</v>
-      </c>
-      <c r="U18" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2149,8 +2151,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
-        <v>46082</v>
+      <c r="N19" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2163,19 +2165,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.03779245836741563</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.03285957752865201</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.0243400411037322</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.02391201432150015</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v>0.02653304114557758</v>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.02696443916493949</v>
       </c>
     </row>
     <row r="20">
@@ -2224,8 +2226,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46082</v>
+      <c r="N20" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2238,19 +2240,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>0.00376460730477457</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.001957950538511444</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>0.002160502174024082</v>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="T20" s="38" t="n">
         <v>0.002950448142634121</v>
       </c>
-      <c r="T20" s="38" t="n">
+      <c r="U20" s="23" t="n">
         <v>0.002329002576704653</v>
-      </c>
-      <c r="U20" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="21">
@@ -2299,8 +2301,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46082</v>
+      <c r="N21" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2313,19 +2315,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.02743309430968526</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.0260216770548682</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.02472462476764023</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.02512028782828883</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v>0.02646484707309002</v>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v>0.02599044806094405</v>
       </c>
     </row>
     <row r="22">
@@ -2378,8 +2380,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46082</v>
+      <c r="N22" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2392,19 +2394,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.005123318605152027</v>
+        <v>0.01375897183427033</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.004965106516948259</v>
+        <v>0.006992824527071173</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.005526756624853135</v>
+        <v>0.005674549808114993</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.003786725277053149</v>
+        <v>0.005560979471212146</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.004088035682236812</v>
+        <v>0.00356164020813754</v>
       </c>
     </row>
     <row r="23">
@@ -2448,8 +2450,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46082</v>
+      <c r="N23" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2462,19 +2464,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.04019452230589979</v>
+        <v>0.05987606244285672</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.03364972711879271</v>
+        <v>0.04266657661004361</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.03033620544010816</v>
+        <v>0.03418267187468382</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.03110464325544714</v>
+        <v>0.03014022638959289</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.03145847985960791</v>
+        <v>0.0308734325272694</v>
       </c>
     </row>
     <row r="24">
@@ -2642,8 +2644,10 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n">
-        <v>46023</v>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2656,19 +2660,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.02495869599850553</v>
+        <v>1</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>0.005923787970366412</v>
+        <v>1</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>0.007794617579222285</v>
+        <v>1</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>0.01778138610314484</v>
+        <v>1</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>0.02303791460563676</v>
+        <v>1</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2721,8 +2725,10 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="48" t="n">
-        <v>46023</v>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2735,19 +2741,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.02054026778170115</v>
+        <v>1</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>-0.004277328978805506</v>
+        <v>1</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>-0.01832684674964358</v>
+        <v>1</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>-0.01299350008050415</v>
+        <v>1</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>-0.002410568051752549</v>
+        <v>1</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2835,8 +2841,10 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
-        <v>46082</v>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'MICH' not found in values file."</t>
+        </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2849,19 +2857,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>3.8</v>
+        <v>1</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2910,8 +2918,10 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="49" t="n">
-        <v>46150</v>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'T5YIFR' not found in values file."</t>
+        </is>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2934,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.28</v>
+        <v>1</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>2.29</v>
+        <v>1</v>
       </c>
       <c r="S29" s="6" t="n">
-        <v>2.26</v>
+        <v>1</v>
       </c>
       <c r="T29" s="6" t="n">
-        <v>2.27</v>
+        <v>1</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.28</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +3000,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46150</v>
+        <v>46154</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3013,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="R30" s="6" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.45</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.45</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.42</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.5</v>
       </c>
     </row>
     <row r="31">
@@ -3329,8 +3339,10 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="49" t="n">
-        <v>46023</v>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PRS85006092' not found in values file."</t>
+        </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -3343,19 +3355,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G35" s="41" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="H35" s="41" t="n">
-        <v>5.2</v>
+        <v>1</v>
       </c>
       <c r="I35" s="41" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="J35" s="41" t="n">
-        <v>-0.9</v>
+        <v>1</v>
       </c>
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -3668,7 +3680,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="49" t="n">
+      <c r="N39" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3708,7 +3720,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n">
+      <c r="C40" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3743,7 +3755,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="49" t="n">
+      <c r="N40" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3779,7 +3791,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n">
+      <c r="C41" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3859,7 +3871,7 @@
         </is>
       </c>
       <c r="C42" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3872,19 +3884,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>3980000</v>
+        <v>4020000</v>
       </c>
       <c r="G42" s="39" t="n">
+        <v>4010000</v>
+      </c>
+      <c r="H42" s="39" t="n">
         <v>4130000</v>
       </c>
-      <c r="H42" s="39" t="n">
+      <c r="I42" s="39" t="n">
         <v>4020000</v>
       </c>
-      <c r="I42" s="39" t="n">
+      <c r="J42" s="39" t="n">
         <v>4270000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4090000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3930,7 +3942,7 @@
         </is>
       </c>
       <c r="C43" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3943,7 +3955,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>-0.009950248756218905</v>
+        <v>0</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4008,8 +4020,10 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="48" t="n">
-        <v>46023</v>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GCE' not found in values file."</t>
+        </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4022,19 +4036,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5418.445</v>
+        <v>1</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>5343.513</v>
+        <v>1</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>5324.402</v>
+        <v>1</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>5236.97</v>
+        <v>1</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>5195.517</v>
+        <v>1</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4079,8 +4093,10 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="48" t="n">
-        <v>46023</v>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GCE' not found in values file."</t>
+        </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4093,19 +4109,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.01402298450476303</v>
+        <v>1</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>0.003589323270481781</v>
+        <v>1</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>0.01669515005814426</v>
+        <v>1</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>0.007978609251013902</v>
+        <v>1</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>0.008696251498575336</v>
+        <v>1</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4130,7 +4146,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
+      <c r="C46" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4217,7 +4233,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
+      <c r="C47" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4256,8 +4272,10 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="49" t="n">
-        <v>46149</v>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DFF' not found in values file."</t>
+        </is>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4270,19 +4288,19 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>3.63</v>
+        <v>1</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.64</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -4296,7 +4314,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
+      <c r="C48" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4335,8 +4353,10 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
-        <v>46149</v>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
+        </is>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4369,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>3.92</v>
+        <v>1</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>3.87</v>
+        <v>1</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>3.93</v>
+        <v>1</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>3.95</v>
+        <v>1</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.88</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -4371,7 +4391,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
+      <c r="C49" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4411,7 +4431,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4444,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="R49" s="6" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="S49" s="6" t="n">
         <v>4.04</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.08</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>4.08</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.02</v>
       </c>
     </row>
     <row r="50">
@@ -4450,7 +4470,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
+      <c r="C50" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4490,7 +4510,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4523,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="R50" s="6" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.41</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.36</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.43</v>
-      </c>
-      <c r="T50" s="6" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.39</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4525,7 +4545,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
+      <c r="C51" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4564,8 +4584,10 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
-        <v>46146</v>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'MORTGAGE30US' not found in values file."</t>
+        </is>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4578,19 +4600,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>6.37</v>
+        <v>1</v>
       </c>
       <c r="R51" s="6" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="S51" s="6" t="n">
-        <v>6.23</v>
+        <v>1</v>
       </c>
       <c r="T51" s="6" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="U51" s="21" t="n">
-        <v>6.37</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4616,7 +4638,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46149</v>
+        <v>46154</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4651,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="S52" s="9" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.02</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.14</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.08</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -360,13 +360,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -898,8 +901,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
-        <v>46023</v>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -912,19 +917,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24174.527</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24055.749</v>
+        <v>1</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>24026.834</v>
+        <v>1</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>23770.976</v>
+        <v>1</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23548.21</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -937,7 +942,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N3" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -973,8 +978,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
-        <v>46023</v>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -987,19 +994,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.004937613873506885</v>
+        <v>1</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>1</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>1</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>1</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>-0.001625164044818495</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1008,7 +1015,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="49" t="n">
+      <c r="N4" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1048,7 +1055,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
+      <c r="C5" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1087,7 +1094,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
+      <c r="N5" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1123,7 +1130,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
+      <c r="C6" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1162,7 +1169,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="49" t="n">
+      <c r="N6" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1202,8 +1209,10 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
-        <v>46113</v>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPNOW' not found in values file."</t>
+        </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1216,19 +1225,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.7469</v>
+        <v>1</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>1.2392</v>
+        <v>1</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>4.2373</v>
+        <v>1</v>
       </c>
       <c r="I7" s="41" t="n">
-        <v>3.4728</v>
+        <v>1</v>
       </c>
       <c r="J7" s="41" t="n">
-        <v>2.902</v>
+        <v>1</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1241,7 +1250,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1281,7 +1290,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1320,8 +1329,10 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="49" t="n">
-        <v>46113</v>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
+        </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1334,19 +1345,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>61.8</v>
+        <v>1</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>61.9</v>
+        <v>1</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>62.1</v>
+        <v>1</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>62.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1360,8 +1371,10 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="48" t="n">
-        <v>46023</v>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -1374,19 +1387,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16731.167</v>
+        <v>1</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>16665.219</v>
+        <v>1</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>16585.878</v>
+        <v>1</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>16445.685</v>
+        <v>1</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>16345.793</v>
+        <v>1</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1399,8 +1412,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="49" t="n">
-        <v>46113</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1413,19 +1428,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.1</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1435,8 +1450,10 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="48" t="n">
-        <v>46023</v>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -1449,19 +1466,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.00395722372445273</v>
+        <v>1</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>0.004783647872002916</v>
+        <v>1</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>0.008524606910566446</v>
+        <v>1</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>0.006111174905983452</v>
+        <v>1</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>0.001525835907232986</v>
+        <v>1</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1474,8 +1491,10 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
-        <v>46082</v>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
+        </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1488,19 +1507,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1514,7 +1533,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
+      <c r="C11" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1553,7 +1572,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1589,7 +1608,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
+      <c r="C12" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1628,7 +1647,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1668,7 +1687,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
+      <c r="C13" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1745,7 +1764,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1784,8 +1803,10 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
-        <v>46132</v>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1798,19 +1819,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1766000</v>
+        <v>1</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1776000</v>
+        <v>1</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1808000</v>
+        <v>1</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1809000</v>
+        <v>1</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1787000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1824,7 +1845,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
+      <c r="C15" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1863,7 +1884,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="49" t="n">
+      <c r="N15" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1899,7 +1920,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1951,7 +1972,7 @@
         </is>
       </c>
       <c r="C17" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1964,19 +1985,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.01661457854582227</v>
+        <v>0.004931175916216501</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.007173558174711436</v>
+        <v>0.01631236863902608</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>0.009223924204530221</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>-0.0002912686109073359</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="51" t="n">
         <v>-1.361066422789214e-06</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>0.005016065910586232</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2038,7 +2059,7 @@
         </is>
       </c>
       <c r="C18" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2051,19 +2072,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.03969447708578144</v>
+        <v>0.04873507936661851</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.03962618135825458</v>
+        <v>0.04151718627089097</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.04174261321715912</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.03267862666254253</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="51" t="n">
         <v>0.02433131408893505</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.03212039564348258</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2076,7 +2097,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
+      <c r="N18" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2116,7 +2137,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2151,7 +2172,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2187,7 +2208,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
+      <c r="C20" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2226,7 +2247,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
+      <c r="N20" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2266,7 +2287,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
+      <c r="C21" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2301,7 +2322,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
+      <c r="N21" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2341,7 +2362,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C22" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2380,7 +2401,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2416,7 +2437,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
+      <c r="C23" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2450,7 +2471,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2490,8 +2511,10 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
-        <v>46082</v>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2504,19 +2527,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.007561302505515899</v>
+        <v>1</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.0002854040755513321</v>
+        <v>1</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.001701852596202258</v>
+        <v>1</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.006198562656960505</v>
+        <v>1</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>-0.0007477594964454548</v>
+        <v>1</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2529,7 +2552,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
+      <c r="N24" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2569,8 +2592,10 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
-        <v>46082</v>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2583,19 +2608,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.003911989748358602</v>
+        <v>1</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.0022395833833464</v>
+        <v>1</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.001310703086948806</v>
+        <v>1</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.001967095543671693</v>
+        <v>1</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.001164097695629751</v>
+        <v>1</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2604,7 +2629,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
+      <c r="N25" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2685,7 +2710,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
+      <c r="N26" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2762,7 +2787,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
+      <c r="N27" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2802,8 +2827,10 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
-        <v>46082</v>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
+        </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2816,19 +2843,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.008462114959539413</v>
+        <v>1</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.01169466364559735</v>
+        <v>1</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>-0.004254034642219184</v>
+        <v>1</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>-0.00913646104747079</v>
+        <v>1</v>
       </c>
       <c r="J28" s="25" t="n">
-        <v>0.05441037812530491</v>
+        <v>1</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2841,10 +2868,8 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'MICH' not found in values file."</t>
-        </is>
+      <c r="N28" s="49" t="n">
+        <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2857,19 +2882,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="S28" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="U28" s="21" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="29">
@@ -2879,8 +2904,10 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
-        <v>46082</v>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
+        </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2893,19 +2920,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.008519519946871591</v>
+        <v>1</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.07567733047604469</v>
+        <v>1</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>0.09883411459674789</v>
+        <v>1</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>0.1059440595541697</v>
+        <v>1</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>0.1247312200873968</v>
+        <v>1</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2918,10 +2945,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'T5YIFR' not found in values file."</t>
-        </is>
+      <c r="N29" s="48" t="n">
+        <v>46155</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2934,19 +2959,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>1</v>
+        <v>2.24</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
       <c r="S29" s="6" t="n">
-        <v>1</v>
+        <v>2.27</v>
       </c>
       <c r="T29" s="6" t="n">
-        <v>1</v>
+        <v>2.28</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>1</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="30">
@@ -2960,7 +2985,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
+      <c r="C30" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2999,8 +3024,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="49" t="n">
-        <v>46154</v>
+      <c r="N30" s="48" t="n">
+        <v>46155</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3019,13 +3044,13 @@
         <v>2.47</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.45</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.42</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="31">
@@ -3035,7 +3060,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
+      <c r="C31" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3074,8 +3099,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="48" t="n">
-        <v>46023</v>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3088,19 +3115,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>0.007177997310378714</v>
+        <v>1</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>0.007345039668930076</v>
+        <v>1</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>0.007979811365325773</v>
+        <v>1</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>0.01026193247962737</v>
+        <v>1</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>0.007624633431085215</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3114,8 +3141,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
-        <v>46082</v>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3128,19 +3157,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>-0.005415070741811912</v>
+        <v>1</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.007368443846867079</v>
+        <v>1</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>-0.0001564786593617473</v>
+        <v>1</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.005246287630711999</v>
+        <v>1</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.001368313417869027</v>
+        <v>1</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3149,8 +3178,10 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="48" t="n">
-        <v>46023</v>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
+        </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3163,19 +3194,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>0.03316647264260756</v>
+        <v>1</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>0.03362463343108507</v>
+        <v>1</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>0.0358081705150977</v>
+        <v>1</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>0.03557875894988063</v>
+        <v>1</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>0.03369434416365838</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3185,8 +3216,10 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
-        <v>46082</v>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
+        </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3199,19 +3232,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.007416835246099523</v>
+        <v>1</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01231165794421915</v>
+        <v>1</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01529710277450485</v>
+        <v>1</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01279811178014365</v>
+        <v>1</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.0180124379988418</v>
+        <v>1</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3224,7 +3257,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="49" t="n">
+      <c r="N33" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -3264,8 +3297,10 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46082</v>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'TCU' not found in values file."</t>
+        </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3278,19 +3313,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>75.6596</v>
+        <v>1</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.1407</v>
+        <v>1</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.6564</v>
+        <v>1</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.7296</v>
+        <v>1</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.42489999999999</v>
+        <v>1</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3299,7 +3334,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="48" t="n">
+      <c r="N34" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
@@ -3380,7 +3415,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="48" t="n">
+      <c r="N35" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
@@ -3420,7 +3455,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
+      <c r="C36" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3455,7 +3490,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="48" t="n">
+      <c r="N36" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
@@ -3491,7 +3526,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
+      <c r="C37" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3530,7 +3565,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
+      <c r="N37" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3570,7 +3605,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
+      <c r="C38" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3605,7 +3640,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
+      <c r="N38" s="49" t="n">
         <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -3641,7 +3676,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
+      <c r="C39" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3680,7 +3715,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
+      <c r="N39" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3720,7 +3755,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
+      <c r="C40" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3755,7 +3790,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
+      <c r="N40" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3791,7 +3826,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
+      <c r="C41" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3831,7 +3866,7 @@
         </is>
       </c>
       <c r="N41" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3844,19 +3879,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.01641414141414144</v>
+        <v>0.03296019900497504</v>
       </c>
       <c r="R41" s="38" t="n">
+        <v>0.01515151515151514</v>
+      </c>
+      <c r="S41" s="38" t="n">
         <v>0.01930501930501927</v>
       </c>
-      <c r="S41" s="38" t="n">
+      <c r="T41" s="38" t="n">
         <v>0.005174644243208348</v>
       </c>
-      <c r="T41" s="38" t="n">
+      <c r="U41" s="23" t="n">
         <v>0.005855562784645496</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="42">
@@ -3870,8 +3905,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="48" t="n">
-        <v>46113</v>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3884,19 +3921,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>4020000</v>
+        <v>1000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>4010000</v>
+        <v>1000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>4130000</v>
+        <v>1000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>4020000</v>
+        <v>1000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>4270000</v>
+        <v>1000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3906,7 +3943,7 @@
         </is>
       </c>
       <c r="N42" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3919,19 +3956,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.05573770491803279</v>
+        <v>0.08846657929226737</v>
       </c>
       <c r="R42" s="38" t="n">
+        <v>0.0544262295081968</v>
+      </c>
+      <c r="S42" s="38" t="n">
         <v>0.03800786369593716</v>
       </c>
-      <c r="S42" s="38" t="n">
+      <c r="T42" s="38" t="n">
         <v>0.02506596306068609</v>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v>0.0341137123745819</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.03293010752688157</v>
       </c>
     </row>
     <row r="43">
@@ -3941,8 +3978,10 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="48" t="n">
-        <v>46113</v>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
+        </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3955,19 +3994,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="I43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="J43" s="38" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -3981,7 +4020,7 @@
         </is>
       </c>
       <c r="N43" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3994,19 +4033,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.007665505226480906</v>
+        <v>0.01933701657458542</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>0.009142053445851062</v>
+        <v>0.009059233449477455</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v>0.005657708628005631</v>
+        <v>0.009852216748768461</v>
       </c>
       <c r="T43" s="38" t="n">
+        <v>0.004950495049504955</v>
+      </c>
+      <c r="U43" s="23" t="n">
         <v>0.00141643059490093</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v/>
       </c>
     </row>
     <row r="44">
@@ -4058,7 +4097,7 @@
         </is>
       </c>
       <c r="N44" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4071,19 +4110,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.0211864406779661</v>
+        <v>0.0416372618207481</v>
       </c>
       <c r="R44" s="38" t="n">
+        <v>0.0225988700564973</v>
+      </c>
+      <c r="S44" s="38" t="n">
         <v>0.009852216748768513</v>
       </c>
-      <c r="S44" s="38" t="n">
-        <v>0.002820874471085876</v>
-      </c>
       <c r="T44" s="38" t="n">
+        <v>0.002115655853314407</v>
+      </c>
+      <c r="U44" s="23" t="n">
         <v>0</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>-0.0007077140835104227</v>
       </c>
     </row>
     <row r="45">
@@ -4146,7 +4185,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
+      <c r="C46" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4233,7 +4272,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
+      <c r="C47" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4314,7 +4353,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
+      <c r="C48" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4353,10 +4392,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS2' not found in values file."</t>
-        </is>
+      <c r="N48" s="48" t="n">
+        <v>46154</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4369,19 +4406,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R48" s="6" t="n">
-        <v>1</v>
+        <v>3.95</v>
       </c>
       <c r="S48" s="6" t="n">
-        <v>1</v>
+        <v>3.9</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>1</v>
+        <v>3.92</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>1</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="49">
@@ -4391,7 +4428,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
+      <c r="C49" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4430,8 +4467,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
-        <v>46153</v>
+      <c r="N49" s="48" t="n">
+        <v>46154</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4444,19 +4481,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.02</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.04</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>3.99</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.08</v>
       </c>
     </row>
     <row r="50">
@@ -4470,7 +4507,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
+      <c r="C50" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4509,8 +4546,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
-        <v>46153</v>
+      <c r="N50" s="48" t="n">
+        <v>46154</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4523,19 +4560,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.42</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.38</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.41</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.36</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.43</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4545,7 +4582,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
+      <c r="C51" s="49" t="n">
         <v>46082</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4637,8 +4674,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="51" t="n">
-        <v>46154</v>
+      <c r="N52" s="52" t="n">
+        <v>46155</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4654,16 +4691,16 @@
         <v>6.12</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.07</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.03</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.06</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.02</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -360,10 +360,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -901,10 +901,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C3" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -917,19 +915,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>1</v>
+        <v>24174.527</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>1</v>
+        <v>24055.749</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>1</v>
+        <v>24026.834</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>1</v>
+        <v>23770.976</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>1</v>
+        <v>23548.21</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -978,10 +976,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C4" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -994,19 +990,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>1</v>
+        <v>0.004937613873506885</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>1</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>1</v>
+        <v>0.0107634621312982</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>1</v>
+        <v>0.009459997171759493</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>1</v>
+        <v>-0.001625164044818495</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1055,7 +1051,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="48" t="n">
+      <c r="C5" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1094,7 +1090,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -1130,7 +1126,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="48" t="n">
+      <c r="C6" s="49" t="n">
         <v>46023</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1209,10 +1205,8 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPNOW' not found in values file."</t>
-        </is>
+      <c r="C7" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -1225,19 +1219,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1</v>
+        <v>3.9912</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>1</v>
+        <v>1.2392</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>1</v>
+        <v>4.2373</v>
       </c>
       <c r="I7" s="41" t="n">
-        <v>1</v>
+        <v>3.4728</v>
       </c>
       <c r="J7" s="41" t="n">
-        <v>1</v>
+        <v>2.902</v>
       </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1290,7 +1284,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1329,10 +1323,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CIVPART' not found in values file."</t>
-        </is>
+      <c r="N8" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1345,19 +1337,19 @@
         </is>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>1</v>
+        <v>61.8</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>1</v>
+        <v>61.9</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>1</v>
+        <v>62.1</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>1</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="9">
@@ -1371,10 +1363,8 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
-        </is>
+      <c r="C9" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -1387,19 +1377,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>1</v>
+        <v>16731.167</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1</v>
+        <v>16665.219</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>1</v>
+        <v>16585.878</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>1</v>
+        <v>16445.685</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>1</v>
+        <v>16345.793</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1412,10 +1402,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1428,19 +1416,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="10">
@@ -1450,10 +1438,8 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
-        </is>
+      <c r="C10" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -1466,19 +1452,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>1</v>
+        <v>0.00395722372445273</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>1</v>
+        <v>0.004783647872002916</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>1</v>
+        <v>0.008524606910566446</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>1</v>
+        <v>0.006111174905983452</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>1</v>
+        <v>0.001525835907232986</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1491,10 +1477,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
-        </is>
+      <c r="N10" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1507,19 +1491,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>1</v>
+        <v>4.1</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>1</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="11">
@@ -1533,7 +1517,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n">
+      <c r="C11" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1572,7 +1556,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1608,7 +1592,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="49" t="n">
+      <c r="C12" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1647,7 +1631,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1687,7 +1671,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="49" t="n">
+      <c r="C13" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1726,10 +1710,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
-        </is>
+      <c r="N13" s="49" t="n">
+        <v>46146</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1742,19 +1724,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>1</v>
+        <v>211000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>1</v>
+        <v>199000</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>1</v>
+        <v>190000</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>1</v>
+        <v>215000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>1</v>
+        <v>208000</v>
       </c>
     </row>
     <row r="14">
@@ -1764,7 +1746,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1803,10 +1785,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
-        </is>
+      <c r="N14" s="49" t="n">
+        <v>46139</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1819,19 +1799,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1</v>
+        <v>1782000</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1</v>
+        <v>1758000</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1</v>
+        <v>1776000</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1</v>
+        <v>1808000</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1</v>
+        <v>1809000</v>
       </c>
     </row>
     <row r="15">
@@ -1845,7 +1825,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1920,7 +1900,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1971,7 +1951,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
+      <c r="C17" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2058,7 +2038,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
+      <c r="C18" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2097,7 +2077,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
+      <c r="N18" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2137,7 +2117,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="49" t="n">
+      <c r="C19" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2172,7 +2152,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
+      <c r="N19" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2208,7 +2188,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2247,7 +2227,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
+      <c r="N20" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2287,7 +2267,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n">
+      <c r="C21" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2322,7 +2302,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
+      <c r="N21" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2362,7 +2342,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2401,7 +2381,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
+      <c r="N22" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2437,7 +2417,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2471,7 +2451,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
+      <c r="N23" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2511,10 +2491,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
-        </is>
+      <c r="C24" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2527,19 +2505,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>1</v>
+        <v>0.007561302505515899</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>1</v>
+        <v>0.0002854040755513321</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>1</v>
+        <v>0.001701852596202258</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>1</v>
+        <v>0.006198562656960505</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>1</v>
+        <v>-0.0007477594964454548</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2552,7 +2530,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="49" t="n">
+      <c r="N24" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2592,10 +2570,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'NONREVSL' not found in values file."</t>
-        </is>
+      <c r="C25" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2608,19 +2584,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>1</v>
+        <v>0.003911989748358602</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>1</v>
+        <v>0.0022395833833464</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>1</v>
+        <v>0.001310703086948806</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>1</v>
+        <v>0.001967095543671693</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>1</v>
+        <v>0.001164097695629751</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2629,7 +2605,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="49" t="n">
+      <c r="N25" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2669,10 +2645,8 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
-        </is>
+      <c r="C26" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2685,19 +2659,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>1</v>
+        <v>0.02495869599850553</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>1</v>
+        <v>0.005923787970366412</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>1</v>
+        <v>0.007794617579222285</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>1</v>
+        <v>0.01778138610314484</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>1</v>
+        <v>0.02303791460563676</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2710,7 +2684,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="49" t="n">
+      <c r="N26" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2750,10 +2724,8 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PRFIC1' not found in values file."</t>
-        </is>
+      <c r="C27" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -2766,19 +2738,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>1</v>
+        <v>-0.02054026778170115</v>
       </c>
       <c r="G27" s="38" t="n">
-        <v>1</v>
+        <v>-0.004277328978805506</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01832684674964358</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>1</v>
+        <v>-0.01299350008050415</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>1</v>
+        <v>-0.002410568051752549</v>
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2787,7 +2759,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="49" t="n">
+      <c r="N27" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2827,10 +2799,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
-        </is>
+      <c r="C28" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2843,19 +2813,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>1</v>
+        <v>0.008462114959539413</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>1</v>
+        <v>-0.01169466364559735</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>1</v>
+        <v>-0.004254034642219184</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>1</v>
+        <v>-0.00913646104747079</v>
       </c>
       <c r="J28" s="25" t="n">
-        <v>1</v>
+        <v>0.05441037812530491</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2868,7 +2838,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="49" t="n">
+      <c r="N28" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -2904,10 +2874,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGORDER' not found in values file."</t>
-        </is>
+      <c r="C29" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2920,19 +2888,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>1</v>
+        <v>0.008519519946871591</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>1</v>
+        <v>0.07567733047604469</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>1</v>
+        <v>0.09883411459674789</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>1</v>
+        <v>0.1059440595541697</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>1</v>
+        <v>0.1247312200873968</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2945,8 +2913,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="48" t="n">
-        <v>46155</v>
+      <c r="N29" s="49" t="n">
+        <v>46156</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2959,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.25</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="30">
@@ -2985,7 +2953,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="49" t="n">
+      <c r="C30" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -3024,8 +2992,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="48" t="n">
-        <v>46155</v>
+      <c r="N30" s="49" t="n">
+        <v>46156</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3047,7 +3015,7 @@
         <v>2.47</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.45</v>
@@ -3060,7 +3028,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="49" t="n">
+      <c r="C31" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3099,10 +3067,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N31" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
@@ -3115,19 +3081,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
-        <v>1</v>
+        <v>0.007177997310378714</v>
       </c>
       <c r="R31" s="38" t="n">
-        <v>1</v>
+        <v>0.007345039668930076</v>
       </c>
       <c r="S31" s="38" t="n">
-        <v>1</v>
+        <v>0.007979811365325773</v>
       </c>
       <c r="T31" s="38" t="n">
-        <v>1</v>
+        <v>0.01026193247962737</v>
       </c>
       <c r="U31" s="23" t="n">
-        <v>1</v>
+        <v>0.007624633431085215</v>
       </c>
     </row>
     <row r="32">
@@ -3141,10 +3107,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C32" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3157,19 +3121,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>1</v>
+        <v>0.006780543386440963</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>1</v>
+        <v>-0.002888319299829911</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>1</v>
+        <v>0.006180911901310315</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>1</v>
+        <v>-0.0004590214961934791</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>1</v>
+        <v>0.004809253086077714</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3178,10 +3142,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ECIWAG' not found in values file."</t>
-        </is>
+      <c r="N32" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
@@ -3194,19 +3156,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
-        <v>1</v>
+        <v>0.03316647264260756</v>
       </c>
       <c r="R32" s="38" t="n">
-        <v>1</v>
+        <v>0.03362463343108507</v>
       </c>
       <c r="S32" s="38" t="n">
-        <v>1</v>
+        <v>0.0358081705150977</v>
       </c>
       <c r="T32" s="38" t="n">
-        <v>1</v>
+        <v>0.03557875894988063</v>
       </c>
       <c r="U32" s="23" t="n">
-        <v>1</v>
+        <v>0.03369434416365838</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3216,10 +3178,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'INDPRO' not found in values file."</t>
-        </is>
+      <c r="C33" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3232,19 +3192,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>1</v>
+        <v>0.01353137956983195</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>1</v>
+        <v>0.007577167152940725</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>1</v>
+        <v>0.00990709134484607</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>1</v>
+        <v>0.01408088966438706</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>1</v>
+        <v>0.01189108049354475</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3297,10 +3257,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'TCU' not found in values file."</t>
-        </is>
+      <c r="C34" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3313,19 +3271,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>1</v>
+        <v>76.1194</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>1</v>
+        <v>75.6716</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>1</v>
+        <v>75.9598</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>1</v>
+        <v>75.5658</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>1</v>
+        <v>75.6618</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3334,7 +3292,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="49" t="n">
+      <c r="N34" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
@@ -3374,10 +3332,8 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PRS85006092' not found in values file."</t>
-        </is>
+      <c r="C35" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
@@ -3390,19 +3346,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G35" s="41" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="H35" s="41" t="n">
-        <v>1</v>
+        <v>5.2</v>
       </c>
       <c r="I35" s="41" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="J35" s="41" t="n">
-        <v>1</v>
+        <v>-0.9</v>
       </c>
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -3415,7 +3371,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="49" t="n">
+      <c r="N35" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
@@ -3455,7 +3411,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="49" t="n">
+      <c r="C36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3490,7 +3446,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="49" t="n">
+      <c r="N36" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
@@ -3526,7 +3482,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n">
+      <c r="C37" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3565,7 +3521,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="49" t="n">
+      <c r="N37" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3605,7 +3561,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="49" t="n">
+      <c r="C38" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3640,7 +3596,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="49" t="n">
+      <c r="N38" s="48" t="n">
         <v>46054</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -3676,7 +3632,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="49" t="n">
+      <c r="C39" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3715,7 +3671,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="49" t="n">
+      <c r="N39" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3755,7 +3711,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n">
+      <c r="C40" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3790,7 +3746,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="49" t="n">
+      <c r="N40" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3826,7 +3782,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n">
+      <c r="C41" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3865,7 +3821,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
+      <c r="N41" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3905,10 +3861,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C42" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3921,19 +3875,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>1000</v>
+        <v>4020000</v>
       </c>
       <c r="G42" s="39" t="n">
-        <v>1000</v>
+        <v>4010000</v>
       </c>
       <c r="H42" s="39" t="n">
-        <v>1000</v>
+        <v>4130000</v>
       </c>
       <c r="I42" s="39" t="n">
-        <v>1000</v>
+        <v>4020000</v>
       </c>
       <c r="J42" s="39" t="n">
-        <v>1000</v>
+        <v>4270000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3942,7 +3896,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
+      <c r="N42" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3978,10 +3932,8 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EXHOSLUSM495S' not found in values file."</t>
-        </is>
+      <c r="C43" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3994,19 +3946,19 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="H43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="I43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="J43" s="38" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="K43" s="5" t="n"/>
       <c r="L43" s="28" t="inlineStr">
@@ -4019,7 +3971,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
+      <c r="N43" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4059,10 +4011,8 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GCE' not found in values file."</t>
-        </is>
+      <c r="C44" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
@@ -4075,19 +4025,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>1</v>
+        <v>5418.445</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>1</v>
+        <v>5343.513</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>1</v>
+        <v>5324.402</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>1</v>
+        <v>5236.97</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>1</v>
+        <v>5195.517</v>
       </c>
       <c r="K44" s="5" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4096,7 +4046,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
+      <c r="N44" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4132,10 +4082,8 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GCE' not found in values file."</t>
-        </is>
+      <c r="C45" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
@@ -4148,19 +4096,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>1</v>
+        <v>0.01402298450476303</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>1</v>
+        <v>0.003589323270481781</v>
       </c>
       <c r="H45" s="38" t="n">
-        <v>1</v>
+        <v>0.01669515005814426</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>1</v>
+        <v>0.007978609251013902</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>1</v>
+        <v>0.008696251498575336</v>
       </c>
       <c r="K45" s="5" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4185,7 +4133,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
+      <c r="C46" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4272,7 +4220,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
+      <c r="C47" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4311,10 +4259,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DFF' not found in values file."</t>
-        </is>
+      <c r="N47" s="49" t="n">
+        <v>46155</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4327,19 +4273,19 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>1</v>
+        <v>3.63</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>1</v>
+        <v>3.63</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>1</v>
+        <v>3.63</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>1</v>
+        <v>3.63</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>1</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="48">
@@ -4353,7 +4299,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
+      <c r="C48" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4392,8 +4338,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="48" t="n">
-        <v>46154</v>
+      <c r="N48" s="49" t="n">
+        <v>46155</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4406,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.9</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.92</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.87</v>
       </c>
     </row>
     <row r="49">
@@ -4428,7 +4374,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
+      <c r="C49" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4467,8 +4413,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="48" t="n">
-        <v>46154</v>
+      <c r="N49" s="49" t="n">
+        <v>46155</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4484,16 +4430,16 @@
         <v>4.12</v>
       </c>
       <c r="R49" s="6" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="S49" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.02</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.04</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>3.99</v>
       </c>
     </row>
     <row r="50">
@@ -4507,7 +4453,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
+      <c r="C50" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4546,8 +4492,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="48" t="n">
-        <v>46154</v>
+      <c r="N50" s="49" t="n">
+        <v>46155</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4563,16 +4509,16 @@
         <v>4.46</v>
       </c>
       <c r="R50" s="6" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.42</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.38</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.41</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.36</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4582,7 +4528,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
+      <c r="C51" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4621,10 +4567,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'MORTGAGE30US' not found in values file."</t>
-        </is>
+      <c r="N51" s="49" t="n">
+        <v>46153</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4637,19 +4581,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>1</v>
+        <v>6.36</v>
       </c>
       <c r="R51" s="6" t="n">
-        <v>1</v>
+        <v>6.37</v>
       </c>
       <c r="S51" s="6" t="n">
-        <v>1</v>
+        <v>6.3</v>
       </c>
       <c r="T51" s="6" t="n">
-        <v>1</v>
+        <v>6.23</v>
       </c>
       <c r="U51" s="21" t="n">
-        <v>1</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4675,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4688,19 +4632,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.12</v>
+        <v>6.09</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.12</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.07</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.03</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.06</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.25</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,7 +3006,7 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.47</v>
+        <v>2.49</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.47</v>
@@ -3018,7 +3018,7 @@
         <v>2.47</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="31">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.95</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.9</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.92</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>4.12</v>
+        <v>4.13</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>4.12</v>
       </c>
       <c r="S49" s="6" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="T49" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.02</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.04</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.46</v>
+        <v>4.47</v>
       </c>
       <c r="R50" s="6" t="n">
         <v>4.46</v>
       </c>
       <c r="S50" s="6" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="T50" s="6" t="n">
         <v>4.42</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.38</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.41</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -77,14 +77,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -363,16 +363,16 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1051,7 +1051,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
+      <c r="C5" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1109,7 +1109,7 @@
       <c r="R5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="S5" s="50" t="n">
+      <c r="S5" s="49" t="n">
         <v>66000</v>
       </c>
       <c r="T5" s="24" t="n">
@@ -1126,7 +1126,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
+      <c r="C6" s="48" t="n">
         <v>46023</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1710,7 +1710,7 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
+      <c r="N13" s="50" t="n">
         <v>46146</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1785,7 +1785,7 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
+      <c r="N14" s="50" t="n">
         <v>46139</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -1951,7 +1951,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
+      <c r="C17" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2038,7 +2038,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="49" t="n">
+      <c r="C18" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2077,7 +2077,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
+      <c r="N18" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2152,7 +2152,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2227,7 +2227,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
+      <c r="N20" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2302,7 +2302,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
+      <c r="N21" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2381,7 +2381,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2451,7 +2451,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2913,7 +2913,7 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="49" t="n">
+      <c r="N29" s="50" t="n">
         <v>46157</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
@@ -2992,7 +2992,7 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="49" t="n">
+      <c r="N30" s="50" t="n">
         <v>46157</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
@@ -3107,7 +3107,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="49" t="n">
+      <c r="C32" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3178,7 +3178,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="49" t="n">
+      <c r="C33" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3257,7 +3257,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="49" t="n">
+      <c r="C34" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -3821,7 +3821,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3896,7 +3896,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="49" t="n">
+      <c r="N42" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3971,7 +3971,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4046,7 +4046,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4259,7 +4259,7 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="49" t="n">
+      <c r="N47" s="50" t="n">
         <v>46156</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
@@ -4338,7 +4338,7 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
+      <c r="N48" s="50" t="n">
         <v>46156</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
@@ -4413,7 +4413,7 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
+      <c r="N49" s="50" t="n">
         <v>46156</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
@@ -4492,7 +4492,7 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
+      <c r="N50" s="50" t="n">
         <v>46156</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
@@ -4567,7 +4567,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="50" t="n">
         <v>46153</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,19 +4632,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.09</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.12</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.12</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.07</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.03</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-19
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2077,7 +2077,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="50" t="n">
+      <c r="N18" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2152,7 +2152,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="50" t="n">
+      <c r="N19" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2227,7 +2227,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="50" t="n">
+      <c r="N20" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2302,7 +2302,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="50" t="n">
+      <c r="N21" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.25</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,10 +3006,10 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.49</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.47</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.47</v>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.95</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.9</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.13</v>
-      </c>
-      <c r="R49" s="6" t="n">
-        <v>4.12</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>4.12</v>
       </c>
       <c r="T49" s="6" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.07</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.02</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.47</v>
-      </c>
-      <c r="R50" s="6" t="n">
-        <v>4.46</v>
       </c>
       <c r="S50" s="6" t="n">
         <v>4.46</v>
       </c>
       <c r="T50" s="6" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.42</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.38</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,19 +4632,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.21</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.09</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.12</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.12</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.07</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-20
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2381,7 +2381,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="50" t="n">
+      <c r="N22" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2451,7 +2451,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="50" t="n">
+      <c r="N23" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,13 +3006,13 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.48</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.49</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.47</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.47</v>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.95</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.13</v>
-      </c>
-      <c r="S49" s="6" t="n">
-        <v>4.12</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>4.12</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.07</v>
+        <v>4.12</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.59</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.47</v>
-      </c>
-      <c r="S50" s="6" t="n">
-        <v>4.46</v>
       </c>
       <c r="T50" s="6" t="n">
         <v>4.46</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.42</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,16 +4632,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.2</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.21</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.09</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.12</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.12</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-05-21
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.9912</v>
+        <v>4.2573</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="N13" s="50" t="n">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1724,19 +1724,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>211000</v>
+        <v>209000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>212000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>199000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>190000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>215000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>208000</v>
       </c>
     </row>
     <row r="14">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="N14" s="50" t="n">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1802,16 +1802,16 @@
         <v>1782000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1776000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1758000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1776000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1808000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1809000</v>
       </c>
     </row>
     <row r="15">
@@ -1951,7 +1951,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="50" t="n">
+      <c r="C17" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2038,7 +2038,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="50" t="n">
+      <c r="C18" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,16 +3006,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.49</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.48</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.49</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.47</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.47</v>
@@ -3411,8 +3411,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
-        <v>46082</v>
+      <c r="C36" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3425,19 +3425,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1502</v>
+        <v>1465</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1356</v>
+        <v>1507</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1398</v>
+        <v>1346</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1373</v>
+        <v>1385</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1324</v>
+        <v>1378</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3482,8 +3482,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
-        <v>46082</v>
+      <c r="C37" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3496,19 +3496,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.1084870848708487</v>
+        <v>0.04642857142857143</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.08993288590604027</v>
+        <v>0.1196136701337296</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>0.02945508100147275</v>
+        <v>-0.09725016767270288</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>-0.09313077939233817</v>
+        <v>0.02365114560236511</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>0.02239382239382239</v>
+        <v>-0.07764390896921017</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3561,8 +3561,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>46082</v>
+      <c r="C38" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3575,19 +3575,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
+        <v>1442</v>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>1363</v>
       </c>
-      <c r="G38" s="24" t="n">
-        <v>1538</v>
-      </c>
       <c r="H38" s="24" t="n">
-        <v>1386</v>
+        <v>1540</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>1455</v>
+        <v>1393</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>1388</v>
+        <v>1482</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3632,8 +3632,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>46082</v>
+      <c r="C39" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3646,19 +3646,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.07967589466576637</v>
+        <v>-0.002076124567474049</v>
       </c>
       <c r="G39" s="38" t="n">
-        <v>0.0577716643741403</v>
+        <v>-0.08646112600536193</v>
       </c>
       <c r="H39" s="38" t="n">
-        <v>-0.05068493150684932</v>
+        <v>0.06500691562932227</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>-0.01689189189189189</v>
+        <v>-0.04784688995215311</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>-0.07957559681697612</v>
+        <v>0.01022494887525562</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3821,7 +3821,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="50" t="n">
+      <c r="N41" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3896,7 +3896,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="50" t="n">
+      <c r="N42" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3971,7 +3971,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="50" t="n">
+      <c r="N43" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4046,7 +4046,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="50" t="n">
+      <c r="N44" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="R47" s="6" t="n">
         <v>3.63</v>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.98</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,16 +4427,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.13</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>4.12</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.12</v>
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,16 +4506,16 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.61</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.59</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.47</v>
-      </c>
-      <c r="T50" s="6" t="n">
-        <v>4.46</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.46</v>
@@ -4568,7 +4568,7 @@
         </is>
       </c>
       <c r="N51" s="50" t="n">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4581,19 +4581,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.36</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.37</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.23</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.3</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,19 +4632,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.24</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.2</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.21</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.09</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.12</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="N28" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
@@ -2852,19 +2852,19 @@
         </is>
       </c>
       <c r="Q28" s="6" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="R28" s="6" t="n">
         <v>3.8</v>
       </c>
-      <c r="R28" s="6" t="n">
+      <c r="S28" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="S28" s="6" t="n">
+      <c r="T28" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T28" s="6" t="n">
+      <c r="U28" s="21" t="n">
         <v>4.2</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>4.5</v>
       </c>
     </row>
     <row r="29">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,19 +3006,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.44</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.49</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.48</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.49</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.47</v>
       </c>
     </row>
     <row r="31">
@@ -3107,7 +3107,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="50" t="n">
+      <c r="C32" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3178,7 +3178,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="50" t="n">
+      <c r="C33" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3257,7 +3257,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="50" t="n">
+      <c r="C34" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
         <v>3.62</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="S47" s="6" t="n">
         <v>3.63</v>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.98</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.32</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.26</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.12</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.67</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.61</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.59</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.47</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.46</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4635,16 +4635,16 @@
         <v>6.16</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.24</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.2</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.21</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.09</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,19 +3006,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.44</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.49</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.48</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.49</v>
       </c>
     </row>
     <row r="31">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4279,7 +4279,7 @@
         <v>3.62</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="T47" s="6" t="n">
         <v>3.63</v>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.04</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.09</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.22</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.32</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4509,16 +4509,16 @@
         <v>4.57</v>
       </c>
       <c r="R50" s="6" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.67</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.61</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.59</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.47</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-26
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -3521,8 +3521,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
-        <v>46054</v>
+      <c r="N37" s="50" t="n">
+        <v>46082</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3535,19 +3535,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.002917033083199794</v>
+        <v>0.007161347041441779</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>-0.001828986686322698</v>
+        <v>0.003402954536404934</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>-0.002571690054911535</v>
+        <v>-0.001489442391916063</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.001325270004722268</v>
+        <v>-0.002589859586293541</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.001961201654098743</v>
+        <v>-0.001285648567050157</v>
       </c>
     </row>
     <row r="38">
@@ -3596,8 +3596,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
-        <v>46054</v>
+      <c r="N38" s="50" t="n">
+        <v>46082</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3610,19 +3610,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.00667093146994231</v>
+        <v>0.006657391474145452</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.00830161397958413</v>
+        <v>0.007541366795841786</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.01125517292572641</v>
+        <v>0.008681655137469846</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01266604881062719</v>
+        <v>0.01129232301425539</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01312727250279332</v>
+        <v>0.01271856657398832</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46164</v>
+        <v>46168</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46164</v>
+        <v>46168</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3009,16 +3009,16 @@
         <v>2.4</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.44</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.49</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.48</v>
       </c>
     </row>
     <row r="31">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46163</v>
+        <v>46167</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4282,10 +4282,10 @@
         <v>3.62</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="48">
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.08</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.04</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.07</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.09</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.25</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.22</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.32</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.57</v>
+        <v>4.56</v>
       </c>
       <c r="R50" s="6" t="n">
         <v>4.57</v>
       </c>
       <c r="S50" s="6" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="T50" s="6" t="n">
         <v>4.67</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.61</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.59</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46163</v>
+        <v>46168</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,19 +4632,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.16</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.16</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.24</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.21</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24174.527</v>
+        <v>24152.656</v>
       </c>
       <c r="G3" s="24" t="n">
         <v>24055.749</v>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.004937613873506885</v>
+        <v>0.004028434117765434</v>
       </c>
       <c r="G4" s="25" t="n">
         <v>0.001203446113624551</v>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.2573</v>
+        <v>3.8233</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16731.167</v>
+        <v>16723.347</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>16665.219</v>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.00395722372445273</v>
+        <v>0.003487982966200454</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>0.004783647872002916</v>
@@ -1517,8 +1517,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
-        <v>46082</v>
+      <c r="C11" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
@@ -1531,19 +1531,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>0.009363644833690454</v>
+        <v>-0.005560917321568049</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.01734597156398099</v>
+        <v>0.01275308354666049</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>-0.01314250970487807</v>
+        <v>0.02042270244597488</v>
       </c>
       <c r="I11" s="25" t="n">
+        <v>-0.0152471820775455</v>
+      </c>
+      <c r="J11" s="25" t="n">
         <v>-0.00581233144238813</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>0.007353974425031495</v>
       </c>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1592,8 +1592,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
-        <v>46082</v>
+      <c r="C12" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -1606,19 +1606,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>-0.005690422651553436</v>
+        <v>-0.0005542725173209322</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.02619753322497357</v>
+        <v>-0.001468496168142728</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.009762633996937256</v>
+        <v>0.02710584185868621</v>
       </c>
       <c r="I12" s="25" t="n">
+        <v>0.007609111791730519</v>
+      </c>
+      <c r="J12" s="25" t="n">
         <v>-0.02262753702687877</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>0.008866163156166484</v>
       </c>
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1671,8 +1671,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
-        <v>46082</v>
+      <c r="C13" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -1685,19 +1685,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>0.003475754493048377</v>
+        <v>0.001712376835190765</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0</v>
+        <v>0.0047667400011282</v>
       </c>
       <c r="H13" s="25" t="n">
+        <v>0.001865038996269996</v>
+      </c>
+      <c r="I13" s="25" t="n">
         <v>-0.0006495156872157182</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="J13" s="25" t="n">
         <v>-0.002197864126912585</v>
-      </c>
-      <c r="J13" s="25" t="n">
-        <v>0.001326110264657787</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="N13" s="50" t="n">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1724,19 +1724,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>209000</v>
+        <v>215000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>210000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>212000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>199000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>190000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>215000</v>
       </c>
     </row>
     <row r="14">
@@ -1746,8 +1746,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
-        <v>46082</v>
+      <c r="C14" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -1760,19 +1760,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.0137310876391664</v>
+        <v>0.01881513204853678</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01412809858145871</v>
+        <v>0.0169283471310306</v>
       </c>
       <c r="H14" s="25" t="n">
+        <v>0.01601948703252618</v>
+      </c>
+      <c r="I14" s="25" t="n">
         <v>0.01859420873870254</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="J14" s="25" t="n">
         <v>0.01400263444247182</v>
-      </c>
-      <c r="J14" s="25" t="n">
-        <v>0.02601983289485096</v>
       </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="N14" s="50" t="n">
-        <v>46146</v>
+        <v>46153</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1799,19 +1799,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1782000</v>
+        <v>1786000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1771000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1776000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1758000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1776000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1808000</v>
       </c>
     </row>
     <row r="15">
@@ -1825,8 +1825,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
-        <v>46082</v>
+      <c r="C15" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1839,19 +1839,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.0009659131941934795</v>
+        <v>0.00194183526011571</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.001283511397942805</v>
+        <v>0.001184566276935417</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.002828085060096797</v>
+        <v>0.0003980279524176122</v>
       </c>
       <c r="I15" s="25" t="n">
+        <v>0.002021355667953806</v>
+      </c>
+      <c r="J15" s="25" t="n">
         <v>0.002845221754583793</v>
-      </c>
-      <c r="J15" s="25" t="n">
-        <v>-9.089339114154438e-05</v>
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1900,8 +1900,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
-        <v>46082</v>
+      <c r="C16" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -1914,19 +1914,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02780790300603432</v>
+        <v>0.02508778414341157</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.03057028560796356</v>
+        <v>0.02629700694270652</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02594680811602797</v>
+        <v>0.02883058889198992</v>
       </c>
       <c r="I16" s="25" t="n">
+        <v>0.02512148076709073</v>
+      </c>
+      <c r="J16" s="25" t="n">
         <v>0.02311045163683583</v>
-      </c>
-      <c r="J16" s="25" t="n">
-        <v>0.02359662426842094</v>
       </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2117,8 +2117,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
-        <v>46082</v>
+      <c r="C19" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -2131,19 +2131,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.0005629480818372112</v>
+        <v>-0.004828076094918865</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>-0.003744432836641498</v>
+        <v>-0.001601241100368522</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>0.006441402056378998</v>
+        <v>-0.004616097329612545</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>-0.0004425121414268762</v>
+        <v>0.00631018120265292</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>0.0008581029834302534</v>
+        <v>-0.0009204273888139269</v>
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2188,8 +2188,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
-        <v>46082</v>
+      <c r="C20" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -2202,19 +2202,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.004415084502276996</v>
+        <v>-0.01104621985451874</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.01163563272940462</v>
+        <v>-0.0005269259142164612</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.01661281847756826</v>
+        <v>0.007704977527148879</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.01134436615382877</v>
+        <v>0.0135496204541136</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01272729309745998</v>
+        <v>0.008428522657950768</v>
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2267,8 +2267,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
-        <v>46082</v>
+      <c r="C21" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -2281,19 +2281,19 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H21" s="6" t="n">
         <v>3.6</v>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>4.5</v>
-      </c>
       <c r="I21" s="6" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2342,8 +2342,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
-        <v>46082</v>
+      <c r="C22" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2356,19 +2356,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.696</v>
+        <v>16.318</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.098</v>
+        <v>16.537</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>15.197</v>
+        <v>15.881</v>
       </c>
       <c r="I22" s="24" t="n">
+        <v>14.987</v>
+      </c>
+      <c r="J22" s="24" t="n">
         <v>16.4</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>16.006</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2417,8 +2417,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
-        <v>46082</v>
+      <c r="C23" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2431,19 +2431,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.09013623978201633</v>
+        <v>-0.07194449183870769</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.01955052073816928</v>
+        <v>-0.09880108991825626</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.04721003134796239</v>
+        <v>-0.0327669163773677</v>
       </c>
       <c r="I23" s="25" t="n">
+        <v>-0.0603761755485893</v>
+      </c>
+      <c r="J23" s="25" t="n">
         <v>-0.05207791457141205</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>-0.05334752779749237</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2530,8 +2530,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
-        <v>46082</v>
+      <c r="N24" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
@@ -2544,19 +2544,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.006641747242902563</v>
+        <v>0.003995981009502714</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.003751937984496134</v>
+        <v>0.006647621988882024</v>
       </c>
       <c r="S24" s="38" t="n">
-        <v>0.003297660527625812</v>
+        <v>0.004015441621060045</v>
       </c>
       <c r="T24" s="38" t="n">
+        <v>0.003313215530114544</v>
+      </c>
+      <c r="U24" s="23" t="n">
         <v>0.003308571071852118</v>
-      </c>
-      <c r="U24" s="23" t="n">
-        <v>0.00219752719537647</v>
       </c>
     </row>
     <row r="25">
@@ -2605,8 +2605,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
-        <v>46082</v>
+      <c r="N25" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
@@ -2619,19 +2619,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.0349608149847944</v>
+        <v>0.03766944114149807</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.02829551861881658</v>
+        <v>0.03525460334601121</v>
       </c>
       <c r="S25" s="38" t="n">
-        <v>0.02856869483403365</v>
+        <v>0.02858141215524022</v>
       </c>
       <c r="T25" s="38" t="n">
+        <v>0.02858464163550402</v>
+      </c>
+      <c r="U25" s="23" t="n">
         <v>0.02878083518031025</v>
-      </c>
-      <c r="U25" s="23" t="n">
-        <v>0.02820189831269997</v>
       </c>
     </row>
     <row r="26">
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.02495869599850553</v>
+        <v>0.0243486718158854</v>
       </c>
       <c r="G26" s="38" t="n">
         <v>0.005923787970366412</v>
@@ -2684,8 +2684,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
-        <v>46082</v>
+      <c r="N26" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
@@ -2698,19 +2698,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.002932483068401215</v>
+        <v>0.002389403113183475</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.003675182396499332</v>
+        <v>0.002954862726849639</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.004245969066199562</v>
+        <v>0.003955400523234065</v>
       </c>
       <c r="T26" s="38" t="n">
+        <v>0.00426942745883041</v>
+      </c>
+      <c r="U26" s="23" t="n">
         <v>0.003271383630529812</v>
-      </c>
-      <c r="U26" s="23" t="n">
-        <v>0.001776129138734595</v>
       </c>
     </row>
     <row r="27">
@@ -2738,7 +2738,7 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.02054026778170115</v>
+        <v>-0.01596729536276953</v>
       </c>
       <c r="G27" s="38" t="n">
         <v>-0.004277328978805506</v>
@@ -2759,8 +2759,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
-        <v>46082</v>
+      <c r="N27" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
@@ -2773,19 +2773,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03202758906974702</v>
+        <v>0.03289190610508199</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03001318470574146</v>
+        <v>0.03236287290347819</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.03083788838321814</v>
+        <v>0.03032482320508212</v>
       </c>
       <c r="T27" s="38" t="n">
+        <v>0.03086196794208051</v>
+      </c>
+      <c r="U27" s="23" t="n">
         <v>0.02971110180682146</v>
-      </c>
-      <c r="U27" s="23" t="n">
-        <v>0.02829092786499081</v>
       </c>
     </row>
     <row r="28">
@@ -2799,8 +2799,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
-        <v>46082</v>
+      <c r="C28" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -2813,19 +2813,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.008462114959539413</v>
+        <v>0.07946631387134628</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>0.01345526874171887</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>-0.01169466364559735</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>-0.004254034642219184</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>-0.00913646104747079</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>0.05441037812530491</v>
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2874,8 +2874,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
-        <v>46082</v>
+      <c r="C29" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -2888,19 +2888,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.008519519946871591</v>
+        <v>0.171822551307629</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.0135129579558212</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.07567733047604469</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.09883411459674789</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.1059440595541697</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.1247312200873968</v>
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.29</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="30">
@@ -2953,8 +2953,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
-        <v>46082</v>
+      <c r="C30" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -2967,19 +2967,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.002810142088861101</v>
+        <v>0.08083364547795258</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>-0.002695717141530163</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>-0.01222345960141613</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>0.002385879326488816</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>-0.01921059426035288</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>0.06592882125886601</v>
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,19 +3006,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.4</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.44</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.49</v>
       </c>
     </row>
     <row r="31">
@@ -3028,8 +3028,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
-        <v>46082</v>
+      <c r="C31" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
@@ -3042,19 +3042,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>-0.01830187491510037</v>
+        <v>0.1492280257336716</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>-0.0181892276038923</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.07288240242929306</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.09283155684402497</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.1010908210327026</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.1265306873826442</v>
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="N34" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
@@ -3306,19 +3306,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.0006003095351817524</v>
+        <v>-0.00188417944067203</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>0.008470913795465586</v>
+        <v>-0.0008839228572701012</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>0.007760924955011093</v>
+        <v>0.008190609959018323</v>
       </c>
       <c r="T34" s="38" t="n">
+        <v>0.007745300996855934</v>
+      </c>
+      <c r="U34" s="23" t="n">
         <v>0.008247145515396716</v>
-      </c>
-      <c r="U34" s="23" t="n">
-        <v>0.01081883276249912</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3372,7 +3372,7 @@
         </is>
       </c>
       <c r="N35" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
@@ -3385,19 +3385,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.004465589402518066</v>
+        <v>-0.00238004469329578</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>-0.0005198395303640524</v>
+        <v>-0.004471399292342637</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>0.0002132515841006821</v>
+        <v>-0.0007821528833659164</v>
       </c>
       <c r="T35" s="38" t="n">
+        <v>0.0001977446423231388</v>
+      </c>
+      <c r="U35" s="23" t="n">
         <v>-0.002758902506289296</v>
-      </c>
-      <c r="U35" s="23" t="n">
-        <v>0.001868922106829984</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3411,7 +3411,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="50" t="n">
+      <c r="C36" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="N36" s="48" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
@@ -3460,19 +3460,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.0006003095351817524</v>
+        <v>-0.00188417944067203</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>0.008470913795465586</v>
+        <v>-0.0008839228572701012</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>0.007760924955011093</v>
+        <v>0.008190609959018323</v>
       </c>
       <c r="T36" s="38" t="n">
+        <v>0.007745300996855934</v>
+      </c>
+      <c r="U36" s="23" t="n">
         <v>0.008247145515396716</v>
-      </c>
-      <c r="U36" s="23" t="n">
-        <v>0.01081883276249912</v>
       </c>
     </row>
     <row r="37">
@@ -3482,7 +3482,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="50" t="n">
+      <c r="C37" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3561,7 +3561,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="50" t="n">
+      <c r="C38" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1442</v>
+        <v>1423</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1363</v>
@@ -3632,7 +3632,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="50" t="n">
+      <c r="C39" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3646,7 +3646,7 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.002076124567474049</v>
+        <v>-0.01522491349480969</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>-0.08646112600536193</v>
@@ -3711,8 +3711,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
-        <v>46082</v>
+      <c r="C40" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -3725,19 +3725,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>682</v>
+        <v>622</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>635</v>
+        <v>663</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>583</v>
+        <v>641</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>728</v>
+        <v>576</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>748</v>
+        <v>723</v>
       </c>
       <c r="K40" s="5" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3782,8 +3782,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
-        <v>46082</v>
+      <c r="C41" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
@@ -3796,19 +3796,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>0.03333333333333333</v>
+        <v>-0.1126961483594865</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.01090342679127726</v>
+        <v>0.01067073170731707</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>-0.1193353474320242</v>
+        <v>0</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>0.01392757660167131</v>
+        <v>-0.1338345864661654</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>0.1081481481481481</v>
+        <v>0.02991452991452992</v>
       </c>
       <c r="K41" s="5" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5418.445</v>
+        <v>5416.4</v>
       </c>
       <c r="G44" s="24" t="n">
         <v>5343.513</v>
@@ -4096,7 +4096,7 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.01402298450476303</v>
+        <v>0.01364027747289098</v>
       </c>
       <c r="G45" s="38" t="n">
         <v>0.003589323270481781</v>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46167</v>
+        <v>46168</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46164</v>
+        <v>46168</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.08</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.04</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.07</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46164</v>
+        <v>46168</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.25</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.22</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.32</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46164</v>
+        <v>46168</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.56</v>
-      </c>
-      <c r="R50" s="6" t="n">
-        <v>4.57</v>
       </c>
       <c r="S50" s="6" t="n">
         <v>4.57</v>
       </c>
       <c r="T50" s="6" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.67</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.61</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4568,7 +4568,7 @@
         </is>
       </c>
       <c r="N51" s="50" t="n">
-        <v>46160</v>
+        <v>46167</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4581,19 +4581,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.51</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.36</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.37</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.3</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.23</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,19 +4632,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.13</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.16</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.16</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.24</v>
+        <v>6.16</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-05-29
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,19 +2927,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.25</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3009,16 +3009,16 @@
         <v>2.39</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.4</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.39</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.44</v>
       </c>
     </row>
     <row r="31">
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4352,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.01</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.08</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.04</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="49">
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4427,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.19</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.25</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.22</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.32</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,19 +4506,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.56</v>
-      </c>
-      <c r="S50" s="6" t="n">
-        <v>4.57</v>
       </c>
       <c r="T50" s="6" t="n">
         <v>4.57</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.67</v>
+        <v>4.57</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="N52" s="52" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,16 +4632,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.13</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.16</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.16</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-05-31
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -901,8 +901,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
-        <v>46023</v>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -915,19 +917,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24152.656</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24055.749</v>
+        <v>1</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>24026.834</v>
+        <v>1</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>23770.976</v>
+        <v>1</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23548.21</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -976,8 +978,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
-        <v>46023</v>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -990,19 +994,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.004028434117765434</v>
+        <v>1</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>1</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>1</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>1</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>-0.001625164044818495</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1402,8 +1406,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46113</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1416,19 +1422,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.1</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2077,8 +2083,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
-        <v>46113</v>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2091,19 +2099,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>0.006400377846336402</v>
+        <v>1</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>0.008651438343614481</v>
+        <v>1</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>0.00267003074209704</v>
+        <v>1</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>0.00170842649932057</v>
+        <v>1</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v>0.00297788428704604</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2152,8 +2160,10 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
-        <v>46113</v>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
+        </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2166,19 +2176,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>0.03779245836741563</v>
+        <v>1</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>0.03285957752865201</v>
+        <v>1</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>0.0243400411037322</v>
+        <v>1</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>0.02391201432150015</v>
+        <v>1</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>0.02653304114557758</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2227,8 +2237,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46113</v>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2241,19 +2253,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>0.00376460730477457</v>
+        <v>1</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.001957950538511444</v>
+        <v>1</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>0.002160502174024082</v>
+        <v>1</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>0.002950448142634121</v>
+        <v>1</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>0.002329002576704653</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2302,8 +2314,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46113</v>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2316,19 +2330,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.02743309430968526</v>
+        <v>1</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.0260216770548682</v>
+        <v>1</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>0.02472462476764023</v>
+        <v>1</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>0.02512028782828883</v>
+        <v>1</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>0.02646484707309002</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2914,7 +2928,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2930,16 +2944,16 @@
         <v>2.24</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.25</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="30">
@@ -2993,7 +3007,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,19 +3020,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.39</v>
+        <v>2.38</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.39</v>
       </c>
       <c r="S30" s="6" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.4</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.39</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="31">
@@ -4133,8 +4147,10 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
-        <v>46082</v>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTEXP' not found in values file."</t>
+        </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -4147,19 +4163,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>320859</v>
+        <v>1</v>
       </c>
       <c r="G46" s="24" t="n">
-        <v>314673</v>
+        <v>1</v>
       </c>
       <c r="H46" s="24" t="n">
-        <v>302224</v>
+        <v>1</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>286301</v>
+        <v>1</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>290906</v>
+        <v>1</v>
       </c>
       <c r="K46" s="5" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4220,8 +4236,10 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
-        <v>46082</v>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTEXP' not found in values file."</t>
+        </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4234,19 +4252,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>0.01965850263606983</v>
+        <v>1</v>
       </c>
       <c r="G47" s="38" t="n">
-        <v>0.04119130181587161</v>
+        <v>1</v>
       </c>
       <c r="H47" s="38" t="n">
-        <v>0.05561629194449202</v>
+        <v>1</v>
       </c>
       <c r="I47" s="38" t="n">
-        <v>-0.01582985569221673</v>
+        <v>1</v>
       </c>
       <c r="J47" s="38" t="n">
-        <v>-0.03410286974104926</v>
+        <v>1</v>
       </c>
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4260,7 +4278,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4299,8 +4317,10 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
-        <v>46082</v>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
+        </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4313,19 +4333,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>381165</v>
+        <v>1</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>372449</v>
+        <v>1</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>356901</v>
+        <v>1</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>359201</v>
+        <v>1</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>346932</v>
+        <v>1</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4339,7 +4359,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4372,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.01</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.08</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.04</v>
       </c>
     </row>
     <row r="49">
@@ -4374,8 +4394,10 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
-        <v>46082</v>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
+        </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4388,19 +4410,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.0234018617314049</v>
+        <v>1</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>0.04356390147407829</v>
+        <v>1</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>-0.006403100214086299</v>
+        <v>1</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>0.03536427887885818</v>
+        <v>1</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>0.04409848350332091</v>
+        <v>1</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4414,7 +4436,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,19 +4449,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.19</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.25</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.22</v>
       </c>
     </row>
     <row r="50">
@@ -4493,7 +4515,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4506,16 +4528,16 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.48</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.56</v>
-      </c>
-      <c r="T50" s="6" t="n">
-        <v>4.57</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.57</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-06-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -901,10 +901,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C3" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -917,19 +915,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>1</v>
+        <v>24152.656</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>1</v>
+        <v>24055.749</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>1</v>
+        <v>24026.834</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>1</v>
+        <v>23770.976</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>1</v>
+        <v>23548.21</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -978,10 +976,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C4" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -994,19 +990,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>1</v>
+        <v>0.004028434117765434</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>1</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>1</v>
+        <v>0.0107634621312982</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>1</v>
+        <v>0.009459997171759493</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>1</v>
+        <v>-0.001625164044818495</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1223,7 +1219,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.8233</v>
+        <v>3.0164</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1367,8 +1363,10 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="48" t="n">
-        <v>46023</v>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -1381,19 +1379,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16723.347</v>
+        <v>1</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>16665.219</v>
+        <v>1</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>16585.878</v>
+        <v>1</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>16445.685</v>
+        <v>1</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>16345.793</v>
+        <v>1</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1406,10 +1404,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1422,19 +1418,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="10">
@@ -1444,8 +1440,10 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="48" t="n">
-        <v>46023</v>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
+        </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -1458,19 +1456,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.003487982966200454</v>
+        <v>1</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>0.004783647872002916</v>
+        <v>1</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>0.008524606910566446</v>
+        <v>1</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>0.006111174905983452</v>
+        <v>1</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>0.001525835907232986</v>
+        <v>1</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1870,8 +1868,10 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
-        <v>46113</v>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
+        </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1884,19 +1884,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>34.3</v>
+        <v>1</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2237,10 +2237,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N20" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2253,19 +2251,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1</v>
+        <v>0.00376460730477457</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>1</v>
+        <v>0.001957950538511444</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>1</v>
+        <v>0.002160502174024082</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>1</v>
+        <v>0.002950448142634121</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>1</v>
+        <v>0.002329002576704653</v>
       </c>
     </row>
     <row r="21">
@@ -2314,10 +2312,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N21" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2330,19 +2326,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1</v>
+        <v>0.02743309430968526</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>1</v>
+        <v>0.0260216770548682</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>1</v>
+        <v>0.02472462476764023</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>1</v>
+        <v>0.02512028782828883</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>1</v>
+        <v>0.02646484707309002</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -368,9 +368,6 @@
     </xf>
     <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1109,10 +1106,10 @@
       <c r="R5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="S5" s="49" t="n">
+      <c r="S5" s="24" t="n">
         <v>66000</v>
       </c>
-      <c r="T5" s="24" t="n">
+      <c r="T5" s="49" t="n">
         <v>11000</v>
       </c>
       <c r="U5" s="26" t="n">
@@ -1284,8 +1281,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
-        <v>46082</v>
+      <c r="C8" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -1298,19 +1295,19 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>1.82</v>
+        <v>0.44</v>
       </c>
       <c r="G8" s="24" t="n">
         <v>0.46</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>0.16</v>
+        <v>0.34</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1404,8 +1401,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46113</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1418,19 +1417,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>59.1</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>59.3</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>59.4</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1481,8 +1480,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
-        <v>46082</v>
+      <c r="N10" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1495,19 +1494,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4.1</v>
+        <v>4.6</v>
       </c>
       <c r="R10" s="6" t="n">
         <v>4.2</v>
       </c>
       <c r="S10" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="T10" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="T10" s="6" t="n">
+      <c r="U10" s="21" t="n">
         <v>4</v>
-      </c>
-      <c r="U10" s="21" t="n">
-        <v>4.1</v>
       </c>
     </row>
     <row r="11">
@@ -1560,8 +1559,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
-        <v>46082</v>
+      <c r="N11" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1574,19 +1573,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="R11" s="6" t="n">
+      <c r="S11" s="6" t="n">
         <v>3.1</v>
       </c>
-      <c r="S11" s="6" t="n">
+      <c r="T11" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="T11" s="6" t="n">
+      <c r="U11" s="21" t="n">
         <v>3.3</v>
-      </c>
-      <c r="U11" s="21" t="n">
-        <v>3.2</v>
       </c>
     </row>
     <row r="12">
@@ -1635,8 +1634,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
-        <v>46082</v>
+      <c r="N12" s="50" t="n">
+        <v>46113</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
@@ -1649,19 +1648,19 @@
         </is>
       </c>
       <c r="Q12" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="R12" s="6" t="n">
         <v>3.4</v>
-      </c>
-      <c r="R12" s="6" t="n">
-        <v>3.2</v>
       </c>
       <c r="S12" s="6" t="n">
         <v>3.2</v>
       </c>
       <c r="T12" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="U12" s="21" t="n">
         <v>3.3</v>
-      </c>
-      <c r="U12" s="21" t="n">
-        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -1714,8 +1713,10 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="50" t="n">
-        <v>46160</v>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1728,19 +1729,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>215000</v>
+        <v>1</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>210000</v>
+        <v>1</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>212000</v>
+        <v>1</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>199000</v>
+        <v>1</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>190000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1868,10 +1869,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'AWHAETP' not found in values file."</t>
-        </is>
+      <c r="N15" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1884,19 +1883,19 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="R15" s="24" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
       <c r="S15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
-        <v>1</v>
+        <v>34.3</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>1</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="16">
@@ -1982,7 +1981,7 @@
       <c r="I17" s="25" t="n">
         <v>-0.0002912686109073359</v>
       </c>
-      <c r="J17" s="51" t="n">
+      <c r="J17" s="25" t="n">
         <v>-1.361066422789214e-06</v>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -2069,7 +2068,7 @@
       <c r="I18" s="25" t="n">
         <v>0.03267862666254253</v>
       </c>
-      <c r="J18" s="51" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.02433131408893505</v>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -2237,8 +2236,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46113</v>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2251,19 +2252,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>0.00376460730477457</v>
+        <v>1</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.001957950538511444</v>
+        <v>1</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>0.002160502174024082</v>
+        <v>1</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>0.002950448142634121</v>
+        <v>1</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>0.002329002576704653</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2312,8 +2313,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46113</v>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2326,19 +2329,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.02743309430968526</v>
+        <v>1</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.0260216770548682</v>
+        <v>1</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>0.02472462476764023</v>
+        <v>1</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>0.02512028782828883</v>
+        <v>1</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>0.02646484707309002</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2924,7 +2927,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2937,19 +2940,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.24</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.25</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="30">
@@ -3003,7 +3006,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3016,16 +3019,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.38</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.39</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.39</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.4</v>
@@ -3531,7 +3534,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="50" t="n">
+      <c r="N37" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -3606,7 +3609,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="50" t="n">
+      <c r="N38" s="48" t="n">
         <v>46082</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
@@ -3681,8 +3684,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
-        <v>46113</v>
+      <c r="N39" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
         <is>
@@ -3695,19 +3698,19 @@
         </is>
       </c>
       <c r="Q39" s="6" t="n">
+        <v>118.7792</v>
+      </c>
+      <c r="R39" s="6" t="n">
         <v>119.0363</v>
       </c>
-      <c r="R39" s="6" t="n">
+      <c r="S39" s="6" t="n">
         <v>119.9199</v>
       </c>
-      <c r="S39" s="6" t="n">
+      <c r="T39" s="6" t="n">
         <v>117.906</v>
       </c>
-      <c r="T39" s="6" t="n">
+      <c r="U39" s="21" t="n">
         <v>119.2298</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>120.1883</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3756,8 +3759,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
-        <v>46113</v>
+      <c r="N40" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
@@ -3770,19 +3773,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.0291232297604588</v>
+      </c>
+      <c r="R40" s="38" t="n">
         <v>-0.04111399852747133</v>
       </c>
-      <c r="R40" s="38" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.05008673748247425</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.07796471263522881</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.07456792269916472</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.05790675033979801</v>
       </c>
     </row>
     <row r="41">
@@ -4274,7 +4277,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4355,7 +4358,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4368,19 +4371,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.01</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.08</v>
       </c>
     </row>
     <row r="49">
@@ -4432,7 +4435,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4445,19 +4448,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.19</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.25</v>
       </c>
     </row>
     <row r="50">
@@ -4511,7 +4514,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4527,16 +4530,16 @@
         <v>4.45</v>
       </c>
       <c r="R50" s="6" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="S50" s="6" t="n">
         <v>4.48</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.56</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.57</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4636,8 +4639,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="52" t="n">
-        <v>46170</v>
+      <c r="N52" s="51" t="n">
+        <v>46171</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4653,16 +4656,16 @@
         <v>6.02</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.13</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.16</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -77,14 +77,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -363,13 +363,13 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -898,8 +898,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
-        <v>46023</v>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -912,19 +914,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24152.656</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>24055.749</v>
+        <v>1</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>24026.834</v>
+        <v>1</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>23770.976</v>
+        <v>1</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>23548.21</v>
+        <v>1</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -973,8 +975,10 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
-        <v>46023</v>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -987,19 +991,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.004028434117765434</v>
+        <v>1</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>0.001203446113624551</v>
+        <v>1</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>0.0107634621312982</v>
+        <v>1</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>0.009459997171759493</v>
+        <v>1</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>-0.001625164044818495</v>
+        <v>1</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1087,8 +1091,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
-        <v>46113</v>
+      <c r="N5" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
@@ -1101,19 +1105,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>109000</v>
+        <v>122000</v>
       </c>
       <c r="R5" s="24" t="n">
+        <v>105000</v>
+      </c>
+      <c r="S5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="S5" s="24" t="n">
+      <c r="T5" s="50" t="n">
         <v>66000</v>
       </c>
-      <c r="T5" s="49" t="n">
+      <c r="U5" s="26" t="n">
         <v>11000</v>
-      </c>
-      <c r="U5" s="26" t="n">
-        <v>37000</v>
       </c>
     </row>
     <row r="6">
@@ -1241,8 +1245,10 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46113</v>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1255,19 +1261,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>8.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1281,7 +1287,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="50" t="n">
+      <c r="C8" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1401,10 +1407,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1417,19 +1421,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>59.3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>59.4</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="10">
@@ -1480,8 +1484,10 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="50" t="n">
-        <v>46113</v>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
+        </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1494,19 +1500,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1520,7 +1526,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="50" t="n">
+      <c r="C11" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1559,8 +1565,10 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="50" t="n">
-        <v>46113</v>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
+        </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1573,19 +1581,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1595,7 +1603,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="50" t="n">
+      <c r="C12" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1634,7 +1642,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="50" t="n">
+      <c r="N12" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1674,7 +1682,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="50" t="n">
+      <c r="C13" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1751,7 +1759,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="50" t="n">
+      <c r="C14" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1790,8 +1798,10 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="50" t="n">
-        <v>46153</v>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1804,19 +1814,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1786000</v>
+        <v>1</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1771000</v>
+        <v>1</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1776000</v>
+        <v>1</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1758000</v>
+        <v>1</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1776000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1830,7 +1840,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="50" t="n">
+      <c r="C15" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1905,7 +1915,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="50" t="n">
+      <c r="C16" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2124,7 +2134,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="50" t="n">
+      <c r="C19" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2197,7 +2207,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="50" t="n">
+      <c r="C20" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2278,7 +2288,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="50" t="n">
+      <c r="C21" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2355,7 +2365,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="50" t="n">
+      <c r="C22" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2394,8 +2404,10 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46113</v>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
+        </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2408,19 +2420,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.01375897183427033</v>
+        <v>1</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.006992824527071173</v>
+        <v>1</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.005674549808114993</v>
+        <v>1</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.005560979471212146</v>
+        <v>1</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.00356164020813754</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2430,7 +2442,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="50" t="n">
+      <c r="C23" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2464,8 +2476,10 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46113</v>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
+        </is>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2478,19 +2492,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.05987606244285672</v>
+        <v>1</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.04266657661004361</v>
+        <v>1</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.03418267187468382</v>
+        <v>1</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.03014022638959289</v>
+        <v>1</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.0308734325272694</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -2543,7 +2557,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="50" t="n">
+      <c r="N24" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2618,7 +2632,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="50" t="n">
+      <c r="N25" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2658,8 +2672,10 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n">
-        <v>46023</v>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
+        </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2672,19 +2688,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.0243486718158854</v>
+        <v>1</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>0.005923787970366412</v>
+        <v>1</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>0.007794617579222285</v>
+        <v>1</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>0.01778138610314484</v>
+        <v>1</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>0.02303791460563676</v>
+        <v>1</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2697,7 +2713,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="50" t="n">
+      <c r="N26" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2772,7 +2788,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="50" t="n">
+      <c r="N27" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2812,7 +2828,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="50" t="n">
+      <c r="C28" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2826,10 +2842,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.07946631387134628</v>
+        <v>0.08018159976285943</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>0.01345526874171887</v>
+        <v>0.01344578206575542</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>-0.01169466364559735</v>
@@ -2887,7 +2903,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="50" t="n">
+      <c r="C29" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2901,10 +2917,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.171822551307629</v>
+        <v>0.1725880587611651</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.0135129579558212</v>
+        <v>0.01350347073984473</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.07567733047604469</v>
@@ -2926,8 +2942,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="50" t="n">
-        <v>46174</v>
+      <c r="N29" s="49" t="n">
+        <v>46175</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2943,16 +2959,16 @@
         <v>2.26</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.24</v>
       </c>
       <c r="T29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.25</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -2966,7 +2982,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="50" t="n">
+      <c r="C30" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2980,10 +2996,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.08083364547795258</v>
+        <v>0.08141853927844678</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>-0.002695717141530163</v>
+        <v>-0.002709178900039744</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>-0.01222345960141613</v>
@@ -3005,8 +3021,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="50" t="n">
-        <v>46174</v>
+      <c r="N30" s="49" t="n">
+        <v>46175</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3019,19 +3035,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.38</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.39</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.39</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="31">
@@ -3041,7 +3057,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="50" t="n">
+      <c r="C31" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3055,10 +3071,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.1492280257336716</v>
+        <v>0.1498344103537483</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>-0.0181892276038923</v>
+        <v>-0.0182024802287403</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>0.07288240242929306</v>
@@ -3534,8 +3550,10 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
-        <v>46082</v>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3548,19 +3566,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.007161347041441779</v>
+        <v>1</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>0.003402954536404934</v>
+        <v>1</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>-0.001489442391916063</v>
+        <v>1</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.002589859586293541</v>
+        <v>1</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.001285648567050157</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -3609,8 +3627,10 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
-        <v>46082</v>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3623,19 +3643,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.006657391474145452</v>
+        <v>1</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.007541366795841786</v>
+        <v>1</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.008681655137469846</v>
+        <v>1</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01129232301425539</v>
+        <v>1</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01271856657398832</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3684,7 +3704,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="50" t="n">
+      <c r="N39" s="49" t="n">
         <v>46143</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3724,7 +3744,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="50" t="n">
+      <c r="C40" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3759,7 +3779,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="50" t="n">
+      <c r="N40" s="49" t="n">
         <v>46143</v>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -3795,7 +3815,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="50" t="n">
+      <c r="C41" s="49" t="n">
         <v>46113</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -4276,8 +4296,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="50" t="n">
-        <v>46171</v>
+      <c r="N47" s="49" t="n">
+        <v>46174</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4357,8 +4377,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="50" t="n">
-        <v>46171</v>
+      <c r="N48" s="49" t="n">
+        <v>46174</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4371,19 +4391,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.01</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="49">
@@ -4434,8 +4454,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="50" t="n">
-        <v>46171</v>
+      <c r="N49" s="49" t="n">
+        <v>46174</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4448,19 +4468,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.19</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4474,8 +4494,10 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
-        <v>46082</v>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
+        </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4488,19 +4510,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>28406</v>
+        <v>1</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>26846</v>
+        <v>1</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>27460</v>
+        <v>1</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>26347</v>
+        <v>1</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>27608</v>
+        <v>1</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4513,8 +4535,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="50" t="n">
-        <v>46171</v>
+      <c r="N50" s="49" t="n">
+        <v>46174</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4527,19 +4549,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
-        <v>4.45</v>
+        <v>4.47</v>
       </c>
       <c r="R50" s="6" t="n">
         <v>4.45</v>
       </c>
       <c r="S50" s="6" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="T50" s="6" t="n">
         <v>4.48</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.5</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.56</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4549,8 +4571,10 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
-        <v>46082</v>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
+        </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4563,19 +4587,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.05810921552559045</v>
+        <v>1</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>-0.02235979606700655</v>
+        <v>1</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>0.04224389873609891</v>
+        <v>1</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>-0.04567516661837145</v>
+        <v>1</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>0.004804192750036407</v>
+        <v>1</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4588,7 +4612,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="50" t="n">
+      <c r="N51" s="49" t="n">
         <v>46167</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4640,7 +4664,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4653,19 +4677,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.02</v>
+        <v>6.01</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.02</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.05</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.06</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.13</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -898,10 +898,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C3" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -914,19 +912,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>1</v>
+        <v>24152.656</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>1</v>
+        <v>24055.749</v>
       </c>
       <c r="H3" s="24" t="n">
-        <v>1</v>
+        <v>24026.834</v>
       </c>
       <c r="I3" s="24" t="n">
-        <v>1</v>
+        <v>23770.976</v>
       </c>
       <c r="J3" s="24" t="n">
-        <v>1</v>
+        <v>23548.21</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -975,10 +973,8 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'GDPC1' not found in values file."</t>
-        </is>
+      <c r="C4" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
@@ -991,19 +987,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>1</v>
+        <v>0.004028434117765434</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>1</v>
+        <v>0.001203446113624551</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>1</v>
+        <v>0.0107634621312982</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>1</v>
+        <v>0.009459997171759493</v>
       </c>
       <c r="J4" s="25" t="n">
-        <v>1</v>
+        <v>-0.001625164044818495</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1245,10 +1241,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
-        </is>
+      <c r="N7" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1261,19 +1255,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>8.1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>1</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1366,10 +1360,8 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
-        </is>
+      <c r="C9" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -1382,19 +1374,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>1</v>
+        <v>16723.347</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1</v>
+        <v>16665.219</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>1</v>
+        <v>16585.878</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>1</v>
+        <v>16445.685</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>1</v>
+        <v>16345.793</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1443,10 +1435,8 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PCECC96' not found in values file."</t>
-        </is>
+      <c r="C10" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -1459,19 +1449,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>1</v>
+        <v>0.003487982966200454</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>1</v>
+        <v>0.004783647872002916</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>1</v>
+        <v>0.008524606910566446</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>1</v>
+        <v>0.006111174905983452</v>
       </c>
       <c r="J10" s="25" t="n">
-        <v>1</v>
+        <v>0.001525835907232986</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1484,10 +1474,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
-        </is>
+      <c r="N10" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
@@ -1500,19 +1488,19 @@
         </is>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>1</v>
+        <v>4.6</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="S10" s="6" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1526,7 +1514,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n">
+      <c r="C11" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1565,10 +1553,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
-        </is>
+      <c r="N11" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
@@ -1581,19 +1567,19 @@
         </is>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="12">
@@ -1603,7 +1589,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="49" t="n">
+      <c r="C12" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1682,7 +1668,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="49" t="n">
+      <c r="C13" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1721,10 +1707,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ICSA' not found in values file."</t>
-        </is>
+      <c r="N13" s="49" t="n">
+        <v>46167</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1737,19 +1721,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>1</v>
+        <v>225000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>1</v>
+        <v>212000</v>
       </c>
       <c r="S13" s="24" t="n">
-        <v>1</v>
+        <v>210000</v>
       </c>
       <c r="T13" s="24" t="n">
-        <v>1</v>
+        <v>212000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>1</v>
+        <v>199000</v>
       </c>
     </row>
     <row r="14">
@@ -1759,7 +1743,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1798,10 +1782,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CCSA' not found in values file."</t>
-        </is>
+      <c r="N14" s="49" t="n">
+        <v>46160</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1814,19 +1796,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1</v>
+        <v>1777000</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>1</v>
+        <v>1785000</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>1</v>
+        <v>1771000</v>
       </c>
       <c r="T14" s="24" t="n">
-        <v>1</v>
+        <v>1776000</v>
       </c>
       <c r="U14" s="26" t="n">
-        <v>1</v>
+        <v>1758000</v>
       </c>
     </row>
     <row r="15">
@@ -1840,7 +1822,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1915,7 +1897,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2092,10 +2074,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N18" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2108,19 +2088,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>1</v>
+        <v>0.006400377846336402</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>1</v>
+        <v>0.008651438343614481</v>
       </c>
       <c r="S18" s="38" t="n">
-        <v>1</v>
+        <v>0.00267003074209704</v>
       </c>
       <c r="T18" s="38" t="n">
-        <v>1</v>
+        <v>0.00170842649932057</v>
       </c>
       <c r="U18" s="23" t="n">
-        <v>1</v>
+        <v>0.00297788428704604</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2134,7 +2114,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="49" t="n">
+      <c r="C19" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2169,10 +2149,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPIAUCSL' not found in values file."</t>
-        </is>
+      <c r="N19" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2185,19 +2163,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>1</v>
+        <v>0.03779245836741563</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>1</v>
+        <v>0.03285957752865201</v>
       </c>
       <c r="S19" s="38" t="n">
-        <v>1</v>
+        <v>0.0243400411037322</v>
       </c>
       <c r="T19" s="38" t="n">
-        <v>1</v>
+        <v>0.02391201432150015</v>
       </c>
       <c r="U19" s="23" t="n">
-        <v>1</v>
+        <v>0.02653304114557758</v>
       </c>
     </row>
     <row r="20">
@@ -2207,7 +2185,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2246,10 +2224,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N20" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2262,19 +2238,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1</v>
+        <v>0.00376460730477457</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>1</v>
+        <v>0.001957950538511444</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>1</v>
+        <v>0.002160502174024082</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>1</v>
+        <v>0.002950448142634121</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>1</v>
+        <v>0.002329002576704653</v>
       </c>
     </row>
     <row r="21">
@@ -2288,7 +2264,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n">
+      <c r="C21" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2323,10 +2299,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N21" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2339,19 +2313,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1</v>
+        <v>0.02743309430968526</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>1</v>
+        <v>0.0260216770548682</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>1</v>
+        <v>0.02472462476764023</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>1</v>
+        <v>0.02512028782828883</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>1</v>
+        <v>0.02646484707309002</v>
       </c>
     </row>
     <row r="22">
@@ -2365,7 +2339,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2404,10 +2378,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
-        </is>
+      <c r="N22" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2420,19 +2392,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>1</v>
+        <v>0.01375897183427033</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>1</v>
+        <v>0.006992824527071173</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>1</v>
+        <v>0.005674549808114993</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>1</v>
+        <v>0.005560979471212146</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>1</v>
+        <v>0.00356164020813754</v>
       </c>
     </row>
     <row r="23">
@@ -2442,7 +2414,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2476,10 +2448,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PPIFIS' not found in values file."</t>
-        </is>
+      <c r="N23" s="48" t="n">
+        <v>46113</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2492,19 +2462,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>1</v>
+        <v>0.05987606244285672</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>1</v>
+        <v>0.04266657661004361</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>1</v>
+        <v>0.03418267187468382</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>1</v>
+        <v>0.03014022638959289</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>1</v>
+        <v>0.0308734325272694</v>
       </c>
     </row>
     <row r="24">
@@ -2557,7 +2527,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="49" t="n">
+      <c r="N24" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2632,7 +2602,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="49" t="n">
+      <c r="N25" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O25" s="6" t="inlineStr">
@@ -2672,10 +2642,8 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PNFIC1' not found in values file."</t>
-        </is>
+      <c r="C26" s="48" t="n">
+        <v>46023</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -2688,19 +2656,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>1</v>
+        <v>0.0243486718158854</v>
       </c>
       <c r="G26" s="38" t="n">
-        <v>1</v>
+        <v>0.005923787970366412</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>1</v>
+        <v>0.007794617579222285</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>1</v>
+        <v>0.01778138610314484</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>1</v>
+        <v>0.02303791460563676</v>
       </c>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2713,7 +2681,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="49" t="n">
+      <c r="N26" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2788,7 +2756,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="49" t="n">
+      <c r="N27" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2943,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2956,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.26</v>
+        <v>2.23</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.26</v>
       </c>
       <c r="S29" s="6" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.24</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.25</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -3022,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3035,16 +3003,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.38</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.39</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.39</v>
@@ -3375,7 +3343,7 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G35" s="41" t="n">
         <v>1.6</v>
@@ -3550,10 +3518,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
-        </is>
+      <c r="N37" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
@@ -3566,19 +3532,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>1</v>
+        <v>0.007161347041441779</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>1</v>
+        <v>0.003402954536404934</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>1</v>
+        <v>-0.001489442391916063</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>1</v>
+        <v>-0.002589859586293541</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>1</v>
+        <v>-0.001285648567050157</v>
       </c>
     </row>
     <row r="38">
@@ -3627,10 +3593,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CSUSHPINSA' not found in values file."</t>
-        </is>
+      <c r="N38" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
@@ -3643,19 +3607,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>1</v>
+        <v>0.006657391474145452</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>1</v>
+        <v>0.007541366795841786</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>1</v>
+        <v>0.008681655137469846</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>1</v>
+        <v>0.01129232301425539</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>1</v>
+        <v>0.01271856657398832</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3744,7 +3708,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n">
+      <c r="C40" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3815,7 +3779,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n">
+      <c r="C41" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -4166,10 +4130,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTEXP' not found in values file."</t>
-        </is>
+      <c r="C46" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -4182,19 +4144,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>1</v>
+        <v>320859</v>
       </c>
       <c r="G46" s="24" t="n">
-        <v>1</v>
+        <v>314673</v>
       </c>
       <c r="H46" s="24" t="n">
-        <v>1</v>
+        <v>302224</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>1</v>
+        <v>286301</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>1</v>
+        <v>290906</v>
       </c>
       <c r="K46" s="5" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4255,10 +4217,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTEXP' not found in values file."</t>
-        </is>
+      <c r="C47" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4271,19 +4231,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>1</v>
+        <v>0.01965850263606983</v>
       </c>
       <c r="G47" s="38" t="n">
-        <v>1</v>
+        <v>0.04119130181587161</v>
       </c>
       <c r="H47" s="38" t="n">
-        <v>1</v>
+        <v>0.05561629194449202</v>
       </c>
       <c r="I47" s="38" t="n">
-        <v>1</v>
+        <v>-0.01582985569221673</v>
       </c>
       <c r="J47" s="38" t="n">
-        <v>1</v>
+        <v>-0.03410286974104926</v>
       </c>
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4297,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,10 +4296,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
-        </is>
+      <c r="C48" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4352,19 +4310,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>1</v>
+        <v>381165</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>1</v>
+        <v>372449</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>1</v>
+        <v>356901</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>1</v>
+        <v>359201</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>1</v>
+        <v>346932</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4378,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4394,16 +4352,16 @@
         <v>4.05</v>
       </c>
       <c r="R48" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="S48" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>3.99</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.01</v>
       </c>
     </row>
     <row r="49">
@@ -4413,10 +4371,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPTIMP' not found in values file."</t>
-        </is>
+      <c r="C49" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4429,19 +4385,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>1</v>
+        <v>0.0234018617314049</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>1</v>
+        <v>0.04356390147407829</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>1</v>
+        <v>-0.006403100214086299</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>1</v>
+        <v>0.03536427887885818</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>1</v>
+        <v>0.04409848350332091</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4455,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4468,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.19</v>
       </c>
     </row>
     <row r="50">
@@ -4494,10 +4450,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
-        </is>
+      <c r="C50" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4510,19 +4464,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>1</v>
+        <v>28406</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>1</v>
+        <v>26846</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>1</v>
+        <v>27460</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>1</v>
+        <v>26347</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>1</v>
+        <v>27608</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4536,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4549,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.47</v>
-      </c>
-      <c r="R50" s="6" t="n">
-        <v>4.45</v>
       </c>
       <c r="S50" s="6" t="n">
         <v>4.45</v>
       </c>
       <c r="T50" s="6" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.48</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.5</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4571,10 +4525,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'BOPSTB' not found in values file."</t>
-        </is>
+      <c r="C51" s="48" t="n">
+        <v>46082</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4587,19 +4539,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>1</v>
+        <v>0.05810921552559045</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>1</v>
+        <v>-0.02235979606700655</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>1</v>
+        <v>0.04224389873609891</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>1</v>
+        <v>-0.04567516661837145</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>1</v>
+        <v>0.004804192750036407</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4613,7 +4565,7 @@
         </is>
       </c>
       <c r="N51" s="49" t="n">
-        <v>46167</v>
+        <v>46174</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4626,19 +4578,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.53</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.51</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.36</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.37</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.3</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4664,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4677,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.01</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.02</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.02</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.05</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.06</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-05
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -937,8 +937,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
-        <v>46113</v>
+      <c r="N3" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
@@ -951,19 +951,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>115</v>
+        <v>172</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>214</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>-156</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>160</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>-17</v>
       </c>
     </row>
     <row r="4">
@@ -1008,8 +1008,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
-        <v>46113</v>
+      <c r="N4" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
@@ -1022,19 +1022,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.001583746095845033</v>
+        <v>0.003173541621976303</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.001540627742664655</v>
+        <v>0.002170552418209925</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.001723735138309224</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.0007959067652075042</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.002047160512548336</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.0007327117916066601</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1162,8 +1162,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
-        <v>46113</v>
+      <c r="N6" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
@@ -1182,13 +1182,13 @@
         <v>4.3</v>
       </c>
       <c r="S6" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="T6" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="U6" s="21" t="n">
         <v>4.3</v>
-      </c>
-      <c r="U6" s="21" t="n">
-        <v>4.4</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1241,8 +1241,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46113</v>
+      <c r="N7" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
@@ -1255,19 +1255,19 @@
         </is>
       </c>
       <c r="Q7" s="6" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="R7" s="6" t="n">
+      <c r="S7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="S7" s="6" t="n">
+      <c r="T7" s="6" t="n">
         <v>7.9</v>
       </c>
-      <c r="T7" s="6" t="n">
+      <c r="U7" s="21" t="n">
         <v>8.1</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>8.4</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1320,8 +1320,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
-        <v>46113</v>
+      <c r="N8" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
@@ -1337,16 +1337,16 @@
         <v>61.8</v>
       </c>
       <c r="R8" s="6" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="S8" s="6" t="n">
         <v>61.9</v>
       </c>
-      <c r="S8" s="6" t="n">
+      <c r="T8" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="T8" s="6" t="n">
+      <c r="U8" s="21" t="n">
         <v>62.1</v>
-      </c>
-      <c r="U8" s="21" t="n">
-        <v>62.4</v>
       </c>
     </row>
     <row r="9">
@@ -1399,8 +1399,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46113</v>
+      <c r="N9" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
@@ -1413,19 +1413,19 @@
         </is>
       </c>
       <c r="Q9" s="6" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="R9" s="6" t="n">
         <v>59.1</v>
       </c>
-      <c r="R9" s="6" t="n">
+      <c r="S9" s="6" t="n">
         <v>59.2</v>
       </c>
-      <c r="S9" s="6" t="n">
+      <c r="T9" s="6" t="n">
         <v>59.3</v>
       </c>
-      <c r="T9" s="6" t="n">
+      <c r="U9" s="21" t="n">
         <v>59.4</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>59.7</v>
       </c>
     </row>
     <row r="10">
@@ -1861,8 +1861,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
-        <v>46113</v>
+      <c r="N15" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
         <v>34.3</v>
       </c>
       <c r="R15" s="24" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="S15" s="24" t="n">
         <v>34.2</v>
-      </c>
-      <c r="S15" s="24" t="n">
-        <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
         <v>34.3</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="16">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,16 +2924,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.23</v>
-      </c>
-      <c r="R29" s="6" t="n">
-        <v>2.26</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.26</v>
       </c>
       <c r="T29" s="6" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.24</v>
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.38</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.39</v>
       </c>
     </row>
     <row r="31">
@@ -3214,8 +3214,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
-        <v>46113</v>
+      <c r="N33" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
@@ -3228,19 +3228,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
+        <v>0.00320769847634339</v>
+      </c>
+      <c r="R33" s="38" t="n">
         <v>0.001606425702811221</v>
       </c>
-      <c r="R33" s="38" t="n">
+      <c r="S33" s="38" t="n">
         <v>0.002146498524282281</v>
       </c>
-      <c r="S33" s="38" t="n">
+      <c r="T33" s="38" t="n">
         <v>0.003230148048452453</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.003511615343057661</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.000540540540540535</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>4.05</v>
+        <v>4.08</v>
       </c>
       <c r="R48" s="6" t="n">
         <v>4.05</v>
       </c>
       <c r="S48" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="T48" s="6" t="n">
         <v>3.98</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>3.99</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.13</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.15</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.17</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.46</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.47</v>
-      </c>
-      <c r="S50" s="6" t="n">
-        <v>4.45</v>
       </c>
       <c r="T50" s="6" t="n">
         <v>4.45</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.48</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.01</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.02</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.02</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.05</v>
+        <v>6.02</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-06
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2339,8 +2339,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
-        <v>46113</v>
+      <c r="C22" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -2353,19 +2353,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.318</v>
+        <v>16.485</v>
       </c>
       <c r="G22" s="24" t="n">
+        <v>16.395</v>
+      </c>
+      <c r="H22" s="24" t="n">
         <v>16.537</v>
       </c>
-      <c r="H22" s="24" t="n">
+      <c r="I22" s="24" t="n">
         <v>15.881</v>
       </c>
-      <c r="I22" s="24" t="n">
+      <c r="J22" s="24" t="n">
         <v>14.987</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>16.4</v>
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2414,8 +2414,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
-        <v>46113</v>
+      <c r="C23" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -2428,19 +2428,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.07194449183870769</v>
+        <v>0.02755095680359036</v>
       </c>
       <c r="G23" s="25" t="n">
+        <v>-0.06756526190069947</v>
+      </c>
+      <c r="H23" s="25" t="n">
         <v>-0.09880108991825626</v>
       </c>
-      <c r="H23" s="25" t="n">
+      <c r="I23" s="25" t="n">
         <v>-0.0327669163773677</v>
       </c>
-      <c r="I23" s="25" t="n">
+      <c r="J23" s="25" t="n">
         <v>-0.0603761755485893</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>-0.05207791457141205</v>
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2488,8 +2488,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
-        <v>46082</v>
+      <c r="C24" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2502,19 +2502,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.007561302505515899</v>
+        <v>0.008703141071390919</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.0002854040755513321</v>
+        <v>0.007795687606403368</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.001701852596202258</v>
+        <v>0.000649622056177801</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.006198562656960505</v>
+        <v>0.001151758694675653</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>-0.0007477594964454548</v>
+        <v>0.005868657238478958</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2567,8 +2567,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="48" t="n">
-        <v>46082</v>
+      <c r="C25" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -2581,19 +2581,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.003911989748358602</v>
+        <v>0.00239671579372791</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.0022395833833464</v>
+        <v>0.003140798606426021</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.001310703086948806</v>
+        <v>0.001559499677996179</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.001967095543671693</v>
+        <v>0.0006476910419241921</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.001164097695629751</v>
+        <v>0.001971303273869296</v>
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2927,16 +2927,16 @@
         <v>2.24</v>
       </c>
       <c r="R29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="S29" s="6" t="n">
         <v>2.23</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <v>2.26</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.26</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3006,16 +3006,16 @@
         <v>2.36</v>
       </c>
       <c r="R30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="S30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.4</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.38</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.08</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>4.05</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>4.05</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>3.98</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>3.99</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.15</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,16 +4503,16 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.49</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.46</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.47</v>
-      </c>
-      <c r="T50" s="6" t="n">
-        <v>4.45</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.45</v>
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.03</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.01</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.02</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.02</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-06-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7964064.3</v>
+        <v>7954866</v>
       </c>
       <c r="G5" s="24" t="n">
         <v>7855631.5</v>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.01380319328878898</v>
+        <v>0.01263227533012468</v>
       </c>
       <c r="G6" s="25" t="n">
         <v>0.0104347069321491</v>
@@ -1281,7 +1281,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -2488,8 +2488,10 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
-        <v>46113</v>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
+        </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2502,19 +2504,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.008703141071390919</v>
+        <v>1</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.007795687606403368</v>
+        <v>1</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.000649622056177801</v>
+        <v>1</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.001151758694675653</v>
+        <v>1</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.005868657238478958</v>
+        <v>1</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -3668,7 +3670,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="49" t="n">
+      <c r="N39" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3743,7 +3745,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="49" t="n">
+      <c r="N40" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O40" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-09
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.0164</v>
+        <v>3.2906</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1474,7 +1474,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="49" t="n">
+      <c r="N10" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1553,7 +1553,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1628,7 +1628,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -2488,10 +2488,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'REVOLSL' not found in values file."</t>
-        </is>
+      <c r="C24" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -2504,19 +2502,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>1</v>
+        <v>0.008703141071390919</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>1</v>
+        <v>0.007795687606403368</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>1</v>
+        <v>0.000649622056177801</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>1</v>
+        <v>0.001151758694675653</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>1</v>
+        <v>0.005868657238478958</v>
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2913,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2926,16 +2924,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="R29" s="6" t="n">
         <v>2.24</v>
       </c>
       <c r="S29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="T29" s="6" t="n">
         <v>2.23</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.26</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.26</v>
@@ -2992,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3005,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="R30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="S30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="T30" s="6" t="n">
         <v>2.38</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.39</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.4</v>
       </c>
     </row>
     <row r="31">
@@ -3861,7 +3859,7 @@
         </is>
       </c>
       <c r="C42" s="48" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -3874,19 +3872,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
+        <v>4170000</v>
+      </c>
+      <c r="G42" s="39" t="n">
+        <v>4040000</v>
+      </c>
+      <c r="H42" s="39" t="n">
+        <v>4010000</v>
+      </c>
+      <c r="I42" s="39" t="n">
+        <v>4130000</v>
+      </c>
+      <c r="J42" s="39" t="n">
         <v>4020000</v>
-      </c>
-      <c r="G42" s="39" t="n">
-        <v>4010000</v>
-      </c>
-      <c r="H42" s="39" t="n">
-        <v>4130000</v>
-      </c>
-      <c r="I42" s="39" t="n">
-        <v>4020000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4270000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3932,7 +3930,7 @@
         </is>
       </c>
       <c r="C43" s="48" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -3945,7 +3943,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>0</v>
+        <v>0.03217821782178218</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4132,8 +4130,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
-        <v>46082</v>
+      <c r="C46" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
@@ -4146,19 +4144,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>320859</v>
+        <v>327101</v>
       </c>
       <c r="G46" s="24" t="n">
-        <v>314673</v>
+        <v>318776</v>
       </c>
       <c r="H46" s="24" t="n">
-        <v>302224</v>
+        <v>311803</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>286301</v>
+        <v>299806</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>290906</v>
+        <v>285282</v>
       </c>
       <c r="K46" s="5" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4219,8 +4217,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
-        <v>46082</v>
+      <c r="C47" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -4233,19 +4231,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>0.01965850263606983</v>
+        <v>0.02611551685195868</v>
       </c>
       <c r="G47" s="38" t="n">
-        <v>0.04119130181587161</v>
+        <v>0.0223634795046872</v>
       </c>
       <c r="H47" s="38" t="n">
-        <v>0.05561629194449202</v>
+        <v>0.04001587693375042</v>
       </c>
       <c r="I47" s="38" t="n">
-        <v>-0.01582985569221673</v>
+        <v>0.05091102838594797</v>
       </c>
       <c r="J47" s="38" t="n">
-        <v>-0.03410286974104926</v>
+        <v>-0.01458356361224711</v>
       </c>
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4259,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4298,8 +4296,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
-        <v>46082</v>
+      <c r="C48" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
@@ -4312,19 +4310,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>381165</v>
+        <v>382982</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>372449</v>
+        <v>375360</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>356901</v>
+        <v>366783</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>359201</v>
+        <v>353991</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>346932</v>
+        <v>361360</v>
       </c>
       <c r="K48" s="5" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4338,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4351,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.08</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>4.05</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>4.05</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>3.98</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="49">
@@ -4373,8 +4371,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
-        <v>46082</v>
+      <c r="C49" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
@@ -4387,19 +4385,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.0234018617314049</v>
+        <v>0.02030583972719513</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>0.04356390147407829</v>
+        <v>0.02338439894978772</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>-0.006403100214086299</v>
+        <v>0.03613651194521905</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>0.03536427887885818</v>
+        <v>-0.02039240646446761</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>0.04409848350332091</v>
+        <v>0.02260507340706108</v>
       </c>
       <c r="K49" s="5" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4413,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4426,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="50">
@@ -4452,8 +4450,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
-        <v>46082</v>
+      <c r="C50" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
@@ -4466,19 +4464,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>28406</v>
+        <v>27806</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>26846</v>
+        <v>29493</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>27460</v>
+        <v>27541</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>26347</v>
+        <v>28077</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>27608</v>
+        <v>26539</v>
       </c>
       <c r="K50" s="5" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4492,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4505,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.47</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.49</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.46</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.47</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.45</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4527,8 +4525,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
-        <v>46082</v>
+      <c r="C51" s="49" t="n">
+        <v>46113</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
@@ -4541,19 +4539,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.05810921552559045</v>
+        <v>-0.05720001356254023</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>-0.02235979606700655</v>
+        <v>0.07087614828800692</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>0.04224389873609891</v>
+        <v>-0.01909035865655162</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>-0.04567516661837145</v>
+        <v>0.05795244734164817</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>0.004804192750036407</v>
+        <v>-0.03858136501956233</v>
       </c>
       <c r="K51" s="5" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4618,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4631,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.03</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.01</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.02</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1087,7 +1087,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -2074,8 +2074,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
-        <v>46113</v>
+      <c r="N18" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
@@ -2088,19 +2088,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>0.004729142286413968</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>0.006400377846336402</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>0.008651438343614481</v>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="T18" s="38" t="n">
         <v>0.00267003074209704</v>
       </c>
-      <c r="T18" s="38" t="n">
+      <c r="U18" s="23" t="n">
         <v>0.00170842649932057</v>
-      </c>
-      <c r="U18" s="23" t="n">
-        <v>0.00297788428704604</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2149,8 +2149,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
-        <v>46113</v>
+      <c r="N19" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
@@ -2163,19 +2163,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.04166614684049648</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.03779245836741563</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.03285957752865201</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.0243400411037322</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v>0.02391201432150015</v>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.02653304114557758</v>
       </c>
     </row>
     <row r="20">
@@ -2224,8 +2224,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46113</v>
+      <c r="N20" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
@@ -2238,19 +2238,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>0.002080954496262777</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.00376460730477457</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>0.001957950538511444</v>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="T20" s="38" t="n">
         <v>0.002160502174024082</v>
       </c>
-      <c r="T20" s="38" t="n">
+      <c r="U20" s="23" t="n">
         <v>0.002950448142634121</v>
-      </c>
-      <c r="U20" s="23" t="n">
-        <v>0.002329002576704653</v>
       </c>
     </row>
     <row r="21">
@@ -2299,8 +2299,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46113</v>
+      <c r="N21" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
@@ -2313,19 +2313,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.02822942063611032</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.02743309430968526</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.0260216770548682</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.02472462476764023</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v>0.02512028782828883</v>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v>0.02646484707309002</v>
       </c>
     </row>
     <row r="22">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.23</v>
-      </c>
-      <c r="R29" s="6" t="n">
-        <v>2.24</v>
       </c>
       <c r="S29" s="6" t="n">
         <v>2.24</v>
       </c>
       <c r="T29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="S30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="T30" s="6" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.38</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.39</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,16 +4349,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.08</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>4.05</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.05</v>
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4427,16 +4427,16 @@
         <v>4.29</v>
       </c>
       <c r="R49" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="S49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.18</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.47</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.49</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.46</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.47</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4632,16 +4632,16 @@
         <v>6.06</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="S52" s="9" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.03</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.01</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="N13" s="49" t="n">
-        <v>46167</v>
+        <v>46174</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1721,19 +1721,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
+        <v>229000</v>
+      </c>
+      <c r="R13" s="24" t="n">
         <v>225000</v>
       </c>
-      <c r="R13" s="24" t="n">
+      <c r="S13" s="24" t="n">
         <v>212000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>210000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>212000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>199000</v>
       </c>
     </row>
     <row r="14">
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="N14" s="49" t="n">
-        <v>46160</v>
+        <v>46167</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1796,19 +1796,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1777000</v>
+        <v>1795000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1771000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1785000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1771000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1776000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1758000</v>
       </c>
     </row>
     <row r="15">
@@ -2378,8 +2378,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46113</v>
+      <c r="N22" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
@@ -2392,19 +2392,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.01375897183427033</v>
+        <v>0.01056335771195616</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.006992824527071173</v>
+        <v>0.01055174826080751</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.005674549808114993</v>
+        <v>0.00747866036701561</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.005560979471212146</v>
+        <v>0.005037122543746886</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.00356164020813754</v>
+        <v>0.00577866905905311</v>
       </c>
     </row>
     <row r="23">
@@ -2448,8 +2448,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46113</v>
+      <c r="N23" s="49" t="n">
+        <v>46143</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
@@ -2462,19 +2462,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.05987606244285672</v>
+        <v>0.06416339864869426</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.04266657661004361</v>
+        <v>0.05659137855135278</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.03418267187468382</v>
+        <v>0.04273411907736988</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.03014022638959289</v>
+        <v>0.03375091916105041</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.0308734325272694</v>
+        <v>0.03036323703328262</v>
       </c>
     </row>
     <row r="24">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.23</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <v>2.24</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>2.24</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.08</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.05</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>4.29</v>
+        <v>4.26</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>4.29</v>
       </c>
       <c r="S49" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="T49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.17</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.56</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.47</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.49</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.46</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="N51" s="49" t="n">
-        <v>46174</v>
+        <v>46181</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4578,19 +4578,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.48</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.53</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.51</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.36</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.37</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.01</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.03</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-12
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -77,14 +77,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -363,13 +363,13 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -937,7 +937,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N3" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -1008,7 +1008,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="49" t="n">
+      <c r="N4" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -1109,7 +1109,7 @@
       <c r="S5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="T5" s="50" t="n">
+      <c r="T5" s="49" t="n">
         <v>66000</v>
       </c>
       <c r="U5" s="26" t="n">
@@ -1162,7 +1162,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="49" t="n">
+      <c r="N6" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1320,7 +1320,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="49" t="n">
+      <c r="N8" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -1399,7 +1399,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="49" t="n">
+      <c r="N9" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1707,7 +1707,7 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="49" t="n">
+      <c r="N13" s="50" t="n">
         <v>46174</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1782,7 +1782,7 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="49" t="n">
+      <c r="N14" s="50" t="n">
         <v>46167</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -1861,7 +1861,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="49" t="n">
+      <c r="N15" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -2074,7 +2074,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="49" t="n">
+      <c r="N18" s="50" t="n">
         <v>46143</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2149,7 +2149,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="50" t="n">
         <v>46143</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2224,7 +2224,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="49" t="n">
+      <c r="N20" s="50" t="n">
         <v>46143</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2299,7 +2299,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="49" t="n">
+      <c r="N21" s="50" t="n">
         <v>46143</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2339,7 +2339,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n">
+      <c r="C22" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2378,7 +2378,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="49" t="n">
+      <c r="N22" s="50" t="n">
         <v>46143</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2414,7 +2414,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n">
+      <c r="C23" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2448,7 +2448,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="49" t="n">
+      <c r="N23" s="50" t="n">
         <v>46143</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2488,7 +2488,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n">
+      <c r="C24" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2567,7 +2567,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n">
+      <c r="C25" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2910,8 +2910,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="49" t="n">
-        <v>46183</v>
+      <c r="N29" s="50" t="n">
+        <v>46184</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,16 +2924,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.23</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>2.24</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.24</v>
@@ -2989,8 +2989,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="49" t="n">
-        <v>46183</v>
+      <c r="N30" s="50" t="n">
+        <v>46184</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T30" s="6" t="n">
-        <v>2.36</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.36</v>
@@ -3214,7 +3214,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="49" t="n">
+      <c r="N33" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O33" s="6" t="inlineStr">
@@ -4130,7 +4130,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="49" t="n">
+      <c r="C46" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4217,7 +4217,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="49" t="n">
+      <c r="C47" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4256,8 +4256,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="49" t="n">
-        <v>46182</v>
+      <c r="N47" s="50" t="n">
+        <v>46183</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4296,7 +4296,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="49" t="n">
+      <c r="C48" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4335,8 +4335,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="49" t="n">
-        <v>46182</v>
+      <c r="N48" s="50" t="n">
+        <v>46183</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4352,16 +4352,16 @@
         <v>4.13</v>
       </c>
       <c r="R48" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="S48" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.05</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.08</v>
       </c>
     </row>
     <row r="49">
@@ -4371,7 +4371,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="49" t="n">
+      <c r="C49" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4410,8 +4410,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="49" t="n">
-        <v>46182</v>
+      <c r="N49" s="50" t="n">
+        <v>46183</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.26</v>
-      </c>
-      <c r="R49" s="6" t="n">
-        <v>4.29</v>
       </c>
       <c r="S49" s="6" t="n">
         <v>4.29</v>
       </c>
       <c r="T49" s="6" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="50">
@@ -4450,7 +4450,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="49" t="n">
+      <c r="C50" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4489,8 +4489,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="49" t="n">
-        <v>46182</v>
+      <c r="N50" s="50" t="n">
+        <v>46183</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.53</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.56</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.47</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.49</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4525,7 +4525,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="49" t="n">
+      <c r="C51" s="50" t="n">
         <v>46113</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4564,7 +4564,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="49" t="n">
+      <c r="N51" s="50" t="n">
         <v>46181</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.06</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.01</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.18</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.33</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.36</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>4.13</v>
+        <v>4.05</v>
       </c>
       <c r="R48" s="6" t="n">
         <v>4.13</v>
       </c>
       <c r="S48" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="T48" s="6" t="n">
         <v>4.15</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.05</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.26</v>
-      </c>
-      <c r="S49" s="6" t="n">
-        <v>4.29</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>4.29</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.18</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.53</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.56</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.55</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.47</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -3104,8 +3104,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
-        <v>46113</v>
+      <c r="C32" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -3118,19 +3118,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.006780543386440963</v>
+        <v>0.001351100878947076</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>-0.002888319299829911</v>
+        <v>0.008675818407061886</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>0.006180911901310315</v>
+        <v>-0.003158432671926059</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>-0.0004590214961934791</v>
+        <v>0.00816625215701583</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>0.004809253086077714</v>
+        <v>-0.003651443778505348</v>
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3175,8 +3175,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
-        <v>46113</v>
+      <c r="C33" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
@@ -3189,19 +3189,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.01353137956983195</v>
+        <v>0.01665915585026556</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.007577167152940725</v>
+        <v>0.01365696311304797</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.00990709134484607</v>
+        <v>0.005808567662044093</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.01408088966438706</v>
+        <v>0.008407575522283481</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.01189108049354475</v>
+        <v>0.01058115399336634</v>
       </c>
       <c r="K33" s="5" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3254,8 +3254,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
-        <v>46113</v>
+      <c r="C34" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
@@ -3268,19 +3268,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.1194</v>
+        <v>76.16630000000001</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>75.6716</v>
+        <v>76.1289</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.9598</v>
+        <v>75.53879999999999</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.5658</v>
+        <v>75.84699999999999</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.6618</v>
+        <v>75.30500000000001</v>
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.06</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.08</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.06</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.2906</v>
+        <v>2.8314</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.18</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.31</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.34</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="31">
@@ -3408,8 +3408,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
-        <v>46113</v>
+      <c r="C36" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -3422,19 +3422,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1465</v>
+        <v>1177</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1507</v>
+        <v>1392</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1522</v>
+      </c>
+      <c r="I36" s="24" t="n">
         <v>1346</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="J36" s="24" t="n">
         <v>1385</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1378</v>
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3479,8 +3479,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
-        <v>46113</v>
+      <c r="C37" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
@@ -3493,19 +3493,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.04642857142857143</v>
+        <v>-0.08688906128782002</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>0.1196136701337296</v>
+        <v>-0.005714285714285714</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>0.1307578008915305</v>
+      </c>
+      <c r="I37" s="25" t="n">
         <v>-0.09725016767270288</v>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="J37" s="25" t="n">
         <v>0.02365114560236511</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>-0.07764390896921017</v>
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3558,8 +3558,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
-        <v>46113</v>
+      <c r="C38" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
@@ -3572,19 +3572,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
+        <v>1413</v>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>1423</v>
       </c>
-      <c r="G38" s="24" t="n">
+      <c r="H38" s="24" t="n">
         <v>1363</v>
       </c>
-      <c r="H38" s="24" t="n">
+      <c r="I38" s="24" t="n">
         <v>1540</v>
       </c>
-      <c r="I38" s="24" t="n">
+      <c r="J38" s="24" t="n">
         <v>1393</v>
-      </c>
-      <c r="J38" s="24" t="n">
-        <v>1482</v>
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3629,8 +3629,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
-        <v>46113</v>
+      <c r="C39" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
@@ -3643,19 +3643,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
+        <v>-0.00211864406779661</v>
+      </c>
+      <c r="G39" s="38" t="n">
         <v>-0.01522491349480969</v>
       </c>
-      <c r="G39" s="38" t="n">
+      <c r="H39" s="38" t="n">
         <v>-0.08646112600536193</v>
       </c>
-      <c r="H39" s="38" t="n">
+      <c r="I39" s="38" t="n">
         <v>0.06500691562932227</v>
       </c>
-      <c r="I39" s="38" t="n">
+      <c r="J39" s="38" t="n">
         <v>-0.04784688995215311</v>
-      </c>
-      <c r="J39" s="38" t="n">
-        <v>0.01022494887525562</v>
       </c>
       <c r="K39" s="5" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3818,8 +3818,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
-        <v>46113</v>
+      <c r="N41" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
         <is>
@@ -3832,19 +3832,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.03296019900497504</v>
+        <v>0.01261261261261248</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v>0.01515151515151514</v>
+        <v>0.03480422622747037</v>
       </c>
       <c r="S41" s="38" t="n">
+        <v>0.01578282828282829</v>
+      </c>
+      <c r="T41" s="38" t="n">
         <v>0.01930501930501927</v>
       </c>
-      <c r="T41" s="38" t="n">
+      <c r="U41" s="23" t="n">
         <v>0.005174644243208348</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0.005855562784645496</v>
       </c>
     </row>
     <row r="42">
@@ -3893,8 +3893,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
-        <v>46113</v>
+      <c r="N42" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
@@ -3907,19 +3907,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.08846657929226737</v>
+        <v>0.1121372031662269</v>
       </c>
       <c r="R42" s="38" t="n">
-        <v>0.0544262295081968</v>
+        <v>0.09108781127129754</v>
       </c>
       <c r="S42" s="38" t="n">
+        <v>0.05508196721311479</v>
+      </c>
+      <c r="T42" s="38" t="n">
         <v>0.03800786369593716</v>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v>0.02506596306068609</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.0341137123745819</v>
       </c>
     </row>
     <row r="43">
@@ -3968,8 +3968,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
-        <v>46113</v>
+      <c r="N43" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
@@ -3982,19 +3982,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.01933701657458542</v>
+        <v>0.01895734597156395</v>
       </c>
       <c r="R43" s="38" t="n">
+        <v>0.0200276243093922</v>
+      </c>
+      <c r="S43" s="38" t="n">
         <v>0.009059233449477455</v>
       </c>
-      <c r="S43" s="38" t="n">
+      <c r="T43" s="38" t="n">
         <v>0.009852216748768461</v>
       </c>
-      <c r="T43" s="38" t="n">
+      <c r="U43" s="23" t="n">
         <v>0.004950495049504955</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>0.00141643059490093</v>
       </c>
     </row>
     <row r="44">
@@ -4043,8 +4043,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
-        <v>46113</v>
+      <c r="N44" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
         <is>
@@ -4057,19 +4057,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.0416372618207481</v>
+        <v>0.0673758865248227</v>
       </c>
       <c r="R44" s="38" t="n">
+        <v>0.04234297812279464</v>
+      </c>
+      <c r="S44" s="38" t="n">
         <v>0.0225988700564973</v>
       </c>
-      <c r="S44" s="38" t="n">
+      <c r="T44" s="38" t="n">
         <v>0.009852216748768513</v>
       </c>
-      <c r="T44" s="38" t="n">
+      <c r="U44" s="23" t="n">
         <v>0.002115655853314407</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -4130,7 +4130,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="50" t="n">
+      <c r="C46" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -4217,7 +4217,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="50" t="n">
+      <c r="C47" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4296,7 +4296,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="50" t="n">
+      <c r="C48" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.05</v>
-      </c>
-      <c r="R48" s="6" t="n">
-        <v>4.13</v>
       </c>
       <c r="S48" s="6" t="n">
         <v>4.13</v>
       </c>
       <c r="T48" s="6" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>4.15</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.17</v>
       </c>
     </row>
     <row r="49">
@@ -4371,7 +4371,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="50" t="n">
+      <c r="C49" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,16 +4424,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.26</v>
-      </c>
-      <c r="T49" s="6" t="n">
-        <v>4.29</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.29</v>
@@ -4450,7 +4450,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="50" t="n">
+      <c r="C50" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.45</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.53</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.56</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.55</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4525,7 +4525,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="50" t="n">
+      <c r="C51" s="48" t="n">
         <v>46113</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.08</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.06</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.08</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-17
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>2.8314</v>
+        <v>3.0377</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1948,8 +1948,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
-        <v>46113</v>
+      <c r="C17" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.004931175916216501</v>
+        <v>0.008809356490312226</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.01631236863902608</v>
+        <v>0.004009214695237295</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>0.01717978949867671</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>0.009223924204530221</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>-0.0002912686109073359</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>-1.361066422789214e-06</v>
       </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2035,8 +2035,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
-        <v>46113</v>
+      <c r="C18" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -2049,19 +2049,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.04873507936661851</v>
+        <v>0.06876462422050805</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.04151718627089097</v>
+        <v>0.0478848128984749</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.04240611939906461</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.04174261321715912</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.03267862666254253</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.02433131408893505</v>
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2074,7 +2074,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="50" t="n">
+      <c r="N18" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O18" s="6" t="inlineStr">
@@ -2149,7 +2149,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="50" t="n">
+      <c r="N19" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2224,7 +2224,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="50" t="n">
+      <c r="N20" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2299,7 +2299,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="50" t="n">
+      <c r="N21" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O21" s="6" t="inlineStr">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.18</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.31</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="Q47" s="6" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="R47" s="6" t="n">
         <v>3.62</v>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.05</v>
-      </c>
-      <c r="S48" s="6" t="n">
-        <v>4.13</v>
       </c>
       <c r="T48" s="6" t="n">
         <v>4.13</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>4.15</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.29</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.48</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.45</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.53</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.56</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="N13" s="50" t="n">
-        <v>46174</v>
+        <v>46181</v>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
@@ -1721,19 +1721,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>229000</v>
+        <v>226000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>230000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>225000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>212000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>210000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>212000</v>
       </c>
     </row>
     <row r="14">
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="N14" s="50" t="n">
-        <v>46167</v>
+        <v>46174</v>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
@@ -1796,19 +1796,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1795000</v>
+        <v>1810000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1786000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1771000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1785000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1771000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1776000</v>
       </c>
     </row>
     <row r="15">
@@ -2378,7 +2378,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="50" t="n">
+      <c r="N22" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2448,7 +2448,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="50" t="n">
+      <c r="N23" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.18</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.31</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.29</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
         <v>3.63</v>
       </c>
       <c r="R47" s="6" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="S47" s="6" t="n">
         <v>3.62</v>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,16 +4349,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.05</v>
-      </c>
-      <c r="T48" s="6" t="n">
-        <v>4.13</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.13</v>
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.47</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.48</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.45</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.55</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.53</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="N51" s="50" t="n">
-        <v>46181</v>
+        <v>46188</v>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
@@ -4578,19 +4578,19 @@
         </is>
       </c>
       <c r="Q51" s="6" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="R51" s="6" t="n">
         <v>6.52</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="S51" s="6" t="n">
         <v>6.48</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="T51" s="6" t="n">
         <v>6.53</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.51</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.36</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.08</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.06</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-19
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.24</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.18</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="31">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
         <v>3.63</v>
       </c>
       <c r="S47" s="6" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="T47" s="6" t="n">
         <v>3.62</v>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.09</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.05</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.16</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.21</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.43</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.47</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.48</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.45</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.55</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,19 +4629,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.98</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.08</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -3104,7 +3104,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="50" t="n">
+      <c r="C32" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3175,7 +3175,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="50" t="n">
+      <c r="C33" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3254,7 +3254,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="50" t="n">
+      <c r="C34" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="N29" s="50" t="n">
-        <v>46191</v>
+        <v>46195</v>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="Q29" s="6" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="R29" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="S29" s="6" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="6" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="30">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="N30" s="50" t="n">
-        <v>46191</v>
+        <v>46195</v>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
@@ -3003,19 +3003,19 @@
         </is>
       </c>
       <c r="Q30" s="6" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R30" s="6" t="n">
         <v>2.25</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="6" t="n">
         <v>2.26</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="6" t="n">
         <v>2.29</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -3408,7 +3408,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="50" t="n">
+      <c r="C36" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3479,7 +3479,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="50" t="n">
+      <c r="C37" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3558,7 +3558,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="50" t="n">
+      <c r="C38" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3629,7 +3629,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="50" t="n">
+      <c r="C39" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3818,7 +3818,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="50" t="n">
+      <c r="N41" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3893,7 +3893,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="50" t="n">
+      <c r="N42" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O42" s="6" t="inlineStr">
@@ -3968,7 +3968,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="50" t="n">
+      <c r="N43" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4043,7 +4043,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="50" t="n">
+      <c r="N44" s="48" t="n">
         <v>46143</v>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="N47" s="50" t="n">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="O47" s="6" t="inlineStr">
         <is>
@@ -4279,10 +4279,10 @@
         <v>3.63</v>
       </c>
       <c r="T47" s="6" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="48">
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="N48" s="50" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
@@ -4349,19 +4349,19 @@
         </is>
       </c>
       <c r="Q48" s="6" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R48" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="6" t="n">
         <v>4.05</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.09</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.05</v>
       </c>
     </row>
     <row r="49">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="N49" s="50" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="O49" s="6" t="inlineStr">
         <is>
@@ -4424,19 +4424,19 @@
         </is>
       </c>
       <c r="Q49" s="6" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="R49" s="6" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="6" t="n">
         <v>4.16</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="6" t="n">
         <v>4.18</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.18</v>
       </c>
     </row>
     <row r="50">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="N50" s="50" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="O50" s="6" t="inlineStr">
         <is>
@@ -4503,19 +4503,19 @@
         </is>
       </c>
       <c r="Q50" s="6" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="R50" s="6" t="n">
         <v>4.49</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="6" t="n">
         <v>4.43</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="6" t="n">
         <v>4.47</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.48</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.45</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="N52" s="51" t="n">
-        <v>46190</v>
+        <v>46195</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>5.99</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.98</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.01</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-06-24
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -354,6 +354,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -735,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U80"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1328125" defaultRowHeight="15.75"/>
   <cols>
     <col width="29.3984375" customWidth="1" style="30" min="1" max="1"/>
@@ -758,31 +767,31 @@
   </cols>
   <sheetData>
     <row r="1" ht="16.15" customHeight="1" thickBot="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="48" t="inlineStr">
         <is>
           <t>Macro Dashboard</t>
         </is>
       </c>
-      <c r="B1" s="46" t="n"/>
-      <c r="C1" s="46" t="n"/>
-      <c r="D1" s="46" t="n"/>
-      <c r="E1" s="46" t="n"/>
-      <c r="F1" s="46" t="n"/>
-      <c r="G1" s="46" t="n"/>
-      <c r="H1" s="46" t="n"/>
-      <c r="I1" s="46" t="n"/>
-      <c r="J1" s="46" t="n"/>
-      <c r="K1" s="46" t="n"/>
-      <c r="L1" s="46" t="n"/>
-      <c r="M1" s="46" t="n"/>
-      <c r="N1" s="46" t="n"/>
-      <c r="O1" s="46" t="n"/>
-      <c r="P1" s="46" t="n"/>
-      <c r="Q1" s="46" t="n"/>
-      <c r="R1" s="46" t="n"/>
-      <c r="S1" s="46" t="n"/>
-      <c r="T1" s="46" t="n"/>
-      <c r="U1" s="47" t="n"/>
+      <c r="B1" s="49" t="n"/>
+      <c r="C1" s="49" t="n"/>
+      <c r="D1" s="49" t="n"/>
+      <c r="E1" s="49" t="n"/>
+      <c r="F1" s="49" t="n"/>
+      <c r="G1" s="49" t="n"/>
+      <c r="H1" s="49" t="n"/>
+      <c r="I1" s="49" t="n"/>
+      <c r="J1" s="49" t="n"/>
+      <c r="K1" s="49" t="n"/>
+      <c r="L1" s="49" t="n"/>
+      <c r="M1" s="49" t="n"/>
+      <c r="N1" s="49" t="n"/>
+      <c r="O1" s="49" t="n"/>
+      <c r="P1" s="49" t="n"/>
+      <c r="Q1" s="49" t="n"/>
+      <c r="R1" s="49" t="n"/>
+      <c r="S1" s="49" t="n"/>
+      <c r="T1" s="49" t="n"/>
+      <c r="U1" s="50" t="n"/>
     </row>
     <row r="2" ht="16.15" customHeight="1" thickBot="1">
       <c r="A2" s="32" t="inlineStr">
@@ -835,7 +844,7 @@
           <t>Lag 4</t>
         </is>
       </c>
-      <c r="K2" s="5" t="n"/>
+      <c r="K2" s="46" t="n"/>
       <c r="L2" s="27" t="inlineStr">
         <is>
           <t>Labor</t>
@@ -898,15 +907,15 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C3" s="48" t="n">
+      <c r="C3" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="45" t="inlineStr">
         <is>
           <t>Trln $</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -926,7 +935,7 @@
       <c r="J3" s="24" t="n">
         <v>23548.21</v>
       </c>
-      <c r="K3" s="5" t="n"/>
+      <c r="K3" s="46" t="n"/>
       <c r="L3" s="28" t="inlineStr">
         <is>
           <t>NFP, Total NonFarm</t>
@@ -937,15 +946,15 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
+      <c r="N3" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="O3" s="45" t="inlineStr">
         <is>
           <t>M/M Delta (Thousands)</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="P3" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -973,15 +982,15 @@
           <t>GDPC1</t>
         </is>
       </c>
-      <c r="C4" s="48" t="n">
+      <c r="C4" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -1001,22 +1010,22 @@
       <c r="J4" s="25" t="n">
         <v>-0.001625164044818495</v>
       </c>
-      <c r="K4" s="5" t="n"/>
+      <c r="K4" s="46" t="n"/>
       <c r="L4" s="28" t="n"/>
       <c r="M4" s="15" t="inlineStr">
         <is>
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
+      <c r="N4" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O4" s="6" t="inlineStr">
+      <c r="O4" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P4" s="6" t="inlineStr">
+      <c r="P4" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1048,15 +1057,15 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="48" t="n">
+      <c r="C5" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="45" t="inlineStr">
         <is>
           <t>Trln $</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -1076,7 +1085,7 @@
       <c r="J5" s="24" t="n">
         <v>7510528.3</v>
       </c>
-      <c r="K5" s="5" t="n"/>
+      <c r="K5" s="46" t="n"/>
       <c r="L5" s="28" t="inlineStr">
         <is>
           <t>ADP, Total NonFarm Private</t>
@@ -1087,15 +1096,15 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
+      <c r="N5" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="O5" s="45" t="inlineStr">
         <is>
           <t>M/M Delta (Thousands)</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr">
+      <c r="P5" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1109,7 +1118,7 @@
       <c r="S5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="T5" s="49" t="n">
+      <c r="T5" s="52" t="n">
         <v>66000</v>
       </c>
       <c r="U5" s="26" t="n">
@@ -1123,15 +1132,15 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="48" t="n">
+      <c r="C6" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -1151,7 +1160,7 @@
       <c r="J6" s="25" t="n">
         <v>0.007273424182290045</v>
       </c>
-      <c r="K6" s="5" t="n"/>
+      <c r="K6" s="46" t="n"/>
       <c r="L6" s="28" t="inlineStr">
         <is>
           <t>UR</t>
@@ -1162,29 +1171,29 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
+      <c r="N6" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O6" s="6" t="inlineStr">
+      <c r="O6" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P6" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q6" s="6" t="n">
+      <c r="P6" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q6" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="R6" s="6" t="n">
+      <c r="R6" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="S6" s="6" t="n">
+      <c r="S6" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="T6" s="45" t="n">
         <v>4.4</v>
       </c>
       <c r="U6" s="21" t="n">
@@ -1202,15 +1211,15 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
+      <c r="C7" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -1230,7 +1239,7 @@
       <c r="J7" s="41" t="n">
         <v>2.902</v>
       </c>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="46" t="n"/>
       <c r="L7" s="28" t="inlineStr">
         <is>
           <t>U-6</t>
@@ -1241,29 +1250,29 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
+      <c r="N7" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O7" s="6" t="inlineStr">
+      <c r="O7" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P7" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q7" s="6" t="n">
+      <c r="P7" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q7" s="45" t="n">
         <v>8.1</v>
       </c>
-      <c r="R7" s="6" t="n">
+      <c r="R7" s="45" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="S7" s="6" t="n">
+      <c r="S7" s="45" t="n">
         <v>8</v>
       </c>
-      <c r="T7" s="6" t="n">
+      <c r="T7" s="45" t="n">
         <v>7.9</v>
       </c>
       <c r="U7" s="21" t="n">
@@ -1281,35 +1290,35 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="45" t="inlineStr">
         <is>
           <t>% (5=5%)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F8" s="24" t="n">
+      <c r="E8" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="n">
         <v>0.44</v>
       </c>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="45" t="n">
         <v>0.46</v>
       </c>
-      <c r="H8" s="24" t="n">
+      <c r="H8" s="45" t="n">
         <v>0.3</v>
       </c>
-      <c r="I8" s="24" t="n">
+      <c r="I8" s="45" t="n">
         <v>0.34</v>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="45" t="n">
         <v>0.4</v>
       </c>
-      <c r="K8" s="5" t="n"/>
+      <c r="K8" s="46" t="n"/>
       <c r="L8" s="28" t="inlineStr">
         <is>
           <t>LFPR</t>
@@ -1320,29 +1329,29 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
+      <c r="N8" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O8" s="6" t="inlineStr">
+      <c r="O8" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q8" s="6" t="n">
+      <c r="P8" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q8" s="45" t="n">
         <v>61.8</v>
       </c>
-      <c r="R8" s="6" t="n">
+      <c r="R8" s="45" t="n">
         <v>61.8</v>
       </c>
-      <c r="S8" s="6" t="n">
+      <c r="S8" s="45" t="n">
         <v>61.9</v>
       </c>
-      <c r="T8" s="6" t="n">
+      <c r="T8" s="45" t="n">
         <v>62</v>
       </c>
       <c r="U8" s="21" t="n">
@@ -1360,15 +1369,15 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C9" s="48" t="n">
+      <c r="C9" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="45" t="inlineStr">
         <is>
           <t>Trln $</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -1388,7 +1397,7 @@
       <c r="J9" s="24" t="n">
         <v>16345.793</v>
       </c>
-      <c r="K9" s="5" t="n"/>
+      <c r="K9" s="46" t="n"/>
       <c r="L9" s="28" t="inlineStr">
         <is>
           <t>EPop</t>
@@ -1399,29 +1408,29 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
+      <c r="N9" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="O9" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q9" s="6" t="n">
+      <c r="P9" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q9" s="45" t="n">
         <v>59.2</v>
       </c>
-      <c r="R9" s="6" t="n">
+      <c r="R9" s="45" t="n">
         <v>59.1</v>
       </c>
-      <c r="S9" s="6" t="n">
+      <c r="S9" s="45" t="n">
         <v>59.2</v>
       </c>
-      <c r="T9" s="6" t="n">
+      <c r="T9" s="45" t="n">
         <v>59.3</v>
       </c>
       <c r="U9" s="21" t="n">
@@ -1435,15 +1444,15 @@
           <t>PCECC96</t>
         </is>
       </c>
-      <c r="C10" s="48" t="n">
+      <c r="C10" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -1463,7 +1472,7 @@
       <c r="J10" s="25" t="n">
         <v>0.001525835907232986</v>
       </c>
-      <c r="K10" s="5" t="n"/>
+      <c r="K10" s="46" t="n"/>
       <c r="L10" s="28" t="inlineStr">
         <is>
           <t>JOLTS Openings Rate</t>
@@ -1474,29 +1483,29 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
+      <c r="N10" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O10" s="6" t="inlineStr">
+      <c r="O10" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P10" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q10" s="6" t="n">
+      <c r="P10" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q10" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="R10" s="6" t="n">
+      <c r="R10" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S10" s="6" t="n">
+      <c r="S10" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="T10" s="6" t="n">
+      <c r="T10" s="45" t="n">
         <v>4.4</v>
       </c>
       <c r="U10" s="21" t="n">
@@ -1514,15 +1523,15 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
+      <c r="C11" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1542,7 +1551,7 @@
       <c r="J11" s="25" t="n">
         <v>-0.00581233144238813</v>
       </c>
-      <c r="K11" s="5" t="n"/>
+      <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
         <is>
           <t>JOLTS Hires Rate</t>
@@ -1553,29 +1562,29 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O11" s="6" t="inlineStr">
+      <c r="O11" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P11" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q11" s="6" t="n">
+      <c r="P11" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q11" s="45" t="n">
         <v>3.2</v>
       </c>
-      <c r="R11" s="6" t="n">
+      <c r="R11" s="45" t="n">
         <v>3.5</v>
       </c>
-      <c r="S11" s="6" t="n">
+      <c r="S11" s="45" t="n">
         <v>3.1</v>
       </c>
-      <c r="T11" s="6" t="n">
+      <c r="T11" s="45" t="n">
         <v>3.4</v>
       </c>
       <c r="U11" s="21" t="n">
@@ -1589,15 +1598,15 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
+      <c r="C12" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1617,7 +1626,7 @@
       <c r="J12" s="25" t="n">
         <v>-0.02262753702687877</v>
       </c>
-      <c r="K12" s="5" t="n"/>
+      <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
         <is>
           <t>JOLTS Separations Rate</t>
@@ -1628,29 +1637,29 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O12" s="6" t="inlineStr">
+      <c r="O12" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P12" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q12" s="6" t="n">
+      <c r="P12" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q12" s="45" t="n">
         <v>3.1</v>
       </c>
-      <c r="R12" s="6" t="n">
+      <c r="R12" s="45" t="n">
         <v>3.4</v>
       </c>
-      <c r="S12" s="6" t="n">
+      <c r="S12" s="45" t="n">
         <v>3.2</v>
       </c>
-      <c r="T12" s="6" t="n">
+      <c r="T12" s="45" t="n">
         <v>3.2</v>
       </c>
       <c r="U12" s="21" t="n">
@@ -1668,15 +1677,15 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
+      <c r="C13" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1696,7 +1705,7 @@
       <c r="J13" s="25" t="n">
         <v>-0.002197864126912585</v>
       </c>
-      <c r="K13" s="5" t="n"/>
+      <c r="K13" s="46" t="n"/>
       <c r="L13" s="28" t="inlineStr">
         <is>
           <t>UI Initial Claims</t>
@@ -1707,15 +1716,15 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="50" t="n">
+      <c r="N13" s="53" t="n">
         <v>46181</v>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="O13" s="45" t="inlineStr">
         <is>
           <t># People</t>
         </is>
       </c>
-      <c r="P13" s="6" t="inlineStr">
+      <c r="P13" s="45" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -1743,15 +1752,15 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1771,7 +1780,7 @@
       <c r="J14" s="25" t="n">
         <v>0.01400263444247182</v>
       </c>
-      <c r="K14" s="5" t="n"/>
+      <c r="K14" s="46" t="n"/>
       <c r="L14" s="28" t="inlineStr">
         <is>
           <t>UI Continuing Claims</t>
@@ -1782,15 +1791,15 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="50" t="n">
+      <c r="N14" s="53" t="n">
         <v>46174</v>
       </c>
-      <c r="O14" s="6" t="inlineStr">
+      <c r="O14" s="45" t="inlineStr">
         <is>
           <t># People</t>
         </is>
       </c>
-      <c r="P14" s="6" t="inlineStr">
+      <c r="P14" s="45" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -1822,15 +1831,15 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
+      <c r="C15" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1850,7 +1859,7 @@
       <c r="J15" s="25" t="n">
         <v>0.002845221754583793</v>
       </c>
-      <c r="K15" s="5" t="n"/>
+      <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
         <is>
           <t>Avg Weekly Hours</t>
@@ -1861,15 +1870,15 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
+      <c r="N15" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="O15" s="45" t="inlineStr">
         <is>
           <t>Hrs</t>
         </is>
       </c>
-      <c r="P15" s="6" t="inlineStr">
+      <c r="P15" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1897,15 +1906,15 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1925,16 +1934,16 @@
       <c r="J16" s="25" t="n">
         <v>0.02311045163683583</v>
       </c>
-      <c r="K16" s="5" t="n"/>
+      <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
       <c r="M16" s="15" t="n"/>
       <c r="N16" s="7" t="n"/>
-      <c r="O16" s="6" t="n"/>
-      <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="6" t="n"/>
-      <c r="S16" s="6" t="n"/>
-      <c r="T16" s="6" t="n"/>
+      <c r="O16" s="45" t="n"/>
+      <c r="P16" s="45" t="n"/>
+      <c r="Q16" s="45" t="n"/>
+      <c r="R16" s="45" t="n"/>
+      <c r="S16" s="45" t="n"/>
+      <c r="T16" s="45" t="n"/>
       <c r="U16" s="21" t="n"/>
     </row>
     <row r="17" ht="16.15" customHeight="1" thickBot="1">
@@ -1948,15 +1957,15 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="50" t="n">
+      <c r="C17" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1976,7 +1985,7 @@
       <c r="J17" s="25" t="n">
         <v>-0.0002912686109073359</v>
       </c>
-      <c r="K17" s="5" t="n"/>
+      <c r="K17" s="46" t="n"/>
       <c r="L17" s="29" t="inlineStr">
         <is>
           <t>Prices</t>
@@ -2035,15 +2044,15 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="50" t="n">
+      <c r="C18" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2063,7 +2072,7 @@
       <c r="J18" s="25" t="n">
         <v>0.03267862666254253</v>
       </c>
-      <c r="K18" s="5" t="n"/>
+      <c r="K18" s="46" t="n"/>
       <c r="L18" s="28" t="inlineStr">
         <is>
           <t>CPI</t>
@@ -2074,15 +2083,15 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
+      <c r="N18" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O18" s="6" t="inlineStr">
+      <c r="O18" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P18" s="6" t="inlineStr">
+      <c r="P18" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2114,15 +2123,15 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2142,22 +2151,22 @@
       <c r="J19" s="25" t="n">
         <v>-0.0009204273888139269</v>
       </c>
-      <c r="K19" s="5" t="n"/>
+      <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
       <c r="M19" s="15" t="inlineStr">
         <is>
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
+      <c r="N19" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O19" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P19" s="6" t="inlineStr">
+      <c r="P19" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2185,15 +2194,15 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
+      <c r="C20" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2213,7 +2222,7 @@
       <c r="J20" s="25" t="n">
         <v>0.008428522657950768</v>
       </c>
-      <c r="K20" s="5" t="n"/>
+      <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
         <is>
           <t>Core CPI</t>
@@ -2224,15 +2233,15 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
+      <c r="N20" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O20" s="6" t="inlineStr">
+      <c r="O20" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P20" s="6" t="inlineStr">
+      <c r="P20" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2264,50 +2273,50 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
+      <c r="C21" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="45" t="inlineStr">
         <is>
           <t>%, SAAR</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
+      <c r="E21" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F21" s="45" t="n">
         <v>2.6</v>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G21" s="45" t="n">
         <v>3.2</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="H21" s="45" t="n">
         <v>3.6</v>
       </c>
-      <c r="I21" s="6" t="n">
+      <c r="I21" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="J21" s="6" t="n">
+      <c r="J21" s="45" t="n">
         <v>3.6</v>
       </c>
-      <c r="K21" s="5" t="n"/>
+      <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
       <c r="M21" s="15" t="inlineStr">
         <is>
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
+      <c r="N21" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O21" s="6" t="inlineStr">
+      <c r="O21" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P21" s="6" t="inlineStr">
+      <c r="P21" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2339,15 +2348,15 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C22" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="45" t="inlineStr">
         <is>
           <t>Mln Units</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2367,7 +2376,7 @@
       <c r="J22" s="24" t="n">
         <v>14.987</v>
       </c>
-      <c r="K22" s="5" t="n"/>
+      <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
         <is>
           <t>PPI-FD</t>
@@ -2378,15 +2387,15 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
+      <c r="N22" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O22" s="6" t="inlineStr">
+      <c r="O22" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P22" s="6" t="inlineStr">
+      <c r="P22" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2414,15 +2423,15 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="48" t="n">
+      <c r="C23" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2442,21 +2451,21 @@
       <c r="J23" s="25" t="n">
         <v>-0.0603761755485893</v>
       </c>
-      <c r="K23" s="5" t="n"/>
+      <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">
         <is>
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
+      <c r="N23" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O23" s="6" t="inlineStr">
+      <c r="O23" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P23" s="6" t="inlineStr">
+      <c r="P23" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2488,15 +2497,15 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n">
+      <c r="C24" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta SAAR</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2516,7 +2525,7 @@
       <c r="J24" s="38" t="n">
         <v>0.005868657238478958</v>
       </c>
-      <c r="K24" s="5" t="n"/>
+      <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
         <is>
           <t>PCE Deflator</t>
@@ -2527,15 +2536,15 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
+      <c r="N24" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O24" s="6" t="inlineStr">
+      <c r="O24" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P24" s="6" t="inlineStr">
+      <c r="P24" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2567,15 +2576,15 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="48" t="n">
+      <c r="C25" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta SAAR</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2595,22 +2604,22 @@
       <c r="J25" s="38" t="n">
         <v>0.001971303273869296</v>
       </c>
-      <c r="K25" s="5" t="n"/>
+      <c r="K25" s="46" t="n"/>
       <c r="L25" s="28" t="n"/>
       <c r="M25" s="15" t="inlineStr">
         <is>
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
+      <c r="N25" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O25" s="6" t="inlineStr">
+      <c r="O25" s="45" t="inlineStr">
         <is>
           <t xml:space="preserve">Y/Y % Delta </t>
         </is>
       </c>
-      <c r="P25" s="6" t="inlineStr">
+      <c r="P25" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2642,15 +2651,15 @@
           <t>PNFIC1</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n">
+      <c r="C26" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E26" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -2670,7 +2679,7 @@
       <c r="J26" s="38" t="n">
         <v>0.02303791460563676</v>
       </c>
-      <c r="K26" s="5" t="n"/>
+      <c r="K26" s="46" t="n"/>
       <c r="L26" s="28" t="inlineStr">
         <is>
           <t>Core PCE Deflator</t>
@@ -2681,15 +2690,15 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
+      <c r="N26" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O26" s="6" t="inlineStr">
+      <c r="O26" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P26" s="6" t="inlineStr">
+      <c r="P26" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2721,15 +2730,15 @@
           <t>PRFIC1</t>
         </is>
       </c>
-      <c r="C27" s="48" t="n">
+      <c r="C27" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -2749,22 +2758,22 @@
       <c r="J27" s="38" t="n">
         <v>-0.002410568051752549</v>
       </c>
-      <c r="K27" s="5" t="n"/>
+      <c r="K27" s="46" t="n"/>
       <c r="L27" s="28" t="n"/>
       <c r="M27" s="15" t="inlineStr">
         <is>
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
+      <c r="N27" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O27" s="6" t="inlineStr">
+      <c r="O27" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P27" s="6" t="inlineStr">
+      <c r="P27" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2796,15 +2805,15 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="48" t="n">
+      <c r="C28" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2824,7 +2833,7 @@
       <c r="J28" s="25" t="n">
         <v>-0.00913646104747079</v>
       </c>
-      <c r="K28" s="5" t="n"/>
+      <c r="K28" s="46" t="n"/>
       <c r="L28" s="28" t="inlineStr">
         <is>
           <t>Mich NTM Inflation Exp</t>
@@ -2835,29 +2844,29 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
+      <c r="N28" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O28" s="6" t="inlineStr">
+      <c r="O28" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="P28" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q28" s="6" t="n">
+      <c r="P28" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q28" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="R28" s="6" t="n">
+      <c r="R28" s="45" t="n">
         <v>3.8</v>
       </c>
-      <c r="S28" s="6" t="n">
+      <c r="S28" s="45" t="n">
         <v>3.4</v>
       </c>
-      <c r="T28" s="6" t="n">
+      <c r="T28" s="45" t="n">
         <v>4</v>
       </c>
       <c r="U28" s="21" t="n">
@@ -2871,15 +2880,15 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="48" t="n">
+      <c r="C29" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2899,7 +2908,7 @@
       <c r="J29" s="25" t="n">
         <v>0.1059440595541697</v>
       </c>
-      <c r="K29" s="5" t="n"/>
+      <c r="K29" s="46" t="n"/>
       <c r="L29" s="28" t="inlineStr">
         <is>
           <t>5yr, 5yr Forward</t>
@@ -2910,33 +2919,33 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="50" t="n">
-        <v>46195</v>
-      </c>
-      <c r="O29" s="6" t="inlineStr">
+      <c r="N29" s="53" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O29" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P29" s="6" t="inlineStr">
+      <c r="P29" s="45" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="Q29" s="6" t="n">
+      <c r="Q29" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="R29" s="6" t="n">
+      <c r="R29" s="45" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="S29" s="6" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="6" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -2950,15 +2959,15 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="48" t="n">
+      <c r="C30" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E30" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2978,7 +2987,7 @@
       <c r="J30" s="25" t="n">
         <v>-0.01921059426035288</v>
       </c>
-      <c r="K30" s="5" t="n"/>
+      <c r="K30" s="46" t="n"/>
       <c r="L30" s="28" t="inlineStr">
         <is>
           <t>10yr TIPS</t>
@@ -2989,33 +2998,33 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="50" t="n">
-        <v>46195</v>
-      </c>
-      <c r="O30" s="6" t="inlineStr">
+      <c r="N30" s="53" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O30" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P30" s="6" t="inlineStr">
+      <c r="P30" s="45" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="Q30" s="6" t="n">
+      <c r="Q30" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="R30" s="6" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="S30" s="6" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T30" s="6" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.29</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="31">
@@ -3025,15 +3034,15 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="48" t="n">
+      <c r="C31" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3053,7 +3062,7 @@
       <c r="J31" s="25" t="n">
         <v>0.1010908210327026</v>
       </c>
-      <c r="K31" s="5" t="n"/>
+      <c r="K31" s="46" t="n"/>
       <c r="L31" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">ECI </t>
@@ -3064,15 +3073,15 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="48" t="n">
+      <c r="N31" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="O31" s="6" t="inlineStr">
+      <c r="O31" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta</t>
         </is>
       </c>
-      <c r="P31" s="6" t="inlineStr">
+      <c r="P31" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -3104,15 +3113,15 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="48" t="n">
+      <c r="C32" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E32" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3132,22 +3141,22 @@
       <c r="J32" s="25" t="n">
         <v>-0.003651443778505348</v>
       </c>
-      <c r="K32" s="5" t="n"/>
+      <c r="K32" s="46" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="7" t="inlineStr">
         <is>
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="48" t="n">
+      <c r="N32" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="O32" s="6" t="inlineStr">
+      <c r="O32" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P32" s="6" t="inlineStr">
+      <c r="P32" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -3175,15 +3184,15 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="48" t="n">
+      <c r="C33" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E33" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3203,7 +3212,7 @@
       <c r="J33" s="25" t="n">
         <v>0.01058115399336634</v>
       </c>
-      <c r="K33" s="5" t="n"/>
+      <c r="K33" s="46" t="n"/>
       <c r="L33" s="28" t="inlineStr">
         <is>
           <t>Avg Hrly Earnings</t>
@@ -3214,15 +3223,15 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
+      <c r="N33" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O33" s="6" t="inlineStr">
+      <c r="O33" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P33" s="6" t="inlineStr">
+      <c r="P33" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3254,15 +3263,15 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="48" t="n">
+      <c r="C34" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" s="45" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E34" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3282,22 +3291,22 @@
       <c r="J34" s="24" t="n">
         <v>75.30500000000001</v>
       </c>
-      <c r="K34" s="5" t="n"/>
+      <c r="K34" s="46" t="n"/>
       <c r="L34" s="28" t="n"/>
       <c r="M34" s="15" t="inlineStr">
         <is>
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="48" t="n">
+      <c r="N34" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O34" s="6" t="inlineStr">
+      <c r="O34" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P34" s="6" t="inlineStr">
+      <c r="P34" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3329,15 +3338,15 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="48" t="n">
+      <c r="C35" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E35" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -3357,7 +3366,7 @@
       <c r="J35" s="41" t="n">
         <v>-0.9</v>
       </c>
-      <c r="K35" s="5" t="n"/>
+      <c r="K35" s="46" t="n"/>
       <c r="L35" s="28" t="inlineStr">
         <is>
           <t>Real Avg. Hourly Earnings</t>
@@ -3368,15 +3377,15 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="48" t="n">
+      <c r="N35" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O35" s="6" t="inlineStr">
+      <c r="O35" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P35" s="6" t="inlineStr">
+      <c r="P35" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3408,15 +3417,15 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="48" t="n">
+      <c r="C36" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" s="45" t="inlineStr">
         <is>
           <t>SAAR (Thousands)</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3436,22 +3445,22 @@
       <c r="J36" s="24" t="n">
         <v>1385</v>
       </c>
-      <c r="K36" s="5" t="n"/>
+      <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
       <c r="M36" s="15" t="inlineStr">
         <is>
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="48" t="n">
+      <c r="N36" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="O36" s="6" t="inlineStr">
+      <c r="O36" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P36" s="6" t="inlineStr">
+      <c r="P36" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3479,15 +3488,15 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="48" t="n">
+      <c r="C37" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E37" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3507,7 +3516,7 @@
       <c r="J37" s="25" t="n">
         <v>0.02365114560236511</v>
       </c>
-      <c r="K37" s="5" t="n"/>
+      <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
         <is>
           <t>Case Shiller HPI</t>
@@ -3518,15 +3527,15 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
+      <c r="N37" s="51" t="n">
         <v>46082</v>
       </c>
-      <c r="O37" s="6" t="inlineStr">
+      <c r="O37" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P37" s="6" t="inlineStr">
+      <c r="P37" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3558,21 +3567,21 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="48" t="n">
+      <c r="C38" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" s="45" t="inlineStr">
         <is>
           <t>SAAR (Thousands)</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E38" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1423</v>
@@ -3586,22 +3595,22 @@
       <c r="J38" s="24" t="n">
         <v>1393</v>
       </c>
-      <c r="K38" s="5" t="n"/>
+      <c r="K38" s="46" t="n"/>
       <c r="L38" s="28" t="n"/>
       <c r="M38" s="15" t="inlineStr">
         <is>
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
+      <c r="N38" s="51" t="n">
         <v>46082</v>
       </c>
-      <c r="O38" s="6" t="inlineStr">
+      <c r="O38" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P38" s="6" t="inlineStr">
+      <c r="P38" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3629,21 +3638,21 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="48" t="n">
+      <c r="C39" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.00211864406779661</v>
+        <v>-0.00423728813559322</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>-0.01522491349480969</v>
@@ -3657,7 +3666,7 @@
       <c r="J39" s="38" t="n">
         <v>-0.04784688995215311</v>
       </c>
-      <c r="K39" s="5" t="n"/>
+      <c r="K39" s="46" t="n"/>
       <c r="L39" s="28" t="inlineStr">
         <is>
           <t>Nominal Broad US Dollar Index</t>
@@ -3668,29 +3677,29 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
+      <c r="N39" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O39" s="6" t="inlineStr">
+      <c r="O39" s="45" t="inlineStr">
         <is>
           <t>Index Jan2006=100</t>
         </is>
       </c>
-      <c r="P39" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q39" s="6" t="n">
+      <c r="P39" s="45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q39" s="45" t="n">
         <v>118.7792</v>
       </c>
-      <c r="R39" s="6" t="n">
+      <c r="R39" s="45" t="n">
         <v>119.0363</v>
       </c>
-      <c r="S39" s="6" t="n">
+      <c r="S39" s="45" t="n">
         <v>119.9199</v>
       </c>
-      <c r="T39" s="6" t="n">
+      <c r="T39" s="45" t="n">
         <v>117.906</v>
       </c>
       <c r="U39" s="21" t="n">
@@ -3708,50 +3717,50 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="48" t="n">
-        <v>46113</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="C40" s="53" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D40" s="45" t="inlineStr">
         <is>
           <t>SAAR (Thousands)</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E40" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>622</v>
+        <v>580</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>663</v>
+        <v>626</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>641</v>
+        <v>664</v>
       </c>
       <c r="I40" s="24" t="n">
+        <v>630</v>
+      </c>
+      <c r="J40" s="24" t="n">
         <v>576</v>
       </c>
-      <c r="J40" s="24" t="n">
-        <v>723</v>
-      </c>
-      <c r="K40" s="5" t="n"/>
+      <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
       <c r="M40" s="15" t="inlineStr">
         <is>
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
+      <c r="N40" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O40" s="6" t="inlineStr">
+      <c r="O40" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P40" s="6" t="inlineStr">
+      <c r="P40" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3779,35 +3788,35 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="48" t="n">
-        <v>46113</v>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="C41" s="53" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.1126961483594865</v>
+        <v>-0.06752411575562701</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>0.01067073170731707</v>
+        <v>-0.1069900142653352</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>0</v>
+        <v>0.01219512195121951</v>
       </c>
       <c r="I41" s="38" t="n">
+        <v>-0.0171606864274571</v>
+      </c>
+      <c r="J41" s="38" t="n">
         <v>-0.1338345864661654</v>
       </c>
-      <c r="J41" s="38" t="n">
-        <v>0.02991452991452992</v>
-      </c>
-      <c r="K41" s="5" t="n"/>
+      <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
         <is>
           <t>Export Prices</t>
@@ -3818,15 +3827,15 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
+      <c r="N41" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O41" s="6" t="inlineStr">
+      <c r="O41" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P41" s="6" t="inlineStr">
+      <c r="P41" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3858,15 +3867,15 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="48" t="n">
+      <c r="C42" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D42" s="45" t="inlineStr">
         <is>
           <t>SAAR (Thousands)</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E42" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3893,15 +3902,15 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
+      <c r="N42" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O42" s="6" t="inlineStr">
+      <c r="O42" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P42" s="6" t="inlineStr">
+      <c r="P42" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3929,15 +3938,15 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="48" t="n">
+      <c r="C43" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D43" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E43" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3957,7 +3966,7 @@
       <c r="J43" s="38" t="n">
         <v/>
       </c>
-      <c r="K43" s="5" t="n"/>
+      <c r="K43" s="46" t="n"/>
       <c r="L43" s="28" t="inlineStr">
         <is>
           <t>Import Prices</t>
@@ -3968,15 +3977,15 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
+      <c r="N43" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O43" s="6" t="inlineStr">
+      <c r="O43" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta</t>
         </is>
       </c>
-      <c r="P43" s="6" t="inlineStr">
+      <c r="P43" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4008,15 +4017,15 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C44" s="48" t="n">
+      <c r="C44" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D44" s="45" t="inlineStr">
         <is>
           <t>Trln $</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="E44" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -4036,22 +4045,22 @@
       <c r="J44" s="24" t="n">
         <v>5195.517</v>
       </c>
-      <c r="K44" s="5" t="n"/>
+      <c r="K44" s="46" t="n"/>
       <c r="L44" s="28" t="n"/>
       <c r="M44" s="15" t="inlineStr">
         <is>
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
+      <c r="N44" s="51" t="n">
         <v>46143</v>
       </c>
-      <c r="O44" s="6" t="inlineStr">
+      <c r="O44" s="45" t="inlineStr">
         <is>
           <t>Y/Y % Delta</t>
         </is>
       </c>
-      <c r="P44" s="6" t="inlineStr">
+      <c r="P44" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4079,15 +4088,15 @@
           <t>GCE</t>
         </is>
       </c>
-      <c r="C45" s="48" t="n">
+      <c r="C45" s="51" t="n">
         <v>46023</v>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D45" s="45" t="inlineStr">
         <is>
           <t>Q/Q % Delta SAAR</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E45" s="45" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
@@ -4107,16 +4116,16 @@
       <c r="J45" s="38" t="n">
         <v>0.008696251498575336</v>
       </c>
-      <c r="K45" s="5" t="n"/>
+      <c r="K45" s="46" t="n"/>
       <c r="L45" s="28" t="n"/>
       <c r="M45" s="15" t="n"/>
       <c r="N45" s="7" t="n"/>
-      <c r="O45" s="6" t="n"/>
-      <c r="P45" s="6" t="n"/>
-      <c r="Q45" s="6" t="n"/>
-      <c r="R45" s="6" t="n"/>
-      <c r="S45" s="6" t="n"/>
-      <c r="T45" s="6" t="n"/>
+      <c r="O45" s="45" t="n"/>
+      <c r="P45" s="45" t="n"/>
+      <c r="Q45" s="45" t="n"/>
+      <c r="R45" s="45" t="n"/>
+      <c r="S45" s="45" t="n"/>
+      <c r="T45" s="45" t="n"/>
       <c r="U45" s="21" t="n"/>
     </row>
     <row r="46" ht="16.15" customHeight="1" thickBot="1">
@@ -4130,15 +4139,15 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="48" t="n">
+      <c r="C46" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D46" s="45" t="inlineStr">
         <is>
           <t>Bln $</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E46" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4158,7 +4167,7 @@
       <c r="J46" s="24" t="n">
         <v>285282</v>
       </c>
-      <c r="K46" s="5" t="n"/>
+      <c r="K46" s="46" t="n"/>
       <c r="L46" s="29" t="inlineStr">
         <is>
           <t>Rates</t>
@@ -4217,15 +4226,15 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="48" t="n">
+      <c r="C47" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D47" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta SA</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4245,7 +4254,7 @@
       <c r="J47" s="38" t="n">
         <v>-0.01458356361224711</v>
       </c>
-      <c r="K47" s="5" t="n"/>
+      <c r="K47" s="46" t="n"/>
       <c r="L47" s="28" t="inlineStr">
         <is>
           <t>FFR</t>
@@ -4256,29 +4265,29 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="50" t="n">
-        <v>46192</v>
-      </c>
-      <c r="O47" s="6" t="inlineStr">
+      <c r="N47" s="53" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O47" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P47" s="6" t="inlineStr">
+      <c r="P47" s="45" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="Q47" s="6" t="n">
+      <c r="Q47" s="45" t="n">
         <v>3.63</v>
       </c>
-      <c r="R47" s="6" t="n">
+      <c r="R47" s="45" t="n">
         <v>3.63</v>
       </c>
-      <c r="S47" s="6" t="n">
+      <c r="S47" s="45" t="n">
         <v>3.63</v>
       </c>
-      <c r="T47" s="6" t="n">
+      <c r="T47" s="45" t="n">
         <v>3.63</v>
       </c>
       <c r="U47" s="21" t="n">
@@ -4296,15 +4305,15 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="48" t="n">
+      <c r="C48" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D48" s="45" t="inlineStr">
         <is>
           <t>Bln $</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E48" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4324,7 +4333,7 @@
       <c r="J48" s="24" t="n">
         <v>361360</v>
       </c>
-      <c r="K48" s="5" t="n"/>
+      <c r="K48" s="46" t="n"/>
       <c r="L48" s="28" t="inlineStr">
         <is>
           <t>2y UST</t>
@@ -4335,33 +4344,33 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="50" t="n">
-        <v>46191</v>
-      </c>
-      <c r="O48" s="6" t="inlineStr">
+      <c r="N48" s="53" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O48" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P48" s="6" t="inlineStr">
+      <c r="P48" s="45" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="Q48" s="6" t="n">
+      <c r="Q48" s="45" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="R48" s="6" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S48" s="6" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.05</v>
       </c>
-      <c r="T48" s="6" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.07</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.09</v>
       </c>
     </row>
     <row r="49">
@@ -4371,15 +4380,15 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="48" t="n">
+      <c r="C49" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta SA</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4399,7 +4408,7 @@
       <c r="J49" s="38" t="n">
         <v>0.02260507340706108</v>
       </c>
-      <c r="K49" s="5" t="n"/>
+      <c r="K49" s="46" t="n"/>
       <c r="L49" s="28" t="inlineStr">
         <is>
           <t>5y UST</t>
@@ -4410,33 +4419,33 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="50" t="n">
-        <v>46191</v>
-      </c>
-      <c r="O49" s="6" t="inlineStr">
+      <c r="N49" s="53" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O49" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P49" s="6" t="inlineStr">
+      <c r="P49" s="45" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="Q49" s="6" t="n">
+      <c r="Q49" s="45" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="R49" s="6" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="6" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="T49" s="6" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="50">
@@ -4450,15 +4459,15 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="48" t="n">
+      <c r="C50" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D50" s="45" t="inlineStr">
         <is>
           <t>Bln $</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4478,7 +4487,7 @@
       <c r="J50" s="24" t="n">
         <v>26539</v>
       </c>
-      <c r="K50" s="5" t="n"/>
+      <c r="K50" s="46" t="n"/>
       <c r="L50" s="28" t="inlineStr">
         <is>
           <t>10y UST</t>
@@ -4489,33 +4498,33 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="50" t="n">
-        <v>46191</v>
-      </c>
-      <c r="O50" s="6" t="inlineStr">
+      <c r="N50" s="53" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O50" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P50" s="6" t="inlineStr">
+      <c r="P50" s="45" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="Q50" s="6" t="n">
+      <c r="Q50" s="45" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.46</v>
       </c>
-      <c r="R50" s="6" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="S50" s="6" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="T50" s="6" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.47</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.48</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4525,15 +4534,15 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="48" t="n">
+      <c r="C51" s="51" t="n">
         <v>46113</v>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="45" t="inlineStr">
         <is>
           <t>M/M % Delta SA</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="45" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4553,7 +4562,7 @@
       <c r="J51" s="38" t="n">
         <v>-0.03858136501956233</v>
       </c>
-      <c r="K51" s="5" t="n"/>
+      <c r="K51" s="46" t="n"/>
       <c r="L51" s="28" t="inlineStr">
         <is>
           <t>30y Mtg.</t>
@@ -4564,29 +4573,29 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="50" t="n">
+      <c r="N51" s="53" t="n">
         <v>46188</v>
       </c>
-      <c r="O51" s="6" t="inlineStr">
+      <c r="O51" s="45" t="inlineStr">
         <is>
           <t>%, NSA</t>
         </is>
       </c>
-      <c r="P51" s="6" t="inlineStr">
+      <c r="P51" s="45" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="Q51" s="6" t="n">
+      <c r="Q51" s="45" t="n">
         <v>6.47</v>
       </c>
-      <c r="R51" s="6" t="n">
+      <c r="R51" s="45" t="n">
         <v>6.52</v>
       </c>
-      <c r="S51" s="6" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.48</v>
       </c>
-      <c r="T51" s="6" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.53</v>
       </c>
       <c r="U51" s="21" t="n">
@@ -4615,8 +4624,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="51" t="n">
-        <v>46195</v>
+      <c r="N52" s="54" t="n">
+        <v>46196</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4629,23 +4638,23 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.02</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.97</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.99</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.98</v>
       </c>
-      <c r="U52" s="22" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="53" ht="21" customHeight="1">
-      <c r="A53" s="37" t="inlineStr">
+      <c r="A53" s="47" t="inlineStr">
         <is>
           <t>Footnote: All data is Seasonally Adjusted unless otherwise indicated by NSA</t>
         </is>
@@ -4656,105 +4665,80 @@
         </is>
       </c>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="6" t="n"/>
-      <c r="K53" s="5" t="n"/>
+      <c r="D53" s="45" t="n"/>
+      <c r="E53" s="45" t="n"/>
+      <c r="F53" s="45" t="n"/>
+      <c r="G53" s="45" t="n"/>
+      <c r="H53" s="45" t="n"/>
+      <c r="I53" s="45" t="n"/>
+      <c r="J53" s="45" t="n"/>
+      <c r="K53" s="46" t="n"/>
       <c r="L53" s="28" t="n"/>
       <c r="M53" s="15" t="n"/>
       <c r="N53" s="7" t="n"/>
-      <c r="O53" s="6" t="n"/>
-      <c r="P53" s="6" t="n"/>
-      <c r="Q53" s="6" t="n"/>
-      <c r="R53" s="6" t="n"/>
-      <c r="S53" s="6" t="n"/>
-      <c r="T53" s="6" t="n"/>
-      <c r="U53" s="6" t="n"/>
+      <c r="O53" s="45" t="n"/>
+      <c r="P53" s="45" t="n"/>
+      <c r="Q53" s="45" t="n"/>
+      <c r="R53" s="45" t="n"/>
+      <c r="S53" s="45" t="n"/>
+      <c r="T53" s="45" t="n"/>
+      <c r="U53" s="45" t="n"/>
     </row>
     <row r="54" ht="21" customHeight="1">
-      <c r="A54" s="37" t="inlineStr">
+      <c r="A54" s="47" t="inlineStr">
         <is>
           <t>Source: All data collected via FRED from the St. Louis Fed</t>
         </is>
       </c>
       <c r="B54" s="15" t="n"/>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="6" t="n"/>
-      <c r="E54" s="6" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
-      <c r="H54" s="6" t="n"/>
-      <c r="I54" s="6" t="n"/>
-      <c r="J54" s="6" t="n"/>
-      <c r="K54" s="5" t="n"/>
+      <c r="D54" s="45" t="n"/>
+      <c r="E54" s="45" t="n"/>
+      <c r="F54" s="45" t="n"/>
+      <c r="G54" s="45" t="n"/>
+      <c r="H54" s="45" t="n"/>
+      <c r="I54" s="45" t="n"/>
+      <c r="J54" s="45" t="n"/>
+      <c r="K54" s="46" t="n"/>
       <c r="L54" s="28" t="n"/>
       <c r="M54" s="15" t="n"/>
       <c r="N54" s="7" t="n"/>
-      <c r="O54" s="6" t="n"/>
-      <c r="P54" s="6" t="n"/>
-      <c r="Q54" s="6" t="n"/>
-      <c r="R54" s="6" t="n"/>
-      <c r="S54" s="6" t="n"/>
-      <c r="T54" s="6" t="n"/>
-      <c r="U54" s="6" t="n"/>
-    </row>
-    <row r="55" ht="21" customHeight="1">
-      <c r="A55" s="37" t="inlineStr">
-        <is>
-          <t>Mike Aguilar | mike.aguilar@duke.edu | www.market-observatory.com</t>
+      <c r="O54" s="45" t="n"/>
+      <c r="P54" s="45" t="n"/>
+      <c r="Q54" s="45" t="n"/>
+      <c r="R54" s="45" t="n"/>
+      <c r="S54" s="45" t="n"/>
+      <c r="T54" s="45" t="n"/>
+      <c r="U54" s="45" t="n"/>
+    </row>
+    <row r="55" ht="31.5" customHeight="1">
+      <c r="A55" s="47" t="inlineStr">
+        <is>
+          <t>Mike Aguilar | mike.aguilar@duke.edu |
+Jacky Yang    | jacky.yang@duke.edu    |
+www.market-observatory.com</t>
         </is>
       </c>
       <c r="B55" s="15" t="n"/>
       <c r="C55" s="7" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
-      <c r="I55" s="6" t="n"/>
-      <c r="J55" s="6" t="n"/>
-      <c r="K55" s="5" t="n"/>
+      <c r="D55" s="45" t="n"/>
+      <c r="E55" s="45" t="n"/>
+      <c r="F55" s="45" t="n"/>
+      <c r="G55" s="45" t="n"/>
+      <c r="H55" s="45" t="n"/>
+      <c r="I55" s="45" t="n"/>
+      <c r="J55" s="45" t="n"/>
+      <c r="K55" s="46" t="n"/>
       <c r="L55" s="28" t="n"/>
       <c r="M55" s="15" t="n"/>
       <c r="N55" s="7" t="n"/>
-      <c r="O55" s="6" t="n"/>
-      <c r="P55" s="6" t="n"/>
-      <c r="Q55" s="6" t="n"/>
-      <c r="R55" s="6" t="n"/>
-      <c r="S55" s="6" t="n"/>
-      <c r="T55" s="6" t="n"/>
-      <c r="U55" s="6" t="n"/>
-    </row>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80">
-      <c r="A80" s="4" t="n"/>
+      <c r="O55" s="45" t="n"/>
+      <c r="P55" s="45" t="n"/>
+      <c r="Q55" s="45" t="n"/>
+      <c r="R55" s="45" t="n"/>
+      <c r="S55" s="45" t="n"/>
+      <c r="T55" s="45" t="n"/>
+      <c r="U55" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-25
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24152.656</v>
+        <v>24180.419</v>
       </c>
       <c r="G3" s="24" t="n">
         <v>24055.749</v>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.004028434117765434</v>
+        <v>0.00518254492928083</v>
       </c>
       <c r="G4" s="25" t="n">
         <v>0.001203446113624551</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>3.0377</v>
+        <v>2.5438</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16723.347</v>
+        <v>16687.728</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>16665.219</v>
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.003487982966200454</v>
+        <v>0.001350657318094584</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>0.004783647872002916</v>
@@ -1523,8 +1523,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="51" t="n">
-        <v>46113</v>
+      <c r="C11" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1537,19 +1537,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>-0.005560917321568049</v>
+        <v>0.008520743120547625</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.01275308354666049</v>
+        <v>-0.01368541905855347</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>0.02042270244597488</v>
+        <v>0.01363932594730488</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>-0.0152471820775455</v>
+        <v>0.0203286786358885</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>-0.00581233144238813</v>
+        <v>-0.01529395257471577</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1598,8 +1598,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="51" t="n">
-        <v>46113</v>
+      <c r="C12" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1612,19 +1612,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>-0.0005542725173209322</v>
+        <v>0.02280776313925494</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>-0.001468496168142728</v>
+        <v>-0.007990762124711401</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.02710584185868621</v>
+        <v>-0.000734248084071364</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>0.007609111791730519</v>
+        <v>0.02696242470599466</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>-0.02262753702687877</v>
+        <v>0.007561255742725968</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1677,8 +1677,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="51" t="n">
-        <v>46113</v>
+      <c r="C13" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
@@ -1691,19 +1691,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>0.001712376835190765</v>
+        <v>0.002576669934182929</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.0047667400011282</v>
+        <v>0.00137424276419118</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>0.001865038996269996</v>
+        <v>0.005754259280153384</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>-0.0006495156872157182</v>
+        <v>0.001865144407392716</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>-0.002197864126912585</v>
+        <v>-0.0007059953121911766</v>
       </c>
       <c r="K13" s="46" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="N13" s="53" t="n">
-        <v>46181</v>
+        <v>46188</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1730,19 +1730,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>226000</v>
+        <v>215000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>227000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>230000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>225000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>212000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>210000</v>
       </c>
     </row>
     <row r="14">
@@ -1752,8 +1752,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="51" t="n">
-        <v>46113</v>
+      <c r="C14" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
@@ -1766,19 +1766,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.01881513204853678</v>
+        <v>0.02326844467312684</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.0169283471310306</v>
+        <v>0.01941470378301213</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.01601948703252618</v>
+        <v>0.01787039680274048</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>0.01859420873870254</v>
+        <v>0.0159621722309786</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>0.01400263444247182</v>
+        <v>0.01853664152898512</v>
       </c>
       <c r="K14" s="46" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="N14" s="53" t="n">
-        <v>46174</v>
+        <v>46181</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1805,19 +1805,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1810000</v>
+        <v>1821000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1786000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1771000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1785000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1771000</v>
       </c>
     </row>
     <row r="15">
@@ -1831,8 +1831,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="51" t="n">
-        <v>46113</v>
+      <c r="C15" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1845,19 +1845,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.00194183526011571</v>
+        <v>0.001720282126268735</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.001184566276935417</v>
+        <v>0.001714161330697239</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.0003980279524176122</v>
+        <v>0.0001360630606932478</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>0.002021355667953806</v>
+        <v>-0.0004895872054544448</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>0.002845221754583793</v>
+        <v>-0.0002266093798154456</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1906,8 +1906,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="51" t="n">
-        <v>46113</v>
+      <c r="C16" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1920,19 +1920,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02508778414341157</v>
+        <v>0.02046708111199261</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02629700694270652</v>
+        <v>0.02057845130290156</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02883058889198992</v>
+        <v>0.02201458987977717</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>0.02512148076709073</v>
+        <v>0.02561168480788904</v>
       </c>
       <c r="J16" s="25" t="n">
-        <v>0.02311045163683583</v>
+        <v>0.02282169219926558</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2123,8 +2123,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="51" t="n">
-        <v>46113</v>
+      <c r="C19" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2137,19 +2137,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>-0.004828076094918865</v>
+        <v>0.002508528998595327</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>-0.001601241100368522</v>
+        <v>-0.005085826793488901</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>-0.004616097329612545</v>
+        <v>-0.001185470781469022</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>0.00631018120265292</v>
+        <v>-0.004560343211319595</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>-0.0009204273888139269</v>
+        <v>0.006443377639647974</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2194,8 +2194,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="51" t="n">
-        <v>46113</v>
+      <c r="C20" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2208,19 +2208,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>-0.01104621985451874</v>
+        <v>0.0001612822494979571</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>-0.0005269259142164612</v>
+        <v>-0.01070429991893201</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>0.007704977527148879</v>
+        <v>7.7652239989875e-05</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>0.0135496204541136</v>
+        <v>0.007894810306803354</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.008428522657950768</v>
+        <v>0.013683775112075</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2273,8 +2273,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="51" t="n">
-        <v>46113</v>
+      <c r="C21" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2287,19 +2287,19 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="G21" s="45" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H21" s="45" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="I21" s="45" t="n">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
       <c r="J21" s="45" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2362,13 +2362,13 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.485</v>
+        <v>16.508</v>
       </c>
       <c r="G22" s="24" t="n">
         <v>16.395</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.537</v>
+        <v>16.536</v>
       </c>
       <c r="I22" s="24" t="n">
         <v>15.881</v>
@@ -2437,13 +2437,13 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.02755095680359036</v>
+        <v>0.02898460387708034</v>
       </c>
       <c r="G23" s="25" t="n">
         <v>-0.06756526190069947</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.09880108991825626</v>
+        <v>-0.09885558583106266</v>
       </c>
       <c r="I23" s="25" t="n">
         <v>-0.0327669163773677</v>
@@ -2536,8 +2536,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="51" t="n">
-        <v>46113</v>
+      <c r="N24" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
         <is>
@@ -2550,19 +2550,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.003995981009502714</v>
+        <v>0.004498312178282893</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.006647621988882024</v>
+        <v>0.004102666349700579</v>
       </c>
       <c r="S24" s="38" t="n">
-        <v>0.004015441621060045</v>
+        <v>0.006669806004369283</v>
       </c>
       <c r="T24" s="38" t="n">
-        <v>0.003313215530114544</v>
+        <v>0.003999286948838554</v>
       </c>
       <c r="U24" s="23" t="n">
-        <v>0.003308571071852118</v>
+        <v>0.003476543056246895</v>
       </c>
     </row>
     <row r="25">
@@ -2611,8 +2611,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="51" t="n">
-        <v>46113</v>
+      <c r="N25" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
@@ -2625,19 +2625,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.03766944114149807</v>
+        <v>0.04072638075644874</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.03525460334601121</v>
+        <v>0.03795481569560034</v>
       </c>
       <c r="S25" s="38" t="n">
-        <v>0.02858141215524022</v>
+        <v>0.03542928831754543</v>
       </c>
       <c r="T25" s="38" t="n">
-        <v>0.02858464163550402</v>
+        <v>0.02873230041057473</v>
       </c>
       <c r="U25" s="23" t="n">
-        <v>0.02878083518031025</v>
+        <v>0.02875208305094201</v>
       </c>
     </row>
     <row r="26">
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.0243486718158854</v>
+        <v>0.02552585944536068</v>
       </c>
       <c r="G26" s="38" t="n">
         <v>0.005923787970366412</v>
@@ -2690,8 +2690,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="51" t="n">
-        <v>46113</v>
+      <c r="N26" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
         <is>
@@ -2704,19 +2704,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.002389403113183475</v>
+        <v>0.003200505911295837</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.002954862726849639</v>
+        <v>0.002504967412229497</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.003955400523234065</v>
+        <v>0.002962135839517099</v>
       </c>
       <c r="T26" s="38" t="n">
-        <v>0.00426942745883041</v>
+        <v>0.003939122649955218</v>
       </c>
       <c r="U26" s="23" t="n">
-        <v>0.003271383630529812</v>
+        <v>0.00444927513566773</v>
       </c>
     </row>
     <row r="27">
@@ -2744,7 +2744,7 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>-0.01596729536276953</v>
+        <v>-0.0201499882390509</v>
       </c>
       <c r="G27" s="38" t="n">
         <v>-0.004277328978805506</v>
@@ -2765,8 +2765,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="51" t="n">
-        <v>46113</v>
+      <c r="N27" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
@@ -2779,19 +2779,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03289190610508199</v>
+        <v>0.03412035932904036</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03236287290347819</v>
+        <v>0.03318672212395027</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.03032482320508212</v>
+        <v>0.03253849776876586</v>
       </c>
       <c r="T27" s="38" t="n">
-        <v>0.03086196794208051</v>
+        <v>0.03049262855088111</v>
       </c>
       <c r="U27" s="23" t="n">
-        <v>0.02971110180682146</v>
+        <v>0.03104657789335973</v>
       </c>
     </row>
     <row r="28">
@@ -2805,8 +2805,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="51" t="n">
-        <v>46113</v>
+      <c r="C28" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
         <is>
@@ -2819,19 +2819,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.08018159976285943</v>
+        <v>-0.04478479250211442</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>0.08466230868839419</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>0.01344578206575542</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>-0.01169466364559735</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>-0.004254034642219184</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>-0.00913646104747079</v>
       </c>
       <c r="K28" s="46" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2880,8 +2880,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="51" t="n">
-        <v>46113</v>
+      <c r="C29" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
         <is>
@@ -2894,19 +2894,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.1725880587611651</v>
+        <v>-0.03493194678974276</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.1774520795721287</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.01350347073984473</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.07567733047604469</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.09883411459674789</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.1059440595541697</v>
       </c>
       <c r="K29" s="46" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.18</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -2959,8 +2959,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="51" t="n">
-        <v>46113</v>
+      <c r="C30" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
         <is>
@@ -2973,19 +2973,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.08141853927844678</v>
+        <v>-0.04626546072493454</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>0.08424643897237227</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>-0.002709178900039744</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>-0.01222345960141613</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>0.002385879326488816</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>-0.01921059426035288</v>
       </c>
       <c r="K30" s="46" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="31">
@@ -3034,8 +3034,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="51" t="n">
-        <v>46113</v>
+      <c r="C31" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
         <is>
@@ -3048,19 +3048,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.1498344103537483</v>
+        <v>-0.04975533214668908</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.1528412169314068</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>-0.0182024802287403</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.07288240242929306</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.09283155684402497</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.1010908210327026</v>
       </c>
       <c r="K31" s="46" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3299,7 +3299,7 @@
         </is>
       </c>
       <c r="N34" s="51" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
         <is>
@@ -3312,19 +3312,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.00188417944067203</v>
+        <v>-0.006026690693604906</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.0008839228572701012</v>
+        <v>-0.00215860068996659</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>0.008190609959018323</v>
+        <v>-0.001052481507739263</v>
       </c>
       <c r="T34" s="38" t="n">
-        <v>0.007745300996855934</v>
+        <v>0.008042734635068088</v>
       </c>
       <c r="U34" s="23" t="n">
-        <v>0.008247145515396716</v>
+        <v>0.007581278680517641</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3378,7 +3378,7 @@
         </is>
       </c>
       <c r="N35" s="51" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
         <is>
@@ -3391,19 +3391,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.00238004469329578</v>
+        <v>-0.001284834116984102</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>-0.004471399292342637</v>
+        <v>-0.002486041249112891</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>-0.0007821528833659164</v>
+        <v>-0.004493337788724072</v>
       </c>
       <c r="T35" s="38" t="n">
-        <v>0.0001977446423231388</v>
+        <v>-0.0007660751460527582</v>
       </c>
       <c r="U35" s="23" t="n">
-        <v>-0.002758902506289296</v>
+        <v>3.495077892301524e-05</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="N36" s="51" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
         <is>
@@ -3466,19 +3466,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.00188417944067203</v>
+        <v>-0.006026690693604906</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.0008839228572701012</v>
+        <v>-0.00215860068996659</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>0.008190609959018323</v>
+        <v>-0.001052481507739263</v>
       </c>
       <c r="T36" s="38" t="n">
-        <v>0.007745300996855934</v>
+        <v>0.008042734635068088</v>
       </c>
       <c r="U36" s="23" t="n">
-        <v>0.008247145515396716</v>
+        <v>0.007581278680517641</v>
       </c>
     </row>
     <row r="37">
@@ -4031,7 +4031,7 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5416.4</v>
+        <v>5416.715</v>
       </c>
       <c r="G44" s="24" t="n">
         <v>5343.513</v>
@@ -4102,7 +4102,7 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.01364027747289098</v>
+        <v>0.01369922745579544</v>
       </c>
       <c r="G45" s="38" t="n">
         <v>0.003589323270481781</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4358,19 +4358,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.05</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.07</v>
       </c>
     </row>
     <row r="49">
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4433,19 +4433,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.29</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.16</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.18</v>
       </c>
     </row>
     <row r="50">
@@ -4499,7 +4499,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4512,19 +4512,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.51</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.46</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.43</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.47</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4574,7 +4574,7 @@
         </is>
       </c>
       <c r="N51" s="53" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4587,19 +4587,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.47</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.52</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.48</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.53</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.51</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="N52" s="54" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4638,19 +4638,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.02</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.97</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.99</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.98</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-26
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.17</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.18</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.18</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="30">
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.25</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="31">
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4358,19 +4358,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.2</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.05</v>
       </c>
     </row>
     <row r="49">
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4433,19 +4433,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.29</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.16</v>
       </c>
     </row>
     <row r="50">
@@ -4499,7 +4499,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4512,19 +4512,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.5</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.51</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.46</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.49</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.43</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="N52" s="54" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4638,19 +4638,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.93</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.02</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.97</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.99</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="N28" s="51" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
@@ -2858,19 +2858,19 @@
         </is>
       </c>
       <c r="Q28" s="45" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="R28" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="R28" s="45" t="n">
+      <c r="S28" s="45" t="n">
         <v>3.8</v>
       </c>
-      <c r="S28" s="45" t="n">
+      <c r="T28" s="45" t="n">
         <v>3.4</v>
       </c>
-      <c r="T28" s="45" t="n">
+      <c r="U28" s="21" t="n">
         <v>4</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>4.2</v>
       </c>
     </row>
     <row r="29">
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,16 +2936,16 @@
         <v>2.19</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.17</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.18</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.18</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.23</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="30">
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4358,19 +4358,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.11</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.19</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.2</v>
       </c>
     </row>
     <row r="49">
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4433,19 +4433,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.29</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.23</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4499,7 +4499,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4512,19 +4512,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.5</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.51</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.46</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.49</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-29
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7954866</v>
+        <v>7966430.3</v>
       </c>
       <c r="G5" s="24" t="n">
         <v>7855631.5</v>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0.01263227533012468</v>
+        <v>0.01410437849585988</v>
       </c>
       <c r="G6" s="25" t="n">
         <v>0.0104347069321491</v>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="N52" s="54" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         <v>5.94</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>5.93</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.01</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.02</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.97</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-06-30
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1483,8 +1483,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="51" t="n">
-        <v>46113</v>
+      <c r="N10" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
         <is>
@@ -1500,16 +1500,16 @@
         <v>4.6</v>
       </c>
       <c r="R10" s="45" t="n">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="S10" s="45" t="n">
         <v>4.2</v>
       </c>
       <c r="T10" s="45" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="U10" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U10" s="21" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1562,8 +1562,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
-        <v>46113</v>
+      <c r="N11" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
         <is>
@@ -1576,19 +1576,19 @@
         </is>
       </c>
       <c r="Q11" s="45" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="R11" s="45" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="S11" s="45" t="n">
         <v>3.5</v>
       </c>
-      <c r="S11" s="45" t="n">
+      <c r="T11" s="45" t="n">
         <v>3.1</v>
       </c>
-      <c r="T11" s="45" t="n">
+      <c r="U11" s="21" t="n">
         <v>3.4</v>
-      </c>
-      <c r="U11" s="21" t="n">
-        <v>3.3</v>
       </c>
     </row>
     <row r="12">
@@ -1637,8 +1637,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="51" t="n">
-        <v>46113</v>
+      <c r="N12" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
         <is>
@@ -1651,19 +1651,19 @@
         </is>
       </c>
       <c r="Q12" s="45" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="R12" s="45" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S12" s="45" t="n">
         <v>3.4</v>
-      </c>
-      <c r="S12" s="45" t="n">
-        <v>3.2</v>
       </c>
       <c r="T12" s="45" t="n">
         <v>3.2</v>
       </c>
       <c r="U12" s="21" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2933,16 +2933,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.19</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.17</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.18</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.18</v>
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="31">
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4358,19 +4358,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.09</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.11</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.24</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.19</v>
       </c>
     </row>
     <row r="49">
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4433,19 +4433,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.15</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.29</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.23</v>
       </c>
     </row>
     <row r="50">
@@ -4499,7 +4499,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4512,19 +4512,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.5</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.51</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.46</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="N52" s="54" t="n">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4638,19 +4638,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>5.94</v>
+        <v>5.93</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>5.94</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>5.93</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.01</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.02</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -77,14 +77,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -372,13 +372,13 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1096,8 +1096,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="51" t="n">
-        <v>46143</v>
+      <c r="N5" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
@@ -1110,19 +1110,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
+        <v>98000</v>
+      </c>
+      <c r="R5" s="24" t="n">
         <v>122000</v>
       </c>
-      <c r="R5" s="24" t="n">
+      <c r="S5" s="24" t="n">
         <v>105000</v>
       </c>
-      <c r="S5" s="24" t="n">
+      <c r="T5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="T5" s="52" t="n">
+      <c r="U5" s="53" t="n">
         <v>66000</v>
-      </c>
-      <c r="U5" s="26" t="n">
-        <v>11000</v>
       </c>
     </row>
     <row r="6">
@@ -1290,8 +1290,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
-        <v>46113</v>
+      <c r="C8" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
@@ -1304,19 +1304,19 @@
         </is>
       </c>
       <c r="F8" s="45" t="n">
-        <v>0.44</v>
+        <v>0.54</v>
       </c>
       <c r="G8" s="45" t="n">
-        <v>0.46</v>
+        <v>0.26</v>
       </c>
       <c r="H8" s="45" t="n">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="I8" s="45" t="n">
-        <v>0.34</v>
+        <v>0.16</v>
       </c>
       <c r="J8" s="45" t="n">
-        <v>0.4</v>
+        <v>0.18</v>
       </c>
       <c r="K8" s="46" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1483,7 +1483,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="53" t="n">
+      <c r="N10" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1523,7 +1523,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="53" t="n">
+      <c r="C11" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
@@ -1562,7 +1562,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="53" t="n">
+      <c r="N11" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1598,7 +1598,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="53" t="n">
+      <c r="C12" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
@@ -1637,7 +1637,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="53" t="n">
+      <c r="N12" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -1677,7 +1677,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="53" t="n">
+      <c r="C13" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -1716,7 +1716,7 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="53" t="n">
+      <c r="N13" s="52" t="n">
         <v>46188</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
@@ -1752,7 +1752,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="53" t="n">
+      <c r="C14" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
@@ -1791,7 +1791,7 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="53" t="n">
+      <c r="N14" s="52" t="n">
         <v>46181</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
@@ -1831,7 +1831,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="53" t="n">
+      <c r="C15" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
@@ -1906,7 +1906,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="53" t="n">
+      <c r="C16" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
@@ -2123,7 +2123,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="53" t="n">
+      <c r="C19" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
@@ -2194,7 +2194,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="53" t="n">
+      <c r="C20" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
@@ -2273,7 +2273,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="53" t="n">
+      <c r="C21" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
@@ -2536,7 +2536,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="53" t="n">
+      <c r="N24" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
@@ -2611,7 +2611,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="53" t="n">
+      <c r="N25" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
@@ -2690,7 +2690,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="53" t="n">
+      <c r="N26" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
@@ -2765,7 +2765,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="53" t="n">
+      <c r="N27" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
@@ -2805,7 +2805,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="53" t="n">
+      <c r="C28" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2880,7 +2880,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="53" t="n">
+      <c r="C29" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2919,8 +2919,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="53" t="n">
-        <v>46202</v>
+      <c r="N29" s="52" t="n">
+        <v>46203</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.2</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.19</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.19</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.17</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.18</v>
       </c>
     </row>
     <row r="30">
@@ -2959,7 +2959,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="53" t="n">
+      <c r="C30" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -2998,8 +2998,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="53" t="n">
-        <v>46202</v>
+      <c r="N30" s="52" t="n">
+        <v>46203</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.18</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="31">
@@ -3034,7 +3034,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="53" t="n">
+      <c r="C31" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3717,7 +3717,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="53" t="n">
+      <c r="C40" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3788,7 +3788,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="53" t="n">
+      <c r="C41" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -4265,8 +4265,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="53" t="n">
-        <v>46199</v>
+      <c r="N47" s="52" t="n">
+        <v>46202</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4344,8 +4344,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="53" t="n">
-        <v>46199</v>
+      <c r="N48" s="52" t="n">
+        <v>46202</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4358,19 +4358,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.07</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.09</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.11</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.16</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.24</v>
       </c>
     </row>
     <row r="49">
@@ -4419,8 +4419,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="53" t="n">
-        <v>46199</v>
+      <c r="N49" s="52" t="n">
+        <v>46202</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4433,19 +4433,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.12</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.15</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.29</v>
       </c>
     </row>
     <row r="50">
@@ -4498,8 +4498,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="53" t="n">
-        <v>46199</v>
+      <c r="N50" s="52" t="n">
+        <v>46202</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,16 +4515,16 @@
         <v>4.38</v>
       </c>
       <c r="R50" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.5</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.51</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4573,7 +4573,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="53" t="n">
+      <c r="N51" s="52" t="n">
         <v>46195</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="N52" s="54" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4638,19 +4638,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.93</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>5.94</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>5.94</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>5.93</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.01</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -376,6 +376,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -946,8 +952,10 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="51" t="n">
-        <v>46143</v>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
+        </is>
       </c>
       <c r="O3" s="45" t="inlineStr">
         <is>
@@ -960,19 +968,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>172</v>
+        <v>1</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>179</v>
+        <v>1</v>
       </c>
       <c r="S3" s="24" t="n">
-        <v>214</v>
+        <v>1</v>
       </c>
       <c r="T3" s="24" t="n">
-        <v>-156</v>
+        <v>1</v>
       </c>
       <c r="U3" s="26" t="n">
-        <v>160</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1017,8 +1025,10 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="51" t="n">
-        <v>46143</v>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
+        </is>
       </c>
       <c r="O4" s="45" t="inlineStr">
         <is>
@@ -1031,19 +1041,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.003173541621976303</v>
+        <v>1</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.002170552418209925</v>
+        <v>1</v>
       </c>
       <c r="S4" s="38" t="n">
-        <v>0.001723735138309224</v>
+        <v>1</v>
       </c>
       <c r="T4" s="38" t="n">
-        <v>0.0007959067652075042</v>
+        <v>1</v>
       </c>
       <c r="U4" s="23" t="n">
-        <v>0.002047160512548336</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1171,8 +1181,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="51" t="n">
-        <v>46143</v>
+      <c r="N6" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
         <is>
@@ -1185,7 +1195,7 @@
         </is>
       </c>
       <c r="Q6" s="45" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="R6" s="45" t="n">
         <v>4.3</v>
@@ -1194,10 +1204,10 @@
         <v>4.3</v>
       </c>
       <c r="T6" s="45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U6" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U6" s="21" t="n">
-        <v>4.3</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1225,7 +1235,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>2.5438</v>
+        <v>1.1889</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1250,8 +1260,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="51" t="n">
-        <v>46143</v>
+      <c r="N7" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
         <is>
@@ -1264,19 +1274,19 @@
         </is>
       </c>
       <c r="Q7" s="45" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="R7" s="45" t="n">
         <v>8.1</v>
       </c>
-      <c r="R7" s="45" t="n">
+      <c r="S7" s="45" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="S7" s="45" t="n">
+      <c r="T7" s="45" t="n">
         <v>8</v>
       </c>
-      <c r="T7" s="45" t="n">
+      <c r="U7" s="21" t="n">
         <v>7.9</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>8.1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1329,8 +1339,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="51" t="n">
-        <v>46143</v>
+      <c r="N8" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
         <is>
@@ -1343,19 +1353,19 @@
         </is>
       </c>
       <c r="Q8" s="45" t="n">
-        <v>61.8</v>
+        <v>61.5</v>
       </c>
       <c r="R8" s="45" t="n">
         <v>61.8</v>
       </c>
       <c r="S8" s="45" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="T8" s="45" t="n">
         <v>61.9</v>
       </c>
-      <c r="T8" s="45" t="n">
+      <c r="U8" s="21" t="n">
         <v>62</v>
-      </c>
-      <c r="U8" s="21" t="n">
-        <v>62.1</v>
       </c>
     </row>
     <row r="9">
@@ -1408,8 +1418,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="51" t="n">
-        <v>46143</v>
+      <c r="N9" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1422,19 +1432,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
+        <v>59</v>
+      </c>
+      <c r="R9" s="45" t="n">
         <v>59.2</v>
       </c>
-      <c r="R9" s="45" t="n">
+      <c r="S9" s="45" t="n">
         <v>59.1</v>
       </c>
-      <c r="S9" s="45" t="n">
+      <c r="T9" s="45" t="n">
         <v>59.2</v>
       </c>
-      <c r="T9" s="45" t="n">
+      <c r="U9" s="21" t="n">
         <v>59.3</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>59.4</v>
       </c>
     </row>
     <row r="10">
@@ -1523,7 +1533,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="52" t="n">
+      <c r="C11" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
@@ -1598,7 +1608,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="52" t="n">
+      <c r="C12" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
@@ -1677,7 +1687,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="52" t="n">
+      <c r="C13" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -1717,7 +1727,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,16 +1743,16 @@
         <v>215000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>216000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>227000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>230000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>225000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>212000</v>
       </c>
     </row>
     <row r="14">
@@ -1752,7 +1762,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="52" t="n">
+      <c r="C14" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
@@ -1792,7 +1802,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46181</v>
+        <v>46188</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1805,19 +1815,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1821000</v>
+        <v>1814000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1812000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1800000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1786000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1771000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1785000</v>
       </c>
     </row>
     <row r="15">
@@ -1831,7 +1841,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="52" t="n">
+      <c r="C15" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
@@ -1870,8 +1880,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="51" t="n">
-        <v>46143</v>
+      <c r="N15" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
@@ -1890,10 +1900,10 @@
         <v>34.3</v>
       </c>
       <c r="S15" s="24" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="T15" s="24" t="n">
         <v>34.2</v>
-      </c>
-      <c r="T15" s="24" t="n">
-        <v>34.3</v>
       </c>
       <c r="U15" s="26" t="n">
         <v>34.3</v>
@@ -1906,7 +1916,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="52" t="n">
+      <c r="C16" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
@@ -2123,7 +2133,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="52" t="n">
+      <c r="C19" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
@@ -2194,7 +2204,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="52" t="n">
+      <c r="C20" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
@@ -2273,7 +2283,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="52" t="n">
+      <c r="C21" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
@@ -2536,7 +2546,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="52" t="n">
+      <c r="N24" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
@@ -2611,7 +2621,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="52" t="n">
+      <c r="N25" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
@@ -2690,7 +2700,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="52" t="n">
+      <c r="N26" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
@@ -2765,7 +2775,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="52" t="n">
+      <c r="N27" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
@@ -2805,7 +2815,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="52" t="n">
+      <c r="C28" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2819,10 +2829,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.04478479250211442</v>
+        <v>-0.04471097027607562</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>0.08466230868839419</v>
+        <v>0.08512722904348102</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>0.01344578206575542</v>
@@ -2880,7 +2890,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="52" t="n">
+      <c r="C29" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2894,10 +2904,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>-0.03493194678974276</v>
+        <v>-0.03444367263543068</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.1774520795721287</v>
+        <v>0.1779567725392831</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.01350347073984473</v>
@@ -2920,7 +2930,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2933,19 +2943,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.2</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.19</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.19</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="30">
@@ -2959,7 +2969,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="52" t="n">
+      <c r="C30" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -2973,10 +2983,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.04626546072493454</v>
+        <v>-0.04608210348174513</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>0.08424643897237227</v>
+        <v>0.08475262626842106</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>-0.002709178900039744</v>
@@ -2999,7 +3009,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3012,19 +3022,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.18</v>
       </c>
     </row>
     <row r="31">
@@ -3034,7 +3044,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="52" t="n">
+      <c r="C31" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3048,10 +3058,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>-0.04975533214668908</v>
+        <v>-0.04912893282642537</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.1528412169314068</v>
+        <v>0.1533794281326583</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>-0.0182024802287403</v>
@@ -3223,8 +3233,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="51" t="n">
-        <v>46143</v>
+      <c r="N33" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
         <is>
@@ -3237,19 +3247,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
-        <v>0.00320769847634339</v>
+        <v>0.003465742468675037</v>
       </c>
       <c r="R33" s="38" t="n">
+        <v>0.002673082063619381</v>
+      </c>
+      <c r="S33" s="38" t="n">
         <v>0.001606425702811221</v>
       </c>
-      <c r="S33" s="38" t="n">
+      <c r="T33" s="38" t="n">
         <v>0.002146498524282281</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.003230148048452453</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.003511615343057661</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -3312,7 +3322,7 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.006026690693604906</v>
+        <v>-0.006556386035628131</v>
       </c>
       <c r="R34" s="38" t="n">
         <v>-0.00215860068996659</v>
@@ -3391,7 +3401,7 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.001284834116984102</v>
+        <v>-0.001817056427606656</v>
       </c>
       <c r="R35" s="38" t="n">
         <v>-0.002486041249112891</v>
@@ -3466,7 +3476,7 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.006026690693604906</v>
+        <v>-0.006556386035628131</v>
       </c>
       <c r="R36" s="38" t="n">
         <v>-0.00215860068996659</v>
@@ -3527,8 +3537,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="51" t="n">
-        <v>46082</v>
+      <c r="N37" s="52" t="n">
+        <v>46113</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
         <is>
@@ -3541,19 +3551,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.007161347041441779</v>
+        <v>0.007712066688476016</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>0.003402954536404934</v>
+        <v>0.007421422032346747</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>-0.001489442391916063</v>
+        <v>0.003076263793446499</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.002589859586293541</v>
+        <v>-0.0009571631275075987</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.001285648567050157</v>
+        <v>-0.002574332320681272</v>
       </c>
     </row>
     <row r="38">
@@ -3602,8 +3612,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="51" t="n">
-        <v>46082</v>
+      <c r="N38" s="52" t="n">
+        <v>46113</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
         <is>
@@ -3616,19 +3626,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.006657391474145452</v>
+        <v>0.008448245026387436</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.007541366795841786</v>
+        <v>0.007298468298041118</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.008681655137469846</v>
+        <v>0.007907630509736042</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.01129232301425539</v>
+        <v>0.009370886912890657</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01271856657398832</v>
+        <v>0.01145670947467402</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -3677,8 +3687,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="51" t="n">
-        <v>46143</v>
+      <c r="N39" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
         <is>
@@ -3691,19 +3701,19 @@
         </is>
       </c>
       <c r="Q39" s="45" t="n">
+        <v>120.0835</v>
+      </c>
+      <c r="R39" s="54" t="n">
         <v>118.7792</v>
       </c>
-      <c r="R39" s="45" t="n">
+      <c r="S39" s="45" t="n">
         <v>119.0363</v>
       </c>
-      <c r="S39" s="45" t="n">
+      <c r="T39" s="45" t="n">
         <v>119.9199</v>
       </c>
-      <c r="T39" s="45" t="n">
+      <c r="U39" s="21" t="n">
         <v>117.906</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>119.2298</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3752,8 +3762,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="51" t="n">
-        <v>46143</v>
+      <c r="N40" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
         <is>
@@ -3766,19 +3776,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.004232386546914929</v>
+      </c>
+      <c r="R40" s="55" t="n">
         <v>-0.0291232297604588</v>
       </c>
-      <c r="R40" s="38" t="n">
+      <c r="S40" s="38" t="n">
         <v>-0.04111399852747133</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.05008673748247425</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.07796471263522881</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.07456792269916472</v>
       </c>
     </row>
     <row r="41">
@@ -4266,7 +4276,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4345,7 +4355,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4358,19 +4368,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.1</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.07</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.09</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.11</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.16</v>
       </c>
     </row>
     <row r="49">
@@ -4420,7 +4430,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4433,19 +4443,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.12</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.15</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4499,7 +4509,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4512,19 +4522,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>4.38</v>
+        <v>4.44</v>
       </c>
       <c r="R50" s="45" t="n">
         <v>4.38</v>
       </c>
       <c r="S50" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="T50" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.41</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.5</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4574,7 +4584,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46195</v>
+        <v>46202</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4587,19 +4597,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.49</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.47</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.52</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.48</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.53</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4624,8 +4634,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="54" t="n">
-        <v>46203</v>
+      <c r="N52" s="56" t="n">
+        <v>46204</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4638,19 +4648,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>5.97</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.93</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>5.94</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>5.94</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>5.93</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -952,10 +952,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
-        </is>
+      <c r="N3" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
         <is>
@@ -968,19 +966,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>1</v>
+        <v>129</v>
       </c>
       <c r="S3" s="24" t="n">
-        <v>1</v>
+        <v>148</v>
       </c>
       <c r="T3" s="24" t="n">
-        <v>1</v>
+        <v>214</v>
       </c>
       <c r="U3" s="26" t="n">
-        <v>1</v>
+        <v>-156</v>
       </c>
     </row>
     <row r="4">
@@ -1025,10 +1023,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PAYEMS' not found in values file."</t>
-        </is>
+      <c r="N4" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
         <is>
@@ -1041,19 +1037,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>1</v>
+        <v>0.003192872196771792</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>1</v>
+        <v>0.002706658759101061</v>
       </c>
       <c r="S4" s="38" t="n">
-        <v>1</v>
+        <v>0.001974950310754961</v>
       </c>
       <c r="T4" s="38" t="n">
-        <v>1</v>
+        <v>0.001723735138309224</v>
       </c>
       <c r="U4" s="23" t="n">
-        <v>1</v>
+        <v>0.0007959067652075042</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -2930,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2943,16 +2939,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.2</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.19</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.19</v>
@@ -3009,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3025,16 +3021,16 @@
         <v>2.23</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="31">
@@ -4276,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4355,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4368,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.1</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.07</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.09</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.11</v>
       </c>
     </row>
     <row r="49">
@@ -4430,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4443,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.12</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.15</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.17</v>
       </c>
     </row>
     <row r="50">
@@ -4509,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4522,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.44</v>
-      </c>
-      <c r="R50" s="45" t="n">
-        <v>4.38</v>
       </c>
       <c r="S50" s="45" t="n">
         <v>4.38</v>
       </c>
       <c r="T50" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.41</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2354,8 +2354,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="51" t="n">
-        <v>46143</v>
+      <c r="C22" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
         <is>
@@ -2368,19 +2368,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.508</v>
+        <v>16.949</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.395</v>
+        <v>16.506</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.536</v>
+        <v>16.588</v>
       </c>
       <c r="I22" s="24" t="n">
+        <v>16.676</v>
+      </c>
+      <c r="J22" s="24" t="n">
         <v>15.881</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>14.987</v>
       </c>
       <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2429,8 +2429,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
-        <v>46143</v>
+      <c r="C23" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
         <is>
@@ -2443,19 +2443,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.02898460387708034</v>
+        <v>0.04096548335585318</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>-0.06756526190069947</v>
+        <v>0.02885993891416824</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.09885558583106266</v>
+        <v>-0.05658875049763962</v>
       </c>
       <c r="I23" s="25" t="n">
+        <v>-0.09122615803814729</v>
+      </c>
+      <c r="J23" s="25" t="n">
         <v>-0.0327669163773677</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>-0.0603761755485893</v>
       </c>
       <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.1889</v>
+        <v>1.3565</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1489,7 +1489,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="52" t="n">
+      <c r="N10" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1568,7 +1568,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="52" t="n">
+      <c r="N11" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1643,7 +1643,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="52" t="n">
+      <c r="N12" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.19</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.23</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="31">
@@ -3533,7 +3533,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="52" t="n">
+      <c r="N37" s="51" t="n">
         <v>46113</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3608,7 +3608,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="52" t="n">
+      <c r="N38" s="51" t="n">
         <v>46113</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.1</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.07</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.09</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.12</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.15</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.44</v>
-      </c>
-      <c r="S50" s="45" t="n">
-        <v>4.38</v>
       </c>
       <c r="T50" s="45" t="n">
         <v>4.38</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.4</v>
+        <v>4.38</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,16 +4644,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.02</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>5.97</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>5.93</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>5.94</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>5.94</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-07-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1102,7 +1102,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="52" t="n">
+      <c r="N5" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.3565</v>
+        <v>1.2603</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -1296,7 +1296,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="52" t="n">
+      <c r="C8" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.24</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.23</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.23</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="31">
@@ -3683,7 +3683,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="52" t="n">
+      <c r="N39" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3758,7 +3758,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="52" t="n">
+      <c r="N40" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
@@ -4145,8 +4145,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="51" t="n">
-        <v>46113</v>
+      <c r="C46" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
         <is>
@@ -4159,19 +4159,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>327101</v>
+        <v>317677</v>
       </c>
       <c r="G46" s="24" t="n">
+        <v>328187</v>
+      </c>
+      <c r="H46" s="24" t="n">
         <v>318776</v>
       </c>
-      <c r="H46" s="24" t="n">
+      <c r="I46" s="24" t="n">
         <v>311803</v>
       </c>
-      <c r="I46" s="24" t="n">
+      <c r="J46" s="24" t="n">
         <v>299806</v>
-      </c>
-      <c r="J46" s="24" t="n">
-        <v>285282</v>
       </c>
       <c r="K46" s="46" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4232,8 +4232,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="51" t="n">
-        <v>46113</v>
+      <c r="C47" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
         <is>
@@ -4246,19 +4246,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>0.02611551685195868</v>
+        <v>-0.03202442509910508</v>
       </c>
       <c r="G47" s="38" t="n">
+        <v>0.02952229778904303</v>
+      </c>
+      <c r="H47" s="38" t="n">
         <v>0.0223634795046872</v>
       </c>
-      <c r="H47" s="38" t="n">
+      <c r="I47" s="38" t="n">
         <v>0.04001587693375042</v>
       </c>
-      <c r="I47" s="38" t="n">
+      <c r="J47" s="38" t="n">
         <v>0.05091102838594797</v>
-      </c>
-      <c r="J47" s="38" t="n">
-        <v>-0.01458356361224711</v>
       </c>
       <c r="K47" s="46" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4311,8 +4311,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="51" t="n">
-        <v>46113</v>
+      <c r="C48" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
         <is>
@@ -4325,19 +4325,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>382982</v>
+        <v>395263</v>
       </c>
       <c r="G48" s="24" t="n">
+        <v>382758</v>
+      </c>
+      <c r="H48" s="24" t="n">
         <v>375360</v>
       </c>
-      <c r="H48" s="24" t="n">
+      <c r="I48" s="24" t="n">
         <v>366783</v>
       </c>
-      <c r="I48" s="24" t="n">
+      <c r="J48" s="24" t="n">
         <v>353991</v>
-      </c>
-      <c r="J48" s="24" t="n">
-        <v>361360</v>
       </c>
       <c r="K48" s="46" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.1</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.07</v>
       </c>
     </row>
     <row r="49">
@@ -4386,8 +4386,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="51" t="n">
-        <v>46113</v>
+      <c r="C49" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
         <is>
@@ -4400,19 +4400,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.02030583972719513</v>
+        <v>0.03267077370035376</v>
       </c>
       <c r="G49" s="38" t="n">
+        <v>0.01970907928388743</v>
+      </c>
+      <c r="H49" s="38" t="n">
         <v>0.02338439894978772</v>
       </c>
-      <c r="H49" s="38" t="n">
+      <c r="I49" s="38" t="n">
         <v>0.03613651194521905</v>
       </c>
-      <c r="I49" s="38" t="n">
+      <c r="J49" s="38" t="n">
         <v>-0.02039240646446761</v>
-      </c>
-      <c r="J49" s="38" t="n">
-        <v>0.02260507340706108</v>
       </c>
       <c r="K49" s="46" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.14</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.12</v>
       </c>
     </row>
     <row r="50">
@@ -4465,8 +4465,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="51" t="n">
-        <v>46113</v>
+      <c r="C50" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
         <is>
@@ -4479,19 +4479,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>27806</v>
+        <v>28899</v>
       </c>
       <c r="G50" s="24" t="n">
+        <v>28342</v>
+      </c>
+      <c r="H50" s="24" t="n">
         <v>29493</v>
       </c>
-      <c r="H50" s="24" t="n">
+      <c r="I50" s="24" t="n">
         <v>27541</v>
       </c>
-      <c r="I50" s="24" t="n">
+      <c r="J50" s="24" t="n">
         <v>28077</v>
-      </c>
-      <c r="J50" s="24" t="n">
-        <v>26539</v>
       </c>
       <c r="K50" s="46" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,16 +4518,16 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.44</v>
-      </c>
-      <c r="T50" s="45" t="n">
-        <v>4.38</v>
       </c>
       <c r="U50" s="21" t="n">
         <v>4.38</v>
@@ -4540,8 +4540,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="51" t="n">
-        <v>46113</v>
+      <c r="C51" s="52" t="n">
+        <v>46143</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
         <is>
@@ -4554,19 +4554,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>-0.05720001356254023</v>
+        <v>0.01965281208101044</v>
       </c>
       <c r="G51" s="38" t="n">
+        <v>-0.03902620960905978</v>
+      </c>
+      <c r="H51" s="38" t="n">
         <v>0.07087614828800692</v>
       </c>
-      <c r="H51" s="38" t="n">
+      <c r="I51" s="38" t="n">
         <v>-0.01909035865655162</v>
       </c>
-      <c r="I51" s="38" t="n">
+      <c r="J51" s="38" t="n">
         <v>0.05795244734164817</v>
-      </c>
-      <c r="J51" s="38" t="n">
-        <v>-0.03858136501956233</v>
       </c>
       <c r="K51" s="46" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46205</v>
+        <v>46210</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.03</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.02</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>5.97</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>5.93</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.94</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-09
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -77,14 +77,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -372,19 +372,19 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -952,7 +952,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="52" t="n">
+      <c r="N3" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
@@ -1023,7 +1023,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="52" t="n">
+      <c r="N4" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
@@ -1127,7 +1127,7 @@
       <c r="T5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="U5" s="53" t="n">
+      <c r="U5" s="52" t="n">
         <v>66000</v>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="52" t="n">
+      <c r="N6" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
@@ -1256,7 +1256,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="52" t="n">
+      <c r="N7" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
@@ -1335,7 +1335,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="52" t="n">
+      <c r="N8" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
@@ -1414,7 +1414,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="52" t="n">
+      <c r="N9" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
@@ -1722,8 +1722,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="52" t="n">
-        <v>46195</v>
+      <c r="N13" s="53" t="n">
+        <v>46202</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1739,16 +1739,16 @@
         <v>215000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>217000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>216000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>227000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>230000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>225000</v>
       </c>
     </row>
     <row r="14">
@@ -1797,8 +1797,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="52" t="n">
-        <v>46188</v>
+      <c r="N14" s="53" t="n">
+        <v>46195</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1814,16 +1814,16 @@
         <v>1814000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1806000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1812000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1800000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1786000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1771000</v>
       </c>
     </row>
     <row r="15">
@@ -1876,7 +1876,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="52" t="n">
+      <c r="N15" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -2354,7 +2354,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="53" t="n">
         <v>46174</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2429,7 +2429,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="53" t="n">
         <v>46174</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2503,8 +2503,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
-        <v>46113</v>
+      <c r="C24" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -2517,19 +2517,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>0.008703141071390919</v>
+        <v>-0.003925763540534311</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.007795687606403368</v>
+        <v>0.008629783986034756</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.000649622056177801</v>
+        <v>0.008052444128709091</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.001151758694675653</v>
+        <v>0.000857114913422663</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.005868657238478958</v>
+        <v>0.00136865468313907</v>
       </c>
       <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2582,8 +2582,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="51" t="n">
-        <v>46113</v>
+      <c r="C25" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
         <is>
@@ -2596,19 +2596,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.00239671579372791</v>
+        <v>0.001344310133821303</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.003140798606426021</v>
+        <v>0.002443819508178846</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.001559499677996179</v>
+        <v>0.003197428618906484</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.0006476910419241921</v>
+        <v>0.001618006847893483</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.001971303273869296</v>
+        <v>0.0006997747068799853</v>
       </c>
       <c r="K25" s="46" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2925,8 +2925,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="52" t="n">
-        <v>46210</v>
+      <c r="N29" s="53" t="n">
+        <v>46211</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -3004,8 +3004,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="52" t="n">
-        <v>46210</v>
+      <c r="N30" s="53" t="n">
+        <v>46211</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,16 +3021,16 @@
         <v>2.25</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.24</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.23</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.23</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="31">
@@ -3229,7 +3229,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="52" t="n">
+      <c r="N33" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
@@ -3874,7 +3874,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
         <is>
@@ -3887,19 +3887,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>4170000</v>
+        <v>4090000</v>
       </c>
       <c r="G42" s="39" t="n">
+        <v>4190000</v>
+      </c>
+      <c r="H42" s="39" t="n">
         <v>4040000</v>
       </c>
-      <c r="H42" s="39" t="n">
+      <c r="I42" s="39" t="n">
         <v>4010000</v>
       </c>
-      <c r="I42" s="39" t="n">
+      <c r="J42" s="39" t="n">
         <v>4130000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4020000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3945,7 +3945,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>0.03217821782178218</v>
+        <v>0.02763819095477387</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4145,7 +4145,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="52" t="n">
+      <c r="C46" s="53" t="n">
         <v>46143</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4232,7 +4232,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="52" t="n">
+      <c r="C47" s="53" t="n">
         <v>46143</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4271,8 +4271,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="52" t="n">
-        <v>46209</v>
+      <c r="N47" s="53" t="n">
+        <v>46210</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4311,7 +4311,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="52" t="n">
+      <c r="C48" s="53" t="n">
         <v>46143</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4350,8 +4350,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="52" t="n">
-        <v>46209</v>
+      <c r="N48" s="53" t="n">
+        <v>46210</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.13</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.14</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.1</v>
       </c>
     </row>
     <row r="49">
@@ -4386,7 +4386,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="52" t="n">
+      <c r="C49" s="53" t="n">
         <v>46143</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4425,8 +4425,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="52" t="n">
-        <v>46209</v>
+      <c r="N49" s="53" t="n">
+        <v>46210</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.19</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.14</v>
       </c>
     </row>
     <row r="50">
@@ -4465,7 +4465,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="52" t="n">
+      <c r="C50" s="53" t="n">
         <v>46143</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4504,8 +4504,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="52" t="n">
-        <v>46209</v>
+      <c r="N50" s="53" t="n">
+        <v>46210</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.44</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.38</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4540,7 +4540,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="52" t="n">
+      <c r="C51" s="53" t="n">
         <v>46143</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4579,8 +4579,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="52" t="n">
-        <v>46202</v>
+      <c r="N51" s="53" t="n">
+        <v>46209</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4593,19 +4593,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.43</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.49</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.47</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.52</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.48</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.1</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.04</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.03</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.02</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>5.97</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2354,7 +2354,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="53" t="n">
+      <c r="C22" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2429,7 +2429,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="53" t="n">
+      <c r="C23" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.19</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.25</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.24</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.23</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.23</v>
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="Q47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="R47" s="45" t="n">
         <v>3.63</v>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.13</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.14</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.14</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.24</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.19</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.48</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.44</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.12</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.1</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.04</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.03</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.02</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.19</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.23</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.25</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.25</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4288,7 +4288,7 @@
         <v>3.62</v>
       </c>
       <c r="R47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="S47" s="45" t="n">
         <v>3.63</v>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.13</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.14</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.17</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.23</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.24</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.49</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.48</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.1</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.12</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.1</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.04</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.03</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2089,8 +2089,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="51" t="n">
-        <v>46143</v>
+      <c r="N18" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
         <is>
@@ -2103,19 +2103,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>-0.004224816530380648</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>0.004729142286413968</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>0.006400377846336402</v>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="T18" s="38" t="n">
         <v>0.008651438343614481</v>
       </c>
-      <c r="T18" s="38" t="n">
+      <c r="U18" s="23" t="n">
         <v>0.00267003074209704</v>
-      </c>
-      <c r="U18" s="23" t="n">
-        <v>0.00170842649932057</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2164,8 +2164,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="51" t="n">
-        <v>46143</v>
+      <c r="N19" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
         <is>
@@ -2178,19 +2178,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.03463530729385406</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.04166614684049648</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.03779245836741563</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.03285957752865201</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v>0.0243400411037322</v>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.02391201432150015</v>
       </c>
     </row>
     <row r="20">
@@ -2239,8 +2239,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="51" t="n">
-        <v>46143</v>
+      <c r="N20" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
         <is>
@@ -2253,19 +2253,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
+        <v>-0.0001666066684318235</v>
+      </c>
+      <c r="R20" s="38" t="n">
         <v>0.002080954496262777</v>
       </c>
-      <c r="R20" s="38" t="n">
+      <c r="S20" s="38" t="n">
         <v>0.00376460730477457</v>
       </c>
-      <c r="S20" s="38" t="n">
+      <c r="T20" s="38" t="n">
         <v>0.001957950538511444</v>
       </c>
-      <c r="T20" s="38" t="n">
+      <c r="U20" s="23" t="n">
         <v>0.002160502174024082</v>
-      </c>
-      <c r="U20" s="23" t="n">
-        <v>0.002950448142634121</v>
       </c>
     </row>
     <row r="21">
@@ -2314,8 +2314,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="51" t="n">
-        <v>46143</v>
+      <c r="N21" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
+        <v>0.02565785056369746</v>
+      </c>
+      <c r="R21" s="38" t="n">
         <v>0.02822942063611032</v>
       </c>
-      <c r="R21" s="38" t="n">
+      <c r="S21" s="38" t="n">
         <v>0.02743309430968526</v>
       </c>
-      <c r="S21" s="38" t="n">
+      <c r="T21" s="38" t="n">
         <v>0.0260216770548682</v>
       </c>
-      <c r="T21" s="38" t="n">
+      <c r="U21" s="23" t="n">
         <v>0.02472462476764023</v>
-      </c>
-      <c r="U21" s="23" t="n">
-        <v>0.02512028782828883</v>
       </c>
     </row>
     <row r="22">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.19</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.23</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.25</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.25</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -4145,7 +4145,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="53" t="n">
+      <c r="C46" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4232,7 +4232,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="53" t="n">
+      <c r="C47" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
         <v>3.62</v>
       </c>
       <c r="S47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="T47" s="45" t="n">
         <v>3.63</v>
@@ -4311,7 +4311,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="53" t="n">
+      <c r="C48" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.14</v>
       </c>
     </row>
     <row r="49">
@@ -4386,7 +4386,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="53" t="n">
+      <c r="C49" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.23</v>
       </c>
     </row>
     <row r="50">
@@ -4465,7 +4465,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="53" t="n">
+      <c r="C50" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.48</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.49</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4540,7 +4540,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="53" t="n">
+      <c r="C51" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D51" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2393,8 +2393,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="51" t="n">
-        <v>46143</v>
+      <c r="N22" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
         <is>
@@ -2407,19 +2407,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>0.01056335771195616</v>
+        <v>-0.002770682989280293</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.01055174826080751</v>
+        <v>0.006223162212395161</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.00747866036701561</v>
+        <v>0.01052427058709249</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.005037122543746886</v>
+        <v>0.00783922090807021</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.00577866905905311</v>
+        <v>0.004827242437757562</v>
       </c>
     </row>
     <row r="23">
@@ -2463,8 +2463,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="51" t="n">
-        <v>46143</v>
+      <c r="N23" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
         <is>
@@ -2477,19 +2477,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.06416339864869426</v>
+        <v>0.05507672194780078</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.05659137855135278</v>
+        <v>0.05972204410305572</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.04273411907736988</v>
+        <v>0.05672005688937049</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.03375091916105041</v>
+        <v>0.04288946675222042</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.03036323703328262</v>
+        <v>0.0335350428042339</v>
       </c>
     </row>
     <row r="24">
@@ -2503,7 +2503,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="53" t="n">
+      <c r="C24" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2582,7 +2582,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="53" t="n">
+      <c r="C25" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.18</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.19</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.23</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.25</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.25</v>
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4294,10 +4294,10 @@
         <v>3.62</v>
       </c>
       <c r="T47" s="45" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="48">
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.19</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.55</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.48</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.1</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.12</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.1</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.04</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-16
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="N13" s="53" t="n">
-        <v>46202</v>
+        <v>46209</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1736,19 +1736,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>215000</v>
+        <v>208000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>216000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>217000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>216000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>227000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>230000</v>
       </c>
     </row>
     <row r="14">
@@ -1798,7 +1798,7 @@
         </is>
       </c>
       <c r="N14" s="53" t="n">
-        <v>46195</v>
+        <v>46202</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1814000</v>
+        <v>1805000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1821000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1806000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1812000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1800000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1786000</v>
       </c>
     </row>
     <row r="15">
@@ -1963,8 +1963,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="51" t="n">
-        <v>46143</v>
+      <c r="C17" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
@@ -1977,19 +1977,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.008809356490312226</v>
+        <v>0.002186794214449339</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.004009214695237295</v>
+        <v>0.01024770220406612</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>0.006742589318751824</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>0.01717978949867671</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>0.009223924204530221</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>-0.0002912686109073359</v>
       </c>
       <c r="K17" s="46" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2050,8 +2050,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="51" t="n">
-        <v>46143</v>
+      <c r="C18" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
@@ -2064,19 +2064,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.06876462422050805</v>
+        <v>0.06719163968207242</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.0478848128984749</v>
+        <v>0.07328488075094505</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.05073763706982706</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.04240611939906461</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.04174261321715912</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.03267862666254253</v>
       </c>
       <c r="K18" s="46" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.18</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.19</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="Q47" s="45" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="R47" s="45" t="n">
         <v>3.62</v>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.19</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.27</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.31</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.62</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.56</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.55</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4579,7 +4579,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="53" t="n">
+      <c r="N51" s="51" t="n">
         <v>46209</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,16 +4644,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.18</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.14</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.12</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.1</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-07-17
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.2603</v>
+        <v>1.7389</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.18</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="31">
@@ -3119,8 +3119,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n">
-        <v>46143</v>
+      <c r="C32" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
         <is>
@@ -3133,19 +3133,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.001351100878947076</v>
+        <v>0.000769301271638545</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.008675818407061886</v>
+        <v>0.001376689618002747</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>-0.003158432671926059</v>
+        <v>0.007896301019906238</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>0.00816625215701583</v>
+        <v>-0.003032583346986972</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>-0.003651443778505348</v>
+        <v>0.008783754359711349</v>
       </c>
       <c r="K32" s="46" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3190,8 +3190,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n">
-        <v>46143</v>
+      <c r="C33" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
         <is>
@@ -3204,19 +3204,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.01665915585026556</v>
+        <v>0.01144084707598163</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01365696311304797</v>
+        <v>0.01579846581257943</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.005808567662044093</v>
+        <v>0.01277293407655064</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.008407575522283481</v>
+        <v>0.005708607646050407</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.01058115399336634</v>
+        <v>0.008180076419915847</v>
       </c>
       <c r="K33" s="46" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3269,8 +3269,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
-        <v>46143</v>
+      <c r="C34" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
         <is>
@@ -3283,19 +3283,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.16630000000001</v>
+        <v>76.0937</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.1289</v>
+        <v>76.1019</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>75.53879999999999</v>
+        <v>76.0625</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.84699999999999</v>
+        <v>75.5313</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.30500000000001</v>
+        <v>75.82989999999999</v>
       </c>
       <c r="K34" s="46" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3423,8 +3423,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
-        <v>46143</v>
+      <c r="C36" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
@@ -3437,19 +3437,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1177</v>
+        <v>1427</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1392</v>
+        <v>1199</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1414</v>
+      </c>
+      <c r="I36" s="24" t="n">
         <v>1522</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="J36" s="24" t="n">
         <v>1346</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1385</v>
       </c>
       <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3494,8 +3494,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
-        <v>46143</v>
+      <c r="C37" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
@@ -3508,19 +3508,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>-0.08688906128782002</v>
+        <v>0.03480783176214648</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.005714285714285714</v>
+        <v>-0.06982156710628394</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I37" s="25" t="n">
         <v>0.1307578008915305</v>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="J37" s="25" t="n">
         <v>-0.09725016767270288</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>0.02365114560236511</v>
       </c>
       <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3573,8 +3573,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n">
-        <v>46143</v>
+      <c r="C38" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
         <is>
@@ -3587,19 +3587,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
+        <v>1367</v>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>1410</v>
       </c>
-      <c r="G38" s="24" t="n">
+      <c r="H38" s="24" t="n">
         <v>1423</v>
       </c>
-      <c r="H38" s="24" t="n">
+      <c r="I38" s="24" t="n">
         <v>1363</v>
       </c>
-      <c r="I38" s="24" t="n">
+      <c r="J38" s="24" t="n">
         <v>1540</v>
-      </c>
-      <c r="J38" s="24" t="n">
-        <v>1393</v>
       </c>
       <c r="K38" s="46" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3644,8 +3644,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="51" t="n">
-        <v>46143</v>
+      <c r="C39" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
         <is>
@@ -3658,19 +3658,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
+        <v>-0.0228734810578985</v>
+      </c>
+      <c r="G39" s="38" t="n">
         <v>-0.00423728813559322</v>
       </c>
-      <c r="G39" s="38" t="n">
+      <c r="H39" s="38" t="n">
         <v>-0.01522491349480969</v>
       </c>
-      <c r="H39" s="38" t="n">
+      <c r="I39" s="38" t="n">
         <v>-0.08646112600536193</v>
       </c>
-      <c r="I39" s="38" t="n">
+      <c r="J39" s="38" t="n">
         <v>0.06500691562932227</v>
-      </c>
-      <c r="J39" s="38" t="n">
-        <v>-0.04784688995215311</v>
       </c>
       <c r="K39" s="46" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3833,8 +3833,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="51" t="n">
-        <v>46143</v>
+      <c r="N41" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
         <is>
@@ -3847,19 +3847,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>0.01261261261261248</v>
+        <v>-0.005924170616113722</v>
       </c>
       <c r="R41" s="38" t="n">
-        <v>0.03480422622747037</v>
+        <v>0.01199040767386084</v>
       </c>
       <c r="S41" s="38" t="n">
-        <v>0.01578282828282829</v>
+        <v>0.03538175046554937</v>
       </c>
       <c r="T41" s="38" t="n">
+        <v>0.01704545454545436</v>
+      </c>
+      <c r="U41" s="23" t="n">
         <v>0.01930501930501927</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0.005174644243208348</v>
       </c>
     </row>
     <row r="42">
@@ -3908,8 +3908,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="51" t="n">
-        <v>46143</v>
+      <c r="N42" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
         <is>
@@ -3922,19 +3922,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.1121372031662269</v>
+        <v>0.1017728168089297</v>
       </c>
       <c r="R42" s="38" t="n">
-        <v>0.09108781127129754</v>
+        <v>0.1134564643799473</v>
       </c>
       <c r="S42" s="38" t="n">
-        <v>0.05508196721311479</v>
+        <v>0.09305373525557023</v>
       </c>
       <c r="T42" s="38" t="n">
+        <v>0.05639344262295078</v>
+      </c>
+      <c r="U42" s="23" t="n">
         <v>0.03800786369593716</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.02506596306068609</v>
       </c>
     </row>
     <row r="43">
@@ -3983,8 +3983,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="51" t="n">
-        <v>46143</v>
+      <c r="N43" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
         <is>
@@ -3997,19 +3997,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.01895734597156395</v>
+        <v>0.003326679973386648</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>0.0200276243093922</v>
+        <v>0.01691474966170503</v>
       </c>
       <c r="S43" s="38" t="n">
+        <v>0.02071823204419898</v>
+      </c>
+      <c r="T43" s="38" t="n">
         <v>0.009059233449477455</v>
       </c>
-      <c r="T43" s="38" t="n">
+      <c r="U43" s="23" t="n">
         <v>0.009852216748768461</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>0.004950495049504955</v>
       </c>
     </row>
     <row r="44">
@@ -4058,8 +4058,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="51" t="n">
-        <v>46143</v>
+      <c r="N44" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
         <is>
@@ -4072,19 +4072,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.0673758865248227</v>
+        <v>0.07102272727272727</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>0.04234297812279464</v>
+        <v>0.06595744680851072</v>
       </c>
       <c r="S44" s="38" t="n">
+        <v>0.04304869442484138</v>
+      </c>
+      <c r="T44" s="38" t="n">
         <v>0.0225988700564973</v>
       </c>
-      <c r="T44" s="38" t="n">
+      <c r="U44" s="23" t="n">
         <v>0.009852216748768513</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>0.002115655853314407</v>
       </c>
     </row>
     <row r="45">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4288,7 +4288,7 @@
         <v>3.63</v>
       </c>
       <c r="R47" s="45" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="S47" s="45" t="n">
         <v>3.62</v>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.16</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.3</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.27</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.58</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.62</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.56</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.54</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.56</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4579,8 +4579,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="51" t="n">
-        <v>46209</v>
+      <c r="N51" s="53" t="n">
+        <v>46216</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4593,19 +4593,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.49</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.43</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.49</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.47</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.52</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.7389</v>
+        <v>1.6817</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
         <v>3.63</v>
       </c>
       <c r="S47" s="45" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="T47" s="45" t="n">
         <v>3.62</v>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.13</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.16</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.3</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.27</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.58</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.62</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.56</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.54</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.15</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.18</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.18</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.14</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.1</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-20
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.16</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.15</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.18</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.18</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.14</v>
+        <v>6.18</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-21
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2089,7 +2089,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="53" t="n">
+      <c r="N18" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2164,7 +2164,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="53" t="n">
+      <c r="N19" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2239,7 +2239,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="53" t="n">
+      <c r="N20" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2314,7 +2314,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="53" t="n">
+      <c r="N21" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.25</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4294,7 +4294,7 @@
         <v>3.63</v>
       </c>
       <c r="T47" s="45" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="U47" s="21" t="n">
         <v>3.62</v>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.13</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4442,16 +4442,16 @@
         <v>4.28</v>
       </c>
       <c r="R49" s="45" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.37</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.3</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.57</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.58</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.62</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.56</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,16 +4644,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.16</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.15</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.18</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.18</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-07-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2393,7 +2393,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="53" t="n">
+      <c r="N22" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2463,7 +2463,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="53" t="n">
+      <c r="N23" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4297,7 +4297,7 @@
         <v>3.63</v>
       </c>
       <c r="U47" s="21" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="48">
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.13</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>4.28</v>
+        <v>4.33</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>4.28</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.31</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.37</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.57</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.58</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.62</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-23
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="N13" s="53" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1736,19 +1736,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>208000</v>
+        <v>187000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>216000</v>
+        <v>209000</v>
       </c>
       <c r="S13" s="24" t="n">
         <v>217000</v>
       </c>
       <c r="T13" s="24" t="n">
+        <v>217000</v>
+      </c>
+      <c r="U13" s="26" t="n">
         <v>216000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>227000</v>
       </c>
     </row>
     <row r="14">
@@ -1798,7 +1798,7 @@
         </is>
       </c>
       <c r="N14" s="53" t="n">
-        <v>46202</v>
+        <v>46209</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1805000</v>
+        <v>1796000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1798000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1821000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1806000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1812000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1800000</v>
       </c>
     </row>
     <row r="15">
@@ -1963,7 +1963,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="53" t="n">
+      <c r="C17" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2050,7 +2050,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="53" t="n">
+      <c r="C18" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.16</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.13</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.18</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.33</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>4.28</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>4.28</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.57</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.55</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.58</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4579,7 +4579,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="53" t="n">
+      <c r="N51" s="51" t="n">
         <v>46216</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R52" s="9" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.21</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.14</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.16</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.18</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-24
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3021,16 +3021,16 @@
         <v>2.28</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="31">
@@ -3119,7 +3119,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="53" t="n">
+      <c r="C32" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3190,7 +3190,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="53" t="n">
+      <c r="C33" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3269,7 +3269,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="53" t="n">
+      <c r="C34" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -3423,7 +3423,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="53" t="n">
+      <c r="C36" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3494,7 +3494,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="53" t="n">
+      <c r="C37" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3573,7 +3573,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="53" t="n">
+      <c r="C38" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1367</v>
+        <v>1374</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1410</v>
@@ -3644,7 +3644,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="53" t="n">
+      <c r="C39" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3658,7 +3658,7 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>-0.0228734810578985</v>
+        <v>-0.0178699070764832</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>-0.00423728813559322</v>
@@ -3723,8 +3723,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="51" t="n">
-        <v>46143</v>
+      <c r="C40" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
         <is>
@@ -3737,19 +3737,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>580</v>
+        <v>628</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>626</v>
+        <v>618</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>664</v>
+        <v>646</v>
       </c>
       <c r="I40" s="24" t="n">
+        <v>659</v>
+      </c>
+      <c r="J40" s="24" t="n">
         <v>630</v>
-      </c>
-      <c r="J40" s="24" t="n">
-        <v>576</v>
       </c>
       <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3794,8 +3794,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="51" t="n">
-        <v>46143</v>
+      <c r="C41" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
         <is>
@@ -3808,19 +3808,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.06752411575562701</v>
+        <v>-0.0556390977443609</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.1069900142653352</v>
+        <v>-0.006430868167202572</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>0.01219512195121951</v>
+        <v>-0.07845934379457917</v>
       </c>
       <c r="I41" s="38" t="n">
+        <v>0.004573170731707317</v>
+      </c>
+      <c r="J41" s="38" t="n">
         <v>-0.0171606864274571</v>
-      </c>
-      <c r="J41" s="38" t="n">
-        <v>-0.1338345864661654</v>
       </c>
       <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -3833,7 +3833,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="53" t="n">
+      <c r="N41" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3908,7 +3908,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="53" t="n">
+      <c r="N42" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3983,7 +3983,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="53" t="n">
+      <c r="N43" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4058,7 +4058,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="53" t="n">
+      <c r="N44" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.16</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.13</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.33</v>
-      </c>
-      <c r="S49" s="45" t="n">
-        <v>4.28</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>4.28</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.26</v>
+        <v>4.28</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.57</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.55</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4579,8 +4579,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="51" t="n">
-        <v>46216</v>
+      <c r="N51" s="53" t="n">
+        <v>46223</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4593,19 +4593,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.55</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.49</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.43</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.49</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.47</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-25
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.28</v>
+        <v>2.26</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.28</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.25</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.21</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.16</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,16 +4439,16 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.33</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>4.28</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.28</v>
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.55</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.57</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.25</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.23</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.21</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.14</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.16</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.6817</v>
+        <v>1.5811</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -2811,8 +2811,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="51" t="n">
-        <v>46143</v>
+      <c r="C28" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
         <is>
@@ -2825,19 +2825,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>-0.04471097027607562</v>
+        <v>0.003194428628793045</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>-0.04043224342735219</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>0.08512722904348102</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>0.01344578206575542</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>-0.01169466364559735</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>-0.004254034642219184</v>
       </c>
       <c r="K28" s="46" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2886,8 +2886,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="51" t="n">
-        <v>46143</v>
+      <c r="C29" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
         <is>
@@ -2900,19 +2900,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>-0.03444367263543068</v>
+        <v>0.07380974528565151</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>-0.03011895869723805</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>0.1779567725392831</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.01350347073984473</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.07567733047604469</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.09883411459674789</v>
       </c>
       <c r="K29" s="46" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2965,8 +2965,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="51" t="n">
-        <v>46143</v>
+      <c r="C30" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
         <is>
@@ -2979,19 +2979,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>-0.04608210348174513</v>
+        <v>0.003010246541142125</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>-0.04303028794703967</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>0.08475262626842106</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>-0.002709178900039744</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>-0.01222345960141613</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>0.002385879326488816</v>
       </c>
       <c r="K30" s="46" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3040,8 +3040,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="51" t="n">
-        <v>46143</v>
+      <c r="C31" s="53" t="n">
+        <v>46174</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
         <is>
@@ -3054,19 +3054,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>-0.04912893282642537</v>
+        <v>0.05654575401758045</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>-0.04608686484039221</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>0.1533794281326583</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>-0.0182024802287403</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>0.07288240242929306</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.09283155684402497</v>
       </c>
       <c r="K31" s="46" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.25</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.23</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.21</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.14</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>1.5811</v>
+        <v>1.54</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.2392</v>
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.22</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.26</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.28</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.28</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.21</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.18</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.46</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.33</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.28</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.71</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.6</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.55</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.28</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.25</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.23</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.21</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-29
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,16 +2942,16 @@
         <v>2.24</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.26</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.28</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.28</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="31">
@@ -3533,8 +3533,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="51" t="n">
-        <v>46113</v>
+      <c r="N37" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
         <is>
@@ -3547,19 +3547,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.007712066688476016</v>
+        <v>0.006366672272541729</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>0.007421422032346747</v>
+        <v>0.008345748997662161</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>0.003076263793446499</v>
+        <v>0.007532973922912856</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>-0.0009571631275075987</v>
+        <v>0.00315552998212576</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.002574332320681272</v>
+        <v>-0.0009081874474428098</v>
       </c>
     </row>
     <row r="38">
@@ -3608,8 +3608,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="51" t="n">
-        <v>46113</v>
+      <c r="N38" s="53" t="n">
+        <v>46143</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
         <is>
@@ -3622,19 +3622,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.008448245026387436</v>
+        <v>0.01114021218302297</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.007298468298041118</v>
+        <v>0.009369704722440333</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.007907630509736042</v>
+        <v>0.007600606583937686</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.009370886912890657</v>
+        <v>0.008095298145032572</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.01145670947467402</v>
+        <v>0.009482201947111055</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.33</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.21</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.46</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.37</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.33</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="53" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.71</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.63</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.6</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.26</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.28</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.25</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.23</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-30
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -77,14 +77,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -369,22 +369,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="C3" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D3" s="45" t="inlineStr">
         <is>
@@ -927,19 +927,19 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
+        <v>24270.599</v>
+      </c>
+      <c r="G3" s="24" t="n">
         <v>24180.419</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="H3" s="24" t="n">
         <v>24055.749</v>
       </c>
-      <c r="H3" s="24" t="n">
+      <c r="I3" s="24" t="n">
         <v>24026.834</v>
       </c>
-      <c r="I3" s="24" t="n">
+      <c r="J3" s="24" t="n">
         <v>23770.976</v>
-      </c>
-      <c r="J3" s="24" t="n">
-        <v>23548.21</v>
       </c>
       <c r="K3" s="46" t="n"/>
       <c r="L3" s="28" t="inlineStr">
@@ -952,7 +952,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="51" t="n">
+      <c r="N3" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D4" s="45" t="inlineStr">
         <is>
@@ -1002,19 +1002,19 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
+        <v>0.003729463910447484</v>
+      </c>
+      <c r="G4" s="25" t="n">
         <v>0.00518254492928083</v>
       </c>
-      <c r="G4" s="25" t="n">
+      <c r="H4" s="25" t="n">
         <v>0.001203446113624551</v>
       </c>
-      <c r="H4" s="25" t="n">
+      <c r="I4" s="25" t="n">
         <v>0.0107634621312982</v>
       </c>
-      <c r="I4" s="25" t="n">
+      <c r="J4" s="25" t="n">
         <v>0.009459997171759493</v>
-      </c>
-      <c r="J4" s="25" t="n">
-        <v>-0.001625164044818495</v>
       </c>
       <c r="K4" s="46" t="n"/>
       <c r="L4" s="28" t="n"/>
@@ -1023,7 +1023,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="51" t="n">
+      <c r="N4" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
@@ -1063,7 +1063,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="51" t="n">
+      <c r="C5" s="52" t="n">
         <v>46023</v>
       </c>
       <c r="D5" s="45" t="inlineStr">
@@ -1102,7 +1102,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="51" t="n">
+      <c r="N5" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
@@ -1127,7 +1127,7 @@
       <c r="T5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="U5" s="52" t="n">
+      <c r="U5" s="53" t="n">
         <v>66000</v>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="51" t="n">
+      <c r="C6" s="52" t="n">
         <v>46023</v>
       </c>
       <c r="D6" s="45" t="inlineStr">
@@ -1177,7 +1177,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="51" t="n">
+      <c r="N6" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D7" s="45" t="inlineStr">
         <is>
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
+        <v>4.9543</v>
+      </c>
+      <c r="G7" s="41" t="n">
         <v>1.54</v>
       </c>
-      <c r="G7" s="41" t="n">
+      <c r="H7" s="41" t="n">
         <v>1.2392</v>
       </c>
-      <c r="H7" s="41" t="n">
+      <c r="I7" s="41" t="n">
         <v>4.2373</v>
       </c>
-      <c r="I7" s="41" t="n">
+      <c r="J7" s="41" t="n">
         <v>3.4728</v>
-      </c>
-      <c r="J7" s="41" t="n">
-        <v>2.902</v>
       </c>
       <c r="K7" s="46" t="n"/>
       <c r="L7" s="28" t="inlineStr">
@@ -1256,7 +1256,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="51" t="n">
+      <c r="N7" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
@@ -1296,7 +1296,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -1335,7 +1335,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="51" t="n">
+      <c r="N8" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D9" s="45" t="inlineStr">
         <is>
@@ -1389,19 +1389,19 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
+        <v>16817.938</v>
+      </c>
+      <c r="G9" s="24" t="n">
         <v>16687.728</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="H9" s="24" t="n">
         <v>16665.219</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="I9" s="24" t="n">
         <v>16585.878</v>
       </c>
-      <c r="I9" s="24" t="n">
+      <c r="J9" s="24" t="n">
         <v>16445.685</v>
-      </c>
-      <c r="J9" s="24" t="n">
-        <v>16345.793</v>
       </c>
       <c r="K9" s="46" t="n"/>
       <c r="L9" s="28" t="inlineStr">
@@ -1414,7 +1414,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="51" t="n">
+      <c r="N9" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="C10" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D10" s="45" t="inlineStr">
         <is>
@@ -1464,19 +1464,19 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
+        <v>0.007802739833726813</v>
+      </c>
+      <c r="G10" s="25" t="n">
         <v>0.001350657318094584</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="H10" s="25" t="n">
         <v>0.004783647872002916</v>
       </c>
-      <c r="H10" s="25" t="n">
+      <c r="I10" s="25" t="n">
         <v>0.008524606910566446</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="J10" s="25" t="n">
         <v>0.006111174905983452</v>
-      </c>
-      <c r="J10" s="25" t="n">
-        <v>0.001525835907232986</v>
       </c>
       <c r="K10" s="46" t="n"/>
       <c r="L10" s="28" t="inlineStr">
@@ -1489,7 +1489,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="51" t="n">
+      <c r="N10" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C11" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1543,19 +1543,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>0.008520743120547625</v>
+        <v>0.01478556341261816</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>-0.01368541905855347</v>
+        <v>0.01269472215763789</v>
       </c>
       <c r="H11" s="25" t="n">
+        <v>-0.01239954075774974</v>
+      </c>
+      <c r="I11" s="25" t="n">
         <v>0.01363932594730488</v>
       </c>
-      <c r="I11" s="25" t="n">
+      <c r="J11" s="25" t="n">
         <v>0.0203286786358885</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>-0.01529395257471577</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1568,7 +1568,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
+      <c r="N11" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C12" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1618,19 +1618,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.02280776313925494</v>
+        <v>0.04546099626283169</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>-0.007990762124711401</v>
+        <v>0.02837984605940425</v>
       </c>
       <c r="H12" s="25" t="n">
+        <v>-0.006697459584295612</v>
+      </c>
+      <c r="I12" s="25" t="n">
         <v>-0.000734248084071364</v>
       </c>
-      <c r="I12" s="25" t="n">
+      <c r="J12" s="25" t="n">
         <v>0.02696242470599466</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>0.007561255742725968</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1643,7 +1643,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="51" t="n">
+      <c r="N12" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -1683,7 +1683,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="51" t="n">
+      <c r="C13" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -1722,8 +1722,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="53" t="n">
-        <v>46216</v>
+      <c r="N13" s="51" t="n">
+        <v>46223</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1736,19 +1736,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>187000</v>
+        <v>197000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>188000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>209000</v>
-      </c>
-      <c r="S13" s="24" t="n">
-        <v>217000</v>
       </c>
       <c r="T13" s="24" t="n">
         <v>217000</v>
       </c>
       <c r="U13" s="26" t="n">
-        <v>216000</v>
+        <v>217000</v>
       </c>
     </row>
     <row r="14">
@@ -1758,7 +1758,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="51" t="n">
+      <c r="C14" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
@@ -1797,8 +1797,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="53" t="n">
-        <v>46209</v>
+      <c r="N14" s="51" t="n">
+        <v>46216</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1796000</v>
+        <v>1782000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1789000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1798000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1821000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1806000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1812000</v>
       </c>
     </row>
     <row r="15">
@@ -1837,7 +1837,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="51" t="n">
+      <c r="C15" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
@@ -1876,7 +1876,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="51" t="n">
+      <c r="N15" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -1912,7 +1912,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="51" t="n">
+      <c r="C16" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
@@ -1963,7 +1963,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="51" t="n">
+      <c r="C17" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2050,7 +2050,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="51" t="n">
+      <c r="C18" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2089,7 +2089,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="51" t="n">
+      <c r="N18" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2130,7 +2130,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2143,19 +2143,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>0.002508528998595327</v>
+        <v>0.003127812531250385</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>-0.005085826793488901</v>
+        <v>0.002428130673527651</v>
       </c>
       <c r="H19" s="25" t="n">
+        <v>-0.004120795319042747</v>
+      </c>
+      <c r="I19" s="25" t="n">
         <v>-0.001185470781469022</v>
       </c>
-      <c r="I19" s="25" t="n">
+      <c r="J19" s="25" t="n">
         <v>-0.004560343211319595</v>
-      </c>
-      <c r="J19" s="25" t="n">
-        <v>0.006443377639647974</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2164,7 +2164,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="51" t="n">
+      <c r="N19" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2214,19 +2214,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.0001612822494979571</v>
+        <v>0.005233241102098308</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>-0.01070429991893201</v>
+        <v>0.001051115350177011</v>
       </c>
       <c r="H20" s="25" t="n">
+        <v>-0.009744718164220876</v>
+      </c>
+      <c r="I20" s="25" t="n">
         <v>7.7652239989875e-05</v>
       </c>
-      <c r="I20" s="25" t="n">
+      <c r="J20" s="25" t="n">
         <v>0.007894810306803354</v>
-      </c>
-      <c r="J20" s="25" t="n">
-        <v>0.013683775112075</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2239,7 +2239,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="51" t="n">
+      <c r="N20" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2293,19 +2293,19 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G21" s="45" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H21" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="45" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="45" t="n">
+      <c r="I21" s="45" t="n">
         <v>3.5</v>
       </c>
-      <c r="I21" s="45" t="n">
+      <c r="J21" s="45" t="n">
         <v>3.8</v>
-      </c>
-      <c r="J21" s="45" t="n">
-        <v>4.4</v>
       </c>
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2314,7 +2314,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="51" t="n">
+      <c r="N21" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2354,7 +2354,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="51" t="n">
+      <c r="C22" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2393,7 +2393,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="51" t="n">
+      <c r="N22" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2429,7 +2429,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
+      <c r="C23" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2463,7 +2463,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="51" t="n">
+      <c r="N23" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2503,7 +2503,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
+      <c r="C24" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2542,7 +2542,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="51" t="n">
+      <c r="N24" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
@@ -2582,7 +2582,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="51" t="n">
+      <c r="C25" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2617,7 +2617,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="51" t="n">
+      <c r="N25" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
@@ -2658,7 +2658,7 @@
         </is>
       </c>
       <c r="C26" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D26" s="45" t="inlineStr">
         <is>
@@ -2671,19 +2671,19 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
+        <v>0.02041382805407022</v>
+      </c>
+      <c r="G26" s="38" t="n">
         <v>0.02552585944536068</v>
       </c>
-      <c r="G26" s="38" t="n">
+      <c r="H26" s="38" t="n">
         <v>0.005923787970366412</v>
       </c>
-      <c r="H26" s="38" t="n">
+      <c r="I26" s="38" t="n">
         <v>0.007794617579222285</v>
       </c>
-      <c r="I26" s="38" t="n">
+      <c r="J26" s="38" t="n">
         <v>0.01778138610314484</v>
-      </c>
-      <c r="J26" s="38" t="n">
-        <v>0.02303791460563676</v>
       </c>
       <c r="K26" s="46" t="n"/>
       <c r="L26" s="28" t="inlineStr">
@@ -2696,7 +2696,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="51" t="n">
+      <c r="N26" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C27" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D27" s="45" t="inlineStr">
         <is>
@@ -2750,19 +2750,19 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
+        <v>0.003742997804626613</v>
+      </c>
+      <c r="G27" s="38" t="n">
         <v>-0.0201499882390509</v>
       </c>
-      <c r="G27" s="38" t="n">
+      <c r="H27" s="38" t="n">
         <v>-0.004277328978805506</v>
       </c>
-      <c r="H27" s="38" t="n">
+      <c r="I27" s="38" t="n">
         <v>-0.01832684674964358</v>
       </c>
-      <c r="I27" s="38" t="n">
+      <c r="J27" s="38" t="n">
         <v>-0.01299350008050415</v>
-      </c>
-      <c r="J27" s="38" t="n">
-        <v>-0.002410568051752549</v>
       </c>
       <c r="K27" s="46" t="n"/>
       <c r="L27" s="28" t="n"/>
@@ -2771,7 +2771,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="51" t="n">
+      <c r="N27" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
@@ -2811,7 +2811,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="53" t="n">
+      <c r="C28" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2850,7 +2850,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="51" t="n">
+      <c r="N28" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
@@ -2886,7 +2886,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="53" t="n">
+      <c r="C29" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2925,8 +2925,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="53" t="n">
-        <v>46231</v>
+      <c r="N29" s="51" t="n">
+        <v>46232</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.24</v>
+        <v>2.28</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.24</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="30">
@@ -2965,7 +2965,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="53" t="n">
+      <c r="C30" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -3004,8 +3004,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="53" t="n">
-        <v>46231</v>
+      <c r="N30" s="51" t="n">
+        <v>46232</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.28</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.28</v>
@@ -3040,7 +3040,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="53" t="n">
+      <c r="C31" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3079,7 +3079,7 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="51" t="n">
+      <c r="N31" s="52" t="n">
         <v>46023</v>
       </c>
       <c r="O31" s="45" t="inlineStr">
@@ -3119,7 +3119,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n">
+      <c r="C32" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3154,7 +3154,7 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="51" t="n">
+      <c r="N32" s="52" t="n">
         <v>46023</v>
       </c>
       <c r="O32" s="45" t="inlineStr">
@@ -3190,7 +3190,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n">
+      <c r="C33" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3229,7 +3229,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="51" t="n">
+      <c r="N33" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
@@ -3269,7 +3269,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
+      <c r="C34" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -3304,7 +3304,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="51" t="n">
+      <c r="N34" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
@@ -3344,7 +3344,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="51" t="n">
+      <c r="C35" s="52" t="n">
         <v>46023</v>
       </c>
       <c r="D35" s="45" t="inlineStr">
@@ -3383,7 +3383,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="51" t="n">
+      <c r="N35" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
@@ -3423,7 +3423,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
+      <c r="C36" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3458,7 +3458,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="51" t="n">
+      <c r="N36" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
@@ -3494,7 +3494,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
+      <c r="C37" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3533,7 +3533,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="53" t="n">
+      <c r="N37" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3573,7 +3573,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n">
+      <c r="C38" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3608,7 +3608,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="53" t="n">
+      <c r="N38" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -3644,7 +3644,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="51" t="n">
+      <c r="C39" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3683,7 +3683,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="51" t="n">
+      <c r="N39" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3723,7 +3723,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="53" t="n">
+      <c r="C40" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3758,7 +3758,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="51" t="n">
+      <c r="N40" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
@@ -3794,7 +3794,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="53" t="n">
+      <c r="C41" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -3833,7 +3833,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="51" t="n">
+      <c r="N41" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3873,7 +3873,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="51" t="n">
+      <c r="C42" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
@@ -3908,7 +3908,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="51" t="n">
+      <c r="N42" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3944,7 +3944,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="51" t="n">
+      <c r="C43" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
@@ -3983,7 +3983,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="51" t="n">
+      <c r="N43" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4024,7 +4024,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D44" s="45" t="inlineStr">
         <is>
@@ -4037,19 +4037,19 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
+        <v>5546.153</v>
+      </c>
+      <c r="G44" s="24" t="n">
         <v>5416.715</v>
       </c>
-      <c r="G44" s="24" t="n">
+      <c r="H44" s="24" t="n">
         <v>5343.513</v>
       </c>
-      <c r="H44" s="24" t="n">
+      <c r="I44" s="24" t="n">
         <v>5324.402</v>
       </c>
-      <c r="I44" s="24" t="n">
+      <c r="J44" s="24" t="n">
         <v>5236.97</v>
-      </c>
-      <c r="J44" s="24" t="n">
-        <v>5195.517</v>
       </c>
       <c r="K44" s="46" t="n"/>
       <c r="L44" s="28" t="n"/>
@@ -4058,7 +4058,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="51" t="n">
+      <c r="N44" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D45" s="45" t="inlineStr">
         <is>
@@ -4108,19 +4108,19 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
+        <v>0.02389603292770626</v>
+      </c>
+      <c r="G45" s="38" t="n">
         <v>0.01369922745579544</v>
       </c>
-      <c r="G45" s="38" t="n">
+      <c r="H45" s="38" t="n">
         <v>0.003589323270481781</v>
       </c>
-      <c r="H45" s="38" t="n">
+      <c r="I45" s="38" t="n">
         <v>0.01669515005814426</v>
       </c>
-      <c r="I45" s="38" t="n">
+      <c r="J45" s="38" t="n">
         <v>0.007978609251013902</v>
-      </c>
-      <c r="J45" s="38" t="n">
-        <v>0.008696251498575336</v>
       </c>
       <c r="K45" s="46" t="n"/>
       <c r="L45" s="28" t="n"/>
@@ -4145,7 +4145,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="51" t="n">
+      <c r="C46" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4232,7 +4232,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="51" t="n">
+      <c r="C47" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4271,8 +4271,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="53" t="n">
-        <v>46230</v>
+      <c r="N47" s="51" t="n">
+        <v>46231</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4311,7 +4311,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="51" t="n">
+      <c r="C48" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4350,8 +4350,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="53" t="n">
-        <v>46230</v>
+      <c r="N48" s="51" t="n">
+        <v>46231</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.33</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.31</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="49">
@@ -4386,7 +4386,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="51" t="n">
+      <c r="C49" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4425,8 +4425,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="53" t="n">
-        <v>46230</v>
+      <c r="N49" s="51" t="n">
+        <v>46231</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.46</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.41</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.37</v>
       </c>
     </row>
     <row r="50">
@@ -4465,7 +4465,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="51" t="n">
+      <c r="C50" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4504,8 +4504,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="53" t="n">
-        <v>46230</v>
+      <c r="N50" s="51" t="n">
+        <v>46231</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.71</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.67</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.63</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4540,7 +4540,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="51" t="n">
+      <c r="C51" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4579,7 +4579,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="53" t="n">
+      <c r="N51" s="52" t="n">
         <v>46223</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.23</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.26</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.28</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.29</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.25</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-07-31
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1683,8 +1683,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="52" t="n">
-        <v>46143</v>
+      <c r="C13" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
@@ -1697,19 +1697,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>0.002576669934182929</v>
+        <v>0.003373010342039962</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.00137424276419118</v>
+        <v>0.002543178134257529</v>
       </c>
       <c r="H13" s="25" t="n">
+        <v>0.003533767107920083</v>
+      </c>
+      <c r="I13" s="25" t="n">
         <v>0.005754259280153384</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="J13" s="25" t="n">
         <v>0.001865144407392716</v>
-      </c>
-      <c r="J13" s="25" t="n">
-        <v>-0.0007059953121911766</v>
       </c>
       <c r="K13" s="46" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1758,8 +1758,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="52" t="n">
-        <v>46143</v>
+      <c r="C14" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
@@ -1772,19 +1772,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.02326844467312684</v>
+        <v>0.02174406721925738</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.01941470378301213</v>
+        <v>0.02544092845096189</v>
       </c>
       <c r="H14" s="25" t="n">
+        <v>0.02161313347608846</v>
+      </c>
+      <c r="I14" s="25" t="n">
         <v>0.01787039680274048</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="J14" s="25" t="n">
         <v>0.0159621722309786</v>
-      </c>
-      <c r="J14" s="25" t="n">
-        <v>0.01853664152898512</v>
       </c>
       <c r="K14" s="46" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1837,8 +1837,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="52" t="n">
-        <v>46143</v>
+      <c r="C15" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1851,19 +1851,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.001720282126268735</v>
+        <v>0.002561096582198497</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.001714161330697239</v>
+        <v>0.002957589790436366</v>
       </c>
       <c r="H15" s="25" t="n">
+        <v>0.002766239184458286</v>
+      </c>
+      <c r="I15" s="25" t="n">
         <v>0.0001360630606932478</v>
       </c>
-      <c r="I15" s="25" t="n">
+      <c r="J15" s="25" t="n">
         <v>-0.0004895872054544448</v>
-      </c>
-      <c r="J15" s="25" t="n">
-        <v>-0.0002266093798154456</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1912,8 +1912,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="52" t="n">
-        <v>46143</v>
+      <c r="C16" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1926,19 +1926,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02046708111199261</v>
+        <v>0.02340010310037548</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02057845130290156</v>
+        <v>0.02280064195982224</v>
       </c>
       <c r="H16" s="25" t="n">
+        <v>0.02165034189613743</v>
+      </c>
+      <c r="I16" s="25" t="n">
         <v>0.02201458987977717</v>
       </c>
-      <c r="I16" s="25" t="n">
+      <c r="J16" s="25" t="n">
         <v>0.02561168480788904</v>
-      </c>
-      <c r="J16" s="25" t="n">
-        <v>0.02282169219926558</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2368,19 +2368,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.949</v>
+        <v>17.037</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.506</v>
+        <v>16.52</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.588</v>
+        <v>16.605</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.676</v>
+        <v>16.678</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>15.881</v>
+        <v>15.883</v>
       </c>
       <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2443,19 +2443,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.04096548335585318</v>
+        <v>0.04637022478810951</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>0.02885993891416824</v>
+        <v>0.02973259365455341</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.05658875049763962</v>
+        <v>-0.05562190752431315</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>-0.09122615803814729</v>
+        <v>-0.09111716621253409</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.0327669163773677</v>
+        <v>-0.03264510627931064</v>
       </c>
       <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2542,8 +2542,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="52" t="n">
-        <v>46143</v>
+      <c r="N24" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
         <is>
@@ -2556,19 +2556,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>0.004498312178282893</v>
+        <v>-0.001087163112479583</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.004102666349700579</v>
+        <v>0.004605444047291796</v>
       </c>
       <c r="S24" s="38" t="n">
+        <v>0.004056655138302112</v>
+      </c>
+      <c r="T24" s="38" t="n">
         <v>0.006669806004369283</v>
       </c>
-      <c r="T24" s="38" t="n">
+      <c r="U24" s="23" t="n">
         <v>0.003999286948838554</v>
-      </c>
-      <c r="U24" s="23" t="n">
-        <v>0.003476543056246895</v>
       </c>
     </row>
     <row r="25">
@@ -2617,8 +2617,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="52" t="n">
-        <v>46143</v>
+      <c r="N25" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
@@ -2631,19 +2631,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.04072638075644874</v>
+        <v>0.03668052673520432</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.03795481569560034</v>
+        <v>0.0407896819116949</v>
       </c>
       <c r="S25" s="38" t="n">
+        <v>0.03790725326991663</v>
+      </c>
+      <c r="T25" s="38" t="n">
         <v>0.03542928831754543</v>
       </c>
-      <c r="T25" s="38" t="n">
+      <c r="U25" s="23" t="n">
         <v>0.02873230041057473</v>
-      </c>
-      <c r="U25" s="23" t="n">
-        <v>0.02875208305094201</v>
       </c>
     </row>
     <row r="26">
@@ -2696,8 +2696,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="52" t="n">
-        <v>46143</v>
+      <c r="N26" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
         <is>
@@ -2710,19 +2710,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.003200505911295837</v>
+        <v>0.00132212092794437</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.002504967412229497</v>
+        <v>0.003324001449912295</v>
       </c>
       <c r="S26" s="38" t="n">
+        <v>0.002474041888621992</v>
+      </c>
+      <c r="T26" s="38" t="n">
         <v>0.002962135839517099</v>
       </c>
-      <c r="T26" s="38" t="n">
+      <c r="U26" s="23" t="n">
         <v>0.003939122649955218</v>
-      </c>
-      <c r="U26" s="23" t="n">
-        <v>0.00444927513566773</v>
       </c>
     </row>
     <row r="27">
@@ -2771,8 +2771,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="52" t="n">
-        <v>46143</v>
+      <c r="N27" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
@@ -2785,19 +2785,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03412035932904036</v>
+        <v>0.03286526430967084</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03318672212395027</v>
+        <v>0.03421575641942911</v>
       </c>
       <c r="S27" s="38" t="n">
+        <v>0.03315485012191053</v>
+      </c>
+      <c r="T27" s="38" t="n">
         <v>0.03253849776876586</v>
       </c>
-      <c r="T27" s="38" t="n">
+      <c r="U27" s="23" t="n">
         <v>0.03049262855088111</v>
-      </c>
-      <c r="U27" s="23" t="n">
-        <v>0.03104657789335973</v>
       </c>
     </row>
     <row r="28">
@@ -2851,7 +2851,7 @@
         </is>
       </c>
       <c r="N28" s="52" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
@@ -2864,19 +2864,19 @@
         </is>
       </c>
       <c r="Q28" s="45" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="R28" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="R28" s="45" t="n">
+      <c r="S28" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="S28" s="45" t="n">
+      <c r="T28" s="45" t="n">
         <v>3.8</v>
       </c>
-      <c r="T28" s="45" t="n">
+      <c r="U28" s="21" t="n">
         <v>3.4</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,19 +2939,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.28</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.24</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.24</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.21</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="31">
@@ -3079,8 +3079,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N31" s="52" t="n">
-        <v>46023</v>
+      <c r="N31" s="51" t="n">
+        <v>46113</v>
       </c>
       <c r="O31" s="45" t="inlineStr">
         <is>
@@ -3093,19 +3093,19 @@
         </is>
       </c>
       <c r="Q31" s="38" t="n">
+        <v>0.008518405841192678</v>
+      </c>
+      <c r="R31" s="38" t="n">
         <v>0.007177997310378714</v>
       </c>
-      <c r="R31" s="38" t="n">
+      <c r="S31" s="38" t="n">
         <v>0.007345039668930076</v>
       </c>
-      <c r="S31" s="38" t="n">
+      <c r="T31" s="38" t="n">
         <v>0.007979811365325773</v>
       </c>
-      <c r="T31" s="38" t="n">
+      <c r="U31" s="23" t="n">
         <v>0.01026193247962737</v>
-      </c>
-      <c r="U31" s="23" t="n">
-        <v>0.007624633431085215</v>
       </c>
     </row>
     <row r="32">
@@ -3154,8 +3154,8 @@
           <t>ECIWAG</t>
         </is>
       </c>
-      <c r="N32" s="52" t="n">
-        <v>46023</v>
+      <c r="N32" s="51" t="n">
+        <v>46113</v>
       </c>
       <c r="O32" s="45" t="inlineStr">
         <is>
@@ -3168,19 +3168,19 @@
         </is>
       </c>
       <c r="Q32" s="38" t="n">
+        <v>0.03138341697251144</v>
+      </c>
+      <c r="R32" s="38" t="n">
         <v>0.03316647264260756</v>
       </c>
-      <c r="R32" s="38" t="n">
+      <c r="S32" s="38" t="n">
         <v>0.03362463343108507</v>
       </c>
-      <c r="S32" s="38" t="n">
+      <c r="T32" s="38" t="n">
         <v>0.0358081705150977</v>
       </c>
-      <c r="T32" s="38" t="n">
+      <c r="U32" s="23" t="n">
         <v>0.03557875894988063</v>
-      </c>
-      <c r="U32" s="23" t="n">
-        <v>0.03369434416365838</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="N34" s="52" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
         <is>
@@ -3318,19 +3318,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.006556386035628131</v>
+        <v>-0.001424745951214598</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.00215860068996659</v>
+        <v>-0.006616807588155823</v>
       </c>
       <c r="S34" s="38" t="n">
+        <v>-0.002112874294617258</v>
+      </c>
+      <c r="T34" s="38" t="n">
         <v>-0.001052481507739263</v>
       </c>
-      <c r="T34" s="38" t="n">
+      <c r="U34" s="23" t="n">
         <v>0.008042734635068088</v>
-      </c>
-      <c r="U34" s="23" t="n">
-        <v>0.007581278680517641</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3384,7 +3384,7 @@
         </is>
       </c>
       <c r="N35" s="52" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
         <is>
@@ -3397,19 +3397,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.001817056427606656</v>
+        <v>0.004557860719200502</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>-0.002486041249112891</v>
+        <v>-0.00192350339640579</v>
       </c>
       <c r="S35" s="38" t="n">
+        <v>-0.002440329858829915</v>
+      </c>
+      <c r="T35" s="38" t="n">
         <v>-0.004493337788724072</v>
       </c>
-      <c r="T35" s="38" t="n">
+      <c r="U35" s="23" t="n">
         <v>-0.0007660751460527582</v>
-      </c>
-      <c r="U35" s="23" t="n">
-        <v>3.495077892301524e-05</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="N36" s="52" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
         <is>
@@ -3472,19 +3472,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.006556386035628131</v>
+        <v>-0.001424745951214598</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.00215860068996659</v>
+        <v>-0.006616807588155823</v>
       </c>
       <c r="S36" s="38" t="n">
+        <v>-0.002112874294617258</v>
+      </c>
+      <c r="T36" s="38" t="n">
         <v>-0.001052481507739263</v>
       </c>
-      <c r="T36" s="38" t="n">
+      <c r="U36" s="23" t="n">
         <v>0.008042734635068088</v>
-      </c>
-      <c r="U36" s="23" t="n">
-        <v>0.007581278680517641</v>
       </c>
     </row>
     <row r="37">
@@ -3723,7 +3723,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="51" t="n">
+      <c r="C40" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3794,7 +3794,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="51" t="n">
+      <c r="C41" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="51" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="51" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.33</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.37</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="51" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.46</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.41</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="51" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.61</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.71</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.67</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4579,8 +4579,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="52" t="n">
-        <v>46223</v>
+      <c r="N51" s="51" t="n">
+        <v>46230</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4593,19 +4593,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.58</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.55</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.49</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.43</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.49</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.27</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.23</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.26</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.28</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.29</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="N29" s="51" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,16 +2942,16 @@
         <v>2.3</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.28</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.24</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.24</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.28</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="N30" s="51" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.2</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.21</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="31">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="N47" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="N48" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4364,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.22</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.31</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.33</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.37</v>
       </c>
     </row>
     <row r="49">
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="N49" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.43</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.46</v>
       </c>
     </row>
     <row r="50">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="N50" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4518,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.61</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.69</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.71</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1217,7 +1217,7 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n">
+      <c r="C7" s="52" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="45" t="inlineStr">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.9543</v>
+        <v>6.1804</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1296,8 +1296,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="52" t="n">
-        <v>46143</v>
+      <c r="C8" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
@@ -1310,16 +1310,16 @@
         </is>
       </c>
       <c r="F8" s="45" t="n">
-        <v>0.54</v>
+        <v>0.6</v>
       </c>
       <c r="G8" s="45" t="n">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
       <c r="H8" s="45" t="n">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="I8" s="45" t="n">
-        <v>0.16</v>
+        <v>0.3</v>
       </c>
       <c r="J8" s="45" t="n">
         <v>0.18</v>
@@ -2811,7 +2811,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="51" t="n">
+      <c r="C28" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2886,7 +2886,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="51" t="n">
+      <c r="C29" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2965,7 +2965,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="51" t="n">
+      <c r="C30" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -3040,7 +3040,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="51" t="n">
+      <c r="C31" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="N52" s="56" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4644,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.32</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.27</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.23</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.26</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.28</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -223,7 +223,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -374,9 +374,6 @@
     </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1127,7 +1124,7 @@
       <c r="T5" s="24" t="n">
         <v>61000</v>
       </c>
-      <c r="U5" s="53" t="n">
+      <c r="U5" s="26" t="n">
         <v>66000</v>
       </c>
     </row>
@@ -1231,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>6.1804</v>
+        <v>5.859</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1489,8 +1486,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="52" t="n">
-        <v>46143</v>
+      <c r="N10" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
         <is>
@@ -1503,19 +1500,19 @@
         </is>
       </c>
       <c r="Q10" s="45" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="R10" s="45" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S10" s="45" t="n">
         <v>4.6</v>
-      </c>
-      <c r="R10" s="45" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="S10" s="45" t="n">
-        <v>4.2</v>
       </c>
       <c r="T10" s="45" t="n">
         <v>4.2</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="11">
@@ -1568,8 +1565,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="52" t="n">
-        <v>46143</v>
+      <c r="N11" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
         <is>
@@ -1582,19 +1579,19 @@
         </is>
       </c>
       <c r="Q11" s="45" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="R11" s="45" t="n">
         <v>3.3</v>
       </c>
       <c r="S11" s="45" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="T11" s="45" t="n">
         <v>3.5</v>
       </c>
-      <c r="T11" s="45" t="n">
+      <c r="U11" s="21" t="n">
         <v>3.1</v>
-      </c>
-      <c r="U11" s="21" t="n">
-        <v>3.4</v>
       </c>
     </row>
     <row r="12">
@@ -1643,8 +1640,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="52" t="n">
-        <v>46143</v>
+      <c r="N12" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
         <is>
@@ -1657,16 +1654,16 @@
         </is>
       </c>
       <c r="Q12" s="45" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="R12" s="45" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="S12" s="45" t="n">
         <v>3.2</v>
       </c>
-      <c r="R12" s="45" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="S12" s="45" t="n">
+      <c r="T12" s="45" t="n">
         <v>3.4</v>
-      </c>
-      <c r="T12" s="45" t="n">
-        <v>3.2</v>
       </c>
       <c r="U12" s="21" t="n">
         <v>3.2</v>
@@ -2825,10 +2822,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.003194428628793045</v>
+        <v>0.00472079606520448</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>-0.04043224342735219</v>
+        <v>-0.04004117699494203</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>0.08512722904348102</v>
@@ -2900,10 +2897,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.07380974528565151</v>
+        <v>0.07588184538797348</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>-0.03011895869723805</v>
+        <v>-0.02972368914374733</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>0.1779567725392831</v>
@@ -2926,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="51" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,16 +2936,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.3</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.28</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.24</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.24</v>
@@ -2979,10 +2976,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.003010246541142125</v>
+        <v>0.004536178951609848</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>-0.04303028794703967</v>
+        <v>-0.04261964610139124</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>0.08475262626842106</v>
@@ -3005,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="51" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.2</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.21</v>
       </c>
     </row>
     <row r="31">
@@ -3054,10 +3051,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.05654575401758045</v>
+        <v>0.05860719312123111</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>-0.04608686484039221</v>
+        <v>-0.04567753459150702</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>0.1533794281326583</v>
@@ -3533,7 +3530,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="51" t="n">
+      <c r="N37" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3608,7 +3605,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="51" t="n">
+      <c r="N38" s="52" t="n">
         <v>46143</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -3683,8 +3680,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="52" t="n">
-        <v>46174</v>
+      <c r="N39" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
         <is>
@@ -3697,19 +3694,19 @@
         </is>
       </c>
       <c r="Q39" s="45" t="n">
+        <v>120.597</v>
+      </c>
+      <c r="R39" s="53" t="n">
         <v>120.0835</v>
       </c>
-      <c r="R39" s="54" t="n">
+      <c r="S39" s="53" t="n">
         <v>118.7792</v>
       </c>
-      <c r="S39" s="45" t="n">
+      <c r="T39" s="45" t="n">
         <v>119.0363</v>
       </c>
-      <c r="T39" s="45" t="n">
+      <c r="U39" s="21" t="n">
         <v>119.9199</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>117.906</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3758,8 +3755,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="52" t="n">
-        <v>46174</v>
+      <c r="N40" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
         <is>
@@ -3772,19 +3769,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>0.004032046569596641</v>
+      </c>
+      <c r="R40" s="54" t="n">
         <v>-0.004232386546914929</v>
       </c>
-      <c r="R40" s="55" t="n">
+      <c r="S40" s="54" t="n">
         <v>-0.0291232297604588</v>
       </c>
-      <c r="S40" s="38" t="n">
+      <c r="T40" s="38" t="n">
         <v>-0.04111399852747133</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.05008673748247425</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.07796471263522881</v>
       </c>
     </row>
     <row r="41">
@@ -4145,8 +4142,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="52" t="n">
-        <v>46143</v>
+      <c r="C46" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
         <is>
@@ -4159,19 +4156,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>317677</v>
+        <v>314728</v>
       </c>
       <c r="G46" s="24" t="n">
+        <v>317633</v>
+      </c>
+      <c r="H46" s="24" t="n">
         <v>328187</v>
       </c>
-      <c r="H46" s="24" t="n">
+      <c r="I46" s="24" t="n">
         <v>318776</v>
       </c>
-      <c r="I46" s="24" t="n">
+      <c r="J46" s="24" t="n">
         <v>311803</v>
-      </c>
-      <c r="J46" s="24" t="n">
-        <v>299806</v>
       </c>
       <c r="K46" s="46" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4232,8 +4229,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="52" t="n">
-        <v>46143</v>
+      <c r="C47" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
         <is>
@@ -4246,19 +4243,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>-0.03202442509910508</v>
+        <v>-0.009145775155604108</v>
       </c>
       <c r="G47" s="38" t="n">
+        <v>-0.03215849500437251</v>
+      </c>
+      <c r="H47" s="38" t="n">
         <v>0.02952229778904303</v>
       </c>
-      <c r="H47" s="38" t="n">
+      <c r="I47" s="38" t="n">
         <v>0.0223634795046872</v>
       </c>
-      <c r="I47" s="38" t="n">
+      <c r="J47" s="38" t="n">
         <v>0.04001587693375042</v>
-      </c>
-      <c r="J47" s="38" t="n">
-        <v>0.05091102838594797</v>
       </c>
       <c r="K47" s="46" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4272,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="51" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4311,8 +4308,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="52" t="n">
-        <v>46143</v>
+      <c r="C48" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
         <is>
@@ -4325,19 +4322,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>395263</v>
+        <v>387989</v>
       </c>
       <c r="G48" s="24" t="n">
+        <v>395280</v>
+      </c>
+      <c r="H48" s="24" t="n">
         <v>382758</v>
       </c>
-      <c r="H48" s="24" t="n">
+      <c r="I48" s="24" t="n">
         <v>375360</v>
       </c>
-      <c r="I48" s="24" t="n">
+      <c r="J48" s="24" t="n">
         <v>366783</v>
-      </c>
-      <c r="J48" s="24" t="n">
-        <v>353991</v>
       </c>
       <c r="K48" s="46" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4351,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="51" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.22</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.26</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.31</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.33</v>
       </c>
     </row>
     <row r="49">
@@ -4386,8 +4383,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="52" t="n">
-        <v>46143</v>
+      <c r="C49" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
         <is>
@@ -4400,19 +4397,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>0.03267077370035376</v>
+        <v>-0.01844515280307635</v>
       </c>
       <c r="G49" s="38" t="n">
+        <v>0.03271518818679175</v>
+      </c>
+      <c r="H49" s="38" t="n">
         <v>0.01970907928388743</v>
       </c>
-      <c r="H49" s="38" t="n">
+      <c r="I49" s="38" t="n">
         <v>0.02338439894978772</v>
       </c>
-      <c r="I49" s="38" t="n">
+      <c r="J49" s="38" t="n">
         <v>0.03613651194521905</v>
-      </c>
-      <c r="J49" s="38" t="n">
-        <v>-0.02039240646446761</v>
       </c>
       <c r="K49" s="46" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4426,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="51" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4439,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.43</v>
       </c>
     </row>
     <row r="50">
@@ -4465,8 +4462,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="52" t="n">
-        <v>46143</v>
+      <c r="C50" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
         <is>
@@ -4479,19 +4476,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>28899</v>
+        <v>28848</v>
       </c>
       <c r="G50" s="24" t="n">
+        <v>28321</v>
+      </c>
+      <c r="H50" s="24" t="n">
         <v>28342</v>
       </c>
-      <c r="H50" s="24" t="n">
+      <c r="I50" s="24" t="n">
         <v>29493</v>
       </c>
-      <c r="I50" s="24" t="n">
+      <c r="J50" s="24" t="n">
         <v>27541</v>
-      </c>
-      <c r="J50" s="24" t="n">
-        <v>28077</v>
       </c>
       <c r="K50" s="46" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4505,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="51" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.61</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.65</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.69</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4540,8 +4537,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="52" t="n">
-        <v>46143</v>
+      <c r="C51" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
         <is>
@@ -4554,19 +4551,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.01965281208101044</v>
+        <v>0.01860809999646906</v>
       </c>
       <c r="G51" s="38" t="n">
+        <v>-0.0007409498271117032</v>
+      </c>
+      <c r="H51" s="38" t="n">
         <v>-0.03902620960905978</v>
       </c>
-      <c r="H51" s="38" t="n">
+      <c r="I51" s="38" t="n">
         <v>0.07087614828800692</v>
       </c>
-      <c r="I51" s="38" t="n">
+      <c r="J51" s="38" t="n">
         <v>-0.01909035865655162</v>
-      </c>
-      <c r="J51" s="38" t="n">
-        <v>0.05795244734164817</v>
       </c>
       <c r="K51" s="46" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4630,8 +4627,8 @@
           <t>DBAA</t>
         </is>
       </c>
-      <c r="N52" s="56" t="n">
-        <v>46234</v>
+      <c r="N52" s="55" t="n">
+        <v>46237</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.32</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.27</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.23</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.26</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-05
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1099,8 +1099,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="52" t="n">
-        <v>46174</v>
+      <c r="N5" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
@@ -1113,19 +1113,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>98000</v>
+        <v>44000</v>
       </c>
       <c r="R5" s="24" t="n">
+        <v>95000</v>
+      </c>
+      <c r="S5" s="24" t="n">
         <v>122000</v>
       </c>
-      <c r="S5" s="24" t="n">
+      <c r="T5" s="24" t="n">
         <v>105000</v>
       </c>
-      <c r="T5" s="24" t="n">
+      <c r="U5" s="26" t="n">
         <v>61000</v>
-      </c>
-      <c r="U5" s="26" t="n">
-        <v>66000</v>
       </c>
     </row>
     <row r="6">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="51" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.31</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.3</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.3</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="51" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="51" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="51" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.28</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.23</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.22</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.26</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.31</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="51" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.45</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.35</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.4</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="51" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.61</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.65</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.31</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.32</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.27</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.23</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-07
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -369,10 +369,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="N3" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
         <is>
@@ -963,19 +963,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>57</v>
+        <v>-23</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>129</v>
+        <v>20</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>63</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>148</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>214</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>-156</v>
       </c>
     </row>
     <row r="4">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="N4" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
         <is>
@@ -1034,19 +1034,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.003192872196771792</v>
+        <v>0.001993162695058723</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.002706658759101061</v>
+        <v>0.002542939714029707</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.002290249719239359</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.001974950310754961</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.001723735138309224</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.0007959067652075042</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1060,7 +1060,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C5" s="52" t="n">
+      <c r="C5" s="51" t="n">
         <v>46023</v>
       </c>
       <c r="D5" s="45" t="inlineStr">
@@ -1099,7 +1099,7 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="51" t="n">
+      <c r="N5" s="52" t="n">
         <v>46204</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
@@ -1135,7 +1135,7 @@
           <t>NGDPSAXDCUSQ</t>
         </is>
       </c>
-      <c r="C6" s="52" t="n">
+      <c r="C6" s="51" t="n">
         <v>46023</v>
       </c>
       <c r="D6" s="45" t="inlineStr">
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="N6" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         </is>
       </c>
       <c r="Q6" s="45" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="R6" s="45" t="n">
         <v>4.2</v>
-      </c>
-      <c r="R6" s="45" t="n">
-        <v>4.3</v>
       </c>
       <c r="S6" s="45" t="n">
         <v>4.3</v>
@@ -1200,7 +1200,7 @@
         <v>4.3</v>
       </c>
       <c r="U6" s="21" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
@@ -1214,7 +1214,7 @@
           <t>GDPNOW</t>
         </is>
       </c>
-      <c r="C7" s="52" t="n">
+      <c r="C7" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="45" t="inlineStr">
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>5.859</v>
+        <v>5.8334</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="N7" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
         <is>
@@ -1270,16 +1270,16 @@
         <v>7.9</v>
       </c>
       <c r="R7" s="45" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="S7" s="45" t="n">
         <v>8.1</v>
       </c>
-      <c r="S7" s="45" t="n">
+      <c r="T7" s="45" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="T7" s="45" t="n">
+      <c r="U7" s="21" t="n">
         <v>8</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>7.9</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1293,7 +1293,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="N8" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
         <is>
@@ -1346,19 +1346,19 @@
         </is>
       </c>
       <c r="Q8" s="45" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="R8" s="45" t="n">
         <v>61.5</v>
-      </c>
-      <c r="R8" s="45" t="n">
-        <v>61.8</v>
       </c>
       <c r="S8" s="45" t="n">
         <v>61.8</v>
       </c>
       <c r="T8" s="45" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="U8" s="21" t="n">
         <v>61.9</v>
-      </c>
-      <c r="U8" s="21" t="n">
-        <v>62</v>
       </c>
     </row>
     <row r="9">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="N9" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1425,19 +1425,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="R9" s="45" t="n">
         <v>59</v>
       </c>
-      <c r="R9" s="45" t="n">
+      <c r="S9" s="45" t="n">
         <v>59.2</v>
       </c>
-      <c r="S9" s="45" t="n">
+      <c r="T9" s="45" t="n">
         <v>59.1</v>
       </c>
-      <c r="T9" s="45" t="n">
+      <c r="U9" s="21" t="n">
         <v>59.2</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>59.3</v>
       </c>
     </row>
     <row r="10">
@@ -1486,7 +1486,7 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="51" t="n">
+      <c r="N10" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
@@ -1565,7 +1565,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
+      <c r="N11" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1640,7 +1640,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="51" t="n">
+      <c r="N12" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -1719,8 +1719,8 @@
           <t>ICSA</t>
         </is>
       </c>
-      <c r="N13" s="51" t="n">
-        <v>46223</v>
+      <c r="N13" s="52" t="n">
+        <v>46230</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,16 +1733,16 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>197000</v>
+        <v>199000</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>188000</v>
+        <v>198000</v>
       </c>
       <c r="S13" s="24" t="n">
+        <v>189000</v>
+      </c>
+      <c r="T13" s="24" t="n">
         <v>209000</v>
-      </c>
-      <c r="T13" s="24" t="n">
-        <v>217000</v>
       </c>
       <c r="U13" s="26" t="n">
         <v>217000</v>
@@ -1794,8 +1794,8 @@
           <t>CCSA</t>
         </is>
       </c>
-      <c r="N14" s="51" t="n">
-        <v>46216</v>
+      <c r="N14" s="52" t="n">
+        <v>46223</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1782000</v>
+        <v>1801000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1777000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1789000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1798000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1821000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1806000</v>
       </c>
     </row>
     <row r="15">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="N15" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
@@ -1896,10 +1896,10 @@
         <v>34.3</v>
       </c>
       <c r="T15" s="24" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="U15" s="26" t="n">
         <v>34.2</v>
-      </c>
-      <c r="U15" s="26" t="n">
-        <v>34.3</v>
       </c>
     </row>
     <row r="16">
@@ -1960,7 +1960,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="52" t="n">
+      <c r="C17" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2047,7 +2047,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="52" t="n">
+      <c r="C18" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2086,7 +2086,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="52" t="n">
+      <c r="N18" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2161,7 +2161,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="52" t="n">
+      <c r="N19" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2236,7 +2236,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="52" t="n">
+      <c r="N20" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2311,7 +2311,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="52" t="n">
+      <c r="N21" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2351,7 +2351,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2390,7 +2390,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="52" t="n">
+      <c r="N22" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2426,7 +2426,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2460,7 +2460,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="52" t="n">
+      <c r="N23" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2500,7 +2500,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="52" t="n">
+      <c r="C24" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2579,7 +2579,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="52" t="n">
+      <c r="C25" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2808,7 +2808,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="52" t="n">
+      <c r="C28" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2847,7 +2847,7 @@
           <t>MICH</t>
         </is>
       </c>
-      <c r="N28" s="52" t="n">
+      <c r="N28" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
@@ -2883,7 +2883,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="52" t="n">
+      <c r="C29" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2922,8 +2922,8 @@
           <t>T5YIFR</t>
         </is>
       </c>
-      <c r="N29" s="51" t="n">
-        <v>46238</v>
+      <c r="N29" s="52" t="n">
+        <v>46240</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R29" s="45" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.3</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="30">
@@ -2962,7 +2962,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="52" t="n">
+      <c r="C30" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -3001,8 +3001,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="51" t="n">
-        <v>46238</v>
+      <c r="N30" s="52" t="n">
+        <v>46240</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="R30" s="45" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.23</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.28</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.27</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="31">
@@ -3037,7 +3037,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="52" t="n">
+      <c r="C31" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3116,7 +3116,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="52" t="n">
+      <c r="C32" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3187,7 +3187,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="52" t="n">
+      <c r="C33" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="N33" s="52" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
         <is>
@@ -3240,19 +3240,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
-        <v>0.003465742468675037</v>
+        <v>0.0005319148936169249</v>
       </c>
       <c r="R33" s="38" t="n">
-        <v>0.002673082063619381</v>
+        <v>0.002934115764203771</v>
       </c>
       <c r="S33" s="38" t="n">
+        <v>0.002138465650895593</v>
+      </c>
+      <c r="T33" s="38" t="n">
         <v>0.001606425702811221</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.002146498524282281</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.003230148048452453</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -3266,7 +3266,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="52" t="n">
+      <c r="C34" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -3301,7 +3301,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N34" s="52" t="n">
+      <c r="N34" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
@@ -3315,10 +3315,10 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.001424745951214598</v>
+        <v>-0.002485931130862563</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.006616807588155823</v>
+        <v>-0.007146470713941611</v>
       </c>
       <c r="S34" s="38" t="n">
         <v>-0.002112874294617258</v>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="C35" s="52" t="n">
-        <v>46023</v>
+        <v>46113</v>
       </c>
       <c r="D35" s="45" t="inlineStr">
         <is>
@@ -3355,19 +3355,19 @@
         </is>
       </c>
       <c r="F35" s="41" t="n">
-        <v>0.3</v>
+        <v>1.4</v>
       </c>
       <c r="G35" s="41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H35" s="41" t="n">
         <v>1.6</v>
       </c>
-      <c r="H35" s="41" t="n">
+      <c r="I35" s="41" t="n">
         <v>5.2</v>
       </c>
-      <c r="I35" s="41" t="n">
+      <c r="J35" s="41" t="n">
         <v>4.2</v>
-      </c>
-      <c r="J35" s="41" t="n">
-        <v>-0.9</v>
       </c>
       <c r="K35" s="46" t="n"/>
       <c r="L35" s="28" t="inlineStr">
@@ -3380,7 +3380,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N35" s="52" t="n">
+      <c r="N35" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
@@ -3394,10 +3394,10 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>0.004557860719200502</v>
+        <v>0.004025655420760277</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>-0.00192350339640579</v>
+        <v>-0.002455668950446244</v>
       </c>
       <c r="S35" s="38" t="n">
         <v>-0.002440329858829915</v>
@@ -3420,7 +3420,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="52" t="n">
+      <c r="C36" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3455,7 +3455,7 @@
           <t>RCES0500000003*</t>
         </is>
       </c>
-      <c r="N36" s="52" t="n">
+      <c r="N36" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
@@ -3469,10 +3469,10 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.001424745951214598</v>
+        <v>-0.002485931130862563</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.006616807588155823</v>
+        <v>-0.007146470713941611</v>
       </c>
       <c r="S36" s="38" t="n">
         <v>-0.002112874294617258</v>
@@ -3491,7 +3491,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="52" t="n">
+      <c r="C37" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3530,7 +3530,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="52" t="n">
+      <c r="N37" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3570,7 +3570,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="52" t="n">
+      <c r="C38" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3605,7 +3605,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="52" t="n">
+      <c r="N38" s="51" t="n">
         <v>46143</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -3641,7 +3641,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="52" t="n">
+      <c r="C39" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3680,7 +3680,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="51" t="n">
+      <c r="N39" s="52" t="n">
         <v>46204</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3720,7 +3720,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="52" t="n">
+      <c r="C40" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3755,7 +3755,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="51" t="n">
+      <c r="N40" s="52" t="n">
         <v>46204</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
@@ -3791,7 +3791,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="52" t="n">
+      <c r="C41" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -3830,7 +3830,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="52" t="n">
+      <c r="N41" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3870,7 +3870,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C42" s="52" t="n">
+      <c r="C42" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
@@ -3905,7 +3905,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="52" t="n">
+      <c r="N42" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3941,7 +3941,7 @@
           <t>EXHOSLUSM495S</t>
         </is>
       </c>
-      <c r="C43" s="52" t="n">
+      <c r="C43" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
@@ -3980,7 +3980,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="52" t="n">
+      <c r="N43" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4055,7 +4055,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="52" t="n">
+      <c r="N44" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4142,7 +4142,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="51" t="n">
+      <c r="C46" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4229,7 +4229,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="51" t="n">
+      <c r="C47" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4268,8 +4268,8 @@
           <t>DFF</t>
         </is>
       </c>
-      <c r="N47" s="51" t="n">
-        <v>46237</v>
+      <c r="N47" s="52" t="n">
+        <v>46239</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="51" t="n">
+      <c r="C48" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4347,8 +4347,8 @@
           <t>DGS2</t>
         </is>
       </c>
-      <c r="N48" s="51" t="n">
-        <v>46237</v>
+      <c r="N48" s="52" t="n">
+        <v>46239</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="R48" s="45" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="S48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.28</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.23</v>
-      </c>
-      <c r="T48" s="45" t="n">
-        <v>4.22</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.26</v>
       </c>
     </row>
     <row r="49">
@@ -4383,7 +4383,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="51" t="n">
+      <c r="C49" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4422,8 +4422,8 @@
           <t>DGS5</t>
         </is>
       </c>
-      <c r="N49" s="51" t="n">
-        <v>46237</v>
+      <c r="N49" s="52" t="n">
+        <v>46239</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="R49" s="45" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.45</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.38</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>4.37</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.35</v>
       </c>
     </row>
     <row r="50">
@@ -4462,7 +4462,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="51" t="n">
+      <c r="C50" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4501,8 +4501,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="51" t="n">
-        <v>46237</v>
+      <c r="N50" s="52" t="n">
+        <v>46239</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="R50" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.68</v>
-      </c>
-      <c r="T50" s="45" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.61</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4537,7 +4537,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="51" t="n">
+      <c r="C51" s="52" t="n">
         <v>46174</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4576,8 +4576,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="51" t="n">
-        <v>46230</v>
+      <c r="N51" s="52" t="n">
+        <v>46237</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4590,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.66</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.58</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.55</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.49</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.43</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.27</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.31</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.38</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.32</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.27</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-08
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2351,8 +2351,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="51" t="n">
-        <v>46174</v>
+      <c r="C22" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
         <is>
@@ -2365,19 +2365,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>17.037</v>
+        <v>16.782</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>16.52</v>
+        <v>17.043</v>
       </c>
       <c r="H22" s="24" t="n">
-        <v>16.605</v>
+        <v>16.748</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.678</v>
+        <v>16.642</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>15.883</v>
+        <v>16.66</v>
       </c>
       <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2426,8 +2426,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
-        <v>46174</v>
+      <c r="C23" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
         <is>
@@ -2440,19 +2440,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.04637022478810951</v>
+        <v>-0.01270737733851048</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>0.02973259365455341</v>
+        <v>0.04673872988576337</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>-0.05562190752431315</v>
+        <v>0.04394439942654129</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>-0.09111716621253409</v>
+        <v>-0.05351760222942609</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.03264510627931064</v>
+        <v>-0.09209809264305184</v>
       </c>
       <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2500,8 +2500,8 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
-        <v>46143</v>
+      <c r="C24" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -2514,19 +2514,19 @@
         </is>
       </c>
       <c r="F24" s="38" t="n">
-        <v>-0.003925763540534311</v>
+        <v>0.005013854980292054</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>0.008629783986034756</v>
+        <v>-0.00392895391127901</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>0.008052444128709091</v>
+        <v>0.008723867563298793</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>0.000857114913422663</v>
+        <v>0.008102056603516816</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>0.00136865468313907</v>
+        <v>0.0008464850167981819</v>
       </c>
       <c r="K24" s="46" t="n"/>
       <c r="L24" s="28" t="inlineStr">
@@ -2579,8 +2579,8 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="51" t="n">
-        <v>46143</v>
+      <c r="C25" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
         <is>
@@ -2593,19 +2593,19 @@
         </is>
       </c>
       <c r="F25" s="38" t="n">
-        <v>0.001344310133821303</v>
+        <v>0.001951572292765213</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>0.002443819508178846</v>
+        <v>0.001109630592487365</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>0.003197428618906484</v>
+        <v>0.002171973058996635</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>0.001618006847893483</v>
+        <v>0.003192546663167928</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>0.0006997747068799853</v>
+        <v>0.001614188463588073</v>
       </c>
       <c r="K25" s="46" t="n"/>
       <c r="L25" s="28" t="n"/>
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.29</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.3</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.23</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.28</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.23</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
-        <v>4.33</v>
+        <v>4.4</v>
       </c>
       <c r="R49" s="45" t="n">
         <v>4.33</v>
       </c>
       <c r="S49" s="45" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="T49" s="45" t="n">
         <v>4.4</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.45</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.38</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>4.63</v>
+        <v>4.69</v>
       </c>
       <c r="R50" s="45" t="n">
         <v>4.63</v>
       </c>
       <c r="S50" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="T50" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.75</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.68</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.25</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.27</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.31</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.38</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.32</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-10
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1293,7 +1293,7 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="52" t="n">
+      <c r="C8" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
@@ -1411,8 +1411,10 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="52" t="n">
-        <v>46204</v>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
+        </is>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1425,19 +1427,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
-        <v>58.9</v>
+        <v>1</v>
       </c>
       <c r="R9" s="45" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="S9" s="45" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="45" t="n">
-        <v>59.1</v>
+        <v>1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>59.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2276,8 +2278,10 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="51" t="n">
-        <v>46174</v>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
+        </is>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2290,19 +2294,19 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="G21" s="45" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
       <c r="H21" s="45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I21" s="45" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="J21" s="45" t="n">
-        <v>3.8</v>
+        <v>1</v>
       </c>
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -3680,7 +3684,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="52" t="n">
+      <c r="N39" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
@@ -3755,7 +3759,7 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="52" t="n">
+      <c r="N40" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O40" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-11
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1099,8 +1099,10 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="52" t="n">
-        <v>46204</v>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
+        </is>
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
@@ -1113,19 +1115,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>44000</v>
+        <v>1</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>95000</v>
+        <v>1</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>122000</v>
+        <v>1</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>105000</v>
+        <v>1</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>61000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1253,8 +1255,10 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="52" t="n">
-        <v>46204</v>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
+        </is>
       </c>
       <c r="O7" s="45" t="inlineStr">
         <is>
@@ -1267,19 +1271,19 @@
         </is>
       </c>
       <c r="Q7" s="45" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="R7" s="45" t="n">
-        <v>7.9</v>
+        <v>1</v>
       </c>
       <c r="S7" s="45" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="T7" s="45" t="n">
-        <v>8.199999999999999</v>
+        <v>1</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1488,8 +1492,10 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="52" t="n">
-        <v>46174</v>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
+        </is>
       </c>
       <c r="O10" s="45" t="inlineStr">
         <is>
@@ -1502,19 +1508,19 @@
         </is>
       </c>
       <c r="Q10" s="45" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="R10" s="45" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="S10" s="45" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="T10" s="45" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1567,7 +1573,7 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="52" t="n">
+      <c r="N11" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
@@ -1642,7 +1648,7 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="52" t="n">
+      <c r="N12" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
@@ -2238,8 +2244,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="51" t="n">
-        <v>46174</v>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O20" s="45" t="inlineStr">
         <is>
@@ -2252,19 +2260,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>-0.0001666066684318235</v>
+        <v>1</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.002080954496262777</v>
+        <v>1</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>0.00376460730477457</v>
+        <v>1</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>0.001957950538511444</v>
+        <v>1</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>0.002160502174024082</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2278,10 +2286,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'PSAVERT' not found in values file."</t>
-        </is>
+      <c r="C21" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2294,19 +2300,19 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="G21" s="45" t="n">
-        <v>1</v>
+        <v>2.8</v>
       </c>
       <c r="H21" s="45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I21" s="45" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="J21" s="45" t="n">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2315,8 +2321,10 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="51" t="n">
-        <v>46174</v>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
+        </is>
       </c>
       <c r="O21" s="45" t="inlineStr">
         <is>
@@ -2329,19 +2337,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.02565785056369746</v>
+        <v>1</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.02822942063611032</v>
+        <v>1</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>0.02743309430968526</v>
+        <v>1</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>0.0260216770548682</v>
+        <v>1</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>0.02472462476764023</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2927,7 +2935,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2940,19 +2948,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.29</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3006,7 +3014,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3019,19 +3027,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.22</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.23</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="31">
@@ -3875,7 +3883,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="D42" s="45" t="inlineStr">
         <is>
@@ -3888,19 +3896,19 @@
         </is>
       </c>
       <c r="F42" s="39" t="n">
-        <v>4090000</v>
+        <v>4060000</v>
       </c>
       <c r="G42" s="39" t="n">
+        <v>4130000</v>
+      </c>
+      <c r="H42" s="39" t="n">
         <v>4190000</v>
       </c>
-      <c r="H42" s="39" t="n">
+      <c r="I42" s="39" t="n">
         <v>4040000</v>
       </c>
-      <c r="I42" s="39" t="n">
+      <c r="J42" s="39" t="n">
         <v>4010000</v>
-      </c>
-      <c r="J42" s="39" t="n">
-        <v>4130000</v>
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="28" t="n"/>
@@ -3946,7 +3954,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="D43" s="45" t="inlineStr">
         <is>
@@ -3959,7 +3967,7 @@
         </is>
       </c>
       <c r="F43" s="38" t="n">
-        <v>0.02763819095477387</v>
+        <v>0.007444168734491315</v>
       </c>
       <c r="G43" s="38" t="n">
         <v/>
@@ -4146,7 +4154,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="52" t="n">
+      <c r="C46" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
@@ -4233,7 +4241,7 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="52" t="n">
+      <c r="C47" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
@@ -4273,7 +4281,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4312,7 +4320,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="52" t="n">
+      <c r="C48" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
@@ -4352,7 +4360,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4365,19 +4373,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.25</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.28</v>
       </c>
     </row>
     <row r="49">
@@ -4387,7 +4395,7 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="52" t="n">
+      <c r="C49" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
@@ -4427,7 +4435,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4440,19 +4448,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.4</v>
-      </c>
-      <c r="R49" s="45" t="n">
-        <v>4.33</v>
       </c>
       <c r="S49" s="45" t="n">
         <v>4.33</v>
       </c>
       <c r="T49" s="45" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="U49" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.45</v>
       </c>
     </row>
     <row r="50">
@@ -4466,7 +4474,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="52" t="n">
+      <c r="C50" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
@@ -4506,7 +4514,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4519,19 +4527,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.69</v>
-      </c>
-      <c r="R50" s="45" t="n">
-        <v>4.63</v>
       </c>
       <c r="S50" s="45" t="n">
         <v>4.63</v>
       </c>
       <c r="T50" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="U50" s="21" t="n">
         <v>4.7</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.75</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4541,7 +4549,7 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="52" t="n">
+      <c r="C51" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
@@ -4632,7 +4640,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4645,19 +4653,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.3</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.25</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.27</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.31</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.38</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-12
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1099,10 +1099,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'ADPMNUSNERSA' not found in values file."</t>
-        </is>
+      <c r="N5" s="51" t="n">
+        <v>46204</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
@@ -1115,19 +1113,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>1</v>
+        <v>44000</v>
       </c>
       <c r="R5" s="24" t="n">
-        <v>1</v>
+        <v>95000</v>
       </c>
       <c r="S5" s="24" t="n">
-        <v>1</v>
+        <v>122000</v>
       </c>
       <c r="T5" s="24" t="n">
-        <v>1</v>
+        <v>105000</v>
       </c>
       <c r="U5" s="26" t="n">
-        <v>1</v>
+        <v>61000</v>
       </c>
     </row>
     <row r="6">
@@ -1255,10 +1253,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'U6RATE' not found in values file."</t>
-        </is>
+      <c r="N7" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
         <is>
@@ -1271,19 +1267,19 @@
         </is>
       </c>
       <c r="Q7" s="45" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="R7" s="45" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="S7" s="45" t="n">
-        <v>1</v>
+        <v>8.1</v>
       </c>
       <c r="T7" s="45" t="n">
-        <v>1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="U7" s="21" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1415,10 +1411,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'EMRATIO' not found in values file."</t>
-        </is>
+      <c r="N9" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1431,19 +1425,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
-        <v>1</v>
+        <v>58.9</v>
       </c>
       <c r="R9" s="45" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="S9" s="45" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
       <c r="T9" s="45" t="n">
-        <v>1</v>
+        <v>59.1</v>
       </c>
       <c r="U9" s="21" t="n">
-        <v>1</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="10">
@@ -1492,10 +1486,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSJOR' not found in values file."</t>
-        </is>
+      <c r="N10" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
         <is>
@@ -1508,19 +1500,19 @@
         </is>
       </c>
       <c r="Q10" s="45" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="R10" s="45" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="S10" s="45" t="n">
-        <v>1</v>
+        <v>4.6</v>
       </c>
       <c r="T10" s="45" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="U10" s="21" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="11">
@@ -2094,8 +2086,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="51" t="n">
-        <v>46174</v>
+      <c r="N18" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
         <is>
@@ -2108,19 +2100,19 @@
         </is>
       </c>
       <c r="Q18" s="38" t="n">
+        <v>0.0007366914435544825</v>
+      </c>
+      <c r="R18" s="38" t="n">
         <v>-0.004224816530380648</v>
       </c>
-      <c r="R18" s="38" t="n">
+      <c r="S18" s="38" t="n">
         <v>0.004729142286413968</v>
       </c>
-      <c r="S18" s="38" t="n">
+      <c r="T18" s="38" t="n">
         <v>0.006400377846336402</v>
       </c>
-      <c r="T18" s="38" t="n">
+      <c r="U18" s="23" t="n">
         <v>0.008651438343614481</v>
-      </c>
-      <c r="U18" s="23" t="n">
-        <v>0.00267003074209704</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
@@ -2169,8 +2161,8 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="51" t="n">
-        <v>46174</v>
+      <c r="N19" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
         <is>
@@ -2183,19 +2175,19 @@
         </is>
       </c>
       <c r="Q19" s="38" t="n">
+        <v>0.03303856050706308</v>
+      </c>
+      <c r="R19" s="38" t="n">
         <v>0.03463530729385406</v>
       </c>
-      <c r="R19" s="38" t="n">
+      <c r="S19" s="38" t="n">
         <v>0.04166614684049648</v>
       </c>
-      <c r="S19" s="38" t="n">
+      <c r="T19" s="38" t="n">
         <v>0.03779245836741563</v>
       </c>
-      <c r="T19" s="38" t="n">
+      <c r="U19" s="23" t="n">
         <v>0.03285957752865201</v>
-      </c>
-      <c r="U19" s="23" t="n">
-        <v>0.0243400411037322</v>
       </c>
     </row>
     <row r="20">
@@ -2244,10 +2236,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N20" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
         <is>
@@ -2260,19 +2250,19 @@
         </is>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1</v>
+        <v>0.002154345141564873</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>1</v>
+        <v>-0.0001666066684318235</v>
       </c>
       <c r="S20" s="38" t="n">
-        <v>1</v>
+        <v>0.002080954496262777</v>
       </c>
       <c r="T20" s="38" t="n">
-        <v>1</v>
+        <v>0.00376460730477457</v>
       </c>
       <c r="U20" s="23" t="n">
-        <v>1</v>
+        <v>0.001957950538511444</v>
       </c>
     </row>
     <row r="21">
@@ -2321,10 +2311,8 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'CPILFESL' not found in values file."</t>
-        </is>
+      <c r="N21" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
         <is>
@@ -2337,19 +2325,19 @@
         </is>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1</v>
+        <v>0.0246651778923092</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>1</v>
+        <v>0.02565785056369746</v>
       </c>
       <c r="S21" s="38" t="n">
-        <v>1</v>
+        <v>0.02822942063611032</v>
       </c>
       <c r="T21" s="38" t="n">
-        <v>1</v>
+        <v>0.02743309430968526</v>
       </c>
       <c r="U21" s="23" t="n">
-        <v>1</v>
+        <v>0.0260216770548682</v>
       </c>
     </row>
     <row r="22">
@@ -2935,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2948,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.29</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -3014,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3027,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.29</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.25</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.22</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.23</v>
       </c>
     </row>
     <row r="31">
@@ -4281,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4360,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4373,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.18</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.2</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.25</v>
       </c>
     </row>
     <row r="49">
@@ -4435,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4448,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.4</v>
-      </c>
-      <c r="S49" s="45" t="n">
-        <v>4.33</v>
       </c>
       <c r="T49" s="45" t="n">
         <v>4.33</v>
       </c>
       <c r="U49" s="21" t="n">
-        <v>4.4</v>
+        <v>4.33</v>
       </c>
     </row>
     <row r="50">
@@ -4514,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4527,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.69</v>
-      </c>
-      <c r="S50" s="45" t="n">
-        <v>4.63</v>
       </c>
       <c r="T50" s="45" t="n">
         <v>4.63</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.7</v>
+        <v>4.63</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4640,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4653,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.3</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.25</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.27</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.31</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-13
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1565,8 +1565,10 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
-        <v>46174</v>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
+        </is>
       </c>
       <c r="O11" s="45" t="inlineStr">
         <is>
@@ -1579,19 +1581,19 @@
         </is>
       </c>
       <c r="Q11" s="45" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="R11" s="45" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
       <c r="S11" s="45" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
       <c r="T11" s="45" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1720,7 +1722,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46230</v>
+        <v>46237</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,19 +1735,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>199000</v>
+        <v>209000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>200000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>198000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>189000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>209000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>217000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1797,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1810,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1801000</v>
+        <v>1777000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1799000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1777000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1789000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1798000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1821000</v>
       </c>
     </row>
     <row r="15">
@@ -2390,8 +2392,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="51" t="n">
-        <v>46174</v>
+      <c r="N22" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
         <is>
@@ -2404,19 +2406,19 @@
         </is>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>-0.002770682989280293</v>
+        <v>-0.0002809580670085632</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.006223162212395161</v>
+        <v>-0.001122570686872826</v>
       </c>
       <c r="S22" s="38" t="n">
-        <v>0.01052427058709249</v>
+        <v>0.004529844434762564</v>
       </c>
       <c r="T22" s="38" t="n">
-        <v>0.00783922090807021</v>
+        <v>0.01090075327249296</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>0.004827242437757562</v>
+        <v>0.007760893971436644</v>
       </c>
     </row>
     <row r="23">
@@ -2460,8 +2462,8 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="51" t="n">
-        <v>46174</v>
+      <c r="N23" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
         <is>
@@ -2474,19 +2476,19 @@
         </is>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>0.05507672194780078</v>
+        <v>0.04656510491520538</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.05972204410305572</v>
+        <v>0.05535301530395638</v>
       </c>
       <c r="S23" s="38" t="n">
-        <v>0.05672005688937049</v>
+        <v>0.05825059229310237</v>
       </c>
       <c r="T23" s="38" t="n">
-        <v>0.04288946675222042</v>
+        <v>0.05703159391825534</v>
       </c>
       <c r="U23" s="23" t="n">
-        <v>0.0335350428042339</v>
+        <v>0.04280841579142882</v>
       </c>
     </row>
     <row r="24">
@@ -2923,7 +2925,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2938,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.29</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="30">
@@ -3001,8 +3003,10 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="52" t="n">
-        <v>46245</v>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'T10YIE' not found in values file."</t>
+        </is>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3019,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.27</v>
+        <v>1</v>
       </c>
       <c r="R30" s="45" t="n">
-        <v>2.29</v>
+        <v>1</v>
       </c>
       <c r="S30" s="45" t="n">
-        <v>2.25</v>
+        <v>1</v>
       </c>
       <c r="T30" s="45" t="n">
-        <v>2.26</v>
+        <v>1</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -3341,7 +3345,7 @@
           <t>PRS85006092</t>
         </is>
       </c>
-      <c r="C35" s="52" t="n">
+      <c r="C35" s="51" t="n">
         <v>46113</v>
       </c>
       <c r="D35" s="45" t="inlineStr">
@@ -3420,8 +3424,10 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
-        <v>46174</v>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
+        </is>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
@@ -3434,19 +3440,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1427</v>
+        <v>1</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1199</v>
+        <v>1</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1414</v>
+        <v>1</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1522</v>
+        <v>1</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1346</v>
+        <v>1</v>
       </c>
       <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3491,8 +3497,10 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
-        <v>46174</v>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
+        </is>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
@@ -3505,19 +3513,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.03480783176214648</v>
+        <v>1</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.06982156710628394</v>
+        <v>1</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>0.1307578008915305</v>
+        <v>1</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>-0.09725016767270288</v>
+        <v>1</v>
       </c>
       <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -4269,7 +4277,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4356,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4369,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.18</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.2</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4431,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,16 +4444,16 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.4</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>4.33</v>
       </c>
       <c r="U49" s="21" t="n">
         <v>4.33</v>
@@ -4501,8 +4509,10 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="52" t="n">
-        <v>46244</v>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
+        </is>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4525,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>4.72</v>
+        <v>1</v>
       </c>
       <c r="R50" s="45" t="n">
-        <v>4.65</v>
+        <v>1</v>
       </c>
       <c r="S50" s="45" t="n">
-        <v>4.69</v>
+        <v>1</v>
       </c>
       <c r="T50" s="45" t="n">
-        <v>4.63</v>
+        <v>1</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>4.63</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4576,7 +4586,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="52" t="n">
+      <c r="N51" s="51" t="n">
         <v>46237</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
@@ -4628,7 +4638,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,16 +4654,16 @@
         <v>6.34</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.3</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.25</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.27</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-14
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -949,7 +949,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="52" t="n">
+      <c r="N3" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
@@ -1020,7 +1020,7 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="52" t="n">
+      <c r="N4" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
@@ -1174,7 +1174,7 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="52" t="n">
+      <c r="N6" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
@@ -1253,7 +1253,7 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="52" t="n">
+      <c r="N7" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
@@ -1332,7 +1332,7 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="52" t="n">
+      <c r="N8" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
@@ -1411,7 +1411,7 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="52" t="n">
+      <c r="N9" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
@@ -1565,10 +1565,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'JTSHIR' not found in values file."</t>
-        </is>
+      <c r="N11" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
         <is>
@@ -1581,19 +1579,19 @@
         </is>
       </c>
       <c r="Q11" s="45" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="R11" s="45" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="S11" s="45" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="T11" s="45" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="U11" s="21" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="12">
@@ -1875,7 +1873,7 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="52" t="n">
+      <c r="N15" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -1962,8 +1960,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="51" t="n">
-        <v>46174</v>
+      <c r="C17" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
@@ -1976,19 +1974,19 @@
         </is>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.002186794214449339</v>
+        <v>-0.005819766896853373</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>0.01024770220406612</v>
+        <v>0.002453693069100149</v>
       </c>
       <c r="H17" s="25" t="n">
+        <v>0.009346631589902232</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>0.006742589318751824</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="J17" s="25" t="n">
         <v>0.01717978949867671</v>
-      </c>
-      <c r="J17" s="25" t="n">
-        <v>0.009223924204530221</v>
       </c>
       <c r="K17" s="46" t="n"/>
       <c r="L17" s="29" t="inlineStr">
@@ -2049,8 +2047,8 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="51" t="n">
-        <v>46174</v>
+      <c r="C18" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
@@ -2063,19 +2061,19 @@
         </is>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0.06719163968207242</v>
+        <v>0.05009241229083468</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>0.07328488075094505</v>
+        <v>0.06753173107393633</v>
       </c>
       <c r="H18" s="25" t="n">
+        <v>0.0723275853623377</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>0.05073763706982706</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.04240611939906461</v>
-      </c>
-      <c r="J18" s="25" t="n">
-        <v>0.04174261321715912</v>
       </c>
       <c r="K18" s="46" t="n"/>
       <c r="L18" s="28" t="inlineStr">
@@ -2353,7 +2351,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
@@ -2428,7 +2426,7 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
@@ -2502,7 +2500,7 @@
           <t>REVOLSL</t>
         </is>
       </c>
-      <c r="C24" s="52" t="n">
+      <c r="C24" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
@@ -2581,7 +2579,7 @@
           <t>NONREVSL</t>
         </is>
       </c>
-      <c r="C25" s="52" t="n">
+      <c r="C25" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -2925,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2938,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="30">
@@ -3003,10 +3001,8 @@
           <t>T10YIE</t>
         </is>
       </c>
-      <c r="N30" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'T10YIE' not found in values file."</t>
-        </is>
+      <c r="N30" s="52" t="n">
+        <v>46247</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3019,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>1</v>
+        <v>2.24</v>
       </c>
       <c r="R30" s="45" t="n">
-        <v>1</v>
+        <v>2.26</v>
       </c>
       <c r="S30" s="45" t="n">
-        <v>1</v>
+        <v>2.27</v>
       </c>
       <c r="T30" s="45" t="n">
-        <v>1</v>
+        <v>2.29</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -3230,7 +3226,7 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="52" t="n">
+      <c r="N33" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
@@ -3424,10 +3420,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
-        </is>
+      <c r="C36" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
@@ -3440,19 +3434,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1</v>
+        <v>1427</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1</v>
+        <v>1199</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>1</v>
+        <v>1414</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>1</v>
+        <v>1522</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>1</v>
+        <v>1346</v>
       </c>
       <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3497,10 +3491,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HOUST' not found in values file."</t>
-        </is>
+      <c r="C37" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
@@ -3513,19 +3505,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>1</v>
+        <v>0.03480783176214648</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>1</v>
+        <v>-0.06982156710628394</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>1</v>
+        <v>0.1307578008915305</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>1</v>
+        <v>-0.09725016767270288</v>
       </c>
       <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -4277,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4356,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4369,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.22</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.25</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.18</v>
       </c>
     </row>
     <row r="49">
@@ -4431,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4444,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.4</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.33</v>
       </c>
     </row>
     <row r="50">
@@ -4509,10 +4501,8 @@
           <t>DGS10</t>
         </is>
       </c>
-      <c r="N50" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'DGS10' not found in values file."</t>
-        </is>
+      <c r="N50" s="52" t="n">
+        <v>46246</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4525,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>1</v>
+        <v>4.68</v>
       </c>
       <c r="R50" s="45" t="n">
-        <v>1</v>
+        <v>4.7</v>
       </c>
       <c r="S50" s="45" t="n">
-        <v>1</v>
+        <v>4.72</v>
       </c>
       <c r="T50" s="45" t="n">
-        <v>1</v>
+        <v>4.65</v>
       </c>
       <c r="U50" s="21" t="n">
-        <v>1</v>
+        <v>4.69</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4586,8 +4576,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="51" t="n">
-        <v>46237</v>
+      <c r="N51" s="52" t="n">
+        <v>46244</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4600,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.69</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.66</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.58</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.55</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.49</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4638,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4657,13 +4647,13 @@
         <v>6.34</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.3</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.25</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-15
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>5.8334</v>
+        <v>4.312</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.29</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.25</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.22</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.25</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.19</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.25</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.35</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.4</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.72</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.65</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.69</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,7 +4641,7 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.34</v>
+        <v>6.3</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.34</v>
@@ -4650,10 +4650,10 @@
         <v>6.34</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.29</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.3</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-18
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.3</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.26</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.29</v>
       </c>
     </row>
     <row r="31">
@@ -3116,8 +3116,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n">
-        <v>46174</v>
+      <c r="C32" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
         <is>
@@ -3130,19 +3130,19 @@
         </is>
       </c>
       <c r="F32" s="25" t="n">
-        <v>0.000769301271638545</v>
+        <v>0.002014850155856562</v>
       </c>
       <c r="G32" s="25" t="n">
-        <v>0.001376689618002747</v>
+        <v>0.002701202518000656</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>0.007896301019906238</v>
+        <v>-9.656671199120836e-05</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>-0.003032583346986972</v>
+        <v>0.00752302359703716</v>
       </c>
       <c r="J32" s="25" t="n">
-        <v>0.008783754359711349</v>
+        <v>-0.001481767876646223</v>
       </c>
       <c r="K32" s="46" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -3187,8 +3187,8 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n">
-        <v>46174</v>
+      <c r="C33" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
         <is>
@@ -3201,19 +3201,19 @@
         </is>
       </c>
       <c r="F33" s="25" t="n">
-        <v>0.01144084707598163</v>
+        <v>0.01079455120026685</v>
       </c>
       <c r="G33" s="25" t="n">
-        <v>0.01579846581257943</v>
+        <v>0.01289238607192659</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>0.01277293407655064</v>
+        <v>0.01529631408748529</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>0.005708607646050407</v>
+        <v>0.01376375856712151</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>0.008180076419915847</v>
+        <v>0.00706549063542895</v>
       </c>
       <c r="K33" s="46" t="n"/>
       <c r="L33" s="28" t="inlineStr">
@@ -3266,8 +3266,8 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
-        <v>46174</v>
+      <c r="C34" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
         <is>
@@ -3280,19 +3280,19 @@
         </is>
       </c>
       <c r="F34" s="24" t="n">
-        <v>76.0937</v>
+        <v>76.2878</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>76.1019</v>
+        <v>76.2029</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>76.0625</v>
+        <v>76.0642</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>75.5313</v>
+        <v>76.1369</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>75.82989999999999</v>
+        <v>75.6332</v>
       </c>
       <c r="K34" s="46" t="n"/>
       <c r="L34" s="28" t="n"/>
@@ -3420,8 +3420,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="51" t="n">
-        <v>46174</v>
+      <c r="C36" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
@@ -3434,19 +3434,19 @@
         </is>
       </c>
       <c r="F36" s="24" t="n">
-        <v>1427</v>
+        <v>1239</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>1199</v>
+        <v>1415</v>
       </c>
       <c r="H36" s="24" t="n">
+        <v>1182</v>
+      </c>
+      <c r="I36" s="24" t="n">
         <v>1414</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="J36" s="24" t="n">
         <v>1522</v>
-      </c>
-      <c r="J36" s="24" t="n">
-        <v>1346</v>
       </c>
       <c r="K36" s="46" t="n"/>
       <c r="L36" s="28" t="n"/>
@@ -3491,8 +3491,8 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="51" t="n">
-        <v>46174</v>
+      <c r="C37" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
@@ -3505,19 +3505,19 @@
         </is>
       </c>
       <c r="F37" s="25" t="n">
-        <v>0.03480783176214648</v>
+        <v>-0.1347765363128492</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>-0.06982156710628394</v>
+        <v>0.02610587382160986</v>
       </c>
       <c r="H37" s="25" t="n">
+        <v>-0.08301008533747091</v>
+      </c>
+      <c r="I37" s="25" t="n">
         <v>0.01</v>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="J37" s="25" t="n">
         <v>0.1307578008915305</v>
-      </c>
-      <c r="J37" s="25" t="n">
-        <v>-0.09725016767270288</v>
       </c>
       <c r="K37" s="46" t="n"/>
       <c r="L37" s="28" t="inlineStr">
@@ -3570,8 +3570,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n">
-        <v>46174</v>
+      <c r="C38" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
         <is>
@@ -3584,19 +3584,19 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
+        <v>1443</v>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>1374</v>
       </c>
-      <c r="G38" s="24" t="n">
+      <c r="H38" s="24" t="n">
         <v>1410</v>
       </c>
-      <c r="H38" s="24" t="n">
+      <c r="I38" s="24" t="n">
         <v>1423</v>
       </c>
-      <c r="I38" s="24" t="n">
+      <c r="J38" s="24" t="n">
         <v>1363</v>
-      </c>
-      <c r="J38" s="24" t="n">
-        <v>1540</v>
       </c>
       <c r="K38" s="46" t="n"/>
       <c r="L38" s="28" t="n"/>
@@ -3641,8 +3641,8 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="51" t="n">
-        <v>46174</v>
+      <c r="C39" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
         <is>
@@ -3655,19 +3655,19 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
+        <v>0.03071428571428571</v>
+      </c>
+      <c r="G39" s="38" t="n">
         <v>-0.0178699070764832</v>
       </c>
-      <c r="G39" s="38" t="n">
+      <c r="H39" s="38" t="n">
         <v>-0.00423728813559322</v>
       </c>
-      <c r="H39" s="38" t="n">
+      <c r="I39" s="38" t="n">
         <v>-0.01522491349480969</v>
       </c>
-      <c r="I39" s="38" t="n">
+      <c r="J39" s="38" t="n">
         <v>-0.08646112600536193</v>
-      </c>
-      <c r="J39" s="38" t="n">
-        <v>0.06500691562932227</v>
       </c>
       <c r="K39" s="46" t="n"/>
       <c r="L39" s="28" t="inlineStr">
@@ -3830,8 +3830,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="51" t="n">
-        <v>46174</v>
+      <c r="N41" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
         <is>
@@ -3844,19 +3844,19 @@
         </is>
       </c>
       <c r="Q41" s="38" t="n">
-        <v>-0.005924170616113722</v>
+        <v>-0.01312649164677793</v>
       </c>
       <c r="R41" s="38" t="n">
+        <v>-0.007109004739336622</v>
+      </c>
+      <c r="S41" s="38" t="n">
         <v>0.01199040767386084</v>
       </c>
-      <c r="S41" s="38" t="n">
+      <c r="T41" s="38" t="n">
         <v>0.03538175046554937</v>
       </c>
-      <c r="T41" s="38" t="n">
+      <c r="U41" s="23" t="n">
         <v>0.01704545454545436</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0.01930501930501927</v>
       </c>
     </row>
     <row r="42">
@@ -3905,8 +3905,8 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="51" t="n">
-        <v>46174</v>
+      <c r="N42" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
         <is>
@@ -3919,19 +3919,19 @@
         </is>
       </c>
       <c r="Q42" s="38" t="n">
-        <v>0.1017728168089297</v>
+        <v>0.08246073298429316</v>
       </c>
       <c r="R42" s="38" t="n">
+        <v>0.1004596191726854</v>
+      </c>
+      <c r="S42" s="38" t="n">
         <v>0.1134564643799473</v>
       </c>
-      <c r="S42" s="38" t="n">
+      <c r="T42" s="38" t="n">
         <v>0.09305373525557023</v>
       </c>
-      <c r="T42" s="38" t="n">
+      <c r="U42" s="23" t="n">
         <v>0.05639344262295078</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0.03800786369593716</v>
       </c>
     </row>
     <row r="43">
@@ -3980,8 +3980,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="51" t="n">
-        <v>46174</v>
+      <c r="N43" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
         <is>
@@ -3994,19 +3994,19 @@
         </is>
       </c>
       <c r="Q43" s="38" t="n">
-        <v>0.003326679973386648</v>
+        <v>-0.003994673768308865</v>
       </c>
       <c r="R43" s="38" t="n">
-        <v>0.01691474966170503</v>
+        <v>-0.002656042496679945</v>
       </c>
       <c r="S43" s="38" t="n">
-        <v>0.02071823204419898</v>
+        <v>0.01688048615800142</v>
       </c>
       <c r="T43" s="38" t="n">
+        <v>0.02279005524861866</v>
+      </c>
+      <c r="U43" s="23" t="n">
         <v>0.009059233449477455</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>0.009852216748768461</v>
       </c>
     </row>
     <row r="44">
@@ -4055,8 +4055,8 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="51" t="n">
-        <v>46174</v>
+      <c r="N44" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
         <is>
@@ -4069,19 +4069,19 @@
         </is>
       </c>
       <c r="Q44" s="38" t="n">
-        <v>0.07102272727272727</v>
+        <v>0.05949008498583574</v>
       </c>
       <c r="R44" s="38" t="n">
-        <v>0.06595744680851072</v>
+        <v>0.06676136363636347</v>
       </c>
       <c r="S44" s="38" t="n">
-        <v>0.04304869442484138</v>
+        <v>0.06808510638297868</v>
       </c>
       <c r="T44" s="38" t="n">
+        <v>0.04516584333098099</v>
+      </c>
+      <c r="U44" s="23" t="n">
         <v>0.0225988700564973</v>
-      </c>
-      <c r="U44" s="23" t="n">
-        <v>0.009852216748768513</v>
       </c>
     </row>
     <row r="45">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.15</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.22</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.25</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.19</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.32</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.41</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.35</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.72</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.65</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,10 +4641,10 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.3</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.34</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.34</v>
@@ -4653,7 +4653,7 @@
         <v>6.34</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.29</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-19
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.312</v>
+        <v>4.0302</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -2086,7 +2086,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N18" s="52" t="n">
+      <c r="N18" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O18" s="45" t="inlineStr">
@@ -2161,7 +2161,7 @@
           <t>CPIAUCSL</t>
         </is>
       </c>
-      <c r="N19" s="52" t="n">
+      <c r="N19" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O19" s="45" t="inlineStr">
@@ -2236,7 +2236,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N20" s="52" t="n">
+      <c r="N20" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O20" s="45" t="inlineStr">
@@ -2311,7 +2311,7 @@
           <t>CPILFESL</t>
         </is>
       </c>
-      <c r="N21" s="52" t="n">
+      <c r="N21" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O21" s="45" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.3</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.24</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.26</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.15</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.22</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.25</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.36</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.32</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.39</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.41</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.7</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.72</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,13 +4641,13 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.37</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.3</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.34</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.34</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-08-20
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46237</v>
+        <v>46244</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,19 +1733,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>209000</v>
+        <v>206000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>212000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>200000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>198000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>189000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>209000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46230</v>
+        <v>46237</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
+        <v>1799000</v>
+      </c>
+      <c r="R14" s="24" t="n">
+        <v>1781000</v>
+      </c>
+      <c r="S14" s="24" t="n">
+        <v>1799000</v>
+      </c>
+      <c r="T14" s="24" t="n">
         <v>1777000</v>
       </c>
-      <c r="R14" s="24" t="n">
-        <v>1799000</v>
-      </c>
-      <c r="S14" s="24" t="n">
-        <v>1777000</v>
-      </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1789000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1798000</v>
       </c>
     </row>
     <row r="15">
@@ -2390,7 +2390,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N22" s="52" t="n">
+      <c r="N22" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O22" s="45" t="inlineStr">
@@ -2460,7 +2460,7 @@
           <t>PPIFIS</t>
         </is>
       </c>
-      <c r="N23" s="52" t="n">
+      <c r="N23" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O23" s="45" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.3</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.28</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         <v>2.3</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.27</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.24</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.26</v>
       </c>
     </row>
     <row r="31">
@@ -3720,8 +3720,10 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="51" t="n">
-        <v>46174</v>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
+        </is>
       </c>
       <c r="D40" s="45" t="inlineStr">
         <is>
@@ -3734,19 +3736,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>628</v>
+        <v>1</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>618</v>
+        <v>1</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>646</v>
+        <v>1</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>659</v>
+        <v>1</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>630</v>
+        <v>1</v>
       </c>
       <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3791,8 +3793,10 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="51" t="n">
-        <v>46174</v>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
+        </is>
       </c>
       <c r="D41" s="45" t="inlineStr">
         <is>
@@ -3805,19 +3809,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.0556390977443609</v>
+        <v>1</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.006430868167202572</v>
+        <v>1</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>-0.07845934379457917</v>
+        <v>1</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>0.004573170731707317</v>
+        <v>1</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>-0.0171606864274571</v>
+        <v>1</v>
       </c>
       <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4269,7 +4273,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4352,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,16 +4368,16 @@
         <v>4.19</v>
       </c>
       <c r="R48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="S48" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.15</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.2</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.22</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4427,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4440,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.36</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.32</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.38</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.39</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4506,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4519,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.72</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.63</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.68</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.7</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4576,7 +4580,7 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="52" t="n">
+      <c r="N51" s="51" t="n">
         <v>46244</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
@@ -4628,7 +4632,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,16 +4645,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.41</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.37</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.3</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.34</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.34</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-08-21
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1960,7 +1960,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C17" s="52" t="n">
+      <c r="C17" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -2047,7 +2047,7 @@
           <t>RSAFS</t>
         </is>
       </c>
-      <c r="C18" s="52" t="n">
+      <c r="C18" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="45" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.3</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.3</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.28</v>
       </c>
-      <c r="T30" s="45" t="n">
+      <c r="U30" s="21" t="n">
         <v>2.27</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.24</v>
       </c>
     </row>
     <row r="31">
@@ -3720,10 +3720,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
-        </is>
+      <c r="C40" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
         <is>
@@ -3736,19 +3734,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>628</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>1</v>
+        <v>618</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>1</v>
+        <v>646</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>1</v>
+        <v>659</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>1</v>
+        <v>630</v>
       </c>
       <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3793,10 +3791,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>ERR: "Ticker 'HSN1F' not found in values file."</t>
-        </is>
+      <c r="C41" s="51" t="n">
+        <v>46174</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
         <is>
@@ -3809,19 +3805,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>1</v>
+        <v>-0.0556390977443609</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>1</v>
+        <v>-0.006430868167202572</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>1</v>
+        <v>-0.07845934379457917</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>1</v>
+        <v>0.004573170731707317</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>1</v>
+        <v>-0.0171606864274571</v>
       </c>
       <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -4273,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4352,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4371,13 +4367,13 @@
         <v>4.19</v>
       </c>
       <c r="S48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="T48" s="45" t="n">
         <v>4.17</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.15</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.2</v>
       </c>
     </row>
     <row r="49">
@@ -4427,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4440,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.36</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.32</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.38</v>
       </c>
     </row>
     <row r="50">
@@ -4506,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4519,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.71</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.72</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.68</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.63</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.68</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4580,8 +4576,8 @@
           <t>MORTGAGE30US</t>
         </is>
       </c>
-      <c r="N51" s="51" t="n">
-        <v>46244</v>
+      <c r="N51" s="52" t="n">
+        <v>46251</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4594,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.67</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.69</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.66</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.58</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.55</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4632,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4645,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.39</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.41</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.37</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.3</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.34</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-22
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,16 +2939,16 @@
         <v>2.34</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.3</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,16 +3018,16 @@
         <v>2.34</v>
       </c>
       <c r="R30" s="45" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.3</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.28</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.27</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4370,10 +4370,10 @@
         <v>4.19</v>
       </c>
       <c r="T48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.15</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.36</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.32</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.71</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.72</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.68</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.63</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.39</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.41</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.37</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.3</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-25
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="S30" s="45" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.3</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.28</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="31">
@@ -3116,7 +3116,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C32" s="52" t="n">
+      <c r="C32" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D32" s="45" t="inlineStr">
@@ -3187,7 +3187,7 @@
           <t>INDPRO</t>
         </is>
       </c>
-      <c r="C33" s="52" t="n">
+      <c r="C33" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D33" s="45" t="inlineStr">
@@ -3266,7 +3266,7 @@
           <t>TCU</t>
         </is>
       </c>
-      <c r="C34" s="52" t="n">
+      <c r="C34" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D34" s="45" t="inlineStr">
@@ -3420,7 +3420,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C36" s="52" t="n">
+      <c r="C36" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D36" s="45" t="inlineStr">
@@ -3491,7 +3491,7 @@
           <t>HOUST</t>
         </is>
       </c>
-      <c r="C37" s="52" t="n">
+      <c r="C37" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D37" s="45" t="inlineStr">
@@ -3570,7 +3570,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C38" s="52" t="n">
+      <c r="C38" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D38" s="45" t="inlineStr">
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1443</v>
+        <v>1433</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>1374</v>
@@ -3641,7 +3641,7 @@
           <t>PERMIT</t>
         </is>
       </c>
-      <c r="C39" s="52" t="n">
+      <c r="C39" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D39" s="45" t="inlineStr">
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="F39" s="38" t="n">
-        <v>0.03071428571428571</v>
+        <v>0.02357142857142857</v>
       </c>
       <c r="G39" s="38" t="n">
         <v>-0.0178699070764832</v>
@@ -3720,8 +3720,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="51" t="n">
-        <v>46174</v>
+      <c r="C40" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
         <is>
@@ -3734,19 +3734,19 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>628</v>
+        <v>607</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>618</v>
+        <v>678</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>646</v>
+        <v>630</v>
       </c>
       <c r="I40" s="24" t="n">
+        <v>641</v>
+      </c>
+      <c r="J40" s="24" t="n">
         <v>659</v>
-      </c>
-      <c r="J40" s="24" t="n">
-        <v>630</v>
       </c>
       <c r="K40" s="46" t="n"/>
       <c r="L40" s="28" t="n"/>
@@ -3791,8 +3791,8 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="51" t="n">
-        <v>46174</v>
+      <c r="C41" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
         <is>
@@ -3805,19 +3805,19 @@
         </is>
       </c>
       <c r="F41" s="38" t="n">
-        <v>-0.0556390977443609</v>
+        <v>-0.06327160493827161</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>-0.006430868167202572</v>
+        <v>0.01954887218045113</v>
       </c>
       <c r="H41" s="38" t="n">
-        <v>-0.07845934379457917</v>
+        <v>0.01286173633440514</v>
       </c>
       <c r="I41" s="38" t="n">
+        <v>-0.08559201141226819</v>
+      </c>
+      <c r="J41" s="38" t="n">
         <v>0.004573170731707317</v>
-      </c>
-      <c r="J41" s="38" t="n">
-        <v>-0.0171606864274571</v>
       </c>
       <c r="K41" s="46" t="n"/>
       <c r="L41" s="28" t="inlineStr">
@@ -3830,7 +3830,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N41" s="52" t="n">
+      <c r="N41" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O41" s="45" t="inlineStr">
@@ -3905,7 +3905,7 @@
           <t>IQ</t>
         </is>
       </c>
-      <c r="N42" s="52" t="n">
+      <c r="N42" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O42" s="45" t="inlineStr">
@@ -3980,7 +3980,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N43" s="52" t="n">
+      <c r="N43" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O43" s="45" t="inlineStr">
@@ -4055,7 +4055,7 @@
           <t>IR</t>
         </is>
       </c>
-      <c r="N44" s="52" t="n">
+      <c r="N44" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O44" s="45" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,7 +4361,7 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
-        <v>4.19</v>
+        <v>4.24</v>
       </c>
       <c r="R48" s="45" t="n">
         <v>4.19</v>
@@ -4373,7 +4373,7 @@
         <v>4.19</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>4.17</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.38</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.36</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.71</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.72</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.68</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.33</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.39</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.41</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.37</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-26
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>24270.599</v>
+        <v>24269.613</v>
       </c>
       <c r="G3" s="24" t="n">
         <v>24180.419</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0.003729463910447484</v>
+        <v>0.003688687114975053</v>
       </c>
       <c r="G4" s="25" t="n">
         <v>0.00518254492928083</v>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.0302</v>
+        <v>4.6099</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1386,7 +1386,7 @@
         </is>
       </c>
       <c r="F9" s="24" t="n">
-        <v>16817.938</v>
+        <v>16829.681</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>16687.728</v>
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0.007802739833726813</v>
+        <v>0.008506430593787417</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>0.001350657318094584</v>
@@ -1526,8 +1526,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="51" t="n">
-        <v>46174</v>
+      <c r="C11" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
@@ -1540,19 +1540,19 @@
         </is>
       </c>
       <c r="F11" s="25" t="n">
-        <v>0.01478556341261816</v>
+        <v>-0.01390979158115568</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.01269472215763789</v>
+        <v>0.00767463235294108</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>-0.01239954075774974</v>
+        <v>0.01091753774680604</v>
       </c>
       <c r="I11" s="25" t="n">
+        <v>-0.01148105625717566</v>
+      </c>
+      <c r="J11" s="25" t="n">
         <v>0.01363932594730488</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>0.0203286786358885</v>
       </c>
       <c r="K11" s="46" t="n"/>
       <c r="L11" s="28" t="inlineStr">
@@ -1601,8 +1601,8 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="51" t="n">
-        <v>46174</v>
+      <c r="C12" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
@@ -1615,19 +1615,19 @@
         </is>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0.04546099626283169</v>
+        <v>0.009618976466193458</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.02837984605940425</v>
+        <v>0.03727707081697323</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>-0.006697459584295612</v>
+        <v>0.02752986730887292</v>
       </c>
       <c r="I12" s="25" t="n">
+        <v>-0.005773672055427252</v>
+      </c>
+      <c r="J12" s="25" t="n">
         <v>-0.000734248084071364</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>0.02696242470599466</v>
       </c>
       <c r="K12" s="46" t="n"/>
       <c r="L12" s="28" t="inlineStr">
@@ -1680,8 +1680,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="51" t="n">
-        <v>46174</v>
+      <c r="C13" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
@@ -1694,19 +1694,19 @@
         </is>
       </c>
       <c r="F13" s="25" t="n">
-        <v>0.003373010342039962</v>
+        <v>-0.002005291742097182</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.002543178134257529</v>
+        <v>0.004925970500153865</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>0.003533767107920083</v>
+        <v>-0.001648597295182741</v>
       </c>
       <c r="I13" s="25" t="n">
+        <v>0.003702041732106975</v>
+      </c>
+      <c r="J13" s="25" t="n">
         <v>0.005754259280153384</v>
-      </c>
-      <c r="J13" s="25" t="n">
-        <v>0.001865144407392716</v>
       </c>
       <c r="K13" s="46" t="n"/>
       <c r="L13" s="28" t="inlineStr">
@@ -1755,8 +1755,8 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="51" t="n">
-        <v>46174</v>
+      <c r="C14" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
@@ -1769,19 +1769,19 @@
         </is>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0.02174406721925738</v>
+        <v>0.01417978036907063</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.02544092845096189</v>
+        <v>0.01921766776427836</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.02161313347608846</v>
+        <v>0.02132464339822197</v>
       </c>
       <c r="I14" s="25" t="n">
+        <v>0.02178443968593867</v>
+      </c>
+      <c r="J14" s="25" t="n">
         <v>0.01787039680274048</v>
-      </c>
-      <c r="J14" s="25" t="n">
-        <v>0.0159621722309786</v>
       </c>
       <c r="K14" s="46" t="n"/>
       <c r="L14" s="28" t="inlineStr">
@@ -1834,8 +1834,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="51" t="n">
-        <v>46174</v>
+      <c r="C15" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -1848,19 +1848,19 @@
         </is>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.002561096582198497</v>
+        <v>0.002869028833739851</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.002957589790436366</v>
+        <v>0.003770800147592235</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>0.002766239184458286</v>
+        <v>0.004156989616562967</v>
       </c>
       <c r="I15" s="25" t="n">
+        <v>0.003618785031471727</v>
+      </c>
+      <c r="J15" s="25" t="n">
         <v>0.0001360630606932478</v>
-      </c>
-      <c r="J15" s="25" t="n">
-        <v>-0.0004895872054544448</v>
       </c>
       <c r="K15" s="46" t="n"/>
       <c r="L15" s="28" t="inlineStr">
@@ -1909,8 +1909,8 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="51" t="n">
-        <v>46174</v>
+      <c r="C16" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
@@ -1923,19 +1923,19 @@
         </is>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0.02340010310037548</v>
+        <v>0.02533641330253361</v>
       </c>
       <c r="G16" s="25" t="n">
-        <v>0.02280064195982224</v>
+        <v>0.02673245452537002</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>0.02165034189613743</v>
+        <v>0.02489439023040468</v>
       </c>
       <c r="I16" s="25" t="n">
+        <v>0.02251894289410467</v>
+      </c>
+      <c r="J16" s="25" t="n">
         <v>0.02201458987977717</v>
-      </c>
-      <c r="J16" s="25" t="n">
-        <v>0.02561168480788904</v>
       </c>
       <c r="K16" s="46" t="n"/>
       <c r="L16" s="28" t="n"/>
@@ -2126,8 +2126,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="51" t="n">
-        <v>46174</v>
+      <c r="C19" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
         <is>
@@ -2140,19 +2140,19 @@
         </is>
       </c>
       <c r="F19" s="25" t="n">
-        <v>0.003127812531250385</v>
+        <v>0.003744135940935589</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>0.002428130673527651</v>
+        <v>0.003044427530958238</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>-0.004120795319042747</v>
+        <v>0.002394596009377858</v>
       </c>
       <c r="I19" s="25" t="n">
+        <v>-0.004070879897950741</v>
+      </c>
+      <c r="J19" s="25" t="n">
         <v>-0.001185470781469022</v>
-      </c>
-      <c r="J19" s="25" t="n">
-        <v>-0.004560343211319595</v>
       </c>
       <c r="K19" s="46" t="n"/>
       <c r="L19" s="28" t="n"/>
@@ -2197,8 +2197,8 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="51" t="n">
-        <v>46174</v>
+      <c r="C20" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
         <is>
@@ -2211,19 +2211,19 @@
         </is>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0.005233241102098308</v>
+        <v>0.004523055945102436</v>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0.001051115350177011</v>
+        <v>0.005166433768880193</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>-0.009744718164220876</v>
+        <v>0.001067799720814703</v>
       </c>
       <c r="I20" s="25" t="n">
+        <v>-0.009695084625184218</v>
+      </c>
+      <c r="J20" s="25" t="n">
         <v>7.7652239989875e-05</v>
-      </c>
-      <c r="J20" s="25" t="n">
-        <v>0.007894810306803354</v>
       </c>
       <c r="K20" s="46" t="n"/>
       <c r="L20" s="28" t="inlineStr">
@@ -2276,8 +2276,8 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="51" t="n">
-        <v>46174</v>
+      <c r="C21" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -2290,19 +2290,19 @@
         </is>
       </c>
       <c r="F21" s="45" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="G21" s="45" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H21" s="45" t="n">
         <v>2.8</v>
       </c>
-      <c r="H21" s="45" t="n">
-        <v>3</v>
-      </c>
       <c r="I21" s="45" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J21" s="45" t="n">
         <v>3.5</v>
-      </c>
-      <c r="J21" s="45" t="n">
-        <v>3.8</v>
       </c>
       <c r="K21" s="46" t="n"/>
       <c r="L21" s="28" t="n"/>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>16.782</v>
+        <v>16.757</v>
       </c>
       <c r="G22" s="24" t="n">
         <v>17.043</v>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
-        <v>-0.01270737733851048</v>
+        <v>-0.01417813860454169</v>
       </c>
       <c r="G23" s="25" t="n">
         <v>0.04673872988576337</v>
@@ -2539,8 +2539,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="51" t="n">
-        <v>46174</v>
+      <c r="N24" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
         <is>
@@ -2553,19 +2553,19 @@
         </is>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>-0.001087163112479583</v>
+        <v>0.00155948088304636</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>0.004605444047291796</v>
+        <v>-0.0009272207697451629</v>
       </c>
       <c r="S24" s="38" t="n">
-        <v>0.004056655138302112</v>
+        <v>0.004811143524811712</v>
       </c>
       <c r="T24" s="38" t="n">
+        <v>0.004164014631565349</v>
+      </c>
+      <c r="U24" s="23" t="n">
         <v>0.006669806004369283</v>
-      </c>
-      <c r="U24" s="23" t="n">
-        <v>0.003999286948838554</v>
       </c>
     </row>
     <row r="25">
@@ -2614,8 +2614,8 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="51" t="n">
-        <v>46174</v>
+      <c r="N25" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
@@ -2628,19 +2628,19 @@
         </is>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.03668052673520432</v>
+        <v>0.03701165721487081</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>0.0407896819116949</v>
+        <v>0.03716970562476833</v>
       </c>
       <c r="S25" s="38" t="n">
-        <v>0.03790725326991663</v>
+        <v>0.04111410033233105</v>
       </c>
       <c r="T25" s="38" t="n">
+        <v>0.03801823226317869</v>
+      </c>
+      <c r="U25" s="23" t="n">
         <v>0.03542928831754543</v>
-      </c>
-      <c r="U25" s="23" t="n">
-        <v>0.02873230041057473</v>
       </c>
     </row>
     <row r="26">
@@ -2668,7 +2668,7 @@
         </is>
       </c>
       <c r="F26" s="38" t="n">
-        <v>0.02041382805407022</v>
+        <v>0.02059204359604272</v>
       </c>
       <c r="G26" s="38" t="n">
         <v>0.02552585944536068</v>
@@ -2693,8 +2693,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="51" t="n">
-        <v>46174</v>
+      <c r="N26" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
         <is>
@@ -2707,19 +2707,19 @@
         </is>
       </c>
       <c r="Q26" s="38" t="n">
-        <v>0.00132212092794437</v>
+        <v>0.002455155058386671</v>
       </c>
       <c r="R26" s="38" t="n">
-        <v>0.003324001449912295</v>
+        <v>0.001467571284778035</v>
       </c>
       <c r="S26" s="38" t="n">
-        <v>0.002474041888621992</v>
+        <v>0.003593433116647615</v>
       </c>
       <c r="T26" s="38" t="n">
+        <v>0.002613206744856766</v>
+      </c>
+      <c r="U26" s="23" t="n">
         <v>0.002962135839517099</v>
-      </c>
-      <c r="U26" s="23" t="n">
-        <v>0.003939122649955218</v>
       </c>
     </row>
     <row r="27">
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="F27" s="38" t="n">
-        <v>0.003742997804626613</v>
+        <v>0.00317839655928509</v>
       </c>
       <c r="G27" s="38" t="n">
         <v>-0.0201499882390509</v>
@@ -2768,8 +2768,8 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="51" t="n">
-        <v>46174</v>
+      <c r="N27" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
@@ -2782,19 +2782,19 @@
         </is>
       </c>
       <c r="Q27" s="38" t="n">
-        <v>0.03286526430967084</v>
+        <v>0.03344143004033837</v>
       </c>
       <c r="R27" s="38" t="n">
-        <v>0.03421575641942911</v>
+        <v>0.03343614465473631</v>
       </c>
       <c r="S27" s="38" t="n">
-        <v>0.03315485012191053</v>
+        <v>0.03463709356864603</v>
       </c>
       <c r="T27" s="38" t="n">
+        <v>0.03329827413108968</v>
+      </c>
+      <c r="U27" s="23" t="n">
         <v>0.03253849776876586</v>
-      </c>
-      <c r="U27" s="23" t="n">
-        <v>0.03049262855088111</v>
       </c>
     </row>
     <row r="28">
@@ -2808,8 +2808,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="51" t="n">
-        <v>46174</v>
+      <c r="C28" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
         <is>
@@ -2822,19 +2822,19 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.00472079606520448</v>
+        <v>0.01071642440258236</v>
       </c>
       <c r="G28" s="25" t="n">
+        <v>0.005424721874419669</v>
+      </c>
+      <c r="H28" s="25" t="n">
         <v>-0.04004117699494203</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="I28" s="25" t="n">
         <v>0.08512722904348102</v>
       </c>
-      <c r="I28" s="25" t="n">
+      <c r="J28" s="25" t="n">
         <v>0.01344578206575542</v>
-      </c>
-      <c r="J28" s="25" t="n">
-        <v>-0.01169466364559735</v>
       </c>
       <c r="K28" s="46" t="n"/>
       <c r="L28" s="28" t="inlineStr">
@@ -2883,8 +2883,8 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="51" t="n">
-        <v>46174</v>
+      <c r="C29" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
         <is>
@@ -2897,19 +2897,19 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.07588184538797348</v>
+        <v>0.1195187306951081</v>
       </c>
       <c r="G29" s="25" t="n">
+        <v>0.07663562793293581</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <v>-0.02972368914374733</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="I29" s="25" t="n">
         <v>0.1779567725392831</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="J29" s="25" t="n">
         <v>0.01350347073984473</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>0.07567733047604469</v>
       </c>
       <c r="K29" s="46" t="n"/>
       <c r="L29" s="28" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.32</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.34</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -2962,8 +2962,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="51" t="n">
-        <v>46174</v>
+      <c r="C30" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
         <is>
@@ -2976,19 +2976,19 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.004536178951609848</v>
+        <v>0.01289555603784764</v>
       </c>
       <c r="G30" s="25" t="n">
+        <v>0.003129183617765152</v>
+      </c>
+      <c r="H30" s="25" t="n">
         <v>-0.04261964610139124</v>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="I30" s="25" t="n">
         <v>0.08475262626842106</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="J30" s="25" t="n">
         <v>-0.002709178900039744</v>
-      </c>
-      <c r="J30" s="25" t="n">
-        <v>-0.01222345960141613</v>
       </c>
       <c r="K30" s="46" t="n"/>
       <c r="L30" s="28" t="inlineStr">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,13 +3018,13 @@
         <v>2.32</v>
       </c>
       <c r="R30" s="45" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.34</v>
       </c>
       <c r="T30" s="45" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.3</v>
@@ -3037,8 +3037,8 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="51" t="n">
-        <v>46174</v>
+      <c r="C31" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
         <is>
@@ -3051,19 +3051,19 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.05860719312123111</v>
+        <v>0.0971379650324378</v>
       </c>
       <c r="G31" s="25" t="n">
+        <v>0.05712446366627972</v>
+      </c>
+      <c r="H31" s="25" t="n">
         <v>-0.04567753459150702</v>
       </c>
-      <c r="H31" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>0.1533794281326583</v>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>-0.0182024802287403</v>
-      </c>
-      <c r="J31" s="25" t="n">
-        <v>0.07288240242929306</v>
       </c>
       <c r="K31" s="46" t="n"/>
       <c r="L31" s="28" t="inlineStr">
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="N34" s="51" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O34" s="45" t="inlineStr">
         <is>
@@ -3315,19 +3315,19 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.002485931130862563</v>
+        <v>-0.005283345196001861</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.007146470713941611</v>
+        <v>-0.00295640652354665</v>
       </c>
       <c r="S34" s="38" t="n">
-        <v>-0.002112874294617258</v>
+        <v>-0.007455850803781246</v>
       </c>
       <c r="T34" s="38" t="n">
+        <v>-0.002219562698691556</v>
+      </c>
+      <c r="U34" s="23" t="n">
         <v>-0.001052481507739263</v>
-      </c>
-      <c r="U34" s="23" t="n">
-        <v>0.008042734635068088</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
@@ -3381,7 +3381,7 @@
         </is>
       </c>
       <c r="N35" s="51" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O35" s="45" t="inlineStr">
         <is>
@@ -3394,19 +3394,19 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>0.004025655420760277</v>
+        <v>-0.001025966015042346</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>-0.002455668950446244</v>
+        <v>0.00386492016820239</v>
       </c>
       <c r="S35" s="38" t="n">
-        <v>-0.002440329858829915</v>
+        <v>-0.002659880805601422</v>
       </c>
       <c r="T35" s="38" t="n">
+        <v>-0.002546983253221669</v>
+      </c>
+      <c r="U35" s="23" t="n">
         <v>-0.004493337788724072</v>
-      </c>
-      <c r="U35" s="23" t="n">
-        <v>-0.0007660751460527582</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
@@ -3456,7 +3456,7 @@
         </is>
       </c>
       <c r="N36" s="51" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O36" s="45" t="inlineStr">
         <is>
@@ -3469,19 +3469,19 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.002485931130862563</v>
+        <v>-0.005283345196001861</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.007146470713941611</v>
+        <v>-0.00295640652354665</v>
       </c>
       <c r="S36" s="38" t="n">
-        <v>-0.002112874294617258</v>
+        <v>-0.007455850803781246</v>
       </c>
       <c r="T36" s="38" t="n">
+        <v>-0.002219562698691556</v>
+      </c>
+      <c r="U36" s="23" t="n">
         <v>-0.001052481507739263</v>
-      </c>
-      <c r="U36" s="23" t="n">
-        <v>0.008042734635068088</v>
       </c>
     </row>
     <row r="37">
@@ -4034,7 +4034,7 @@
         </is>
       </c>
       <c r="F44" s="24" t="n">
-        <v>5546.153</v>
+        <v>5543.809</v>
       </c>
       <c r="G44" s="24" t="n">
         <v>5416.715</v>
@@ -4105,7 +4105,7 @@
         </is>
       </c>
       <c r="F45" s="38" t="n">
-        <v>0.02389603292770626</v>
+        <v>0.02346329832749183</v>
       </c>
       <c r="G45" s="38" t="n">
         <v>0.01369922745579544</v>
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,7 +4364,7 @@
         <v>4.24</v>
       </c>
       <c r="R48" s="45" t="n">
-        <v>4.19</v>
+        <v>4.24</v>
       </c>
       <c r="S48" s="45" t="n">
         <v>4.19</v>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.39</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.37</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.38</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.74</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.69</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.65</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.71</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.72</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.37</v>
       </c>
-      <c r="R52" s="9" t="n">
+      <c r="S52" s="9" t="n">
         <v>6.33</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.29</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.39</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.41</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-27
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,19 +1733,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>206000</v>
+        <v>203000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>207000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>212000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>200000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>198000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>189000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46237</v>
+        <v>46244</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
+        <v>1778000</v>
+      </c>
+      <c r="R14" s="24" t="n">
+        <v>1796000</v>
+      </c>
+      <c r="S14" s="24" t="n">
+        <v>1781000</v>
+      </c>
+      <c r="T14" s="24" t="n">
         <v>1799000</v>
       </c>
-      <c r="R14" s="24" t="n">
-        <v>1781000</v>
-      </c>
-      <c r="S14" s="24" t="n">
-        <v>1799000</v>
-      </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1777000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1789000</v>
       </c>
     </row>
     <row r="15">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.33</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.32</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="T30" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.34</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.3</v>
       </c>
     </row>
     <row r="31">
@@ -3530,8 +3530,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="51" t="n">
-        <v>46143</v>
+      <c r="N37" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
         <is>
@@ -3544,19 +3544,19 @@
         </is>
       </c>
       <c r="Q37" s="38" t="n">
-        <v>0.006366672272541729</v>
+        <v>0.003675878722833481</v>
       </c>
       <c r="R37" s="38" t="n">
-        <v>0.008345748997662161</v>
+        <v>0.006967689254868681</v>
       </c>
       <c r="S37" s="38" t="n">
-        <v>0.007532973922912856</v>
+        <v>0.00856545961002797</v>
       </c>
       <c r="T37" s="38" t="n">
-        <v>0.00315552998212576</v>
+        <v>0.007608622698956014</v>
       </c>
       <c r="U37" s="23" t="n">
-        <v>-0.0009081874474428098</v>
+        <v>0.003179830266230477</v>
       </c>
     </row>
     <row r="38">
@@ -3605,8 +3605,8 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="51" t="n">
-        <v>46143</v>
+      <c r="N38" s="52" t="n">
+        <v>46174</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
         <is>
@@ -3619,19 +3619,19 @@
         </is>
       </c>
       <c r="Q38" s="38" t="n">
-        <v>0.01114021218302297</v>
+        <v>0.01525308725742975</v>
       </c>
       <c r="R38" s="38" t="n">
-        <v>0.009369704722440333</v>
+        <v>0.01210861241276107</v>
       </c>
       <c r="S38" s="38" t="n">
-        <v>0.007600606583937686</v>
+        <v>0.009742493823792416</v>
       </c>
       <c r="T38" s="38" t="n">
-        <v>0.008095298145032572</v>
+        <v>0.007762345302316447</v>
       </c>
       <c r="U38" s="23" t="n">
-        <v>0.009482201947111055</v>
+        <v>0.008178342616885069</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,16 +4361,16 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="R48" s="45" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="S48" s="45" t="n">
         <v>4.24</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.24</v>
-      </c>
-      <c r="S48" s="45" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="T48" s="45" t="n">
-        <v>4.19</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.19</v>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="R49" s="45" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="S49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.43</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.39</v>
-      </c>
-      <c r="T49" s="45" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.37</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="R50" s="45" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.74</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.69</v>
-      </c>
-      <c r="T50" s="45" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.71</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46251</v>
+        <v>46258</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4590,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.65</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.67</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.69</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.66</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.58</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,19 +4641,19 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.33</v>
+        <v>6.27</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>6.37</v>
+        <v>6.26</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.33</v>
       </c>
       <c r="T52" s="9" t="n">
-        <v>6.29</v>
+        <v>6.37</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.39</v>
+        <v>6.33</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-28
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="N28" s="51" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
@@ -2861,19 +2861,19 @@
         </is>
       </c>
       <c r="Q28" s="45" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="R28" s="45" t="n">
         <v>4.6</v>
       </c>
-      <c r="R28" s="45" t="n">
+      <c r="S28" s="45" t="n">
         <v>4.8</v>
       </c>
-      <c r="S28" s="45" t="n">
+      <c r="T28" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="T28" s="45" t="n">
+      <c r="U28" s="21" t="n">
         <v>3.8</v>
-      </c>
-      <c r="U28" s="21" t="n">
-        <v>3.4</v>
       </c>
     </row>
     <row r="29">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R29" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="S29" s="45" t="n">
         <v>2.33</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.34</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,10 +3015,10 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.33</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.32</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.32</v>
@@ -3027,7 +3027,7 @@
         <v>2.32</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="31">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.17</v>
-      </c>
-      <c r="S48" s="45" t="n">
-        <v>4.24</v>
       </c>
       <c r="T48" s="45" t="n">
         <v>4.24</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>4.19</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.41</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.43</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.39</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.66</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.64</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.7</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.74</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.69</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,16 +4644,16 @@
         <v>6.27</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.26</v>
       </c>
-      <c r="S52" s="9" t="n">
+      <c r="T52" s="9" t="n">
         <v>6.33</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.37</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.33</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-08-31
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4647,13 +4647,13 @@
         <v>6.27</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.26</v>
       </c>
-      <c r="T52" s="9" t="n">
+      <c r="U52" s="22" t="n">
         <v>6.33</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.37</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-01
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.6099</v>
+        <v>4.8158</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1293,8 +1293,8 @@
           <t>RECPROUSM156N</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
-        <v>46174</v>
+      <c r="C8" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D8" s="45" t="inlineStr">
         <is>
@@ -1307,19 +1307,19 @@
         </is>
       </c>
       <c r="F8" s="45" t="n">
-        <v>0.6</v>
+        <v>0.76</v>
       </c>
       <c r="G8" s="45" t="n">
-        <v>0.32</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H8" s="45" t="n">
-        <v>0.3</v>
+        <v>0.54</v>
       </c>
       <c r="I8" s="45" t="n">
-        <v>0.3</v>
+        <v>0.46</v>
       </c>
       <c r="J8" s="45" t="n">
-        <v>0.18</v>
+        <v>0.54</v>
       </c>
       <c r="K8" s="46" t="n"/>
       <c r="L8" s="28" t="inlineStr">
@@ -1486,8 +1486,8 @@
           <t>JTSJOR</t>
         </is>
       </c>
-      <c r="N10" s="51" t="n">
-        <v>46174</v>
+      <c r="N10" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O10" s="45" t="inlineStr">
         <is>
@@ -1503,13 +1503,13 @@
         <v>4.4</v>
       </c>
       <c r="R10" s="45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="S10" s="45" t="n">
         <v>4.5</v>
       </c>
-      <c r="S10" s="45" t="n">
+      <c r="T10" s="45" t="n">
         <v>4.6</v>
-      </c>
-      <c r="T10" s="45" t="n">
-        <v>4.2</v>
       </c>
       <c r="U10" s="21" t="n">
         <v>4.2</v>
@@ -1565,8 +1565,8 @@
           <t>JTSHIR</t>
         </is>
       </c>
-      <c r="N11" s="51" t="n">
-        <v>46174</v>
+      <c r="N11" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O11" s="45" t="inlineStr">
         <is>
@@ -1579,19 +1579,19 @@
         </is>
       </c>
       <c r="Q11" s="45" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R11" s="45" t="n">
         <v>3.4</v>
-      </c>
-      <c r="R11" s="45" t="n">
-        <v>3.3</v>
       </c>
       <c r="S11" s="45" t="n">
         <v>3.3</v>
       </c>
       <c r="T11" s="45" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="U11" s="21" t="n">
         <v>3.5</v>
-      </c>
-      <c r="U11" s="21" t="n">
-        <v>3.1</v>
       </c>
     </row>
     <row r="12">
@@ -1640,8 +1640,8 @@
           <t>JTSTSR</t>
         </is>
       </c>
-      <c r="N12" s="51" t="n">
-        <v>46174</v>
+      <c r="N12" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="O12" s="45" t="inlineStr">
         <is>
@@ -1654,19 +1654,19 @@
         </is>
       </c>
       <c r="Q12" s="45" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R12" s="45" t="n">
         <v>3.4</v>
       </c>
-      <c r="R12" s="45" t="n">
+      <c r="S12" s="45" t="n">
         <v>3.3</v>
       </c>
-      <c r="S12" s="45" t="n">
+      <c r="T12" s="45" t="n">
         <v>3.2</v>
       </c>
-      <c r="T12" s="45" t="n">
+      <c r="U12" s="21" t="n">
         <v>3.4</v>
-      </c>
-      <c r="U12" s="21" t="n">
-        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S29" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="T29" s="45" t="n">
         <v>2.33</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,10 +3018,10 @@
         <v>2.31</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.33</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.32</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.32</v>
@@ -3530,7 +3530,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N37" s="52" t="n">
+      <c r="N37" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O37" s="45" t="inlineStr">
@@ -3605,7 +3605,7 @@
           <t>CSUSHPINSA</t>
         </is>
       </c>
-      <c r="N38" s="52" t="n">
+      <c r="N38" s="51" t="n">
         <v>46174</v>
       </c>
       <c r="O38" s="45" t="inlineStr">
@@ -3720,7 +3720,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C40" s="52" t="n">
+      <c r="C40" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D40" s="45" t="inlineStr">
@@ -3791,7 +3791,7 @@
           <t>HSN1F</t>
         </is>
       </c>
-      <c r="C41" s="52" t="n">
+      <c r="C41" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D41" s="45" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,16 +4361,16 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="R48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="R48" s="45" t="n">
+      <c r="S48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.17</v>
-      </c>
-      <c r="T48" s="45" t="n">
-        <v>4.24</v>
       </c>
       <c r="U48" s="21" t="n">
         <v>4.24</v>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.35</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.41</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.43</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.66</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.64</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.7</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.74</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,7 +4641,7 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.27</v>
+        <v>6.34</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.27</v>
@@ -4650,10 +4650,10 @@
         <v>6.27</v>
       </c>
       <c r="T52" s="9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="U52" s="22" t="n">
         <v>6.26</v>
-      </c>
-      <c r="U52" s="22" t="n">
-        <v>6.33</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-02
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1526,7 +1526,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C11" s="52" t="n">
+      <c r="C11" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="45" t="inlineStr">
@@ -1601,7 +1601,7 @@
           <t>PCEDGC96</t>
         </is>
       </c>
-      <c r="C12" s="52" t="n">
+      <c r="C12" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="45" t="inlineStr">
@@ -1680,7 +1680,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C13" s="52" t="n">
+      <c r="C13" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -1755,7 +1755,7 @@
           <t>PCENDC96</t>
         </is>
       </c>
-      <c r="C14" s="52" t="n">
+      <c r="C14" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="45" t="inlineStr">
@@ -1834,7 +1834,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C15" s="52" t="n">
+      <c r="C15" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
@@ -1909,7 +1909,7 @@
           <t>PCESC96</t>
         </is>
       </c>
-      <c r="C16" s="52" t="n">
+      <c r="C16" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="45" t="inlineStr">
@@ -2126,7 +2126,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C19" s="52" t="n">
+      <c r="C19" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="45" t="inlineStr">
@@ -2197,7 +2197,7 @@
           <t>DSPIC96</t>
         </is>
       </c>
-      <c r="C20" s="52" t="n">
+      <c r="C20" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="45" t="inlineStr">
@@ -2276,7 +2276,7 @@
           <t>PSAVERT</t>
         </is>
       </c>
-      <c r="C21" s="52" t="n">
+      <c r="C21" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
@@ -2539,7 +2539,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N24" s="52" t="n">
+      <c r="N24" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O24" s="45" t="inlineStr">
@@ -2614,7 +2614,7 @@
           <t>PCEPI</t>
         </is>
       </c>
-      <c r="N25" s="52" t="n">
+      <c r="N25" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O25" s="45" t="inlineStr">
@@ -2693,7 +2693,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N26" s="52" t="n">
+      <c r="N26" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O26" s="45" t="inlineStr">
@@ -2768,7 +2768,7 @@
           <t>PCEPILFE</t>
         </is>
       </c>
-      <c r="N27" s="52" t="n">
+      <c r="N27" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="O27" s="45" t="inlineStr">
@@ -2808,7 +2808,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C28" s="52" t="n">
+      <c r="C28" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="45" t="inlineStr">
@@ -2822,10 +2822,10 @@
         </is>
       </c>
       <c r="F28" s="25" t="n">
-        <v>0.01071642440258236</v>
+        <v>0.01076005348756182</v>
       </c>
       <c r="G28" s="25" t="n">
-        <v>0.005424721874419669</v>
+        <v>0.005802145925317914</v>
       </c>
       <c r="H28" s="25" t="n">
         <v>-0.04004117699494203</v>
@@ -2883,7 +2883,7 @@
           <t>DGORDER</t>
         </is>
       </c>
-      <c r="C29" s="52" t="n">
+      <c r="C29" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -2897,10 +2897,10 @@
         </is>
       </c>
       <c r="F29" s="25" t="n">
-        <v>0.1195187306951081</v>
+        <v>0.1199873280709628</v>
       </c>
       <c r="G29" s="25" t="n">
-        <v>0.07663562793293581</v>
+        <v>0.07703978368044752</v>
       </c>
       <c r="H29" s="25" t="n">
         <v>-0.02972368914374733</v>
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2936,16 +2936,16 @@
         </is>
       </c>
       <c r="Q29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="R29" s="45" t="n">
+      <c r="S29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T29" s="45" t="n">
-        <v>2.33</v>
       </c>
       <c r="U29" s="21" t="n">
         <v>2.33</v>
@@ -2962,7 +2962,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C30" s="52" t="n">
+      <c r="C30" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D30" s="45" t="inlineStr">
@@ -2976,10 +2976,10 @@
         </is>
       </c>
       <c r="F30" s="25" t="n">
-        <v>0.01289555603784764</v>
+        <v>0.01294210214449687</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>0.003129183617765152</v>
+        <v>0.003538609511678281</v>
       </c>
       <c r="H30" s="25" t="n">
         <v>-0.04261964610139124</v>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,16 +3015,16 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
-        <v>2.31</v>
+        <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>2.31</v>
       </c>
       <c r="S30" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="T30" s="45" t="n">
         <v>2.33</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.32</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.32</v>
@@ -3037,7 +3037,7 @@
           <t>ADXDNO</t>
         </is>
       </c>
-      <c r="C31" s="52" t="n">
+      <c r="C31" s="51" t="n">
         <v>46204</v>
       </c>
       <c r="D31" s="45" t="inlineStr">
@@ -3051,10 +3051,10 @@
         </is>
       </c>
       <c r="F31" s="25" t="n">
-        <v>0.0971379650324378</v>
+        <v>0.09763619840916188</v>
       </c>
       <c r="G31" s="25" t="n">
-        <v>0.05712446366627972</v>
+        <v>0.05755592766471823</v>
       </c>
       <c r="H31" s="25" t="n">
         <v>-0.04567753459150702</v>
@@ -3680,8 +3680,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N39" s="51" t="n">
-        <v>46204</v>
+      <c r="N39" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O39" s="45" t="inlineStr">
         <is>
@@ -3694,19 +3694,19 @@
         </is>
       </c>
       <c r="Q39" s="45" t="n">
+        <v>118.8512</v>
+      </c>
+      <c r="R39" s="45" t="n">
         <v>120.597</v>
       </c>
-      <c r="R39" s="53" t="n">
+      <c r="S39" s="53" t="n">
         <v>120.0835</v>
       </c>
-      <c r="S39" s="53" t="n">
+      <c r="T39" s="53" t="n">
         <v>118.7792</v>
       </c>
-      <c r="T39" s="45" t="n">
+      <c r="U39" s="21" t="n">
         <v>119.0363</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>119.9199</v>
       </c>
     </row>
     <row r="40" ht="31.5" customHeight="1">
@@ -3755,8 +3755,8 @@
           <t>TWEXBGSMTH</t>
         </is>
       </c>
-      <c r="N40" s="51" t="n">
-        <v>46204</v>
+      <c r="N40" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O40" s="45" t="inlineStr">
         <is>
@@ -3769,19 +3769,19 @@
         </is>
       </c>
       <c r="Q40" s="38" t="n">
+        <v>-0.01430303593258345</v>
+      </c>
+      <c r="R40" s="38" t="n">
         <v>0.004032046569596641</v>
       </c>
-      <c r="R40" s="54" t="n">
+      <c r="S40" s="54" t="n">
         <v>-0.004232386546914929</v>
       </c>
-      <c r="S40" s="54" t="n">
+      <c r="T40" s="54" t="n">
         <v>-0.0291232297604588</v>
       </c>
-      <c r="T40" s="38" t="n">
+      <c r="U40" s="23" t="n">
         <v>-0.04111399852747133</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>-0.05008673748247425</v>
       </c>
     </row>
     <row r="41">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,16 +4364,16 @@
         <v>4.34</v>
       </c>
       <c r="R48" s="45" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="S48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S48" s="45" t="n">
+      <c r="T48" s="45" t="n">
         <v>4.19</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.17</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.24</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.37</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.35</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.41</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.73</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.66</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.64</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.7</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,10 +4641,10 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="R52" s="9" t="n">
         <v>6.34</v>
-      </c>
-      <c r="R52" s="9" t="n">
-        <v>6.27</v>
       </c>
       <c r="S52" s="9" t="n">
         <v>6.27</v>
@@ -4653,7 +4653,7 @@
         <v>6.27</v>
       </c>
       <c r="U52" s="22" t="n">
-        <v>6.26</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="53" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update dashboards - 2026-09-03
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -1099,8 +1099,8 @@
           <t>ADPMNUSNERSA</t>
         </is>
       </c>
-      <c r="N5" s="51" t="n">
-        <v>46204</v>
+      <c r="N5" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
@@ -1113,19 +1113,19 @@
         </is>
       </c>
       <c r="Q5" s="24" t="n">
-        <v>44000</v>
+        <v>38000</v>
       </c>
       <c r="R5" s="24" t="n">
+        <v>46000</v>
+      </c>
+      <c r="S5" s="24" t="n">
         <v>95000</v>
       </c>
-      <c r="S5" s="24" t="n">
+      <c r="T5" s="24" t="n">
         <v>122000</v>
       </c>
-      <c r="T5" s="24" t="n">
+      <c r="U5" s="26" t="n">
         <v>105000</v>
-      </c>
-      <c r="U5" s="26" t="n">
-        <v>61000</v>
       </c>
     </row>
     <row r="6">
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="F7" s="41" t="n">
-        <v>4.8158</v>
+        <v>4.7487</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>1.54</v>
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="N13" s="52" t="n">
-        <v>46251</v>
+        <v>46258</v>
       </c>
       <c r="O13" s="45" t="inlineStr">
         <is>
@@ -1733,19 +1733,19 @@
         </is>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>203000</v>
+        <v>206000</v>
       </c>
       <c r="R13" s="24" t="n">
+        <v>204000</v>
+      </c>
+      <c r="S13" s="24" t="n">
         <v>207000</v>
       </c>
-      <c r="S13" s="24" t="n">
+      <c r="T13" s="24" t="n">
         <v>212000</v>
       </c>
-      <c r="T13" s="24" t="n">
+      <c r="U13" s="26" t="n">
         <v>200000</v>
-      </c>
-      <c r="U13" s="26" t="n">
-        <v>198000</v>
       </c>
     </row>
     <row r="14">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="N14" s="52" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O14" s="45" t="inlineStr">
         <is>
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="Q14" s="24" t="n">
-        <v>1778000</v>
+        <v>1779000</v>
       </c>
       <c r="R14" s="24" t="n">
+        <v>1771000</v>
+      </c>
+      <c r="S14" s="24" t="n">
         <v>1796000</v>
       </c>
-      <c r="S14" s="24" t="n">
+      <c r="T14" s="24" t="n">
         <v>1781000</v>
       </c>
-      <c r="T14" s="24" t="n">
+      <c r="U14" s="26" t="n">
         <v>1799000</v>
-      </c>
-      <c r="U14" s="26" t="n">
-        <v>1777000</v>
       </c>
     </row>
     <row r="15">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2939,16 +2939,16 @@
         <v>2.33</v>
       </c>
       <c r="R29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="S29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="S29" s="45" t="n">
+      <c r="T29" s="45" t="n">
         <v>2.32</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.35</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.33</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="R30" s="45" t="n">
-        <v>2.31</v>
       </c>
       <c r="S30" s="45" t="n">
         <v>2.31</v>
       </c>
       <c r="T30" s="45" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="U30" s="21" t="n">
         <v>2.33</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="31">
@@ -4142,8 +4142,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C46" s="51" t="n">
-        <v>46174</v>
+      <c r="C46" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D46" s="45" t="inlineStr">
         <is>
@@ -4156,19 +4156,19 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>314728</v>
+        <v>310723</v>
       </c>
       <c r="G46" s="24" t="n">
-        <v>317633</v>
+        <v>317335</v>
       </c>
       <c r="H46" s="24" t="n">
-        <v>328187</v>
+        <v>319979</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>318776</v>
+        <v>329893</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>311803</v>
+        <v>321163</v>
       </c>
       <c r="K46" s="46" t="n"/>
       <c r="L46" s="29" t="inlineStr">
@@ -4229,8 +4229,8 @@
           <t>BOPTEXP</t>
         </is>
       </c>
-      <c r="C47" s="51" t="n">
-        <v>46174</v>
+      <c r="C47" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D47" s="45" t="inlineStr">
         <is>
@@ -4243,19 +4243,19 @@
         </is>
       </c>
       <c r="F47" s="38" t="n">
-        <v>-0.009145775155604108</v>
+        <v>-0.020836025020877</v>
       </c>
       <c r="G47" s="38" t="n">
-        <v>-0.03215849500437251</v>
+        <v>-0.008263042262148468</v>
       </c>
       <c r="H47" s="38" t="n">
-        <v>0.02952229778904303</v>
+        <v>-0.03005216843036984</v>
       </c>
       <c r="I47" s="38" t="n">
-        <v>0.0223634795046872</v>
+        <v>0.02718245875147507</v>
       </c>
       <c r="J47" s="38" t="n">
-        <v>0.04001587693375042</v>
+        <v>0.02402527835524881</v>
       </c>
       <c r="K47" s="46" t="n"/>
       <c r="L47" s="28" t="inlineStr">
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4308,8 +4308,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C48" s="51" t="n">
-        <v>46174</v>
+      <c r="C48" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D48" s="45" t="inlineStr">
         <is>
@@ -4322,19 +4322,19 @@
         </is>
       </c>
       <c r="F48" s="24" t="n">
-        <v>387989</v>
+        <v>399299</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>395280</v>
+        <v>388517</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>382758</v>
+        <v>395731</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>375360</v>
+        <v>382776</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>366783</v>
+        <v>374820</v>
       </c>
       <c r="K48" s="46" t="n"/>
       <c r="L48" s="28" t="inlineStr">
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
-        <v>4.34</v>
+        <v>4.39</v>
       </c>
       <c r="R48" s="45" t="n">
         <v>4.34</v>
       </c>
       <c r="S48" s="45" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="T48" s="45" t="n">
         <v>4.2</v>
       </c>
-      <c r="T48" s="45" t="n">
+      <c r="U48" s="21" t="n">
         <v>4.19</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.17</v>
       </c>
     </row>
     <row r="49">
@@ -4383,8 +4383,8 @@
           <t>BOPTIMP</t>
         </is>
       </c>
-      <c r="C49" s="51" t="n">
-        <v>46174</v>
+      <c r="C49" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D49" s="45" t="inlineStr">
         <is>
@@ -4397,19 +4397,19 @@
         </is>
       </c>
       <c r="F49" s="38" t="n">
-        <v>-0.01844515280307635</v>
+        <v>0.02775168139360695</v>
       </c>
       <c r="G49" s="38" t="n">
-        <v>0.03271518818679175</v>
+        <v>-0.01822955492493639</v>
       </c>
       <c r="H49" s="38" t="n">
-        <v>0.01970907928388743</v>
+        <v>0.03384485965682282</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>0.02338439894978772</v>
+        <v>0.02122618857051384</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>0.03613651194521905</v>
+        <v>0.02374312738475992</v>
       </c>
       <c r="K49" s="46" t="n"/>
       <c r="L49" s="28" t="inlineStr">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.38</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.37</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.35</v>
       </c>
     </row>
     <row r="50">
@@ -4462,8 +4462,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C50" s="51" t="n">
-        <v>46174</v>
+      <c r="C50" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D50" s="45" t="inlineStr">
         <is>
@@ -4476,19 +4476,19 @@
         </is>
       </c>
       <c r="F50" s="24" t="n">
-        <v>28848</v>
+        <v>31016</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>28321</v>
+        <v>30791</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>28342</v>
+        <v>30517</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>29493</v>
+        <v>30177</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>27541</v>
+        <v>32455</v>
       </c>
       <c r="K50" s="46" t="n"/>
       <c r="L50" s="28" t="inlineStr">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="R50" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="R50" s="45" t="n">
+      <c r="S50" s="45" t="n">
         <v>4.73</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.67</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.66</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.64</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4537,8 +4537,8 @@
           <t>BOPSTB</t>
         </is>
       </c>
-      <c r="C51" s="51" t="n">
-        <v>46174</v>
+      <c r="C51" s="52" t="n">
+        <v>46204</v>
       </c>
       <c r="D51" s="45" t="inlineStr">
         <is>
@@ -4551,19 +4551,19 @@
         </is>
       </c>
       <c r="F51" s="38" t="n">
-        <v>0.01860809999646906</v>
+        <v>0.007307330063979656</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>-0.0007409498271117032</v>
+        <v>0.008978602090637944</v>
       </c>
       <c r="H51" s="38" t="n">
-        <v>-0.03902620960905978</v>
+        <v>0.01126685886602385</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>0.07087614828800692</v>
+        <v>-0.07018949314435374</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>-0.01909035865655162</v>
+        <v>0.08060864353732433</v>
       </c>
       <c r="K51" s="46" t="n"/>
       <c r="L51" s="28" t="inlineStr">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="N51" s="52" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="O51" s="45" t="inlineStr">
         <is>
@@ -4590,19 +4590,19 @@
         </is>
       </c>
       <c r="Q51" s="45" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="R51" s="45" t="n">
         <v>6.66</v>
       </c>
-      <c r="R51" s="45" t="n">
+      <c r="S51" s="45" t="n">
         <v>6.65</v>
       </c>
-      <c r="S51" s="45" t="n">
+      <c r="T51" s="45" t="n">
         <v>6.67</v>
       </c>
-      <c r="T51" s="45" t="n">
+      <c r="U51" s="21" t="n">
         <v>6.69</v>
-      </c>
-      <c r="U51" s="21" t="n">
-        <v>6.66</v>
       </c>
     </row>
     <row r="52" ht="16.15" customHeight="1" thickBot="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4644,10 +4644,10 @@
         <v>6.37</v>
       </c>
       <c r="R52" s="9" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="S52" s="9" t="n">
         <v>6.34</v>
-      </c>
-      <c r="S52" s="9" t="n">
-        <v>6.27</v>
       </c>
       <c r="T52" s="9" t="n">
         <v>6.27</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-09-04
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -949,8 +949,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N3" s="51" t="n">
-        <v>46204</v>
+      <c r="N3" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O3" s="45" t="inlineStr">
         <is>
@@ -963,19 +963,19 @@
         </is>
       </c>
       <c r="Q3" s="24" t="n">
-        <v>-23</v>
+        <v>162</v>
       </c>
       <c r="R3" s="24" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" s="24" t="n">
+        <v>31</v>
+      </c>
+      <c r="T3" s="24" t="n">
         <v>63</v>
       </c>
-      <c r="T3" s="24" t="n">
+      <c r="U3" s="26" t="n">
         <v>148</v>
-      </c>
-      <c r="U3" s="26" t="n">
-        <v>214</v>
       </c>
     </row>
     <row r="4">
@@ -1020,8 +1020,8 @@
           <t>PAYEMS</t>
         </is>
       </c>
-      <c r="N4" s="51" t="n">
-        <v>46204</v>
+      <c r="N4" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O4" s="45" t="inlineStr">
         <is>
@@ -1034,19 +1034,19 @@
         </is>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>0.001993162695058723</v>
+        <v>0.003805088596092685</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>0.002542939714029707</v>
+        <v>0.00234007392362907</v>
       </c>
       <c r="S4" s="38" t="n">
+        <v>0.00261234997917692</v>
+      </c>
+      <c r="T4" s="38" t="n">
         <v>0.002290249719239359</v>
       </c>
-      <c r="T4" s="38" t="n">
+      <c r="U4" s="23" t="n">
         <v>0.001974950310754961</v>
-      </c>
-      <c r="U4" s="23" t="n">
-        <v>0.001723735138309224</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -1174,8 +1174,8 @@
           <t>UNRATE</t>
         </is>
       </c>
-      <c r="N6" s="51" t="n">
-        <v>46204</v>
+      <c r="N6" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O6" s="45" t="inlineStr">
         <is>
@@ -1191,10 +1191,10 @@
         <v>4.1</v>
       </c>
       <c r="R6" s="45" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="S6" s="45" t="n">
         <v>4.2</v>
-      </c>
-      <c r="S6" s="45" t="n">
-        <v>4.3</v>
       </c>
       <c r="T6" s="45" t="n">
         <v>4.3</v>
@@ -1253,8 +1253,8 @@
           <t>U6RATE</t>
         </is>
       </c>
-      <c r="N7" s="51" t="n">
-        <v>46204</v>
+      <c r="N7" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O7" s="45" t="inlineStr">
         <is>
@@ -1267,19 +1267,19 @@
         </is>
       </c>
       <c r="Q7" s="45" t="n">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
       <c r="R7" s="45" t="n">
         <v>7.9</v>
       </c>
       <c r="S7" s="45" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="T7" s="45" t="n">
         <v>8.1</v>
       </c>
-      <c r="T7" s="45" t="n">
+      <c r="U7" s="21" t="n">
         <v>8.199999999999999</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
@@ -1332,8 +1332,8 @@
           <t>CIVPART</t>
         </is>
       </c>
-      <c r="N8" s="51" t="n">
-        <v>46204</v>
+      <c r="N8" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O8" s="45" t="inlineStr">
         <is>
@@ -1346,19 +1346,19 @@
         </is>
       </c>
       <c r="Q8" s="45" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="R8" s="45" t="n">
         <v>61.4</v>
       </c>
-      <c r="R8" s="45" t="n">
+      <c r="S8" s="45" t="n">
         <v>61.5</v>
-      </c>
-      <c r="S8" s="45" t="n">
-        <v>61.8</v>
       </c>
       <c r="T8" s="45" t="n">
         <v>61.8</v>
       </c>
       <c r="U8" s="21" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="9">
@@ -1411,8 +1411,8 @@
           <t>EMRATIO</t>
         </is>
       </c>
-      <c r="N9" s="51" t="n">
-        <v>46204</v>
+      <c r="N9" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O9" s="45" t="inlineStr">
         <is>
@@ -1425,19 +1425,19 @@
         </is>
       </c>
       <c r="Q9" s="45" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="R9" s="45" t="n">
         <v>58.9</v>
       </c>
-      <c r="R9" s="45" t="n">
+      <c r="S9" s="45" t="n">
         <v>59</v>
       </c>
-      <c r="S9" s="45" t="n">
+      <c r="T9" s="45" t="n">
         <v>59.2</v>
       </c>
-      <c r="T9" s="45" t="n">
+      <c r="U9" s="21" t="n">
         <v>59.1</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>59.2</v>
       </c>
     </row>
     <row r="10">
@@ -1873,8 +1873,8 @@
           <t>AWHAETP</t>
         </is>
       </c>
-      <c r="N15" s="51" t="n">
-        <v>46204</v>
+      <c r="N15" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="Q15" s="24" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="R15" s="24" t="n">
         <v>34.3</v>
@@ -1899,7 +1899,7 @@
         <v>34.3</v>
       </c>
       <c r="U15" s="26" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="16">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2942,13 +2942,13 @@
         <v>2.33</v>
       </c>
       <c r="S29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="T29" s="45" t="n">
         <v>2.31</v>
       </c>
-      <c r="T29" s="45" t="n">
+      <c r="U29" s="21" t="n">
         <v>2.32</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.35</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3015,19 +3015,19 @@
         </is>
       </c>
       <c r="Q30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="R30" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="R30" s="45" t="n">
+      <c r="S30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="S30" s="45" t="n">
-        <v>2.31</v>
       </c>
       <c r="T30" s="45" t="n">
         <v>2.31</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>2.33</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="31">
@@ -3226,8 +3226,8 @@
           <t>CES0500000003</t>
         </is>
       </c>
-      <c r="N33" s="51" t="n">
-        <v>46204</v>
+      <c r="N33" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="O33" s="45" t="inlineStr">
         <is>
@@ -3240,19 +3240,19 @@
         </is>
       </c>
       <c r="Q33" s="38" t="n">
-        <v>0.0005319148936169249</v>
+        <v>0.002656042496679945</v>
       </c>
       <c r="R33" s="38" t="n">
-        <v>0.002934115764203771</v>
+        <v>0.001596169193934349</v>
       </c>
       <c r="S33" s="38" t="n">
+        <v>0.002667377967457973</v>
+      </c>
+      <c r="T33" s="38" t="n">
         <v>0.002138465650895593</v>
       </c>
-      <c r="T33" s="38" t="n">
+      <c r="U33" s="23" t="n">
         <v>0.001606425702811221</v>
-      </c>
-      <c r="U33" s="23" t="n">
-        <v>0.002146498524282281</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
@@ -3315,10 +3315,10 @@
         </is>
       </c>
       <c r="Q34" s="38" t="n">
-        <v>-0.005283345196001861</v>
+        <v>-0.004490110224068822</v>
       </c>
       <c r="R34" s="38" t="n">
-        <v>-0.00295640652354665</v>
+        <v>-0.003221577692024325</v>
       </c>
       <c r="S34" s="38" t="n">
         <v>-0.007455850803781246</v>
@@ -3394,10 +3394,10 @@
         </is>
       </c>
       <c r="Q35" s="38" t="n">
-        <v>-0.001025966015042346</v>
+        <v>3.663118525487619e-05</v>
       </c>
       <c r="R35" s="38" t="n">
-        <v>0.00386492016820239</v>
+        <v>0.003597934817094028</v>
       </c>
       <c r="S35" s="38" t="n">
         <v>-0.002659880805601422</v>
@@ -3469,10 +3469,10 @@
         </is>
       </c>
       <c r="Q36" s="38" t="n">
-        <v>-0.005283345196001861</v>
+        <v>-0.004490110224068822</v>
       </c>
       <c r="R36" s="38" t="n">
-        <v>-0.00295640652354665</v>
+        <v>-0.003221577692024325</v>
       </c>
       <c r="S36" s="38" t="n">
         <v>-0.007455850803781246</v>
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4364,16 +4364,16 @@
         <v>4.39</v>
       </c>
       <c r="R48" s="45" t="n">
-        <v>4.34</v>
+        <v>4.39</v>
       </c>
       <c r="S48" s="45" t="n">
         <v>4.34</v>
       </c>
       <c r="T48" s="45" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="U48" s="21" t="n">
         <v>4.2</v>
-      </c>
-      <c r="U48" s="21" t="n">
-        <v>4.19</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.48</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.38</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.37</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4518,16 +4518,16 @@
         <v>4.79</v>
       </c>
       <c r="R50" s="45" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="S50" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="S50" s="45" t="n">
+      <c r="T50" s="45" t="n">
         <v>4.73</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.67</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.66</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="N52" s="55" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O52" s="9" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         </is>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>6.37</v>
+        <v>6.34</v>
       </c>
       <c r="R52" s="9" t="n">
         <v>6.37</v>
       </c>
       <c r="S52" s="9" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="T52" s="9" t="n">
         <v>6.34</v>
-      </c>
-      <c r="T52" s="9" t="n">
-        <v>6.27</v>
       </c>
       <c r="U52" s="22" t="n">
         <v>6.27</v>

</xml_diff>

<commit_message>
Update dashboards - 2026-09-05
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template-UPDATE.xlsx
@@ -2351,8 +2351,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C22" s="51" t="n">
-        <v>46204</v>
+      <c r="C22" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
         <is>
@@ -2365,19 +2365,19 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
+        <v>17.19</v>
+      </c>
+      <c r="G22" s="24" t="n">
         <v>16.757</v>
       </c>
-      <c r="G22" s="24" t="n">
-        <v>17.043</v>
-      </c>
       <c r="H22" s="24" t="n">
-        <v>16.748</v>
+        <v>17.221</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>16.642</v>
+        <v>16.744</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>16.66</v>
+        <v>16.636</v>
       </c>
       <c r="K22" s="46" t="n"/>
       <c r="L22" s="28" t="inlineStr">
@@ -2426,8 +2426,8 @@
           <t>TOTALSA</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
-        <v>46204</v>
+      <c r="C23" s="52" t="n">
+        <v>46235</v>
       </c>
       <c r="D23" s="45" t="inlineStr">
         <is>
@@ -2440,19 +2440,19 @@
         </is>
       </c>
       <c r="F23" s="25" t="n">
+        <v>0.01715976331360963</v>
+      </c>
+      <c r="G23" s="25" t="n">
         <v>-0.01417813860454169</v>
       </c>
-      <c r="G23" s="25" t="n">
-        <v>0.04673872988576337</v>
-      </c>
       <c r="H23" s="25" t="n">
-        <v>0.04394439942654129</v>
+        <v>0.05767104778282767</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>-0.05351760222942609</v>
+        <v>0.04369506950071686</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>-0.09209809264305184</v>
+        <v>-0.05385884092589429</v>
       </c>
       <c r="K23" s="46" t="n"/>
       <c r="M23" s="15" t="inlineStr">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="N29" s="52" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
@@ -2945,10 +2945,10 @@
         <v>2.33</v>
       </c>
       <c r="T29" s="45" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U29" s="21" t="n">
         <v>2.31</v>
-      </c>
-      <c r="U29" s="21" t="n">
-        <v>2.32</v>
       </c>
     </row>
     <row r="30">
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="N30" s="52" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
@@ -3018,13 +3018,13 @@
         <v>2.35</v>
       </c>
       <c r="R30" s="45" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="S30" s="45" t="n">
         <v>2.34</v>
       </c>
-      <c r="S30" s="45" t="n">
+      <c r="T30" s="45" t="n">
         <v>2.35</v>
-      </c>
-      <c r="T30" s="45" t="n">
-        <v>2.31</v>
       </c>
       <c r="U30" s="21" t="n">
         <v>2.31</v>
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="N47" s="52" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O47" s="45" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="N48" s="52" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O48" s="45" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
         </is>
       </c>
       <c r="Q48" s="45" t="n">
-        <v>4.39</v>
+        <v>4.34</v>
       </c>
       <c r="R48" s="45" t="n">
         <v>4.39</v>
       </c>
       <c r="S48" s="45" t="n">
-        <v>4.34</v>
+        <v>4.39</v>
       </c>
       <c r="T48" s="45" t="n">
         <v>4.34</v>
       </c>
       <c r="U48" s="21" t="n">
-        <v>4.2</v>
+        <v>4.34</v>
       </c>
     </row>
     <row r="49">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="N49" s="52" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O49" s="45" t="inlineStr">
         <is>
@@ -4436,19 +4436,19 @@
         </is>
       </c>
       <c r="Q49" s="45" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="R49" s="45" t="n">
         <v>4.54</v>
       </c>
-      <c r="R49" s="45" t="n">
+      <c r="S49" s="45" t="n">
         <v>4.55</v>
       </c>
-      <c r="S49" s="45" t="n">
+      <c r="T49" s="45" t="n">
         <v>4.49</v>
       </c>
-      <c r="T49" s="45" t="n">
+      <c r="U49" s="21" t="n">
         <v>4.48</v>
-      </c>
-      <c r="U49" s="21" t="n">
-        <v>4.38</v>
       </c>
     </row>
     <row r="50">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="N50" s="52" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="O50" s="45" t="inlineStr">
         <is>
@@ -4515,19 +4515,19 @@
         </is>
       </c>
       <c r="Q50" s="45" t="n">
-        <v>4.79</v>
+        <v>4.77</v>
       </c>
       <c r="R50" s="45" t="n">
         <v>4.79</v>
       </c>
       <c r="S50" s="45" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="T50" s="45" t="n">
         <v>4.75</v>
       </c>
-      <c r="T50" s="45" t="n">
+      <c r="U50" s="21" t="n">
         <v>4.73</v>
-      </c>
-      <c r="U50" s="21" t="n">
-        <v>4.67</v>
       </c>
     </row>
     <row r="51" ht="31.5" customHeight="1">

</xml_diff>